<commit_message>
docs:update usage note for Distribution.rights
</commit_message>
<xml_diff>
--- a/Documents/Metadata_CoreGenericHealth_v2.xlsx
+++ b/Documents/Metadata_CoreGenericHealth_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anakonrad/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{424B36F4-CD4D-ED4C-B2CE-D33BD863D11C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{616AA07E-76D5-7B4D-A220-EE7A7862A61B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="680" windowWidth="30240" windowHeight="17380" firstSheet="2" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17380" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="14" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1888" uniqueCount="691">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1888" uniqueCount="692">
   <si>
     <t>Property label</t>
   </si>
@@ -1841,30 +1841,6 @@
   </si>
   <si>
     <t>fill in in 'Periof of Time' tab</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">A statement that concerns all rights not addressed in fields License or Access rights. In case of not open data (as specified in the dct:licence property), further agreements regarding data reuse (eg. Data Transfer Agreement, DTA,) should be stated in this property.
-The rights statement should be a free-text statement placed at an web-accessible location such that the value of this property is the IRI pointing to that statement.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Display"/>
-      </rPr>
-      <t xml:space="preserve">Current status: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Display"/>
-      </rPr>
-      <t>This recommendation on how to state data transfer/reuse conditions will be pilotted in 2025.</t>
-    </r>
   </si>
   <si>
     <t>resource:rights</t>
@@ -2765,12 +2741,38 @@
   <si>
     <t>This property allows free text description of the rights.</t>
   </si>
+  <si>
+    <t>dct:RightsStatement</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">A statement that concerns all rights not addressed in fields license or access rights. In case of not open data (as specified in the </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Display"/>
+      </rPr>
+      <t>dct:licence</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Display"/>
+      </rPr>
+      <t xml:space="preserve"> property), further agreements regarding data reuse (e.g., Data Transfer Agreement, DTA) should be stated in this property. 
+The rights statement can be a document placed at a web-accessible location, or a free-text statement. See RightsStatement class for further information.</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="56" x14ac:knownFonts="1">
+  <fonts count="57" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3127,6 +3129,12 @@
       <color rgb="FF000000"/>
       <name val="Aptos Display"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Display"/>
     </font>
   </fonts>
   <fills count="14">
@@ -7801,33 +7809,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>558</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>559</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="227" t="s">
         <v>560</v>
       </c>
-      <c r="N1" s="227" t="s">
+      <c r="O1" s="233" t="s">
         <v>561</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>562</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="80" x14ac:dyDescent="0.2">
       <c r="A2" s="196" t="s">
+        <v>562</v>
+      </c>
+      <c r="B2" s="45" t="s">
         <v>563</v>
       </c>
-      <c r="B2" s="45" t="s">
+      <c r="C2" s="76" t="s">
         <v>564</v>
-      </c>
-      <c r="C2" s="76" t="s">
-        <v>565</v>
       </c>
       <c r="D2" s="196" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="197" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="F2" s="198" t="s">
         <v>35</v>
@@ -7836,7 +7844,7 @@
         <v>58</v>
       </c>
       <c r="H2" s="198" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="I2" s="160" t="s">
         <v>20</v>
@@ -7851,13 +7859,13 @@
     </row>
     <row r="3" spans="1:15" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" s="68" t="s">
+        <v>567</v>
+      </c>
+      <c r="B3" s="61" t="s">
         <v>568</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="C3" s="77" t="s">
         <v>569</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>570</v>
       </c>
       <c r="D3" s="68" t="s">
         <v>16</v>
@@ -7996,36 +8004,36 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>570</v>
+      </c>
+      <c r="M1" s="220" t="s">
         <v>571</v>
       </c>
-      <c r="M1" s="220" t="s">
+      <c r="N1" s="226" t="s">
         <v>572</v>
       </c>
-      <c r="N1" s="226" t="s">
+      <c r="O1" s="230" t="s">
         <v>573</v>
       </c>
-      <c r="O1" s="230" t="s">
+      <c r="P1" s="227" t="s">
         <v>574</v>
       </c>
-      <c r="P1" s="227" t="s">
+      <c r="Q1" s="231" t="s">
         <v>575</v>
       </c>
-      <c r="Q1" s="231" t="s">
+      <c r="R1" s="233" t="s">
         <v>576</v>
-      </c>
-      <c r="R1" s="233" t="s">
-        <v>577</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="58" t="s">
+        <v>577</v>
+      </c>
+      <c r="B2" s="44" t="s">
         <v>578</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="C2" s="76" t="s">
         <v>579</v>
-      </c>
-      <c r="C2" s="76" t="s">
-        <v>580</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
@@ -8053,13 +8061,13 @@
     </row>
     <row r="3" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="48" t="s">
+        <v>580</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>581</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>582</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>583</v>
       </c>
       <c r="D3" s="48" t="s">
         <v>16</v>
@@ -8721,33 +8729,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>583</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>584</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="227" t="s">
         <v>585</v>
       </c>
-      <c r="N1" s="227" t="s">
+      <c r="O1" s="233" t="s">
         <v>586</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>587</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="48" x14ac:dyDescent="0.2">
       <c r="A2" s="84" t="s">
+        <v>587</v>
+      </c>
+      <c r="B2" s="44" t="s">
         <v>588</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="C2" s="58" t="s">
         <v>589</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>590</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>17</v>
@@ -8777,19 +8785,19 @@
     </row>
     <row r="3" spans="1:15" ht="144" x14ac:dyDescent="0.2">
       <c r="A3" s="48" t="s">
+        <v>591</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>592</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>593</v>
       </c>
-      <c r="C3" s="77" t="s">
+      <c r="D3" s="234" t="s">
         <v>594</v>
       </c>
-      <c r="D3" s="234" t="s">
+      <c r="E3" s="50" t="s">
         <v>595</v>
-      </c>
-      <c r="E3" s="50" t="s">
-        <v>596</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>17</v>
@@ -8915,33 +8923,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="218" t="s">
+        <v>596</v>
+      </c>
+      <c r="M1" s="229" t="s">
         <v>597</v>
       </c>
-      <c r="M1" s="229" t="s">
+      <c r="N1" s="228" t="s">
         <v>598</v>
       </c>
-      <c r="N1" s="228" t="s">
+      <c r="O1" s="233" t="s">
         <v>599</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>600</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="160" x14ac:dyDescent="0.2">
       <c r="A2" s="84" t="s">
+        <v>600</v>
+      </c>
+      <c r="B2" s="44" t="s">
+        <v>592</v>
+      </c>
+      <c r="C2" s="58" t="s">
+        <v>593</v>
+      </c>
+      <c r="D2" s="59" t="s">
         <v>601</v>
       </c>
-      <c r="B2" s="44" t="s">
-        <v>593</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>594</v>
-      </c>
-      <c r="D2" s="59" t="s">
+      <c r="E2" s="59" t="s">
         <v>602</v>
-      </c>
-      <c r="E2" s="59" t="s">
-        <v>603</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>35</v>
@@ -8962,19 +8970,19 @@
     </row>
     <row r="3" spans="1:15" ht="48" x14ac:dyDescent="0.2">
       <c r="A3" s="48" t="s">
+        <v>603</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>604</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>605</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>606</v>
       </c>
       <c r="D3" s="116" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>35</v>
@@ -9099,33 +9107,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="218" t="s">
+        <v>678</v>
+      </c>
+      <c r="M1" s="229" t="s">
+        <v>688</v>
+      </c>
+      <c r="N1" s="228" t="s">
         <v>679</v>
       </c>
-      <c r="M1" s="229" t="s">
-        <v>689</v>
-      </c>
-      <c r="N1" s="228" t="s">
+      <c r="O1" s="233" t="s">
         <v>680</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>681</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="288" x14ac:dyDescent="0.2">
       <c r="A2" s="84" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="C2" s="58" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="D2" s="59" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="F2" s="51" t="s">
         <v>17</v>
@@ -9144,19 +9152,19 @@
     </row>
     <row r="3" spans="1:15" ht="192" x14ac:dyDescent="0.2">
       <c r="A3" s="48" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="B3" s="49" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="C3" s="77" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="D3" s="116" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>17</v>
@@ -9314,33 +9322,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>607</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>608</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="227" t="s">
         <v>609</v>
       </c>
-      <c r="N1" s="227" t="s">
+      <c r="O1" s="233" t="s">
         <v>610</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>611</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="112" x14ac:dyDescent="0.2">
       <c r="A2" s="84" t="s">
+        <v>611</v>
+      </c>
+      <c r="B2" s="44" t="s">
         <v>612</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="C2" s="58" t="s">
         <v>613</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>614</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>17</v>
@@ -9361,19 +9369,19 @@
     </row>
     <row r="3" spans="1:15" ht="64" x14ac:dyDescent="0.2">
       <c r="A3" s="48" t="s">
+        <v>615</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>616</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>617</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>618</v>
       </c>
       <c r="D3" s="116" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>17</v>
@@ -9477,7 +9485,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="56" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="E1" s="56" t="s">
         <v>4</v>
@@ -9500,13 +9508,13 @@
     </row>
     <row r="2" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="63" t="s">
+        <v>620</v>
+      </c>
+      <c r="B2" s="53" t="s">
         <v>621</v>
       </c>
-      <c r="B2" s="53" t="s">
+      <c r="C2" s="44" t="s">
         <v>622</v>
-      </c>
-      <c r="C2" s="44" t="s">
-        <v>623</v>
       </c>
       <c r="D2" s="43" t="s">
         <v>16</v>
@@ -9514,7 +9522,7 @@
       <c r="E2" s="45"/>
       <c r="F2" s="64"/>
       <c r="G2" s="63" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="H2" s="65" t="s">
         <v>81</v>
@@ -9528,13 +9536,13 @@
     </row>
     <row r="3" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A3" s="67" t="s">
+        <v>624</v>
+      </c>
+      <c r="B3" s="50" t="s">
         <v>625</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="C3" s="49" t="s">
         <v>626</v>
-      </c>
-      <c r="C3" s="49" t="s">
-        <v>627</v>
       </c>
       <c r="D3" s="48" t="s">
         <v>16</v>
@@ -9542,10 +9550,10 @@
       <c r="E3" s="50"/>
       <c r="F3" s="68"/>
       <c r="G3" s="69" t="s">
+        <v>627</v>
+      </c>
+      <c r="H3" s="48" t="s">
         <v>628</v>
-      </c>
-      <c r="H3" s="48" t="s">
-        <v>629</v>
       </c>
       <c r="I3" s="69" t="s">
         <v>20</v>
@@ -9556,13 +9564,13 @@
     </row>
     <row r="4" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A4" s="63" t="s">
+        <v>629</v>
+      </c>
+      <c r="B4" s="53" t="s">
         <v>630</v>
       </c>
-      <c r="B4" s="53" t="s">
+      <c r="C4" s="44" t="s">
         <v>631</v>
-      </c>
-      <c r="C4" s="44" t="s">
-        <v>632</v>
       </c>
       <c r="D4" s="43" t="s">
         <v>16</v>
@@ -9570,10 +9578,10 @@
       <c r="E4" s="53"/>
       <c r="F4" s="64"/>
       <c r="G4" s="63" t="s">
+        <v>632</v>
+      </c>
+      <c r="H4" s="65" t="s">
         <v>633</v>
-      </c>
-      <c r="H4" s="65" t="s">
-        <v>634</v>
       </c>
       <c r="I4" s="66" t="s">
         <v>20</v>
@@ -9584,26 +9592,26 @@
     </row>
     <row r="5" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A5" s="67" t="s">
+        <v>634</v>
+      </c>
+      <c r="B5" s="50" t="s">
         <v>635</v>
       </c>
-      <c r="B5" s="50" t="s">
+      <c r="C5" s="49" t="s">
         <v>636</v>
-      </c>
-      <c r="C5" s="49" t="s">
-        <v>637</v>
       </c>
       <c r="D5" s="48" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="49" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="F5" s="68"/>
       <c r="G5" s="67" t="s">
+        <v>638</v>
+      </c>
+      <c r="H5" s="48" t="s">
         <v>639</v>
-      </c>
-      <c r="H5" s="48" t="s">
-        <v>640</v>
       </c>
       <c r="I5" s="69" t="s">
         <v>20</v>
@@ -9614,13 +9622,13 @@
     </row>
     <row r="6" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="63" t="s">
+        <v>640</v>
+      </c>
+      <c r="B6" s="73" t="s">
         <v>641</v>
       </c>
-      <c r="B6" s="73" t="s">
+      <c r="C6" s="44" t="s">
         <v>642</v>
-      </c>
-      <c r="C6" s="44" t="s">
-        <v>643</v>
       </c>
       <c r="D6" s="43" t="s">
         <v>16</v>
@@ -9631,7 +9639,7 @@
         <v>99</v>
       </c>
       <c r="H6" s="65" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="I6" s="66" t="s">
         <v>20</v>
@@ -9642,13 +9650,13 @@
     </row>
     <row r="7" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="67" t="s">
+        <v>643</v>
+      </c>
+      <c r="B7" s="50" t="s">
         <v>644</v>
       </c>
-      <c r="B7" s="50" t="s">
+      <c r="C7" s="49" t="s">
         <v>645</v>
-      </c>
-      <c r="C7" s="49" t="s">
-        <v>646</v>
       </c>
       <c r="D7" s="48" t="s">
         <v>16</v>
@@ -9670,23 +9678,23 @@
     </row>
     <row r="8" spans="1:10" ht="80" x14ac:dyDescent="0.2">
       <c r="A8" s="63" t="s">
+        <v>646</v>
+      </c>
+      <c r="B8" s="53" t="s">
         <v>647</v>
       </c>
-      <c r="B8" s="53" t="s">
+      <c r="C8" s="44" t="s">
         <v>648</v>
-      </c>
-      <c r="C8" s="44" t="s">
-        <v>649</v>
       </c>
       <c r="D8" s="43" t="s">
         <v>16</v>
       </c>
       <c r="E8" s="71" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="F8" s="47"/>
       <c r="G8" s="63" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="H8" s="65">
         <v>1</v>
@@ -9700,13 +9708,13 @@
     </row>
     <row r="9" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="67" t="s">
+        <v>651</v>
+      </c>
+      <c r="B9" s="50" t="s">
         <v>652</v>
       </c>
-      <c r="B9" s="50" t="s">
+      <c r="C9" s="49" t="s">
         <v>653</v>
-      </c>
-      <c r="C9" s="49" t="s">
-        <v>654</v>
       </c>
       <c r="D9" s="48" t="s">
         <v>16</v>
@@ -9714,7 +9722,7 @@
       <c r="E9" s="50"/>
       <c r="F9" s="68"/>
       <c r="G9" s="69" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
       <c r="H9" s="48" t="s">
         <v>81</v>
@@ -9728,23 +9736,23 @@
     </row>
     <row r="10" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="63" t="s">
+        <v>655</v>
+      </c>
+      <c r="B10" s="72" t="s">
         <v>656</v>
       </c>
-      <c r="B10" s="72" t="s">
+      <c r="C10" s="44" t="s">
         <v>657</v>
-      </c>
-      <c r="C10" s="44" t="s">
-        <v>658</v>
       </c>
       <c r="D10" s="43" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="72" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="F10" s="64"/>
       <c r="G10" s="63" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="H10" s="65" t="s">
         <v>19</v>
@@ -10209,36 +10217,36 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>659</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>660</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="233" t="s">
         <v>661</v>
-      </c>
-      <c r="N1" s="233" t="s">
-        <v>662</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="64" x14ac:dyDescent="0.2">
       <c r="A2" s="44" t="s">
+        <v>662</v>
+      </c>
+      <c r="B2" s="57" t="s">
         <v>663</v>
       </c>
-      <c r="B2" s="57" t="s">
+      <c r="C2" s="58" t="s">
         <v>664</v>
       </c>
-      <c r="C2" s="58" t="s">
+      <c r="D2" s="78" t="s">
         <v>665</v>
       </c>
-      <c r="D2" s="78" t="s">
+      <c r="E2" s="197" t="s">
         <v>666</v>
-      </c>
-      <c r="E2" s="197" t="s">
-        <v>667</v>
       </c>
       <c r="F2" s="46" t="s">
         <v>35</v>
       </c>
       <c r="G2" s="204" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="H2" s="47">
         <v>1</v>
@@ -10252,13 +10260,13 @@
     </row>
     <row r="3" spans="1:14" ht="71.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="49" t="s">
+        <v>668</v>
+      </c>
+      <c r="B3" s="61" t="s">
         <v>669</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="C3" s="48" t="s">
         <v>670</v>
-      </c>
-      <c r="C3" s="48" t="s">
-        <v>671</v>
       </c>
       <c r="D3" s="50" t="s">
         <v>16</v>
@@ -10268,7 +10276,7 @@
         <v>35</v>
       </c>
       <c r="G3" s="51" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="H3" s="52">
         <v>1</v>
@@ -12312,8 +12320,8 @@
       <c r="F2" s="124" t="s">
         <v>35</v>
       </c>
-      <c r="G2" s="124" t="s">
-        <v>115</v>
+      <c r="G2" s="128" t="s">
+        <v>690</v>
       </c>
       <c r="H2" s="124">
         <v>1</v>
@@ -14437,7 +14445,7 @@
         <v>16</v>
       </c>
       <c r="E3" s="184" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="F3" s="163" t="s">
         <v>35</v>
@@ -15507,7 +15515,7 @@
         <v>16</v>
       </c>
       <c r="E3" s="184" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="F3" s="163" t="s">
         <v>35</v>
@@ -17066,7 +17074,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="144" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" ht="112" x14ac:dyDescent="0.2">
       <c r="A20" s="121" t="s">
         <v>111</v>
       </c>
@@ -17080,13 +17088,13 @@
         <v>16</v>
       </c>
       <c r="E20" s="79" t="s">
-        <v>495</v>
+        <v>691</v>
       </c>
       <c r="F20" s="190" t="s">
         <v>35</v>
       </c>
-      <c r="G20" s="124" t="s">
-        <v>115</v>
+      <c r="G20" s="128" t="s">
+        <v>690</v>
       </c>
       <c r="H20" s="133">
         <v>1</v>
@@ -17098,7 +17106,7 @@
         <v>29</v>
       </c>
       <c r="K20" s="99" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="L20" s="107"/>
       <c r="M20" s="107"/>
@@ -17114,10 +17122,10 @@
         <v>327</v>
       </c>
       <c r="D21" s="154" t="s">
+        <v>496</v>
+      </c>
+      <c r="E21" s="81" t="s">
         <v>497</v>
-      </c>
-      <c r="E21" s="81" t="s">
-        <v>498</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>17</v>
@@ -17135,7 +17143,7 @@
         <v>29</v>
       </c>
       <c r="K21" s="98" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="L21" s="129"/>
       <c r="M21" s="129"/>
@@ -17154,7 +17162,7 @@
         <v>16</v>
       </c>
       <c r="E22" s="132" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>17</v>
@@ -17189,7 +17197,7 @@
         <v>16</v>
       </c>
       <c r="E23" s="126" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>17</v>
@@ -17207,7 +17215,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="98" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="L23" s="129"/>
       <c r="M23" s="129"/>
@@ -17689,7 +17697,7 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="16" x14ac:dyDescent="0.2">
@@ -17706,7 +17714,7 @@
         <v>16</v>
       </c>
       <c r="E2" s="74" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>17</v>
@@ -17724,7 +17732,7 @@
         <v>29</v>
       </c>
       <c r="K2" s="98" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="L2" s="129"/>
     </row>
@@ -17760,7 +17768,7 @@
         <v>29</v>
       </c>
       <c r="K3" s="98" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="L3" s="107" t="s">
         <v>39</v>
@@ -17780,7 +17788,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="126" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="F4" s="127" t="s">
         <v>35</v>
@@ -17798,7 +17806,7 @@
         <v>29</v>
       </c>
       <c r="K4" s="99" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="L4" s="129"/>
     </row>
@@ -17816,7 +17824,7 @@
         <v>198</v>
       </c>
       <c r="E5" s="135" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="F5" s="124" t="s">
         <v>17</v>
@@ -17868,7 +17876,7 @@
         <v>66</v>
       </c>
       <c r="K6" s="247" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="L6" s="246"/>
     </row>
@@ -17950,7 +17958,7 @@
         <v>16</v>
       </c>
       <c r="E11" s="132" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="F11" s="124" t="s">
         <v>17</v>
@@ -17968,7 +17976,7 @@
         <v>29</v>
       </c>
       <c r="K11" s="99" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="L11" s="107"/>
     </row>
@@ -17986,7 +17994,7 @@
         <v>16</v>
       </c>
       <c r="E12" s="126" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="F12" s="124" t="s">
         <v>17</v>
@@ -18004,7 +18012,7 @@
         <v>29</v>
       </c>
       <c r="K12" s="98" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="L12" s="129" t="s">
         <v>46</v>
@@ -18024,7 +18032,7 @@
         <v>16</v>
       </c>
       <c r="E13" s="132" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>17</v>
@@ -18042,25 +18050,25 @@
         <v>29</v>
       </c>
       <c r="K13" s="98" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="L13" s="107"/>
     </row>
     <row r="14" spans="1:12" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="125" t="s">
+        <v>674</v>
+      </c>
+      <c r="B14" s="125" t="s">
+        <v>676</v>
+      </c>
+      <c r="C14" s="125" t="s">
         <v>675</v>
-      </c>
-      <c r="B14" s="125" t="s">
-        <v>677</v>
-      </c>
-      <c r="C14" s="125" t="s">
-        <v>676</v>
       </c>
       <c r="D14" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E14" s="126" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
       <c r="F14" s="127" t="s">
         <v>17</v>
@@ -18092,7 +18100,7 @@
         <v>16</v>
       </c>
       <c r="E15" s="132" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>17</v>
@@ -18110,7 +18118,7 @@
         <v>29</v>
       </c>
       <c r="K15" s="98" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="L15" s="107" t="s">
         <v>314</v>
@@ -18130,7 +18138,7 @@
         <v>16</v>
       </c>
       <c r="E16" s="126" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="F16" s="124" t="s">
         <v>35</v>
@@ -18437,7 +18445,7 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="84" x14ac:dyDescent="0.2">
@@ -18454,7 +18462,7 @@
         <v>153</v>
       </c>
       <c r="E2" s="82" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>35</v>
@@ -18472,7 +18480,7 @@
         <v>37</v>
       </c>
       <c r="K2" s="107" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="L2" s="186"/>
     </row>
@@ -18510,7 +18518,7 @@
     </row>
     <row r="4" spans="1:12" ht="92.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="121" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B4" s="35" t="s">
         <v>177</v>
@@ -18522,7 +18530,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="194" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="F4" s="124" t="s">
         <v>17</v>
@@ -18660,7 +18668,7 @@
         <v>16</v>
       </c>
       <c r="E8" s="82" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="F8" s="124" t="s">
         <v>35</v>
@@ -18678,25 +18686,25 @@
         <v>37</v>
       </c>
       <c r="K8" s="107" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="L8" s="107"/>
     </row>
     <row r="9" spans="1:12" ht="48" x14ac:dyDescent="0.2">
       <c r="A9" s="125" t="s">
+        <v>525</v>
+      </c>
+      <c r="B9" s="74" t="s">
         <v>526</v>
       </c>
-      <c r="B9" s="74" t="s">
+      <c r="C9" s="125" t="s">
         <v>527</v>
-      </c>
-      <c r="C9" s="125" t="s">
-        <v>528</v>
       </c>
       <c r="D9" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E9" s="212" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="F9" s="127" t="s">
         <v>35</v>
@@ -18714,25 +18722,25 @@
         <v>37</v>
       </c>
       <c r="K9" s="106" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="L9" s="129"/>
     </row>
     <row r="10" spans="1:12" ht="48" x14ac:dyDescent="0.2">
       <c r="A10" s="121" t="s">
+        <v>530</v>
+      </c>
+      <c r="B10" s="35" t="s">
         <v>531</v>
       </c>
-      <c r="B10" s="35" t="s">
+      <c r="C10" s="121" t="s">
         <v>532</v>
-      </c>
-      <c r="C10" s="121" t="s">
-        <v>533</v>
       </c>
       <c r="D10" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F10" s="124" t="s">
         <v>35</v>
@@ -18750,7 +18758,7 @@
         <v>37</v>
       </c>
       <c r="K10" s="106" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="L10" s="107"/>
     </row>
@@ -18788,13 +18796,13 @@
     </row>
     <row r="12" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" s="121" t="s">
+        <v>535</v>
+      </c>
+      <c r="B12" s="35" t="s">
         <v>536</v>
       </c>
-      <c r="B12" s="35" t="s">
+      <c r="C12" s="121" t="s">
         <v>537</v>
-      </c>
-      <c r="C12" s="121" t="s">
-        <v>538</v>
       </c>
       <c r="D12" s="132" t="s">
         <v>16</v>
@@ -18832,7 +18840,7 @@
         <v>16</v>
       </c>
       <c r="E13" s="126" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>35</v>
@@ -18886,19 +18894,19 @@
     </row>
     <row r="15" spans="1:12" ht="64" x14ac:dyDescent="0.2">
       <c r="A15" s="125" t="s">
+        <v>539</v>
+      </c>
+      <c r="B15" s="74" t="s">
         <v>540</v>
       </c>
-      <c r="B15" s="74" t="s">
+      <c r="C15" s="125" t="s">
         <v>541</v>
-      </c>
-      <c r="C15" s="125" t="s">
-        <v>542</v>
       </c>
       <c r="D15" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E15" s="126" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>17</v>
@@ -18932,7 +18940,7 @@
         <v>85</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="F16" s="124" t="s">
         <v>17</v>
@@ -18966,7 +18974,7 @@
         <v>92</v>
       </c>
       <c r="E17" s="80" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="F17" s="127" t="s">
         <v>35</v>
@@ -18984,7 +18992,7 @@
         <v>37</v>
       </c>
       <c r="K17" s="107" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="L17" s="129"/>
     </row>
@@ -19002,7 +19010,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="35" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="F18" s="124" t="s">
         <v>17</v>
@@ -19053,7 +19061,7 @@
       </c>
       <c r="K19" s="106"/>
       <c r="L19" s="129" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="48" x14ac:dyDescent="0.2">
@@ -19070,7 +19078,7 @@
         <v>16</v>
       </c>
       <c r="E20" s="35" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="F20" s="124" t="s">
         <v>35</v>
@@ -19094,19 +19102,19 @@
     </row>
     <row r="21" spans="1:12" ht="48" x14ac:dyDescent="0.2">
       <c r="A21" s="125" t="s">
+        <v>549</v>
+      </c>
+      <c r="B21" s="74" t="s">
         <v>550</v>
       </c>
-      <c r="B21" s="74" t="s">
+      <c r="C21" s="125" t="s">
         <v>551</v>
-      </c>
-      <c r="C21" s="125" t="s">
-        <v>552</v>
       </c>
       <c r="D21" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E21" s="126" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>17</v>
@@ -19124,10 +19132,10 @@
         <v>29</v>
       </c>
       <c r="K21" s="107" t="s">
+        <v>553</v>
+      </c>
+      <c r="L21" s="192" t="s">
         <v>554</v>
-      </c>
-      <c r="L21" s="192" t="s">
-        <v>555</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="48" x14ac:dyDescent="0.2">
@@ -19144,7 +19152,7 @@
         <v>338</v>
       </c>
       <c r="E22" s="35" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>35</v>
@@ -19178,7 +19186,7 @@
         <v>16</v>
       </c>
       <c r="E23" s="126" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>35</v>
@@ -19196,7 +19204,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="106" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="L23" s="195"/>
     </row>

</xml_diff>

<commit_message>
docs: remove edam example
The Distribution.format property contained an example with a value from EDAM ontology in the usage note. Since this property must be filled with a value from the EU authority, this example was removed.
</commit_message>
<xml_diff>
--- a/Documents/Metadata_CoreGenericHealth_v2.xlsx
+++ b/Documents/Metadata_CoreGenericHealth_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://healthri-my.sharepoint.com/personal/hannah_neikes_health-ri_nl/Documents/Documenten/GitHub/health-ri-metadata/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{B604F9AE-9787-411E-AB68-6C0D2821F0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8958F1D5-0A21-4FE0-BA8C-AACF2C87639E}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{B604F9AE-9787-411E-AB68-6C0D2821F0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75DD3E37-514C-4AE3-A673-1E268BD8AFB0}"/>
   <bookViews>
-    <workbookView xWindow="5295" yWindow="-16320" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="14" r:id="rId1"/>
@@ -1734,9 +1734,6 @@
     <t>http://publications.europa.eu/resource/authority/file-type</t>
   </si>
   <si>
-    <t>This property can be used to describe a media format in more detail than "media type" (using IANA media type) when needed. Instances of this property should use a URL, e.g., from the File Type vocabulary. For instance, for mzML files the value of this property could be: http://edamontology.org/format_3244</t>
-  </si>
-  <si>
     <t>dct:MediaTypeOrExtent (IRI)</t>
   </si>
   <si>
@@ -2618,6 +2615,9 @@
   <si>
     <t>The licence under which the catalogue (with resource description) is made available.
 The licences for Distributions and Data Services are not specified here. They are specified in the licence properties of their respective classes.</t>
+  </si>
+  <si>
+    <t>This property can be used to describe a media format in more detail than "media type" (using IANA media type) when needed. Instances of this property should use a URL from the File Type vocabulary.</t>
   </si>
 </sst>
 </file>
@@ -3765,6 +3765,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3776,13 +3779,16 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3796,12 +3802,6 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -7438,33 +7438,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>557</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>558</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="227" t="s">
         <v>559</v>
       </c>
-      <c r="N1" s="227" t="s">
+      <c r="O1" s="233" t="s">
         <v>560</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>561</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="72">
       <c r="A2" s="196" t="s">
+        <v>561</v>
+      </c>
+      <c r="B2" s="45" t="s">
         <v>562</v>
       </c>
-      <c r="B2" s="45" t="s">
+      <c r="C2" s="76" t="s">
         <v>563</v>
-      </c>
-      <c r="C2" s="76" t="s">
-        <v>564</v>
       </c>
       <c r="D2" s="196" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="197" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="F2" s="198" t="s">
         <v>35</v>
@@ -7473,7 +7473,7 @@
         <v>58</v>
       </c>
       <c r="H2" s="198" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="I2" s="160" t="s">
         <v>20</v>
@@ -7488,13 +7488,13 @@
     </row>
     <row r="3" spans="1:15" ht="28.8">
       <c r="A3" s="68" t="s">
+        <v>566</v>
+      </c>
+      <c r="B3" s="61" t="s">
         <v>567</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="C3" s="77" t="s">
         <v>568</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>569</v>
       </c>
       <c r="D3" s="68" t="s">
         <v>16</v>
@@ -7633,36 +7633,36 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>569</v>
+      </c>
+      <c r="M1" s="220" t="s">
         <v>570</v>
       </c>
-      <c r="M1" s="220" t="s">
+      <c r="N1" s="226" t="s">
         <v>571</v>
       </c>
-      <c r="N1" s="226" t="s">
+      <c r="O1" s="230" t="s">
         <v>572</v>
       </c>
-      <c r="O1" s="230" t="s">
+      <c r="P1" s="227" t="s">
         <v>573</v>
       </c>
-      <c r="P1" s="227" t="s">
+      <c r="Q1" s="231" t="s">
         <v>574</v>
       </c>
-      <c r="Q1" s="231" t="s">
+      <c r="R1" s="233" t="s">
         <v>575</v>
-      </c>
-      <c r="R1" s="233" t="s">
-        <v>576</v>
       </c>
     </row>
     <row r="2" spans="1:18">
       <c r="A2" s="58" t="s">
+        <v>576</v>
+      </c>
+      <c r="B2" s="44" t="s">
         <v>577</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="C2" s="76" t="s">
         <v>578</v>
-      </c>
-      <c r="C2" s="76" t="s">
-        <v>579</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
@@ -7690,13 +7690,13 @@
     </row>
     <row r="3" spans="1:18">
       <c r="A3" s="48" t="s">
+        <v>579</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>580</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>581</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>582</v>
       </c>
       <c r="D3" s="48" t="s">
         <v>16</v>
@@ -8358,33 +8358,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>582</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>583</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="227" t="s">
         <v>584</v>
       </c>
-      <c r="N1" s="227" t="s">
+      <c r="O1" s="233" t="s">
         <v>585</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>586</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="43.2">
       <c r="A2" s="84" t="s">
+        <v>586</v>
+      </c>
+      <c r="B2" s="44" t="s">
         <v>587</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="C2" s="58" t="s">
         <v>588</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>589</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>17</v>
@@ -8414,19 +8414,19 @@
     </row>
     <row r="3" spans="1:15" ht="129.6">
       <c r="A3" s="48" t="s">
+        <v>590</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>591</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>592</v>
       </c>
-      <c r="C3" s="77" t="s">
+      <c r="D3" s="234" t="s">
         <v>593</v>
       </c>
-      <c r="D3" s="234" t="s">
+      <c r="E3" s="50" t="s">
         <v>594</v>
-      </c>
-      <c r="E3" s="50" t="s">
-        <v>595</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>17</v>
@@ -8552,33 +8552,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="218" t="s">
+        <v>595</v>
+      </c>
+      <c r="M1" s="229" t="s">
         <v>596</v>
       </c>
-      <c r="M1" s="229" t="s">
+      <c r="N1" s="228" t="s">
         <v>597</v>
       </c>
-      <c r="N1" s="228" t="s">
+      <c r="O1" s="233" t="s">
         <v>598</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>599</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="158.4">
       <c r="A2" s="84" t="s">
+        <v>599</v>
+      </c>
+      <c r="B2" s="44" t="s">
+        <v>591</v>
+      </c>
+      <c r="C2" s="58" t="s">
+        <v>592</v>
+      </c>
+      <c r="D2" s="59" t="s">
         <v>600</v>
       </c>
-      <c r="B2" s="44" t="s">
-        <v>592</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>593</v>
-      </c>
-      <c r="D2" s="59" t="s">
+      <c r="E2" s="59" t="s">
         <v>601</v>
-      </c>
-      <c r="E2" s="59" t="s">
-        <v>602</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>35</v>
@@ -8599,19 +8599,19 @@
     </row>
     <row r="3" spans="1:15" ht="43.2">
       <c r="A3" s="48" t="s">
+        <v>602</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>603</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>604</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>605</v>
       </c>
       <c r="D3" s="116" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>35</v>
@@ -8737,33 +8737,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>606</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>607</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="227" t="s">
         <v>608</v>
       </c>
-      <c r="N1" s="227" t="s">
+      <c r="O1" s="233" t="s">
         <v>609</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>610</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="100.8">
       <c r="A2" s="84" t="s">
+        <v>610</v>
+      </c>
+      <c r="B2" s="44" t="s">
         <v>611</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="C2" s="58" t="s">
         <v>612</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>613</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>17</v>
@@ -8784,19 +8784,19 @@
     </row>
     <row r="3" spans="1:15" ht="57.6">
       <c r="A3" s="48" t="s">
+        <v>614</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>615</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>616</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>617</v>
       </c>
       <c r="D3" s="116" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>17</v>
@@ -8900,7 +8900,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="56" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="E1" s="56" t="s">
         <v>4</v>
@@ -8923,13 +8923,13 @@
     </row>
     <row r="2" spans="1:10" ht="28.8">
       <c r="A2" s="63" t="s">
+        <v>619</v>
+      </c>
+      <c r="B2" s="53" t="s">
         <v>620</v>
       </c>
-      <c r="B2" s="53" t="s">
+      <c r="C2" s="44" t="s">
         <v>621</v>
-      </c>
-      <c r="C2" s="44" t="s">
-        <v>622</v>
       </c>
       <c r="D2" s="43" t="s">
         <v>16</v>
@@ -8937,7 +8937,7 @@
       <c r="E2" s="45"/>
       <c r="F2" s="64"/>
       <c r="G2" s="63" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="H2" s="65" t="s">
         <v>81</v>
@@ -8951,13 +8951,13 @@
     </row>
     <row r="3" spans="1:10" ht="43.2">
       <c r="A3" s="67" t="s">
+        <v>623</v>
+      </c>
+      <c r="B3" s="50" t="s">
         <v>624</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="C3" s="49" t="s">
         <v>625</v>
-      </c>
-      <c r="C3" s="49" t="s">
-        <v>626</v>
       </c>
       <c r="D3" s="48" t="s">
         <v>16</v>
@@ -8965,10 +8965,10 @@
       <c r="E3" s="50"/>
       <c r="F3" s="68"/>
       <c r="G3" s="69" t="s">
+        <v>626</v>
+      </c>
+      <c r="H3" s="48" t="s">
         <v>627</v>
-      </c>
-      <c r="H3" s="48" t="s">
-        <v>628</v>
       </c>
       <c r="I3" s="69" t="s">
         <v>20</v>
@@ -8979,13 +8979,13 @@
     </row>
     <row r="4" spans="1:10" ht="43.2">
       <c r="A4" s="63" t="s">
+        <v>628</v>
+      </c>
+      <c r="B4" s="53" t="s">
         <v>629</v>
       </c>
-      <c r="B4" s="53" t="s">
+      <c r="C4" s="44" t="s">
         <v>630</v>
-      </c>
-      <c r="C4" s="44" t="s">
-        <v>631</v>
       </c>
       <c r="D4" s="43" t="s">
         <v>16</v>
@@ -8993,10 +8993,10 @@
       <c r="E4" s="53"/>
       <c r="F4" s="64"/>
       <c r="G4" s="63" t="s">
+        <v>631</v>
+      </c>
+      <c r="H4" s="65" t="s">
         <v>632</v>
-      </c>
-      <c r="H4" s="65" t="s">
-        <v>633</v>
       </c>
       <c r="I4" s="66" t="s">
         <v>20</v>
@@ -9007,26 +9007,26 @@
     </row>
     <row r="5" spans="1:10" ht="43.2">
       <c r="A5" s="67" t="s">
+        <v>633</v>
+      </c>
+      <c r="B5" s="50" t="s">
         <v>634</v>
       </c>
-      <c r="B5" s="50" t="s">
+      <c r="C5" s="49" t="s">
         <v>635</v>
-      </c>
-      <c r="C5" s="49" t="s">
-        <v>636</v>
       </c>
       <c r="D5" s="48" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="49" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="F5" s="68"/>
       <c r="G5" s="67" t="s">
+        <v>637</v>
+      </c>
+      <c r="H5" s="48" t="s">
         <v>638</v>
-      </c>
-      <c r="H5" s="48" t="s">
-        <v>639</v>
       </c>
       <c r="I5" s="69" t="s">
         <v>20</v>
@@ -9037,13 +9037,13 @@
     </row>
     <row r="6" spans="1:10" ht="28.8">
       <c r="A6" s="63" t="s">
+        <v>639</v>
+      </c>
+      <c r="B6" s="73" t="s">
         <v>640</v>
       </c>
-      <c r="B6" s="73" t="s">
+      <c r="C6" s="44" t="s">
         <v>641</v>
-      </c>
-      <c r="C6" s="44" t="s">
-        <v>642</v>
       </c>
       <c r="D6" s="43" t="s">
         <v>16</v>
@@ -9054,7 +9054,7 @@
         <v>98</v>
       </c>
       <c r="H6" s="65" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="I6" s="66" t="s">
         <v>20</v>
@@ -9065,13 +9065,13 @@
     </row>
     <row r="7" spans="1:10" ht="28.8">
       <c r="A7" s="67" t="s">
+        <v>642</v>
+      </c>
+      <c r="B7" s="50" t="s">
         <v>643</v>
       </c>
-      <c r="B7" s="50" t="s">
+      <c r="C7" s="49" t="s">
         <v>644</v>
-      </c>
-      <c r="C7" s="49" t="s">
-        <v>645</v>
       </c>
       <c r="D7" s="48" t="s">
         <v>16</v>
@@ -9093,23 +9093,23 @@
     </row>
     <row r="8" spans="1:10" ht="86.4">
       <c r="A8" s="63" t="s">
+        <v>645</v>
+      </c>
+      <c r="B8" s="53" t="s">
         <v>646</v>
       </c>
-      <c r="B8" s="53" t="s">
+      <c r="C8" s="44" t="s">
         <v>647</v>
-      </c>
-      <c r="C8" s="44" t="s">
-        <v>648</v>
       </c>
       <c r="D8" s="43" t="s">
         <v>16</v>
       </c>
       <c r="E8" s="71" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="F8" s="47"/>
       <c r="G8" s="63" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="H8" s="65">
         <v>1</v>
@@ -9123,13 +9123,13 @@
     </row>
     <row r="9" spans="1:10" ht="28.8">
       <c r="A9" s="67" t="s">
+        <v>650</v>
+      </c>
+      <c r="B9" s="50" t="s">
         <v>651</v>
       </c>
-      <c r="B9" s="50" t="s">
+      <c r="C9" s="49" t="s">
         <v>652</v>
-      </c>
-      <c r="C9" s="49" t="s">
-        <v>653</v>
       </c>
       <c r="D9" s="48" t="s">
         <v>16</v>
@@ -9137,7 +9137,7 @@
       <c r="E9" s="50"/>
       <c r="F9" s="68"/>
       <c r="G9" s="69" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="H9" s="48" t="s">
         <v>81</v>
@@ -9151,23 +9151,23 @@
     </row>
     <row r="10" spans="1:10" ht="28.8">
       <c r="A10" s="63" t="s">
+        <v>654</v>
+      </c>
+      <c r="B10" s="72" t="s">
         <v>655</v>
       </c>
-      <c r="B10" s="72" t="s">
+      <c r="C10" s="44" t="s">
         <v>656</v>
-      </c>
-      <c r="C10" s="44" t="s">
-        <v>657</v>
       </c>
       <c r="D10" s="43" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="72" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="F10" s="64"/>
       <c r="G10" s="63" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="H10" s="65" t="s">
         <v>19</v>
@@ -9632,36 +9632,36 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>658</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>659</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="233" t="s">
         <v>660</v>
-      </c>
-      <c r="N1" s="233" t="s">
-        <v>661</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="72">
       <c r="A2" s="44" t="s">
+        <v>661</v>
+      </c>
+      <c r="B2" s="57" t="s">
         <v>662</v>
       </c>
-      <c r="B2" s="57" t="s">
+      <c r="C2" s="58" t="s">
         <v>663</v>
       </c>
-      <c r="C2" s="58" t="s">
+      <c r="D2" s="78" t="s">
         <v>664</v>
       </c>
-      <c r="D2" s="78" t="s">
+      <c r="E2" s="197" t="s">
         <v>665</v>
-      </c>
-      <c r="E2" s="197" t="s">
-        <v>666</v>
       </c>
       <c r="F2" s="46" t="s">
         <v>35</v>
       </c>
       <c r="G2" s="204" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="H2" s="47">
         <v>1</v>
@@ -9675,13 +9675,13 @@
     </row>
     <row r="3" spans="1:14" ht="71.25" customHeight="1">
       <c r="A3" s="49" t="s">
+        <v>667</v>
+      </c>
+      <c r="B3" s="61" t="s">
         <v>668</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="C3" s="48" t="s">
         <v>669</v>
-      </c>
-      <c r="C3" s="48" t="s">
-        <v>670</v>
       </c>
       <c r="D3" s="50" t="s">
         <v>16</v>
@@ -9691,7 +9691,7 @@
         <v>35</v>
       </c>
       <c r="G3" s="51" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="H3" s="52">
         <v>1</v>
@@ -10605,107 +10605,107 @@
       <c r="M7" s="129"/>
     </row>
     <row r="8" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A8" s="236" t="s">
+      <c r="A8" s="237" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="237" t="s">
+      <c r="B8" s="238" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="236" t="s">
+      <c r="C8" s="237" t="s">
         <v>62</v>
       </c>
       <c r="D8" s="213" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="238" t="s">
+      <c r="E8" s="239" t="s">
         <v>64</v>
       </c>
-      <c r="F8" s="235" t="s">
+      <c r="F8" s="236" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="235" t="s">
+      <c r="G8" s="236" t="s">
         <v>65</v>
       </c>
-      <c r="H8" s="235" t="s">
+      <c r="H8" s="236" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="239" t="s">
+      <c r="I8" s="235" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="239" t="s">
+      <c r="J8" s="235" t="s">
         <v>66</v>
       </c>
       <c r="K8" s="137"/>
-      <c r="L8" s="239"/>
-      <c r="M8" s="239"/>
+      <c r="L8" s="235"/>
+      <c r="M8" s="235"/>
     </row>
     <row r="9" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A9" s="236"/>
-      <c r="B9" s="237"/>
-      <c r="C9" s="236"/>
+      <c r="A9" s="237"/>
+      <c r="B9" s="238"/>
+      <c r="C9" s="237"/>
       <c r="D9" s="214" t="s">
         <v>67</v>
       </c>
-      <c r="E9" s="238"/>
-      <c r="F9" s="235"/>
-      <c r="G9" s="235"/>
-      <c r="H9" s="235"/>
-      <c r="I9" s="239"/>
-      <c r="J9" s="239"/>
+      <c r="E9" s="239"/>
+      <c r="F9" s="236"/>
+      <c r="G9" s="236"/>
+      <c r="H9" s="236"/>
+      <c r="I9" s="235"/>
+      <c r="J9" s="235"/>
       <c r="K9" s="137"/>
-      <c r="L9" s="239"/>
-      <c r="M9" s="239"/>
+      <c r="L9" s="235"/>
+      <c r="M9" s="235"/>
     </row>
     <row r="10" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A10" s="236"/>
-      <c r="B10" s="237"/>
-      <c r="C10" s="236"/>
+      <c r="A10" s="237"/>
+      <c r="B10" s="238"/>
+      <c r="C10" s="237"/>
       <c r="D10" s="214" t="s">
         <v>68</v>
       </c>
-      <c r="E10" s="238"/>
-      <c r="F10" s="235"/>
-      <c r="G10" s="235"/>
-      <c r="H10" s="235"/>
-      <c r="I10" s="239"/>
-      <c r="J10" s="239"/>
+      <c r="E10" s="239"/>
+      <c r="F10" s="236"/>
+      <c r="G10" s="236"/>
+      <c r="H10" s="236"/>
+      <c r="I10" s="235"/>
+      <c r="J10" s="235"/>
       <c r="K10" s="137"/>
-      <c r="L10" s="239"/>
-      <c r="M10" s="239"/>
+      <c r="L10" s="235"/>
+      <c r="M10" s="235"/>
     </row>
     <row r="11" spans="1:13" ht="14.4" customHeight="1">
-      <c r="A11" s="236"/>
-      <c r="B11" s="237"/>
-      <c r="C11" s="236"/>
+      <c r="A11" s="237"/>
+      <c r="B11" s="238"/>
+      <c r="C11" s="237"/>
       <c r="D11" s="152" t="s">
         <v>69</v>
       </c>
-      <c r="E11" s="238"/>
-      <c r="F11" s="235"/>
-      <c r="G11" s="235"/>
-      <c r="H11" s="235"/>
-      <c r="I11" s="239"/>
-      <c r="J11" s="239"/>
+      <c r="E11" s="239"/>
+      <c r="F11" s="236"/>
+      <c r="G11" s="236"/>
+      <c r="H11" s="236"/>
+      <c r="I11" s="235"/>
+      <c r="J11" s="235"/>
       <c r="K11" s="153"/>
-      <c r="L11" s="239"/>
-      <c r="M11" s="239"/>
+      <c r="L11" s="235"/>
+      <c r="M11" s="235"/>
     </row>
     <row r="12" spans="1:13" ht="14.4" customHeight="1">
-      <c r="A12" s="236"/>
-      <c r="B12" s="237"/>
-      <c r="C12" s="236"/>
+      <c r="A12" s="237"/>
+      <c r="B12" s="238"/>
+      <c r="C12" s="237"/>
       <c r="D12" s="152" t="s">
         <v>70</v>
       </c>
-      <c r="E12" s="238"/>
-      <c r="F12" s="235"/>
-      <c r="G12" s="235"/>
-      <c r="H12" s="235"/>
-      <c r="I12" s="239"/>
-      <c r="J12" s="239"/>
+      <c r="E12" s="239"/>
+      <c r="F12" s="236"/>
+      <c r="G12" s="236"/>
+      <c r="H12" s="236"/>
+      <c r="I12" s="235"/>
+      <c r="J12" s="235"/>
       <c r="K12" s="137"/>
-      <c r="L12" s="239"/>
-      <c r="M12" s="239"/>
+      <c r="L12" s="235"/>
+      <c r="M12" s="235"/>
     </row>
     <row r="13" spans="1:13" ht="43.2">
       <c r="A13" s="125" t="s">
@@ -10830,7 +10830,7 @@
         <v>92</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="F16" s="124" t="s">
         <v>17</v>
@@ -11524,17 +11524,17 @@
     <sortCondition ref="A2:A24"/>
   </sortState>
   <mergeCells count="11">
-    <mergeCell ref="M8:M12"/>
-    <mergeCell ref="L8:L12"/>
-    <mergeCell ref="H8:H12"/>
-    <mergeCell ref="I8:I12"/>
-    <mergeCell ref="J8:J12"/>
     <mergeCell ref="G8:G12"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="B8:B12"/>
     <mergeCell ref="C8:C12"/>
     <mergeCell ref="E8:E12"/>
     <mergeCell ref="F8:F12"/>
+    <mergeCell ref="M8:M12"/>
+    <mergeCell ref="L8:L12"/>
+    <mergeCell ref="H8:H12"/>
+    <mergeCell ref="I8:I12"/>
+    <mergeCell ref="J8:J12"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F8">
     <cfRule type="cellIs" dxfId="190" priority="16" operator="equal">
@@ -12181,102 +12181,102 @@
       <c r="N13" s="129"/>
     </row>
     <row r="14" spans="1:14" ht="43.2">
-      <c r="A14" s="236" t="s">
+      <c r="A14" s="237" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="240" t="s">
+      <c r="B14" s="241" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="236" t="s">
+      <c r="C14" s="237" t="s">
         <v>62</v>
       </c>
       <c r="D14" s="213" t="s">
         <v>63</v>
       </c>
-      <c r="E14" s="238" t="s">
+      <c r="E14" s="239" t="s">
         <v>200</v>
       </c>
-      <c r="F14" s="235" t="s">
+      <c r="F14" s="236" t="s">
         <v>17</v>
       </c>
-      <c r="G14" s="235" t="s">
+      <c r="G14" s="236" t="s">
         <v>65</v>
       </c>
-      <c r="H14" s="235" t="s">
+      <c r="H14" s="236" t="s">
         <v>19</v>
       </c>
-      <c r="I14" s="239" t="s">
+      <c r="I14" s="235" t="s">
         <v>20</v>
       </c>
-      <c r="J14" s="239" t="s">
+      <c r="J14" s="235" t="s">
         <v>66</v>
       </c>
-      <c r="K14" s="241"/>
-      <c r="L14" s="239"/>
+      <c r="K14" s="240"/>
+      <c r="L14" s="235"/>
     </row>
     <row r="15" spans="1:14" ht="43.2">
-      <c r="A15" s="236"/>
-      <c r="B15" s="240"/>
-      <c r="C15" s="236"/>
+      <c r="A15" s="237"/>
+      <c r="B15" s="241"/>
+      <c r="C15" s="237"/>
       <c r="D15" s="214" t="s">
         <v>67</v>
       </c>
-      <c r="E15" s="238"/>
-      <c r="F15" s="235"/>
-      <c r="G15" s="235"/>
-      <c r="H15" s="235"/>
-      <c r="I15" s="239"/>
-      <c r="J15" s="239"/>
-      <c r="K15" s="241"/>
-      <c r="L15" s="239"/>
+      <c r="E15" s="239"/>
+      <c r="F15" s="236"/>
+      <c r="G15" s="236"/>
+      <c r="H15" s="236"/>
+      <c r="I15" s="235"/>
+      <c r="J15" s="235"/>
+      <c r="K15" s="240"/>
+      <c r="L15" s="235"/>
     </row>
     <row r="16" spans="1:14" ht="28.8">
-      <c r="A16" s="236"/>
-      <c r="B16" s="240"/>
-      <c r="C16" s="236"/>
+      <c r="A16" s="237"/>
+      <c r="B16" s="241"/>
+      <c r="C16" s="237"/>
       <c r="D16" s="214" t="s">
         <v>68</v>
       </c>
-      <c r="E16" s="238"/>
-      <c r="F16" s="235"/>
-      <c r="G16" s="235"/>
-      <c r="H16" s="235"/>
-      <c r="I16" s="239"/>
-      <c r="J16" s="239"/>
-      <c r="K16" s="241"/>
-      <c r="L16" s="239"/>
+      <c r="E16" s="239"/>
+      <c r="F16" s="236"/>
+      <c r="G16" s="236"/>
+      <c r="H16" s="236"/>
+      <c r="I16" s="235"/>
+      <c r="J16" s="235"/>
+      <c r="K16" s="240"/>
+      <c r="L16" s="235"/>
     </row>
     <row r="17" spans="1:14">
-      <c r="A17" s="236"/>
-      <c r="B17" s="240"/>
-      <c r="C17" s="236"/>
+      <c r="A17" s="237"/>
+      <c r="B17" s="241"/>
+      <c r="C17" s="237"/>
       <c r="D17" s="152" t="s">
         <v>69</v>
       </c>
-      <c r="E17" s="238"/>
-      <c r="F17" s="235"/>
-      <c r="G17" s="235"/>
-      <c r="H17" s="235"/>
-      <c r="I17" s="239"/>
-      <c r="J17" s="239"/>
-      <c r="K17" s="241"/>
-      <c r="L17" s="239"/>
+      <c r="E17" s="239"/>
+      <c r="F17" s="236"/>
+      <c r="G17" s="236"/>
+      <c r="H17" s="236"/>
+      <c r="I17" s="235"/>
+      <c r="J17" s="235"/>
+      <c r="K17" s="240"/>
+      <c r="L17" s="235"/>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="236"/>
-      <c r="B18" s="240"/>
-      <c r="C18" s="236"/>
+      <c r="A18" s="237"/>
+      <c r="B18" s="241"/>
+      <c r="C18" s="237"/>
       <c r="D18" s="152" t="s">
         <v>70</v>
       </c>
-      <c r="E18" s="238"/>
-      <c r="F18" s="235"/>
-      <c r="G18" s="235"/>
-      <c r="H18" s="235"/>
-      <c r="I18" s="239"/>
-      <c r="J18" s="239"/>
-      <c r="K18" s="241"/>
-      <c r="L18" s="239"/>
+      <c r="E18" s="239"/>
+      <c r="F18" s="236"/>
+      <c r="G18" s="236"/>
+      <c r="H18" s="236"/>
+      <c r="I18" s="235"/>
+      <c r="J18" s="235"/>
+      <c r="K18" s="240"/>
+      <c r="L18" s="235"/>
     </row>
     <row r="19" spans="1:14" ht="28.8">
       <c r="A19" s="125" t="s">
@@ -13604,17 +13604,17 @@
     <sortCondition ref="A2:A53"/>
   </sortState>
   <mergeCells count="11">
+    <mergeCell ref="A14:A18"/>
+    <mergeCell ref="B14:B18"/>
+    <mergeCell ref="C14:C18"/>
+    <mergeCell ref="F14:F18"/>
+    <mergeCell ref="E14:E18"/>
     <mergeCell ref="L14:L18"/>
     <mergeCell ref="K14:K18"/>
     <mergeCell ref="G14:G18"/>
     <mergeCell ref="H14:H18"/>
     <mergeCell ref="I14:I18"/>
     <mergeCell ref="J14:J18"/>
-    <mergeCell ref="A14:A18"/>
-    <mergeCell ref="B14:B18"/>
-    <mergeCell ref="C14:C18"/>
-    <mergeCell ref="F14:F18"/>
-    <mergeCell ref="E14:E18"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F14 F19:F53">
     <cfRule type="cellIs" dxfId="171" priority="8" operator="equal">
@@ -13860,7 +13860,7 @@
         <v>16</v>
       </c>
       <c r="E3" s="184" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="F3" s="163" t="s">
         <v>35</v>
@@ -14930,7 +14930,7 @@
         <v>16</v>
       </c>
       <c r="E3" s="184" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="F3" s="163" t="s">
         <v>35</v>
@@ -16158,7 +16158,7 @@
       <c r="L10" s="107"/>
       <c r="M10" s="107"/>
     </row>
-    <row r="11" spans="1:13" ht="72">
+    <row r="11" spans="1:13" ht="43.2">
       <c r="A11" s="125" t="s">
         <v>463</v>
       </c>
@@ -16172,13 +16172,13 @@
         <v>466</v>
       </c>
       <c r="E11" s="126" t="s">
-        <v>467</v>
+        <v>674</v>
       </c>
       <c r="F11" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G11" s="127" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="H11" s="127">
         <v>1</v>
@@ -16190,7 +16190,7 @@
         <v>29</v>
       </c>
       <c r="K11" s="99" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="L11" s="129"/>
       <c r="M11" s="129"/>
@@ -16209,7 +16209,7 @@
         <v>85</v>
       </c>
       <c r="E12" s="138" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="F12" s="124" t="s">
         <v>17</v>
@@ -16227,14 +16227,14 @@
         <v>29</v>
       </c>
       <c r="K12" s="98" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="L12" s="107"/>
       <c r="M12" s="107"/>
     </row>
     <row r="13" spans="1:13" ht="72">
       <c r="A13" s="125" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B13" s="74" t="s">
         <v>90</v>
@@ -16246,13 +16246,13 @@
         <v>92</v>
       </c>
       <c r="E13" s="80" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G13" s="127" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="H13" s="127">
         <v>1</v>
@@ -16264,14 +16264,14 @@
         <v>37</v>
       </c>
       <c r="K13" s="98" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L13" s="129"/>
       <c r="M13" s="129"/>
     </row>
     <row r="14" spans="1:13" ht="72">
       <c r="A14" s="121" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B14" s="35" t="s">
         <v>176</v>
@@ -16283,7 +16283,7 @@
         <v>16</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="F14" s="124" t="s">
         <v>17</v>
@@ -16301,26 +16301,26 @@
         <v>29</v>
       </c>
       <c r="K14" s="98" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L14" s="107"/>
       <c r="M14" s="107"/>
     </row>
     <row r="15" spans="1:13" ht="100.8">
       <c r="A15" s="125" t="s">
+        <v>478</v>
+      </c>
+      <c r="B15" s="74" t="s">
         <v>479</v>
       </c>
-      <c r="B15" s="74" t="s">
+      <c r="C15" s="125" t="s">
         <v>480</v>
-      </c>
-      <c r="C15" s="125" t="s">
-        <v>481</v>
       </c>
       <c r="D15" s="185" t="s">
         <v>450</v>
       </c>
       <c r="E15" s="80" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>17</v>
@@ -16338,7 +16338,7 @@
         <v>29</v>
       </c>
       <c r="K15" s="98" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="L15" s="129"/>
       <c r="M15" s="129"/>
@@ -16373,26 +16373,26 @@
         <v>29</v>
       </c>
       <c r="K16" s="98" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="L16" s="107"/>
       <c r="M16" s="107"/>
     </row>
     <row r="17" spans="1:13" ht="57.6">
       <c r="A17" s="125" t="s">
+        <v>484</v>
+      </c>
+      <c r="B17" s="74" t="s">
         <v>485</v>
       </c>
-      <c r="B17" s="74" t="s">
+      <c r="C17" s="125" t="s">
         <v>486</v>
-      </c>
-      <c r="C17" s="125" t="s">
-        <v>487</v>
       </c>
       <c r="D17" s="185" t="s">
         <v>450</v>
       </c>
       <c r="E17" s="74" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="F17" s="127" t="s">
         <v>17</v>
@@ -16410,7 +16410,7 @@
         <v>29</v>
       </c>
       <c r="K17" s="98" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="L17" s="129"/>
       <c r="M17" s="129"/>
@@ -16429,7 +16429,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="132" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="F18" s="124" t="s">
         <v>17</v>
@@ -16447,7 +16447,7 @@
         <v>29</v>
       </c>
       <c r="K18" s="98" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="L18" s="107"/>
       <c r="M18" s="107"/>
@@ -16460,7 +16460,7 @@
         <v>310</v>
       </c>
       <c r="C19" s="125" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="D19" s="126"/>
       <c r="E19" s="80" t="s">
@@ -16483,10 +16483,10 @@
       </c>
       <c r="K19" s="104"/>
       <c r="L19" s="129" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="M19" s="129" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="129.6">
@@ -16503,7 +16503,7 @@
         <v>16</v>
       </c>
       <c r="E20" s="79" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="F20" s="190" t="s">
         <v>35</v>
@@ -16521,7 +16521,7 @@
         <v>29</v>
       </c>
       <c r="K20" s="99" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="L20" s="107"/>
       <c r="M20" s="107"/>
@@ -16537,10 +16537,10 @@
         <v>326</v>
       </c>
       <c r="D21" s="154" t="s">
+        <v>495</v>
+      </c>
+      <c r="E21" s="81" t="s">
         <v>496</v>
-      </c>
-      <c r="E21" s="81" t="s">
-        <v>497</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>17</v>
@@ -16558,7 +16558,7 @@
         <v>29</v>
       </c>
       <c r="K21" s="98" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="L21" s="129"/>
       <c r="M21" s="129"/>
@@ -16577,7 +16577,7 @@
         <v>16</v>
       </c>
       <c r="E22" s="132" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>17</v>
@@ -16612,7 +16612,7 @@
         <v>16</v>
       </c>
       <c r="E23" s="126" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>17</v>
@@ -16630,7 +16630,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="98" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="L23" s="129"/>
       <c r="M23" s="129"/>
@@ -17112,7 +17112,7 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -17129,7 +17129,7 @@
         <v>16</v>
       </c>
       <c r="E2" s="74" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>17</v>
@@ -17147,7 +17147,7 @@
         <v>29</v>
       </c>
       <c r="K2" s="98" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="L2" s="129"/>
     </row>
@@ -17183,7 +17183,7 @@
         <v>29</v>
       </c>
       <c r="K3" s="98" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="L3" s="107" t="s">
         <v>39</v>
@@ -17203,7 +17203,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="126" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="F4" s="127" t="s">
         <v>35</v>
@@ -17221,7 +17221,7 @@
         <v>29</v>
       </c>
       <c r="K4" s="99" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="L4" s="129"/>
     </row>
@@ -17239,7 +17239,7 @@
         <v>197</v>
       </c>
       <c r="E5" s="135" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="F5" s="124" t="s">
         <v>17</v>
@@ -17260,104 +17260,104 @@
       <c r="L5" s="107"/>
     </row>
     <row r="6" spans="1:12" ht="28.8">
-      <c r="A6" s="243" t="s">
+      <c r="A6" s="245" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="244" t="s">
+      <c r="B6" s="246" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="243" t="s">
+      <c r="C6" s="245" t="s">
         <v>62</v>
       </c>
       <c r="D6" s="215" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="245" t="s">
+      <c r="E6" s="247" t="s">
         <v>200</v>
       </c>
-      <c r="F6" s="242" t="s">
+      <c r="F6" s="244" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="242" t="s">
+      <c r="G6" s="244" t="s">
         <v>65</v>
       </c>
-      <c r="H6" s="242" t="s">
+      <c r="H6" s="244" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="246" t="s">
+      <c r="I6" s="242" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="239" t="s">
+      <c r="J6" s="235" t="s">
         <v>66</v>
       </c>
-      <c r="K6" s="247" t="s">
-        <v>509</v>
-      </c>
-      <c r="L6" s="246"/>
+      <c r="K6" s="243" t="s">
+        <v>508</v>
+      </c>
+      <c r="L6" s="242"/>
     </row>
     <row r="7" spans="1:12" ht="28.8">
-      <c r="A7" s="243"/>
-      <c r="B7" s="244"/>
-      <c r="C7" s="243"/>
+      <c r="A7" s="245"/>
+      <c r="B7" s="246"/>
+      <c r="C7" s="245"/>
       <c r="D7" s="216" t="s">
         <v>67</v>
       </c>
-      <c r="E7" s="245"/>
-      <c r="F7" s="242"/>
-      <c r="G7" s="242"/>
-      <c r="H7" s="242"/>
-      <c r="I7" s="246"/>
-      <c r="J7" s="239"/>
-      <c r="K7" s="247"/>
-      <c r="L7" s="246"/>
+      <c r="E7" s="247"/>
+      <c r="F7" s="244"/>
+      <c r="G7" s="244"/>
+      <c r="H7" s="244"/>
+      <c r="I7" s="242"/>
+      <c r="J7" s="235"/>
+      <c r="K7" s="243"/>
+      <c r="L7" s="242"/>
     </row>
     <row r="8" spans="1:12" ht="28.8">
-      <c r="A8" s="243"/>
-      <c r="B8" s="244"/>
-      <c r="C8" s="243"/>
+      <c r="A8" s="245"/>
+      <c r="B8" s="246"/>
+      <c r="C8" s="245"/>
       <c r="D8" s="216" t="s">
         <v>68</v>
       </c>
-      <c r="E8" s="245"/>
-      <c r="F8" s="242"/>
-      <c r="G8" s="242"/>
-      <c r="H8" s="242"/>
-      <c r="I8" s="246"/>
-      <c r="J8" s="239"/>
-      <c r="K8" s="247"/>
-      <c r="L8" s="246"/>
+      <c r="E8" s="247"/>
+      <c r="F8" s="244"/>
+      <c r="G8" s="244"/>
+      <c r="H8" s="244"/>
+      <c r="I8" s="242"/>
+      <c r="J8" s="235"/>
+      <c r="K8" s="243"/>
+      <c r="L8" s="242"/>
     </row>
     <row r="9" spans="1:12">
-      <c r="A9" s="243"/>
-      <c r="B9" s="244"/>
-      <c r="C9" s="243"/>
+      <c r="A9" s="245"/>
+      <c r="B9" s="246"/>
+      <c r="C9" s="245"/>
       <c r="D9" s="139" t="s">
         <v>69</v>
       </c>
-      <c r="E9" s="245"/>
-      <c r="F9" s="242"/>
-      <c r="G9" s="242"/>
-      <c r="H9" s="242"/>
-      <c r="I9" s="246"/>
-      <c r="J9" s="239"/>
-      <c r="K9" s="247"/>
-      <c r="L9" s="246"/>
+      <c r="E9" s="247"/>
+      <c r="F9" s="244"/>
+      <c r="G9" s="244"/>
+      <c r="H9" s="244"/>
+      <c r="I9" s="242"/>
+      <c r="J9" s="235"/>
+      <c r="K9" s="243"/>
+      <c r="L9" s="242"/>
     </row>
     <row r="10" spans="1:12">
-      <c r="A10" s="243"/>
-      <c r="B10" s="244"/>
-      <c r="C10" s="243"/>
+      <c r="A10" s="245"/>
+      <c r="B10" s="246"/>
+      <c r="C10" s="245"/>
       <c r="D10" s="139" t="s">
         <v>70</v>
       </c>
-      <c r="E10" s="245"/>
-      <c r="F10" s="242"/>
-      <c r="G10" s="242"/>
-      <c r="H10" s="242"/>
-      <c r="I10" s="246"/>
-      <c r="J10" s="239"/>
-      <c r="K10" s="247"/>
-      <c r="L10" s="246"/>
+      <c r="E10" s="247"/>
+      <c r="F10" s="244"/>
+      <c r="G10" s="244"/>
+      <c r="H10" s="244"/>
+      <c r="I10" s="242"/>
+      <c r="J10" s="235"/>
+      <c r="K10" s="243"/>
+      <c r="L10" s="242"/>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="121" t="s">
@@ -17373,7 +17373,7 @@
         <v>16</v>
       </c>
       <c r="E11" s="132" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="F11" s="124" t="s">
         <v>17</v>
@@ -17391,7 +17391,7 @@
         <v>29</v>
       </c>
       <c r="K11" s="99" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="L11" s="107"/>
     </row>
@@ -17409,7 +17409,7 @@
         <v>16</v>
       </c>
       <c r="E12" s="126" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="F12" s="124" t="s">
         <v>17</v>
@@ -17427,7 +17427,7 @@
         <v>29</v>
       </c>
       <c r="K12" s="98" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="L12" s="129" t="s">
         <v>46</v>
@@ -17447,7 +17447,7 @@
         <v>16</v>
       </c>
       <c r="E13" s="132" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>17</v>
@@ -17465,7 +17465,7 @@
         <v>29</v>
       </c>
       <c r="K13" s="98" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="L13" s="107"/>
     </row>
@@ -17483,7 +17483,7 @@
         <v>16</v>
       </c>
       <c r="E14" s="126" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="F14" s="124" t="s">
         <v>17</v>
@@ -17501,7 +17501,7 @@
         <v>29</v>
       </c>
       <c r="K14" s="98" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="L14" s="129" t="s">
         <v>313</v>
@@ -17521,7 +17521,7 @@
         <v>16</v>
       </c>
       <c r="E15" s="121" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>35</v>
@@ -17666,17 +17666,17 @@
   </sheetData>
   <autoFilter ref="A1:L15" xr:uid="{FBE7E653-2382-46E4-9C76-9C694EDC9195}"/>
   <mergeCells count="11">
-    <mergeCell ref="L6:L10"/>
-    <mergeCell ref="K6:K10"/>
-    <mergeCell ref="H6:H10"/>
-    <mergeCell ref="I6:I10"/>
-    <mergeCell ref="J6:J10"/>
     <mergeCell ref="G6:G10"/>
     <mergeCell ref="A6:A10"/>
     <mergeCell ref="B6:B10"/>
     <mergeCell ref="C6:C10"/>
     <mergeCell ref="E6:E10"/>
     <mergeCell ref="F6:F10"/>
+    <mergeCell ref="L6:L10"/>
+    <mergeCell ref="K6:K10"/>
+    <mergeCell ref="H6:H10"/>
+    <mergeCell ref="I6:I10"/>
+    <mergeCell ref="J6:J10"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F6 F11:F15">
     <cfRule type="cellIs" dxfId="127" priority="7" operator="equal">
@@ -17820,7 +17820,7 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="92.4">
@@ -17837,7 +17837,7 @@
         <v>152</v>
       </c>
       <c r="E2" s="82" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>35</v>
@@ -17855,7 +17855,7 @@
         <v>37</v>
       </c>
       <c r="K2" s="107" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="L2" s="186"/>
     </row>
@@ -17893,7 +17893,7 @@
     </row>
     <row r="4" spans="1:12" ht="92.25" customHeight="1">
       <c r="A4" s="121" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B4" s="35" t="s">
         <v>176</v>
@@ -17905,7 +17905,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="194" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="F4" s="124" t="s">
         <v>17</v>
@@ -18043,7 +18043,7 @@
         <v>16</v>
       </c>
       <c r="E8" s="82" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="F8" s="124" t="s">
         <v>35</v>
@@ -18061,25 +18061,25 @@
         <v>37</v>
       </c>
       <c r="K8" s="107" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="L8" s="107"/>
     </row>
     <row r="9" spans="1:12" ht="43.2">
       <c r="A9" s="125" t="s">
+        <v>524</v>
+      </c>
+      <c r="B9" s="74" t="s">
         <v>525</v>
       </c>
-      <c r="B9" s="74" t="s">
+      <c r="C9" s="125" t="s">
         <v>526</v>
-      </c>
-      <c r="C9" s="125" t="s">
-        <v>527</v>
       </c>
       <c r="D9" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E9" s="212" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="F9" s="127" t="s">
         <v>35</v>
@@ -18097,25 +18097,25 @@
         <v>37</v>
       </c>
       <c r="K9" s="106" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="L9" s="129"/>
     </row>
     <row r="10" spans="1:12" ht="43.2">
       <c r="A10" s="121" t="s">
+        <v>529</v>
+      </c>
+      <c r="B10" s="35" t="s">
         <v>530</v>
       </c>
-      <c r="B10" s="35" t="s">
+      <c r="C10" s="121" t="s">
         <v>531</v>
-      </c>
-      <c r="C10" s="121" t="s">
-        <v>532</v>
       </c>
       <c r="D10" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="F10" s="124" t="s">
         <v>35</v>
@@ -18133,7 +18133,7 @@
         <v>37</v>
       </c>
       <c r="K10" s="106" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="L10" s="107"/>
     </row>
@@ -18155,7 +18155,7 @@
         <v>17</v>
       </c>
       <c r="G11" s="127" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="H11" s="127" t="s">
         <v>19</v>
@@ -18171,13 +18171,13 @@
     </row>
     <row r="12" spans="1:12" ht="28.8">
       <c r="A12" s="121" t="s">
+        <v>534</v>
+      </c>
+      <c r="B12" s="35" t="s">
         <v>535</v>
       </c>
-      <c r="B12" s="35" t="s">
+      <c r="C12" s="121" t="s">
         <v>536</v>
-      </c>
-      <c r="C12" s="121" t="s">
-        <v>537</v>
       </c>
       <c r="D12" s="132" t="s">
         <v>16</v>
@@ -18215,7 +18215,7 @@
         <v>16</v>
       </c>
       <c r="E13" s="126" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>35</v>
@@ -18269,19 +18269,19 @@
     </row>
     <row r="15" spans="1:12" ht="57.6">
       <c r="A15" s="125" t="s">
+        <v>538</v>
+      </c>
+      <c r="B15" s="74" t="s">
         <v>539</v>
       </c>
-      <c r="B15" s="74" t="s">
+      <c r="C15" s="125" t="s">
         <v>540</v>
-      </c>
-      <c r="C15" s="125" t="s">
-        <v>541</v>
       </c>
       <c r="D15" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E15" s="126" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>17</v>
@@ -18315,7 +18315,7 @@
         <v>85</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="F16" s="124" t="s">
         <v>17</v>
@@ -18349,7 +18349,7 @@
         <v>92</v>
       </c>
       <c r="E17" s="80" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="F17" s="127" t="s">
         <v>35</v>
@@ -18367,7 +18367,7 @@
         <v>37</v>
       </c>
       <c r="K17" s="107" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="L17" s="129"/>
     </row>
@@ -18385,7 +18385,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="35" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="F18" s="124" t="s">
         <v>17</v>
@@ -18436,7 +18436,7 @@
       </c>
       <c r="K19" s="106"/>
       <c r="L19" s="129" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="43.2">
@@ -18453,7 +18453,7 @@
         <v>16</v>
       </c>
       <c r="E20" s="35" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="F20" s="124" t="s">
         <v>35</v>
@@ -18477,19 +18477,19 @@
     </row>
     <row r="21" spans="1:12" ht="57.6">
       <c r="A21" s="125" t="s">
+        <v>548</v>
+      </c>
+      <c r="B21" s="74" t="s">
         <v>549</v>
       </c>
-      <c r="B21" s="74" t="s">
+      <c r="C21" s="125" t="s">
         <v>550</v>
-      </c>
-      <c r="C21" s="125" t="s">
-        <v>551</v>
       </c>
       <c r="D21" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E21" s="126" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>17</v>
@@ -18507,10 +18507,10 @@
         <v>29</v>
       </c>
       <c r="K21" s="107" t="s">
+        <v>552</v>
+      </c>
+      <c r="L21" s="192" t="s">
         <v>553</v>
-      </c>
-      <c r="L21" s="192" t="s">
-        <v>554</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="43.2">
@@ -18527,7 +18527,7 @@
         <v>337</v>
       </c>
       <c r="E22" s="35" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>35</v>
@@ -18561,7 +18561,7 @@
         <v>16</v>
       </c>
       <c r="E23" s="126" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>35</v>
@@ -18579,7 +18579,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="106" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="L23" s="195"/>
     </row>
@@ -19062,6 +19062,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000B1A1CF98C819F4881BB4349588D0C85" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ff8ef391852eaca4511043a54bffd4a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cfc87205-1831-4b6c-a7b4-76d40079a43e" xmlns:ns3="221af607-abea-4d5e-830c-567dcc03c0ec" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="201dd8b781da46d5daa37e3355db44fe" ns2:_="" ns3:_="">
     <xsd:import namespace="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
@@ -19304,15 +19313,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -19326,6 +19326,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19A23828-4FF7-4569-837D-B1B2C775409F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19344,14 +19352,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16D2CAB5-B21B-4A93-9D82-49FE3E36CF14}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
docs: remove edam example (#257)
* docs: remove edam example

The Distribution.format property contained an example with a value from EDAM ontology in the usage note. Since this property must be filled with a value from the EU authority, this example was removed.

* Update README.md

Co-authored-by: sourcery-ai[bot] <58596630+sourcery-ai[bot]@users.noreply.github.com>

---------

Co-authored-by: sourcery-ai[bot] <58596630+sourcery-ai[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Documents/Metadata_CoreGenericHealth_v2.xlsx
+++ b/Documents/Metadata_CoreGenericHealth_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://healthri-my.sharepoint.com/personal/hannah_neikes_health-ri_nl/Documents/Documenten/GitHub/health-ri-metadata/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{B604F9AE-9787-411E-AB68-6C0D2821F0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8958F1D5-0A21-4FE0-BA8C-AACF2C87639E}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{B604F9AE-9787-411E-AB68-6C0D2821F0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75DD3E37-514C-4AE3-A673-1E268BD8AFB0}"/>
   <bookViews>
-    <workbookView xWindow="5295" yWindow="-16320" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="14" r:id="rId1"/>
@@ -1734,9 +1734,6 @@
     <t>http://publications.europa.eu/resource/authority/file-type</t>
   </si>
   <si>
-    <t>This property can be used to describe a media format in more detail than "media type" (using IANA media type) when needed. Instances of this property should use a URL, e.g., from the File Type vocabulary. For instance, for mzML files the value of this property could be: http://edamontology.org/format_3244</t>
-  </si>
-  <si>
     <t>dct:MediaTypeOrExtent (IRI)</t>
   </si>
   <si>
@@ -2618,6 +2615,9 @@
   <si>
     <t>The licence under which the catalogue (with resource description) is made available.
 The licences for Distributions and Data Services are not specified here. They are specified in the licence properties of their respective classes.</t>
+  </si>
+  <si>
+    <t>This property can be used to describe a media format in more detail than "media type" (using IANA media type) when needed. Instances of this property should use a URL from the File Type vocabulary.</t>
   </si>
 </sst>
 </file>
@@ -3765,6 +3765,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3776,13 +3779,16 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3796,12 +3802,6 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -7438,33 +7438,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>557</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>558</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="227" t="s">
         <v>559</v>
       </c>
-      <c r="N1" s="227" t="s">
+      <c r="O1" s="233" t="s">
         <v>560</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>561</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="72">
       <c r="A2" s="196" t="s">
+        <v>561</v>
+      </c>
+      <c r="B2" s="45" t="s">
         <v>562</v>
       </c>
-      <c r="B2" s="45" t="s">
+      <c r="C2" s="76" t="s">
         <v>563</v>
-      </c>
-      <c r="C2" s="76" t="s">
-        <v>564</v>
       </c>
       <c r="D2" s="196" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="197" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="F2" s="198" t="s">
         <v>35</v>
@@ -7473,7 +7473,7 @@
         <v>58</v>
       </c>
       <c r="H2" s="198" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="I2" s="160" t="s">
         <v>20</v>
@@ -7488,13 +7488,13 @@
     </row>
     <row r="3" spans="1:15" ht="28.8">
       <c r="A3" s="68" t="s">
+        <v>566</v>
+      </c>
+      <c r="B3" s="61" t="s">
         <v>567</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="C3" s="77" t="s">
         <v>568</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>569</v>
       </c>
       <c r="D3" s="68" t="s">
         <v>16</v>
@@ -7633,36 +7633,36 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>569</v>
+      </c>
+      <c r="M1" s="220" t="s">
         <v>570</v>
       </c>
-      <c r="M1" s="220" t="s">
+      <c r="N1" s="226" t="s">
         <v>571</v>
       </c>
-      <c r="N1" s="226" t="s">
+      <c r="O1" s="230" t="s">
         <v>572</v>
       </c>
-      <c r="O1" s="230" t="s">
+      <c r="P1" s="227" t="s">
         <v>573</v>
       </c>
-      <c r="P1" s="227" t="s">
+      <c r="Q1" s="231" t="s">
         <v>574</v>
       </c>
-      <c r="Q1" s="231" t="s">
+      <c r="R1" s="233" t="s">
         <v>575</v>
-      </c>
-      <c r="R1" s="233" t="s">
-        <v>576</v>
       </c>
     </row>
     <row r="2" spans="1:18">
       <c r="A2" s="58" t="s">
+        <v>576</v>
+      </c>
+      <c r="B2" s="44" t="s">
         <v>577</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="C2" s="76" t="s">
         <v>578</v>
-      </c>
-      <c r="C2" s="76" t="s">
-        <v>579</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
@@ -7690,13 +7690,13 @@
     </row>
     <row r="3" spans="1:18">
       <c r="A3" s="48" t="s">
+        <v>579</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>580</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>581</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>582</v>
       </c>
       <c r="D3" s="48" t="s">
         <v>16</v>
@@ -8358,33 +8358,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>582</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>583</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="227" t="s">
         <v>584</v>
       </c>
-      <c r="N1" s="227" t="s">
+      <c r="O1" s="233" t="s">
         <v>585</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>586</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="43.2">
       <c r="A2" s="84" t="s">
+        <v>586</v>
+      </c>
+      <c r="B2" s="44" t="s">
         <v>587</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="C2" s="58" t="s">
         <v>588</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>589</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>17</v>
@@ -8414,19 +8414,19 @@
     </row>
     <row r="3" spans="1:15" ht="129.6">
       <c r="A3" s="48" t="s">
+        <v>590</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>591</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>592</v>
       </c>
-      <c r="C3" s="77" t="s">
+      <c r="D3" s="234" t="s">
         <v>593</v>
       </c>
-      <c r="D3" s="234" t="s">
+      <c r="E3" s="50" t="s">
         <v>594</v>
-      </c>
-      <c r="E3" s="50" t="s">
-        <v>595</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>17</v>
@@ -8552,33 +8552,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="218" t="s">
+        <v>595</v>
+      </c>
+      <c r="M1" s="229" t="s">
         <v>596</v>
       </c>
-      <c r="M1" s="229" t="s">
+      <c r="N1" s="228" t="s">
         <v>597</v>
       </c>
-      <c r="N1" s="228" t="s">
+      <c r="O1" s="233" t="s">
         <v>598</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>599</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="158.4">
       <c r="A2" s="84" t="s">
+        <v>599</v>
+      </c>
+      <c r="B2" s="44" t="s">
+        <v>591</v>
+      </c>
+      <c r="C2" s="58" t="s">
+        <v>592</v>
+      </c>
+      <c r="D2" s="59" t="s">
         <v>600</v>
       </c>
-      <c r="B2" s="44" t="s">
-        <v>592</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>593</v>
-      </c>
-      <c r="D2" s="59" t="s">
+      <c r="E2" s="59" t="s">
         <v>601</v>
-      </c>
-      <c r="E2" s="59" t="s">
-        <v>602</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>35</v>
@@ -8599,19 +8599,19 @@
     </row>
     <row r="3" spans="1:15" ht="43.2">
       <c r="A3" s="48" t="s">
+        <v>602</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>603</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>604</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>605</v>
       </c>
       <c r="D3" s="116" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>35</v>
@@ -8737,33 +8737,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>606</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>607</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="227" t="s">
         <v>608</v>
       </c>
-      <c r="N1" s="227" t="s">
+      <c r="O1" s="233" t="s">
         <v>609</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>610</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="100.8">
       <c r="A2" s="84" t="s">
+        <v>610</v>
+      </c>
+      <c r="B2" s="44" t="s">
         <v>611</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="C2" s="58" t="s">
         <v>612</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>613</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>17</v>
@@ -8784,19 +8784,19 @@
     </row>
     <row r="3" spans="1:15" ht="57.6">
       <c r="A3" s="48" t="s">
+        <v>614</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>615</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>616</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>617</v>
       </c>
       <c r="D3" s="116" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>17</v>
@@ -8900,7 +8900,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="56" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="E1" s="56" t="s">
         <v>4</v>
@@ -8923,13 +8923,13 @@
     </row>
     <row r="2" spans="1:10" ht="28.8">
       <c r="A2" s="63" t="s">
+        <v>619</v>
+      </c>
+      <c r="B2" s="53" t="s">
         <v>620</v>
       </c>
-      <c r="B2" s="53" t="s">
+      <c r="C2" s="44" t="s">
         <v>621</v>
-      </c>
-      <c r="C2" s="44" t="s">
-        <v>622</v>
       </c>
       <c r="D2" s="43" t="s">
         <v>16</v>
@@ -8937,7 +8937,7 @@
       <c r="E2" s="45"/>
       <c r="F2" s="64"/>
       <c r="G2" s="63" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="H2" s="65" t="s">
         <v>81</v>
@@ -8951,13 +8951,13 @@
     </row>
     <row r="3" spans="1:10" ht="43.2">
       <c r="A3" s="67" t="s">
+        <v>623</v>
+      </c>
+      <c r="B3" s="50" t="s">
         <v>624</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="C3" s="49" t="s">
         <v>625</v>
-      </c>
-      <c r="C3" s="49" t="s">
-        <v>626</v>
       </c>
       <c r="D3" s="48" t="s">
         <v>16</v>
@@ -8965,10 +8965,10 @@
       <c r="E3" s="50"/>
       <c r="F3" s="68"/>
       <c r="G3" s="69" t="s">
+        <v>626</v>
+      </c>
+      <c r="H3" s="48" t="s">
         <v>627</v>
-      </c>
-      <c r="H3" s="48" t="s">
-        <v>628</v>
       </c>
       <c r="I3" s="69" t="s">
         <v>20</v>
@@ -8979,13 +8979,13 @@
     </row>
     <row r="4" spans="1:10" ht="43.2">
       <c r="A4" s="63" t="s">
+        <v>628</v>
+      </c>
+      <c r="B4" s="53" t="s">
         <v>629</v>
       </c>
-      <c r="B4" s="53" t="s">
+      <c r="C4" s="44" t="s">
         <v>630</v>
-      </c>
-      <c r="C4" s="44" t="s">
-        <v>631</v>
       </c>
       <c r="D4" s="43" t="s">
         <v>16</v>
@@ -8993,10 +8993,10 @@
       <c r="E4" s="53"/>
       <c r="F4" s="64"/>
       <c r="G4" s="63" t="s">
+        <v>631</v>
+      </c>
+      <c r="H4" s="65" t="s">
         <v>632</v>
-      </c>
-      <c r="H4" s="65" t="s">
-        <v>633</v>
       </c>
       <c r="I4" s="66" t="s">
         <v>20</v>
@@ -9007,26 +9007,26 @@
     </row>
     <row r="5" spans="1:10" ht="43.2">
       <c r="A5" s="67" t="s">
+        <v>633</v>
+      </c>
+      <c r="B5" s="50" t="s">
         <v>634</v>
       </c>
-      <c r="B5" s="50" t="s">
+      <c r="C5" s="49" t="s">
         <v>635</v>
-      </c>
-      <c r="C5" s="49" t="s">
-        <v>636</v>
       </c>
       <c r="D5" s="48" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="49" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="F5" s="68"/>
       <c r="G5" s="67" t="s">
+        <v>637</v>
+      </c>
+      <c r="H5" s="48" t="s">
         <v>638</v>
-      </c>
-      <c r="H5" s="48" t="s">
-        <v>639</v>
       </c>
       <c r="I5" s="69" t="s">
         <v>20</v>
@@ -9037,13 +9037,13 @@
     </row>
     <row r="6" spans="1:10" ht="28.8">
       <c r="A6" s="63" t="s">
+        <v>639</v>
+      </c>
+      <c r="B6" s="73" t="s">
         <v>640</v>
       </c>
-      <c r="B6" s="73" t="s">
+      <c r="C6" s="44" t="s">
         <v>641</v>
-      </c>
-      <c r="C6" s="44" t="s">
-        <v>642</v>
       </c>
       <c r="D6" s="43" t="s">
         <v>16</v>
@@ -9054,7 +9054,7 @@
         <v>98</v>
       </c>
       <c r="H6" s="65" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="I6" s="66" t="s">
         <v>20</v>
@@ -9065,13 +9065,13 @@
     </row>
     <row r="7" spans="1:10" ht="28.8">
       <c r="A7" s="67" t="s">
+        <v>642</v>
+      </c>
+      <c r="B7" s="50" t="s">
         <v>643</v>
       </c>
-      <c r="B7" s="50" t="s">
+      <c r="C7" s="49" t="s">
         <v>644</v>
-      </c>
-      <c r="C7" s="49" t="s">
-        <v>645</v>
       </c>
       <c r="D7" s="48" t="s">
         <v>16</v>
@@ -9093,23 +9093,23 @@
     </row>
     <row r="8" spans="1:10" ht="86.4">
       <c r="A8" s="63" t="s">
+        <v>645</v>
+      </c>
+      <c r="B8" s="53" t="s">
         <v>646</v>
       </c>
-      <c r="B8" s="53" t="s">
+      <c r="C8" s="44" t="s">
         <v>647</v>
-      </c>
-      <c r="C8" s="44" t="s">
-        <v>648</v>
       </c>
       <c r="D8" s="43" t="s">
         <v>16</v>
       </c>
       <c r="E8" s="71" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="F8" s="47"/>
       <c r="G8" s="63" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="H8" s="65">
         <v>1</v>
@@ -9123,13 +9123,13 @@
     </row>
     <row r="9" spans="1:10" ht="28.8">
       <c r="A9" s="67" t="s">
+        <v>650</v>
+      </c>
+      <c r="B9" s="50" t="s">
         <v>651</v>
       </c>
-      <c r="B9" s="50" t="s">
+      <c r="C9" s="49" t="s">
         <v>652</v>
-      </c>
-      <c r="C9" s="49" t="s">
-        <v>653</v>
       </c>
       <c r="D9" s="48" t="s">
         <v>16</v>
@@ -9137,7 +9137,7 @@
       <c r="E9" s="50"/>
       <c r="F9" s="68"/>
       <c r="G9" s="69" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="H9" s="48" t="s">
         <v>81</v>
@@ -9151,23 +9151,23 @@
     </row>
     <row r="10" spans="1:10" ht="28.8">
       <c r="A10" s="63" t="s">
+        <v>654</v>
+      </c>
+      <c r="B10" s="72" t="s">
         <v>655</v>
       </c>
-      <c r="B10" s="72" t="s">
+      <c r="C10" s="44" t="s">
         <v>656</v>
-      </c>
-      <c r="C10" s="44" t="s">
-        <v>657</v>
       </c>
       <c r="D10" s="43" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="72" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="F10" s="64"/>
       <c r="G10" s="63" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="H10" s="65" t="s">
         <v>19</v>
@@ -9632,36 +9632,36 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>658</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>659</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="233" t="s">
         <v>660</v>
-      </c>
-      <c r="N1" s="233" t="s">
-        <v>661</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="72">
       <c r="A2" s="44" t="s">
+        <v>661</v>
+      </c>
+      <c r="B2" s="57" t="s">
         <v>662</v>
       </c>
-      <c r="B2" s="57" t="s">
+      <c r="C2" s="58" t="s">
         <v>663</v>
       </c>
-      <c r="C2" s="58" t="s">
+      <c r="D2" s="78" t="s">
         <v>664</v>
       </c>
-      <c r="D2" s="78" t="s">
+      <c r="E2" s="197" t="s">
         <v>665</v>
-      </c>
-      <c r="E2" s="197" t="s">
-        <v>666</v>
       </c>
       <c r="F2" s="46" t="s">
         <v>35</v>
       </c>
       <c r="G2" s="204" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="H2" s="47">
         <v>1</v>
@@ -9675,13 +9675,13 @@
     </row>
     <row r="3" spans="1:14" ht="71.25" customHeight="1">
       <c r="A3" s="49" t="s">
+        <v>667</v>
+      </c>
+      <c r="B3" s="61" t="s">
         <v>668</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="C3" s="48" t="s">
         <v>669</v>
-      </c>
-      <c r="C3" s="48" t="s">
-        <v>670</v>
       </c>
       <c r="D3" s="50" t="s">
         <v>16</v>
@@ -9691,7 +9691,7 @@
         <v>35</v>
       </c>
       <c r="G3" s="51" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="H3" s="52">
         <v>1</v>
@@ -10605,107 +10605,107 @@
       <c r="M7" s="129"/>
     </row>
     <row r="8" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A8" s="236" t="s">
+      <c r="A8" s="237" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="237" t="s">
+      <c r="B8" s="238" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="236" t="s">
+      <c r="C8" s="237" t="s">
         <v>62</v>
       </c>
       <c r="D8" s="213" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="238" t="s">
+      <c r="E8" s="239" t="s">
         <v>64</v>
       </c>
-      <c r="F8" s="235" t="s">
+      <c r="F8" s="236" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="235" t="s">
+      <c r="G8" s="236" t="s">
         <v>65</v>
       </c>
-      <c r="H8" s="235" t="s">
+      <c r="H8" s="236" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="239" t="s">
+      <c r="I8" s="235" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="239" t="s">
+      <c r="J8" s="235" t="s">
         <v>66</v>
       </c>
       <c r="K8" s="137"/>
-      <c r="L8" s="239"/>
-      <c r="M8" s="239"/>
+      <c r="L8" s="235"/>
+      <c r="M8" s="235"/>
     </row>
     <row r="9" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A9" s="236"/>
-      <c r="B9" s="237"/>
-      <c r="C9" s="236"/>
+      <c r="A9" s="237"/>
+      <c r="B9" s="238"/>
+      <c r="C9" s="237"/>
       <c r="D9" s="214" t="s">
         <v>67</v>
       </c>
-      <c r="E9" s="238"/>
-      <c r="F9" s="235"/>
-      <c r="G9" s="235"/>
-      <c r="H9" s="235"/>
-      <c r="I9" s="239"/>
-      <c r="J9" s="239"/>
+      <c r="E9" s="239"/>
+      <c r="F9" s="236"/>
+      <c r="G9" s="236"/>
+      <c r="H9" s="236"/>
+      <c r="I9" s="235"/>
+      <c r="J9" s="235"/>
       <c r="K9" s="137"/>
-      <c r="L9" s="239"/>
-      <c r="M9" s="239"/>
+      <c r="L9" s="235"/>
+      <c r="M9" s="235"/>
     </row>
     <row r="10" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A10" s="236"/>
-      <c r="B10" s="237"/>
-      <c r="C10" s="236"/>
+      <c r="A10" s="237"/>
+      <c r="B10" s="238"/>
+      <c r="C10" s="237"/>
       <c r="D10" s="214" t="s">
         <v>68</v>
       </c>
-      <c r="E10" s="238"/>
-      <c r="F10" s="235"/>
-      <c r="G10" s="235"/>
-      <c r="H10" s="235"/>
-      <c r="I10" s="239"/>
-      <c r="J10" s="239"/>
+      <c r="E10" s="239"/>
+      <c r="F10" s="236"/>
+      <c r="G10" s="236"/>
+      <c r="H10" s="236"/>
+      <c r="I10" s="235"/>
+      <c r="J10" s="235"/>
       <c r="K10" s="137"/>
-      <c r="L10" s="239"/>
-      <c r="M10" s="239"/>
+      <c r="L10" s="235"/>
+      <c r="M10" s="235"/>
     </row>
     <row r="11" spans="1:13" ht="14.4" customHeight="1">
-      <c r="A11" s="236"/>
-      <c r="B11" s="237"/>
-      <c r="C11" s="236"/>
+      <c r="A11" s="237"/>
+      <c r="B11" s="238"/>
+      <c r="C11" s="237"/>
       <c r="D11" s="152" t="s">
         <v>69</v>
       </c>
-      <c r="E11" s="238"/>
-      <c r="F11" s="235"/>
-      <c r="G11" s="235"/>
-      <c r="H11" s="235"/>
-      <c r="I11" s="239"/>
-      <c r="J11" s="239"/>
+      <c r="E11" s="239"/>
+      <c r="F11" s="236"/>
+      <c r="G11" s="236"/>
+      <c r="H11" s="236"/>
+      <c r="I11" s="235"/>
+      <c r="J11" s="235"/>
       <c r="K11" s="153"/>
-      <c r="L11" s="239"/>
-      <c r="M11" s="239"/>
+      <c r="L11" s="235"/>
+      <c r="M11" s="235"/>
     </row>
     <row r="12" spans="1:13" ht="14.4" customHeight="1">
-      <c r="A12" s="236"/>
-      <c r="B12" s="237"/>
-      <c r="C12" s="236"/>
+      <c r="A12" s="237"/>
+      <c r="B12" s="238"/>
+      <c r="C12" s="237"/>
       <c r="D12" s="152" t="s">
         <v>70</v>
       </c>
-      <c r="E12" s="238"/>
-      <c r="F12" s="235"/>
-      <c r="G12" s="235"/>
-      <c r="H12" s="235"/>
-      <c r="I12" s="239"/>
-      <c r="J12" s="239"/>
+      <c r="E12" s="239"/>
+      <c r="F12" s="236"/>
+      <c r="G12" s="236"/>
+      <c r="H12" s="236"/>
+      <c r="I12" s="235"/>
+      <c r="J12" s="235"/>
       <c r="K12" s="137"/>
-      <c r="L12" s="239"/>
-      <c r="M12" s="239"/>
+      <c r="L12" s="235"/>
+      <c r="M12" s="235"/>
     </row>
     <row r="13" spans="1:13" ht="43.2">
       <c r="A13" s="125" t="s">
@@ -10830,7 +10830,7 @@
         <v>92</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="F16" s="124" t="s">
         <v>17</v>
@@ -11524,17 +11524,17 @@
     <sortCondition ref="A2:A24"/>
   </sortState>
   <mergeCells count="11">
-    <mergeCell ref="M8:M12"/>
-    <mergeCell ref="L8:L12"/>
-    <mergeCell ref="H8:H12"/>
-    <mergeCell ref="I8:I12"/>
-    <mergeCell ref="J8:J12"/>
     <mergeCell ref="G8:G12"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="B8:B12"/>
     <mergeCell ref="C8:C12"/>
     <mergeCell ref="E8:E12"/>
     <mergeCell ref="F8:F12"/>
+    <mergeCell ref="M8:M12"/>
+    <mergeCell ref="L8:L12"/>
+    <mergeCell ref="H8:H12"/>
+    <mergeCell ref="I8:I12"/>
+    <mergeCell ref="J8:J12"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F8">
     <cfRule type="cellIs" dxfId="190" priority="16" operator="equal">
@@ -12181,102 +12181,102 @@
       <c r="N13" s="129"/>
     </row>
     <row r="14" spans="1:14" ht="43.2">
-      <c r="A14" s="236" t="s">
+      <c r="A14" s="237" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="240" t="s">
+      <c r="B14" s="241" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="236" t="s">
+      <c r="C14" s="237" t="s">
         <v>62</v>
       </c>
       <c r="D14" s="213" t="s">
         <v>63</v>
       </c>
-      <c r="E14" s="238" t="s">
+      <c r="E14" s="239" t="s">
         <v>200</v>
       </c>
-      <c r="F14" s="235" t="s">
+      <c r="F14" s="236" t="s">
         <v>17</v>
       </c>
-      <c r="G14" s="235" t="s">
+      <c r="G14" s="236" t="s">
         <v>65</v>
       </c>
-      <c r="H14" s="235" t="s">
+      <c r="H14" s="236" t="s">
         <v>19</v>
       </c>
-      <c r="I14" s="239" t="s">
+      <c r="I14" s="235" t="s">
         <v>20</v>
       </c>
-      <c r="J14" s="239" t="s">
+      <c r="J14" s="235" t="s">
         <v>66</v>
       </c>
-      <c r="K14" s="241"/>
-      <c r="L14" s="239"/>
+      <c r="K14" s="240"/>
+      <c r="L14" s="235"/>
     </row>
     <row r="15" spans="1:14" ht="43.2">
-      <c r="A15" s="236"/>
-      <c r="B15" s="240"/>
-      <c r="C15" s="236"/>
+      <c r="A15" s="237"/>
+      <c r="B15" s="241"/>
+      <c r="C15" s="237"/>
       <c r="D15" s="214" t="s">
         <v>67</v>
       </c>
-      <c r="E15" s="238"/>
-      <c r="F15" s="235"/>
-      <c r="G15" s="235"/>
-      <c r="H15" s="235"/>
-      <c r="I15" s="239"/>
-      <c r="J15" s="239"/>
-      <c r="K15" s="241"/>
-      <c r="L15" s="239"/>
+      <c r="E15" s="239"/>
+      <c r="F15" s="236"/>
+      <c r="G15" s="236"/>
+      <c r="H15" s="236"/>
+      <c r="I15" s="235"/>
+      <c r="J15" s="235"/>
+      <c r="K15" s="240"/>
+      <c r="L15" s="235"/>
     </row>
     <row r="16" spans="1:14" ht="28.8">
-      <c r="A16" s="236"/>
-      <c r="B16" s="240"/>
-      <c r="C16" s="236"/>
+      <c r="A16" s="237"/>
+      <c r="B16" s="241"/>
+      <c r="C16" s="237"/>
       <c r="D16" s="214" t="s">
         <v>68</v>
       </c>
-      <c r="E16" s="238"/>
-      <c r="F16" s="235"/>
-      <c r="G16" s="235"/>
-      <c r="H16" s="235"/>
-      <c r="I16" s="239"/>
-      <c r="J16" s="239"/>
-      <c r="K16" s="241"/>
-      <c r="L16" s="239"/>
+      <c r="E16" s="239"/>
+      <c r="F16" s="236"/>
+      <c r="G16" s="236"/>
+      <c r="H16" s="236"/>
+      <c r="I16" s="235"/>
+      <c r="J16" s="235"/>
+      <c r="K16" s="240"/>
+      <c r="L16" s="235"/>
     </row>
     <row r="17" spans="1:14">
-      <c r="A17" s="236"/>
-      <c r="B17" s="240"/>
-      <c r="C17" s="236"/>
+      <c r="A17" s="237"/>
+      <c r="B17" s="241"/>
+      <c r="C17" s="237"/>
       <c r="D17" s="152" t="s">
         <v>69</v>
       </c>
-      <c r="E17" s="238"/>
-      <c r="F17" s="235"/>
-      <c r="G17" s="235"/>
-      <c r="H17" s="235"/>
-      <c r="I17" s="239"/>
-      <c r="J17" s="239"/>
-      <c r="K17" s="241"/>
-      <c r="L17" s="239"/>
+      <c r="E17" s="239"/>
+      <c r="F17" s="236"/>
+      <c r="G17" s="236"/>
+      <c r="H17" s="236"/>
+      <c r="I17" s="235"/>
+      <c r="J17" s="235"/>
+      <c r="K17" s="240"/>
+      <c r="L17" s="235"/>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="236"/>
-      <c r="B18" s="240"/>
-      <c r="C18" s="236"/>
+      <c r="A18" s="237"/>
+      <c r="B18" s="241"/>
+      <c r="C18" s="237"/>
       <c r="D18" s="152" t="s">
         <v>70</v>
       </c>
-      <c r="E18" s="238"/>
-      <c r="F18" s="235"/>
-      <c r="G18" s="235"/>
-      <c r="H18" s="235"/>
-      <c r="I18" s="239"/>
-      <c r="J18" s="239"/>
-      <c r="K18" s="241"/>
-      <c r="L18" s="239"/>
+      <c r="E18" s="239"/>
+      <c r="F18" s="236"/>
+      <c r="G18" s="236"/>
+      <c r="H18" s="236"/>
+      <c r="I18" s="235"/>
+      <c r="J18" s="235"/>
+      <c r="K18" s="240"/>
+      <c r="L18" s="235"/>
     </row>
     <row r="19" spans="1:14" ht="28.8">
       <c r="A19" s="125" t="s">
@@ -13604,17 +13604,17 @@
     <sortCondition ref="A2:A53"/>
   </sortState>
   <mergeCells count="11">
+    <mergeCell ref="A14:A18"/>
+    <mergeCell ref="B14:B18"/>
+    <mergeCell ref="C14:C18"/>
+    <mergeCell ref="F14:F18"/>
+    <mergeCell ref="E14:E18"/>
     <mergeCell ref="L14:L18"/>
     <mergeCell ref="K14:K18"/>
     <mergeCell ref="G14:G18"/>
     <mergeCell ref="H14:H18"/>
     <mergeCell ref="I14:I18"/>
     <mergeCell ref="J14:J18"/>
-    <mergeCell ref="A14:A18"/>
-    <mergeCell ref="B14:B18"/>
-    <mergeCell ref="C14:C18"/>
-    <mergeCell ref="F14:F18"/>
-    <mergeCell ref="E14:E18"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F14 F19:F53">
     <cfRule type="cellIs" dxfId="171" priority="8" operator="equal">
@@ -13860,7 +13860,7 @@
         <v>16</v>
       </c>
       <c r="E3" s="184" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="F3" s="163" t="s">
         <v>35</v>
@@ -14930,7 +14930,7 @@
         <v>16</v>
       </c>
       <c r="E3" s="184" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="F3" s="163" t="s">
         <v>35</v>
@@ -16158,7 +16158,7 @@
       <c r="L10" s="107"/>
       <c r="M10" s="107"/>
     </row>
-    <row r="11" spans="1:13" ht="72">
+    <row r="11" spans="1:13" ht="43.2">
       <c r="A11" s="125" t="s">
         <v>463</v>
       </c>
@@ -16172,13 +16172,13 @@
         <v>466</v>
       </c>
       <c r="E11" s="126" t="s">
-        <v>467</v>
+        <v>674</v>
       </c>
       <c r="F11" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G11" s="127" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="H11" s="127">
         <v>1</v>
@@ -16190,7 +16190,7 @@
         <v>29</v>
       </c>
       <c r="K11" s="99" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="L11" s="129"/>
       <c r="M11" s="129"/>
@@ -16209,7 +16209,7 @@
         <v>85</v>
       </c>
       <c r="E12" s="138" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="F12" s="124" t="s">
         <v>17</v>
@@ -16227,14 +16227,14 @@
         <v>29</v>
       </c>
       <c r="K12" s="98" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="L12" s="107"/>
       <c r="M12" s="107"/>
     </row>
     <row r="13" spans="1:13" ht="72">
       <c r="A13" s="125" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B13" s="74" t="s">
         <v>90</v>
@@ -16246,13 +16246,13 @@
         <v>92</v>
       </c>
       <c r="E13" s="80" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G13" s="127" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="H13" s="127">
         <v>1</v>
@@ -16264,14 +16264,14 @@
         <v>37</v>
       </c>
       <c r="K13" s="98" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="L13" s="129"/>
       <c r="M13" s="129"/>
     </row>
     <row r="14" spans="1:13" ht="72">
       <c r="A14" s="121" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="B14" s="35" t="s">
         <v>176</v>
@@ -16283,7 +16283,7 @@
         <v>16</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="F14" s="124" t="s">
         <v>17</v>
@@ -16301,26 +16301,26 @@
         <v>29</v>
       </c>
       <c r="K14" s="98" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="L14" s="107"/>
       <c r="M14" s="107"/>
     </row>
     <row r="15" spans="1:13" ht="100.8">
       <c r="A15" s="125" t="s">
+        <v>478</v>
+      </c>
+      <c r="B15" s="74" t="s">
         <v>479</v>
       </c>
-      <c r="B15" s="74" t="s">
+      <c r="C15" s="125" t="s">
         <v>480</v>
-      </c>
-      <c r="C15" s="125" t="s">
-        <v>481</v>
       </c>
       <c r="D15" s="185" t="s">
         <v>450</v>
       </c>
       <c r="E15" s="80" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>17</v>
@@ -16338,7 +16338,7 @@
         <v>29</v>
       </c>
       <c r="K15" s="98" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="L15" s="129"/>
       <c r="M15" s="129"/>
@@ -16373,26 +16373,26 @@
         <v>29</v>
       </c>
       <c r="K16" s="98" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="L16" s="107"/>
       <c r="M16" s="107"/>
     </row>
     <row r="17" spans="1:13" ht="57.6">
       <c r="A17" s="125" t="s">
+        <v>484</v>
+      </c>
+      <c r="B17" s="74" t="s">
         <v>485</v>
       </c>
-      <c r="B17" s="74" t="s">
+      <c r="C17" s="125" t="s">
         <v>486</v>
-      </c>
-      <c r="C17" s="125" t="s">
-        <v>487</v>
       </c>
       <c r="D17" s="185" t="s">
         <v>450</v>
       </c>
       <c r="E17" s="74" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="F17" s="127" t="s">
         <v>17</v>
@@ -16410,7 +16410,7 @@
         <v>29</v>
       </c>
       <c r="K17" s="98" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="L17" s="129"/>
       <c r="M17" s="129"/>
@@ -16429,7 +16429,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="132" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="F18" s="124" t="s">
         <v>17</v>
@@ -16447,7 +16447,7 @@
         <v>29</v>
       </c>
       <c r="K18" s="98" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="L18" s="107"/>
       <c r="M18" s="107"/>
@@ -16460,7 +16460,7 @@
         <v>310</v>
       </c>
       <c r="C19" s="125" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="D19" s="126"/>
       <c r="E19" s="80" t="s">
@@ -16483,10 +16483,10 @@
       </c>
       <c r="K19" s="104"/>
       <c r="L19" s="129" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="M19" s="129" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="129.6">
@@ -16503,7 +16503,7 @@
         <v>16</v>
       </c>
       <c r="E20" s="79" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="F20" s="190" t="s">
         <v>35</v>
@@ -16521,7 +16521,7 @@
         <v>29</v>
       </c>
       <c r="K20" s="99" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="L20" s="107"/>
       <c r="M20" s="107"/>
@@ -16537,10 +16537,10 @@
         <v>326</v>
       </c>
       <c r="D21" s="154" t="s">
+        <v>495</v>
+      </c>
+      <c r="E21" s="81" t="s">
         <v>496</v>
-      </c>
-      <c r="E21" s="81" t="s">
-        <v>497</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>17</v>
@@ -16558,7 +16558,7 @@
         <v>29</v>
       </c>
       <c r="K21" s="98" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="L21" s="129"/>
       <c r="M21" s="129"/>
@@ -16577,7 +16577,7 @@
         <v>16</v>
       </c>
       <c r="E22" s="132" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>17</v>
@@ -16612,7 +16612,7 @@
         <v>16</v>
       </c>
       <c r="E23" s="126" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>17</v>
@@ -16630,7 +16630,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="98" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="L23" s="129"/>
       <c r="M23" s="129"/>
@@ -17112,7 +17112,7 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -17129,7 +17129,7 @@
         <v>16</v>
       </c>
       <c r="E2" s="74" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>17</v>
@@ -17147,7 +17147,7 @@
         <v>29</v>
       </c>
       <c r="K2" s="98" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="L2" s="129"/>
     </row>
@@ -17183,7 +17183,7 @@
         <v>29</v>
       </c>
       <c r="K3" s="98" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="L3" s="107" t="s">
         <v>39</v>
@@ -17203,7 +17203,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="126" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="F4" s="127" t="s">
         <v>35</v>
@@ -17221,7 +17221,7 @@
         <v>29</v>
       </c>
       <c r="K4" s="99" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="L4" s="129"/>
     </row>
@@ -17239,7 +17239,7 @@
         <v>197</v>
       </c>
       <c r="E5" s="135" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="F5" s="124" t="s">
         <v>17</v>
@@ -17260,104 +17260,104 @@
       <c r="L5" s="107"/>
     </row>
     <row r="6" spans="1:12" ht="28.8">
-      <c r="A6" s="243" t="s">
+      <c r="A6" s="245" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="244" t="s">
+      <c r="B6" s="246" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="243" t="s">
+      <c r="C6" s="245" t="s">
         <v>62</v>
       </c>
       <c r="D6" s="215" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="245" t="s">
+      <c r="E6" s="247" t="s">
         <v>200</v>
       </c>
-      <c r="F6" s="242" t="s">
+      <c r="F6" s="244" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="242" t="s">
+      <c r="G6" s="244" t="s">
         <v>65</v>
       </c>
-      <c r="H6" s="242" t="s">
+      <c r="H6" s="244" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="246" t="s">
+      <c r="I6" s="242" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="239" t="s">
+      <c r="J6" s="235" t="s">
         <v>66</v>
       </c>
-      <c r="K6" s="247" t="s">
-        <v>509</v>
-      </c>
-      <c r="L6" s="246"/>
+      <c r="K6" s="243" t="s">
+        <v>508</v>
+      </c>
+      <c r="L6" s="242"/>
     </row>
     <row r="7" spans="1:12" ht="28.8">
-      <c r="A7" s="243"/>
-      <c r="B7" s="244"/>
-      <c r="C7" s="243"/>
+      <c r="A7" s="245"/>
+      <c r="B7" s="246"/>
+      <c r="C7" s="245"/>
       <c r="D7" s="216" t="s">
         <v>67</v>
       </c>
-      <c r="E7" s="245"/>
-      <c r="F7" s="242"/>
-      <c r="G7" s="242"/>
-      <c r="H7" s="242"/>
-      <c r="I7" s="246"/>
-      <c r="J7" s="239"/>
-      <c r="K7" s="247"/>
-      <c r="L7" s="246"/>
+      <c r="E7" s="247"/>
+      <c r="F7" s="244"/>
+      <c r="G7" s="244"/>
+      <c r="H7" s="244"/>
+      <c r="I7" s="242"/>
+      <c r="J7" s="235"/>
+      <c r="K7" s="243"/>
+      <c r="L7" s="242"/>
     </row>
     <row r="8" spans="1:12" ht="28.8">
-      <c r="A8" s="243"/>
-      <c r="B8" s="244"/>
-      <c r="C8" s="243"/>
+      <c r="A8" s="245"/>
+      <c r="B8" s="246"/>
+      <c r="C8" s="245"/>
       <c r="D8" s="216" t="s">
         <v>68</v>
       </c>
-      <c r="E8" s="245"/>
-      <c r="F8" s="242"/>
-      <c r="G8" s="242"/>
-      <c r="H8" s="242"/>
-      <c r="I8" s="246"/>
-      <c r="J8" s="239"/>
-      <c r="K8" s="247"/>
-      <c r="L8" s="246"/>
+      <c r="E8" s="247"/>
+      <c r="F8" s="244"/>
+      <c r="G8" s="244"/>
+      <c r="H8" s="244"/>
+      <c r="I8" s="242"/>
+      <c r="J8" s="235"/>
+      <c r="K8" s="243"/>
+      <c r="L8" s="242"/>
     </row>
     <row r="9" spans="1:12">
-      <c r="A9" s="243"/>
-      <c r="B9" s="244"/>
-      <c r="C9" s="243"/>
+      <c r="A9" s="245"/>
+      <c r="B9" s="246"/>
+      <c r="C9" s="245"/>
       <c r="D9" s="139" t="s">
         <v>69</v>
       </c>
-      <c r="E9" s="245"/>
-      <c r="F9" s="242"/>
-      <c r="G9" s="242"/>
-      <c r="H9" s="242"/>
-      <c r="I9" s="246"/>
-      <c r="J9" s="239"/>
-      <c r="K9" s="247"/>
-      <c r="L9" s="246"/>
+      <c r="E9" s="247"/>
+      <c r="F9" s="244"/>
+      <c r="G9" s="244"/>
+      <c r="H9" s="244"/>
+      <c r="I9" s="242"/>
+      <c r="J9" s="235"/>
+      <c r="K9" s="243"/>
+      <c r="L9" s="242"/>
     </row>
     <row r="10" spans="1:12">
-      <c r="A10" s="243"/>
-      <c r="B10" s="244"/>
-      <c r="C10" s="243"/>
+      <c r="A10" s="245"/>
+      <c r="B10" s="246"/>
+      <c r="C10" s="245"/>
       <c r="D10" s="139" t="s">
         <v>70</v>
       </c>
-      <c r="E10" s="245"/>
-      <c r="F10" s="242"/>
-      <c r="G10" s="242"/>
-      <c r="H10" s="242"/>
-      <c r="I10" s="246"/>
-      <c r="J10" s="239"/>
-      <c r="K10" s="247"/>
-      <c r="L10" s="246"/>
+      <c r="E10" s="247"/>
+      <c r="F10" s="244"/>
+      <c r="G10" s="244"/>
+      <c r="H10" s="244"/>
+      <c r="I10" s="242"/>
+      <c r="J10" s="235"/>
+      <c r="K10" s="243"/>
+      <c r="L10" s="242"/>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="121" t="s">
@@ -17373,7 +17373,7 @@
         <v>16</v>
       </c>
       <c r="E11" s="132" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="F11" s="124" t="s">
         <v>17</v>
@@ -17391,7 +17391,7 @@
         <v>29</v>
       </c>
       <c r="K11" s="99" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="L11" s="107"/>
     </row>
@@ -17409,7 +17409,7 @@
         <v>16</v>
       </c>
       <c r="E12" s="126" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="F12" s="124" t="s">
         <v>17</v>
@@ -17427,7 +17427,7 @@
         <v>29</v>
       </c>
       <c r="K12" s="98" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="L12" s="129" t="s">
         <v>46</v>
@@ -17447,7 +17447,7 @@
         <v>16</v>
       </c>
       <c r="E13" s="132" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>17</v>
@@ -17465,7 +17465,7 @@
         <v>29</v>
       </c>
       <c r="K13" s="98" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="L13" s="107"/>
     </row>
@@ -17483,7 +17483,7 @@
         <v>16</v>
       </c>
       <c r="E14" s="126" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="F14" s="124" t="s">
         <v>17</v>
@@ -17501,7 +17501,7 @@
         <v>29</v>
       </c>
       <c r="K14" s="98" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="L14" s="129" t="s">
         <v>313</v>
@@ -17521,7 +17521,7 @@
         <v>16</v>
       </c>
       <c r="E15" s="121" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>35</v>
@@ -17666,17 +17666,17 @@
   </sheetData>
   <autoFilter ref="A1:L15" xr:uid="{FBE7E653-2382-46E4-9C76-9C694EDC9195}"/>
   <mergeCells count="11">
-    <mergeCell ref="L6:L10"/>
-    <mergeCell ref="K6:K10"/>
-    <mergeCell ref="H6:H10"/>
-    <mergeCell ref="I6:I10"/>
-    <mergeCell ref="J6:J10"/>
     <mergeCell ref="G6:G10"/>
     <mergeCell ref="A6:A10"/>
     <mergeCell ref="B6:B10"/>
     <mergeCell ref="C6:C10"/>
     <mergeCell ref="E6:E10"/>
     <mergeCell ref="F6:F10"/>
+    <mergeCell ref="L6:L10"/>
+    <mergeCell ref="K6:K10"/>
+    <mergeCell ref="H6:H10"/>
+    <mergeCell ref="I6:I10"/>
+    <mergeCell ref="J6:J10"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F6 F11:F15">
     <cfRule type="cellIs" dxfId="127" priority="7" operator="equal">
@@ -17820,7 +17820,7 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="92.4">
@@ -17837,7 +17837,7 @@
         <v>152</v>
       </c>
       <c r="E2" s="82" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>35</v>
@@ -17855,7 +17855,7 @@
         <v>37</v>
       </c>
       <c r="K2" s="107" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="L2" s="186"/>
     </row>
@@ -17893,7 +17893,7 @@
     </row>
     <row r="4" spans="1:12" ht="92.25" customHeight="1">
       <c r="A4" s="121" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B4" s="35" t="s">
         <v>176</v>
@@ -17905,7 +17905,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="194" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="F4" s="124" t="s">
         <v>17</v>
@@ -18043,7 +18043,7 @@
         <v>16</v>
       </c>
       <c r="E8" s="82" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="F8" s="124" t="s">
         <v>35</v>
@@ -18061,25 +18061,25 @@
         <v>37</v>
       </c>
       <c r="K8" s="107" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="L8" s="107"/>
     </row>
     <row r="9" spans="1:12" ht="43.2">
       <c r="A9" s="125" t="s">
+        <v>524</v>
+      </c>
+      <c r="B9" s="74" t="s">
         <v>525</v>
       </c>
-      <c r="B9" s="74" t="s">
+      <c r="C9" s="125" t="s">
         <v>526</v>
-      </c>
-      <c r="C9" s="125" t="s">
-        <v>527</v>
       </c>
       <c r="D9" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E9" s="212" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="F9" s="127" t="s">
         <v>35</v>
@@ -18097,25 +18097,25 @@
         <v>37</v>
       </c>
       <c r="K9" s="106" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="L9" s="129"/>
     </row>
     <row r="10" spans="1:12" ht="43.2">
       <c r="A10" s="121" t="s">
+        <v>529</v>
+      </c>
+      <c r="B10" s="35" t="s">
         <v>530</v>
       </c>
-      <c r="B10" s="35" t="s">
+      <c r="C10" s="121" t="s">
         <v>531</v>
-      </c>
-      <c r="C10" s="121" t="s">
-        <v>532</v>
       </c>
       <c r="D10" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="F10" s="124" t="s">
         <v>35</v>
@@ -18133,7 +18133,7 @@
         <v>37</v>
       </c>
       <c r="K10" s="106" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="L10" s="107"/>
     </row>
@@ -18155,7 +18155,7 @@
         <v>17</v>
       </c>
       <c r="G11" s="127" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="H11" s="127" t="s">
         <v>19</v>
@@ -18171,13 +18171,13 @@
     </row>
     <row r="12" spans="1:12" ht="28.8">
       <c r="A12" s="121" t="s">
+        <v>534</v>
+      </c>
+      <c r="B12" s="35" t="s">
         <v>535</v>
       </c>
-      <c r="B12" s="35" t="s">
+      <c r="C12" s="121" t="s">
         <v>536</v>
-      </c>
-      <c r="C12" s="121" t="s">
-        <v>537</v>
       </c>
       <c r="D12" s="132" t="s">
         <v>16</v>
@@ -18215,7 +18215,7 @@
         <v>16</v>
       </c>
       <c r="E13" s="126" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>35</v>
@@ -18269,19 +18269,19 @@
     </row>
     <row r="15" spans="1:12" ht="57.6">
       <c r="A15" s="125" t="s">
+        <v>538</v>
+      </c>
+      <c r="B15" s="74" t="s">
         <v>539</v>
       </c>
-      <c r="B15" s="74" t="s">
+      <c r="C15" s="125" t="s">
         <v>540</v>
-      </c>
-      <c r="C15" s="125" t="s">
-        <v>541</v>
       </c>
       <c r="D15" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E15" s="126" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>17</v>
@@ -18315,7 +18315,7 @@
         <v>85</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="F16" s="124" t="s">
         <v>17</v>
@@ -18349,7 +18349,7 @@
         <v>92</v>
       </c>
       <c r="E17" s="80" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="F17" s="127" t="s">
         <v>35</v>
@@ -18367,7 +18367,7 @@
         <v>37</v>
       </c>
       <c r="K17" s="107" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="L17" s="129"/>
     </row>
@@ -18385,7 +18385,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="35" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="F18" s="124" t="s">
         <v>17</v>
@@ -18436,7 +18436,7 @@
       </c>
       <c r="K19" s="106"/>
       <c r="L19" s="129" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="43.2">
@@ -18453,7 +18453,7 @@
         <v>16</v>
       </c>
       <c r="E20" s="35" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="F20" s="124" t="s">
         <v>35</v>
@@ -18477,19 +18477,19 @@
     </row>
     <row r="21" spans="1:12" ht="57.6">
       <c r="A21" s="125" t="s">
+        <v>548</v>
+      </c>
+      <c r="B21" s="74" t="s">
         <v>549</v>
       </c>
-      <c r="B21" s="74" t="s">
+      <c r="C21" s="125" t="s">
         <v>550</v>
-      </c>
-      <c r="C21" s="125" t="s">
-        <v>551</v>
       </c>
       <c r="D21" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E21" s="126" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>17</v>
@@ -18507,10 +18507,10 @@
         <v>29</v>
       </c>
       <c r="K21" s="107" t="s">
+        <v>552</v>
+      </c>
+      <c r="L21" s="192" t="s">
         <v>553</v>
-      </c>
-      <c r="L21" s="192" t="s">
-        <v>554</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="43.2">
@@ -18527,7 +18527,7 @@
         <v>337</v>
       </c>
       <c r="E22" s="35" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>35</v>
@@ -18561,7 +18561,7 @@
         <v>16</v>
       </c>
       <c r="E23" s="126" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>35</v>
@@ -18579,7 +18579,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="106" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="L23" s="195"/>
     </row>
@@ -19062,6 +19062,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000B1A1CF98C819F4881BB4349588D0C85" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ff8ef391852eaca4511043a54bffd4a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cfc87205-1831-4b6c-a7b4-76d40079a43e" xmlns:ns3="221af607-abea-4d5e-830c-567dcc03c0ec" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="201dd8b781da46d5daa37e3355db44fe" ns2:_="" ns3:_="">
     <xsd:import namespace="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
@@ -19304,15 +19313,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -19326,6 +19326,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19A23828-4FF7-4569-837D-B1B2C775409F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19344,14 +19352,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16D2CAB5-B21B-4A93-9D82-49FE3E36CF14}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
docs: update usage notes after legal check
</commit_message>
<xml_diff>
--- a/Documents/Metadata_CoreGenericHealth_v2.xlsx
+++ b/Documents/Metadata_CoreGenericHealth_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://healthri-my.sharepoint.com/personal/hannah_neikes_health-ri_nl/Documents/Documenten/GitHub/health-ri-metadata/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{B604F9AE-9787-411E-AB68-6C0D2821F0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75DD3E37-514C-4AE3-A673-1E268BD8AFB0}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{B604F9AE-9787-411E-AB68-6C0D2821F0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A5D35E6-B235-466B-BAC2-6DE286A26D1D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-12765" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="14" r:id="rId1"/>
@@ -583,12 +583,6 @@
     <t>If available, add URI to analytics distribution here</t>
   </si>
   <si>
-    <t>The ELI of the EHDS was published in March 2025 and can now be included as the applicable legislation mandating that the dataset has to be made public.
-For health datasets, the value must include the ELI of the EHDS Regulation (http://data.europa.eu/eli/reg/2025/327/oj).
-As multiple legislations may apply to the resource the maximum cardinality is not limited.
-While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property (also in Datasets) described the legal basis for initial collection and processing of (personal) data.</t>
-  </si>
-  <si>
     <t>code values</t>
   </si>
   <si>
@@ -841,11 +835,6 @@
     <t>https://w3c.github.io/dpv/2.0/dpv/modules/legal_basis.html#vocab-legal-basis</t>
   </si>
   <si>
-    <t>The legal basis can be provided as a value from the dpv taxonomy (see Controlled vocabulary column).
-While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property described the legal basis for initial collection and processing of (personal) data.
-Example value for this property could be: dpv:Consent</t>
-  </si>
-  <si>
     <t>dpv:LegalBasis</t>
   </si>
   <si>
@@ -989,10 +978,6 @@
   </si>
   <si>
     <t>https://w3c.github.io/dpv/2.1/dpv/#vocab-purposes</t>
-  </si>
-  <si>
-    <t>One (or many) category or sub-category of the purposes can be chosen from the taxonomy provided by dpv (see controlled vocabulary column).
-Example value could be: dpv:ResearchAndDevelopment.</t>
   </si>
   <si>
     <t>dpv:Purpose</t>
@@ -2618,6 +2603,22 @@
   </si>
   <si>
     <t>This property can be used to describe a media format in more detail than "media type" (using IANA media type) when needed. Instances of this property should use a URL from the File Type vocabulary.</t>
+  </si>
+  <si>
+    <t>The ELI of the EHDS was published in March 2025 and can now be included as the applicable legislation mandating that the dataset has to be made public.
+For health datasets, the value must include the ELI of the EHDS Regulation (http://data.europa.eu/eli/reg/2025/327/oj).
+As multiple legislations may apply to the resource the maximum cardinality is not limited. Note that the relation with other legislations is complex and is being looked into by legal experts.
+While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property (also in Datasets) described the legal basis for initial collection and processing of (personal) data.</t>
+  </si>
+  <si>
+    <t>One (or many) category or sub-category of the purposes can be chosen from the taxonomy provided by dpv (see controlled vocabulary column). Try to be as specific as possible.
+Example value could be: dpv:ResearchAndDevelopment.</t>
+  </si>
+  <si>
+    <t>The legal basis can be provided as a value from the dpv taxonomy (see Controlled vocabulary column).
+While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property described the legal basis for initial collection and processing of (personal) data.
+This property should always be filled if the data contains personal data and the applicable legislation is GDPR.
+Example value for this property could be: dpv:Consent</t>
   </si>
 </sst>
 </file>
@@ -3765,9 +3766,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3779,10 +3777,25 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3790,18 +3803,6 @@
     </xf>
     <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -7438,33 +7439,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>554</v>
+      </c>
+      <c r="M1" s="226" t="s">
+        <v>555</v>
+      </c>
+      <c r="N1" s="227" t="s">
+        <v>556</v>
+      </c>
+      <c r="O1" s="233" t="s">
         <v>557</v>
-      </c>
-      <c r="M1" s="226" t="s">
-        <v>558</v>
-      </c>
-      <c r="N1" s="227" t="s">
-        <v>559</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>560</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="72">
       <c r="A2" s="196" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="B2" s="45" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="C2" s="76" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="D2" s="196" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="197" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="F2" s="198" t="s">
         <v>35</v>
@@ -7473,7 +7474,7 @@
         <v>58</v>
       </c>
       <c r="H2" s="198" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="I2" s="160" t="s">
         <v>20</v>
@@ -7488,13 +7489,13 @@
     </row>
     <row r="3" spans="1:15" ht="28.8">
       <c r="A3" s="68" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="C3" s="77" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="D3" s="68" t="s">
         <v>16</v>
@@ -7633,36 +7634,36 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>566</v>
+      </c>
+      <c r="M1" s="220" t="s">
+        <v>567</v>
+      </c>
+      <c r="N1" s="226" t="s">
+        <v>568</v>
+      </c>
+      <c r="O1" s="230" t="s">
         <v>569</v>
       </c>
-      <c r="M1" s="220" t="s">
+      <c r="P1" s="227" t="s">
         <v>570</v>
       </c>
-      <c r="N1" s="226" t="s">
+      <c r="Q1" s="231" t="s">
         <v>571</v>
       </c>
-      <c r="O1" s="230" t="s">
+      <c r="R1" s="233" t="s">
         <v>572</v>
-      </c>
-      <c r="P1" s="227" t="s">
-        <v>573</v>
-      </c>
-      <c r="Q1" s="231" t="s">
-        <v>574</v>
-      </c>
-      <c r="R1" s="233" t="s">
-        <v>575</v>
       </c>
     </row>
     <row r="2" spans="1:18">
       <c r="A2" s="58" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="C2" s="76" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
@@ -7690,13 +7691,13 @@
     </row>
     <row r="3" spans="1:18">
       <c r="A3" s="48" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="B3" s="49" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="C3" s="77" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="D3" s="48" t="s">
         <v>16</v>
@@ -8358,33 +8359,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>579</v>
+      </c>
+      <c r="M1" s="226" t="s">
+        <v>580</v>
+      </c>
+      <c r="N1" s="227" t="s">
+        <v>581</v>
+      </c>
+      <c r="O1" s="233" t="s">
         <v>582</v>
-      </c>
-      <c r="M1" s="226" t="s">
-        <v>583</v>
-      </c>
-      <c r="N1" s="227" t="s">
-        <v>584</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>585</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="43.2">
       <c r="A2" s="84" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="C2" s="58" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>17</v>
@@ -8414,25 +8415,25 @@
     </row>
     <row r="3" spans="1:15" ht="129.6">
       <c r="A3" s="48" t="s">
+        <v>587</v>
+      </c>
+      <c r="B3" s="49" t="s">
+        <v>588</v>
+      </c>
+      <c r="C3" s="77" t="s">
+        <v>589</v>
+      </c>
+      <c r="D3" s="234" t="s">
         <v>590</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="E3" s="50" t="s">
         <v>591</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>592</v>
-      </c>
-      <c r="D3" s="234" t="s">
-        <v>593</v>
-      </c>
-      <c r="E3" s="50" t="s">
-        <v>594</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>17</v>
       </c>
       <c r="G3" s="51" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H3" s="51" t="s">
         <v>81</v>
@@ -8552,39 +8553,39 @@
         <v>10</v>
       </c>
       <c r="L1" s="218" t="s">
+        <v>592</v>
+      </c>
+      <c r="M1" s="229" t="s">
+        <v>593</v>
+      </c>
+      <c r="N1" s="228" t="s">
+        <v>594</v>
+      </c>
+      <c r="O1" s="233" t="s">
         <v>595</v>
-      </c>
-      <c r="M1" s="229" t="s">
-        <v>596</v>
-      </c>
-      <c r="N1" s="228" t="s">
-        <v>597</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="158.4">
       <c r="A2" s="84" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="C2" s="58" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="D2" s="59" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>35</v>
       </c>
       <c r="G2" s="115" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H2" s="60" t="s">
         <v>52</v>
@@ -8599,25 +8600,25 @@
     </row>
     <row r="3" spans="1:15" ht="43.2">
       <c r="A3" s="48" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="B3" s="49" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="C3" s="77" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="D3" s="116" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>35</v>
       </c>
       <c r="G3" s="51" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H3" s="51" t="s">
         <v>52</v>
@@ -8737,39 +8738,39 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>603</v>
+      </c>
+      <c r="M1" s="226" t="s">
+        <v>604</v>
+      </c>
+      <c r="N1" s="227" t="s">
+        <v>605</v>
+      </c>
+      <c r="O1" s="233" t="s">
         <v>606</v>
-      </c>
-      <c r="M1" s="226" t="s">
-        <v>607</v>
-      </c>
-      <c r="N1" s="227" t="s">
-        <v>608</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>609</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="100.8">
       <c r="A2" s="84" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="C2" s="58" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>17</v>
       </c>
       <c r="G2" s="46" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H2" s="60" t="s">
         <v>81</v>
@@ -8784,25 +8785,25 @@
     </row>
     <row r="3" spans="1:15" ht="57.6">
       <c r="A3" s="48" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="B3" s="49" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="C3" s="77" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
       <c r="D3" s="116" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>17</v>
       </c>
       <c r="G3" s="51" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H3" s="51" t="s">
         <v>81</v>
@@ -8900,7 +8901,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="56" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="E1" s="56" t="s">
         <v>4</v>
@@ -8923,13 +8924,13 @@
     </row>
     <row r="2" spans="1:10" ht="28.8">
       <c r="A2" s="63" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
       <c r="B2" s="53" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="C2" s="44" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="D2" s="43" t="s">
         <v>16</v>
@@ -8937,7 +8938,7 @@
       <c r="E2" s="45"/>
       <c r="F2" s="64"/>
       <c r="G2" s="63" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="H2" s="65" t="s">
         <v>81</v>
@@ -8951,13 +8952,13 @@
     </row>
     <row r="3" spans="1:10" ht="43.2">
       <c r="A3" s="67" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="B3" s="50" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="C3" s="49" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="D3" s="48" t="s">
         <v>16</v>
@@ -8965,10 +8966,10 @@
       <c r="E3" s="50"/>
       <c r="F3" s="68"/>
       <c r="G3" s="69" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="H3" s="48" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="I3" s="69" t="s">
         <v>20</v>
@@ -8979,13 +8980,13 @@
     </row>
     <row r="4" spans="1:10" ht="43.2">
       <c r="A4" s="63" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="B4" s="53" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="C4" s="44" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
       <c r="D4" s="43" t="s">
         <v>16</v>
@@ -8993,10 +8994,10 @@
       <c r="E4" s="53"/>
       <c r="F4" s="64"/>
       <c r="G4" s="63" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="H4" s="65" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="I4" s="66" t="s">
         <v>20</v>
@@ -9007,26 +9008,26 @@
     </row>
     <row r="5" spans="1:10" ht="43.2">
       <c r="A5" s="67" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="B5" s="50" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="C5" s="49" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
       <c r="D5" s="48" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="49" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="F5" s="68"/>
       <c r="G5" s="67" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="H5" s="48" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="I5" s="69" t="s">
         <v>20</v>
@@ -9037,13 +9038,13 @@
     </row>
     <row r="6" spans="1:10" ht="28.8">
       <c r="A6" s="63" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="B6" s="73" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="C6" s="44" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="D6" s="43" t="s">
         <v>16</v>
@@ -9054,7 +9055,7 @@
         <v>98</v>
       </c>
       <c r="H6" s="65" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="I6" s="66" t="s">
         <v>20</v>
@@ -9065,13 +9066,13 @@
     </row>
     <row r="7" spans="1:10" ht="28.8">
       <c r="A7" s="67" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="B7" s="50" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="C7" s="49" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="D7" s="48" t="s">
         <v>16</v>
@@ -9093,23 +9094,23 @@
     </row>
     <row r="8" spans="1:10" ht="86.4">
       <c r="A8" s="63" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="B8" s="53" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="C8" s="44" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="D8" s="43" t="s">
         <v>16</v>
       </c>
       <c r="E8" s="71" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="F8" s="47"/>
       <c r="G8" s="63" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="H8" s="65">
         <v>1</v>
@@ -9123,13 +9124,13 @@
     </row>
     <row r="9" spans="1:10" ht="28.8">
       <c r="A9" s="67" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="B9" s="50" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="C9" s="49" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="D9" s="48" t="s">
         <v>16</v>
@@ -9137,7 +9138,7 @@
       <c r="E9" s="50"/>
       <c r="F9" s="68"/>
       <c r="G9" s="69" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="H9" s="48" t="s">
         <v>81</v>
@@ -9151,23 +9152,23 @@
     </row>
     <row r="10" spans="1:10" ht="28.8">
       <c r="A10" s="63" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="B10" s="72" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="C10" s="44" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="D10" s="43" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="72" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="F10" s="64"/>
       <c r="G10" s="63" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="H10" s="65" t="s">
         <v>19</v>
@@ -9632,36 +9633,36 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="M1" s="226" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="N1" s="233" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="72">
       <c r="A2" s="44" t="s">
+        <v>658</v>
+      </c>
+      <c r="B2" s="57" t="s">
+        <v>659</v>
+      </c>
+      <c r="C2" s="58" t="s">
+        <v>660</v>
+      </c>
+      <c r="D2" s="78" t="s">
         <v>661</v>
       </c>
-      <c r="B2" s="57" t="s">
+      <c r="E2" s="197" t="s">
         <v>662</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>663</v>
-      </c>
-      <c r="D2" s="78" t="s">
-        <v>664</v>
-      </c>
-      <c r="E2" s="197" t="s">
-        <v>665</v>
       </c>
       <c r="F2" s="46" t="s">
         <v>35</v>
       </c>
       <c r="G2" s="204" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
       <c r="H2" s="47">
         <v>1</v>
@@ -9675,13 +9676,13 @@
     </row>
     <row r="3" spans="1:14" ht="71.25" customHeight="1">
       <c r="A3" s="49" t="s">
-        <v>667</v>
+        <v>664</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
       <c r="C3" s="48" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="D3" s="50" t="s">
         <v>16</v>
@@ -9691,7 +9692,7 @@
         <v>35</v>
       </c>
       <c r="G3" s="51" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="H3" s="52">
         <v>1</v>
@@ -10605,107 +10606,107 @@
       <c r="M7" s="129"/>
     </row>
     <row r="8" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A8" s="237" t="s">
+      <c r="A8" s="236" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="238" t="s">
+      <c r="B8" s="237" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="237" t="s">
+      <c r="C8" s="236" t="s">
         <v>62</v>
       </c>
       <c r="D8" s="213" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="239" t="s">
+      <c r="E8" s="238" t="s">
         <v>64</v>
       </c>
-      <c r="F8" s="236" t="s">
+      <c r="F8" s="235" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="236" t="s">
+      <c r="G8" s="235" t="s">
         <v>65</v>
       </c>
-      <c r="H8" s="236" t="s">
+      <c r="H8" s="235" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="235" t="s">
+      <c r="I8" s="239" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="235" t="s">
+      <c r="J8" s="239" t="s">
         <v>66</v>
       </c>
       <c r="K8" s="137"/>
-      <c r="L8" s="235"/>
-      <c r="M8" s="235"/>
+      <c r="L8" s="239"/>
+      <c r="M8" s="239"/>
     </row>
     <row r="9" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A9" s="237"/>
-      <c r="B9" s="238"/>
-      <c r="C9" s="237"/>
+      <c r="A9" s="236"/>
+      <c r="B9" s="237"/>
+      <c r="C9" s="236"/>
       <c r="D9" s="214" t="s">
         <v>67</v>
       </c>
-      <c r="E9" s="239"/>
-      <c r="F9" s="236"/>
-      <c r="G9" s="236"/>
-      <c r="H9" s="236"/>
-      <c r="I9" s="235"/>
-      <c r="J9" s="235"/>
+      <c r="E9" s="238"/>
+      <c r="F9" s="235"/>
+      <c r="G9" s="235"/>
+      <c r="H9" s="235"/>
+      <c r="I9" s="239"/>
+      <c r="J9" s="239"/>
       <c r="K9" s="137"/>
-      <c r="L9" s="235"/>
-      <c r="M9" s="235"/>
+      <c r="L9" s="239"/>
+      <c r="M9" s="239"/>
     </row>
     <row r="10" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A10" s="237"/>
-      <c r="B10" s="238"/>
-      <c r="C10" s="237"/>
+      <c r="A10" s="236"/>
+      <c r="B10" s="237"/>
+      <c r="C10" s="236"/>
       <c r="D10" s="214" t="s">
         <v>68</v>
       </c>
-      <c r="E10" s="239"/>
-      <c r="F10" s="236"/>
-      <c r="G10" s="236"/>
-      <c r="H10" s="236"/>
-      <c r="I10" s="235"/>
-      <c r="J10" s="235"/>
+      <c r="E10" s="238"/>
+      <c r="F10" s="235"/>
+      <c r="G10" s="235"/>
+      <c r="H10" s="235"/>
+      <c r="I10" s="239"/>
+      <c r="J10" s="239"/>
       <c r="K10" s="137"/>
-      <c r="L10" s="235"/>
-      <c r="M10" s="235"/>
+      <c r="L10" s="239"/>
+      <c r="M10" s="239"/>
     </row>
     <row r="11" spans="1:13" ht="14.4" customHeight="1">
-      <c r="A11" s="237"/>
-      <c r="B11" s="238"/>
-      <c r="C11" s="237"/>
+      <c r="A11" s="236"/>
+      <c r="B11" s="237"/>
+      <c r="C11" s="236"/>
       <c r="D11" s="152" t="s">
         <v>69</v>
       </c>
-      <c r="E11" s="239"/>
-      <c r="F11" s="236"/>
-      <c r="G11" s="236"/>
-      <c r="H11" s="236"/>
-      <c r="I11" s="235"/>
-      <c r="J11" s="235"/>
+      <c r="E11" s="238"/>
+      <c r="F11" s="235"/>
+      <c r="G11" s="235"/>
+      <c r="H11" s="235"/>
+      <c r="I11" s="239"/>
+      <c r="J11" s="239"/>
       <c r="K11" s="153"/>
-      <c r="L11" s="235"/>
-      <c r="M11" s="235"/>
+      <c r="L11" s="239"/>
+      <c r="M11" s="239"/>
     </row>
     <row r="12" spans="1:13" ht="14.4" customHeight="1">
-      <c r="A12" s="237"/>
-      <c r="B12" s="238"/>
-      <c r="C12" s="237"/>
+      <c r="A12" s="236"/>
+      <c r="B12" s="237"/>
+      <c r="C12" s="236"/>
       <c r="D12" s="152" t="s">
         <v>70</v>
       </c>
-      <c r="E12" s="239"/>
-      <c r="F12" s="236"/>
-      <c r="G12" s="236"/>
-      <c r="H12" s="236"/>
-      <c r="I12" s="235"/>
-      <c r="J12" s="235"/>
+      <c r="E12" s="238"/>
+      <c r="F12" s="235"/>
+      <c r="G12" s="235"/>
+      <c r="H12" s="235"/>
+      <c r="I12" s="239"/>
+      <c r="J12" s="239"/>
       <c r="K12" s="137"/>
-      <c r="L12" s="235"/>
-      <c r="M12" s="235"/>
+      <c r="L12" s="239"/>
+      <c r="M12" s="239"/>
     </row>
     <row r="13" spans="1:13" ht="43.2">
       <c r="A13" s="125" t="s">
@@ -10830,7 +10831,7 @@
         <v>92</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>673</v>
+        <v>670</v>
       </c>
       <c r="F16" s="124" t="s">
         <v>17</v>
@@ -11524,17 +11525,17 @@
     <sortCondition ref="A2:A24"/>
   </sortState>
   <mergeCells count="11">
+    <mergeCell ref="M8:M12"/>
+    <mergeCell ref="L8:L12"/>
+    <mergeCell ref="H8:H12"/>
+    <mergeCell ref="I8:I12"/>
+    <mergeCell ref="J8:J12"/>
     <mergeCell ref="G8:G12"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="B8:B12"/>
     <mergeCell ref="C8:C12"/>
     <mergeCell ref="E8:E12"/>
     <mergeCell ref="F8:F12"/>
-    <mergeCell ref="M8:M12"/>
-    <mergeCell ref="L8:L12"/>
-    <mergeCell ref="H8:H12"/>
-    <mergeCell ref="I8:I12"/>
-    <mergeCell ref="J8:J12"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F8">
     <cfRule type="cellIs" dxfId="190" priority="16" operator="equal">
@@ -11792,7 +11793,7 @@
       <c r="M3" s="129"/>
       <c r="N3" s="129"/>
     </row>
-    <row r="4" spans="1:14" s="117" customFormat="1" ht="144">
+    <row r="4" spans="1:14" s="117" customFormat="1" ht="158.4">
       <c r="A4" s="131" t="s">
         <v>13</v>
       </c>
@@ -11806,7 +11807,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="132" t="s">
-        <v>162</v>
+        <v>672</v>
       </c>
       <c r="F4" s="124" t="s">
         <v>35</v>
@@ -11830,25 +11831,25 @@
     </row>
     <row r="5" spans="1:14" ht="57.6">
       <c r="A5" s="125" t="s">
+        <v>162</v>
+      </c>
+      <c r="B5" s="74" t="s">
         <v>163</v>
       </c>
-      <c r="B5" s="74" t="s">
+      <c r="C5" s="134" t="s">
         <v>164</v>
-      </c>
-      <c r="C5" s="134" t="s">
-        <v>165</v>
       </c>
       <c r="D5" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="126" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F5" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G5" s="127" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H5" s="127" t="s">
         <v>19</v>
@@ -11860,7 +11861,7 @@
         <v>66</v>
       </c>
       <c r="K5" s="130" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="L5" s="129"/>
       <c r="M5" s="129"/>
@@ -11868,25 +11869,25 @@
     </row>
     <row r="6" spans="1:14" ht="28.8">
       <c r="A6" s="121" t="s">
+        <v>168</v>
+      </c>
+      <c r="B6" s="35" t="s">
         <v>169</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="C6" s="121" t="s">
         <v>170</v>
-      </c>
-      <c r="C6" s="121" t="s">
-        <v>171</v>
       </c>
       <c r="D6" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="132" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F6" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G6" s="124" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H6" s="124" t="s">
         <v>19</v>
@@ -11898,31 +11899,31 @@
         <v>66</v>
       </c>
       <c r="K6" s="106" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="L6" s="107"/>
     </row>
     <row r="7" spans="1:14" ht="43.2">
       <c r="A7" s="125" t="s">
+        <v>174</v>
+      </c>
+      <c r="B7" s="74" t="s">
         <v>175</v>
       </c>
-      <c r="B7" s="74" t="s">
+      <c r="C7" s="125" t="s">
         <v>176</v>
-      </c>
-      <c r="C7" s="125" t="s">
-        <v>177</v>
       </c>
       <c r="D7" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E7" s="74" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F7" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G7" s="127" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H7" s="127" t="s">
         <v>19</v>
@@ -11934,7 +11935,7 @@
         <v>66</v>
       </c>
       <c r="K7" s="130" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="L7" s="129"/>
       <c r="M7" s="129"/>
@@ -11972,7 +11973,7 @@
         <v>37</v>
       </c>
       <c r="K8" s="106" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="L8" s="107" t="s">
         <v>39</v>
@@ -11998,7 +11999,7 @@
         <v>16</v>
       </c>
       <c r="E9" s="74" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F9" s="127" t="s">
         <v>35</v>
@@ -12016,7 +12017,7 @@
         <v>37</v>
       </c>
       <c r="K9" s="130" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="L9" s="129" t="s">
         <v>46</v>
@@ -12042,7 +12043,7 @@
         <v>16</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F10" s="124" t="s">
         <v>35</v>
@@ -12066,19 +12067,19 @@
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="125" t="s">
+        <v>183</v>
+      </c>
+      <c r="B11" s="74" t="s">
         <v>184</v>
       </c>
-      <c r="B11" s="74" t="s">
+      <c r="C11" s="125" t="s">
         <v>185</v>
-      </c>
-      <c r="C11" s="125" t="s">
-        <v>186</v>
       </c>
       <c r="D11" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E11" s="140" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F11" s="127" t="s">
         <v>17</v>
@@ -12097,30 +12098,30 @@
       </c>
       <c r="K11" s="130"/>
       <c r="L11" s="129" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="M11" s="129" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="N11" s="129" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="28.8">
       <c r="A12" s="121" t="s">
+        <v>188</v>
+      </c>
+      <c r="B12" s="35" t="s">
         <v>189</v>
       </c>
-      <c r="B12" s="35" t="s">
+      <c r="C12" s="121" t="s">
         <v>190</v>
-      </c>
-      <c r="C12" s="121" t="s">
-        <v>191</v>
       </c>
       <c r="D12" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E12" s="132" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F12" s="124" t="s">
         <v>17</v>
@@ -12138,31 +12139,31 @@
         <v>66</v>
       </c>
       <c r="K12" s="106" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="L12" s="107"/>
     </row>
     <row r="13" spans="1:14" ht="69.75" customHeight="1">
       <c r="A13" s="125" t="s">
+        <v>193</v>
+      </c>
+      <c r="B13" s="74" t="s">
         <v>194</v>
       </c>
-      <c r="B13" s="74" t="s">
+      <c r="C13" s="125" t="s">
         <v>195</v>
       </c>
-      <c r="C13" s="125" t="s">
+      <c r="D13" s="142" t="s">
         <v>196</v>
       </c>
-      <c r="D13" s="142" t="s">
+      <c r="E13" s="80" t="s">
         <v>197</v>
-      </c>
-      <c r="E13" s="80" t="s">
-        <v>198</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G13" s="127" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H13" s="127" t="s">
         <v>81</v>
@@ -12174,125 +12175,125 @@
         <v>66</v>
       </c>
       <c r="K13" s="130" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="L13" s="129"/>
       <c r="M13" s="129"/>
       <c r="N13" s="129"/>
     </row>
     <row r="14" spans="1:14" ht="43.2">
-      <c r="A14" s="237" t="s">
+      <c r="A14" s="236" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="241" t="s">
+      <c r="B14" s="240" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="237" t="s">
+      <c r="C14" s="236" t="s">
         <v>62</v>
       </c>
       <c r="D14" s="213" t="s">
         <v>63</v>
       </c>
-      <c r="E14" s="239" t="s">
-        <v>200</v>
-      </c>
-      <c r="F14" s="236" t="s">
+      <c r="E14" s="238" t="s">
+        <v>199</v>
+      </c>
+      <c r="F14" s="235" t="s">
         <v>17</v>
       </c>
-      <c r="G14" s="236" t="s">
+      <c r="G14" s="235" t="s">
         <v>65</v>
       </c>
-      <c r="H14" s="236" t="s">
+      <c r="H14" s="235" t="s">
         <v>19</v>
       </c>
-      <c r="I14" s="235" t="s">
+      <c r="I14" s="239" t="s">
         <v>20</v>
       </c>
-      <c r="J14" s="235" t="s">
+      <c r="J14" s="239" t="s">
         <v>66</v>
       </c>
-      <c r="K14" s="240"/>
-      <c r="L14" s="235"/>
+      <c r="K14" s="241"/>
+      <c r="L14" s="239"/>
     </row>
     <row r="15" spans="1:14" ht="43.2">
-      <c r="A15" s="237"/>
-      <c r="B15" s="241"/>
-      <c r="C15" s="237"/>
+      <c r="A15" s="236"/>
+      <c r="B15" s="240"/>
+      <c r="C15" s="236"/>
       <c r="D15" s="214" t="s">
         <v>67</v>
       </c>
-      <c r="E15" s="239"/>
-      <c r="F15" s="236"/>
-      <c r="G15" s="236"/>
-      <c r="H15" s="236"/>
-      <c r="I15" s="235"/>
-      <c r="J15" s="235"/>
-      <c r="K15" s="240"/>
-      <c r="L15" s="235"/>
+      <c r="E15" s="238"/>
+      <c r="F15" s="235"/>
+      <c r="G15" s="235"/>
+      <c r="H15" s="235"/>
+      <c r="I15" s="239"/>
+      <c r="J15" s="239"/>
+      <c r="K15" s="241"/>
+      <c r="L15" s="239"/>
     </row>
     <row r="16" spans="1:14" ht="28.8">
-      <c r="A16" s="237"/>
-      <c r="B16" s="241"/>
-      <c r="C16" s="237"/>
+      <c r="A16" s="236"/>
+      <c r="B16" s="240"/>
+      <c r="C16" s="236"/>
       <c r="D16" s="214" t="s">
         <v>68</v>
       </c>
-      <c r="E16" s="239"/>
-      <c r="F16" s="236"/>
-      <c r="G16" s="236"/>
-      <c r="H16" s="236"/>
-      <c r="I16" s="235"/>
-      <c r="J16" s="235"/>
-      <c r="K16" s="240"/>
-      <c r="L16" s="235"/>
+      <c r="E16" s="238"/>
+      <c r="F16" s="235"/>
+      <c r="G16" s="235"/>
+      <c r="H16" s="235"/>
+      <c r="I16" s="239"/>
+      <c r="J16" s="239"/>
+      <c r="K16" s="241"/>
+      <c r="L16" s="239"/>
     </row>
     <row r="17" spans="1:14">
-      <c r="A17" s="237"/>
-      <c r="B17" s="241"/>
-      <c r="C17" s="237"/>
+      <c r="A17" s="236"/>
+      <c r="B17" s="240"/>
+      <c r="C17" s="236"/>
       <c r="D17" s="152" t="s">
         <v>69</v>
       </c>
-      <c r="E17" s="239"/>
-      <c r="F17" s="236"/>
-      <c r="G17" s="236"/>
-      <c r="H17" s="236"/>
-      <c r="I17" s="235"/>
-      <c r="J17" s="235"/>
-      <c r="K17" s="240"/>
-      <c r="L17" s="235"/>
+      <c r="E17" s="238"/>
+      <c r="F17" s="235"/>
+      <c r="G17" s="235"/>
+      <c r="H17" s="235"/>
+      <c r="I17" s="239"/>
+      <c r="J17" s="239"/>
+      <c r="K17" s="241"/>
+      <c r="L17" s="239"/>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="237"/>
-      <c r="B18" s="241"/>
-      <c r="C18" s="237"/>
+      <c r="A18" s="236"/>
+      <c r="B18" s="240"/>
+      <c r="C18" s="236"/>
       <c r="D18" s="152" t="s">
         <v>70</v>
       </c>
-      <c r="E18" s="239"/>
-      <c r="F18" s="236"/>
-      <c r="G18" s="236"/>
-      <c r="H18" s="236"/>
-      <c r="I18" s="235"/>
-      <c r="J18" s="235"/>
-      <c r="K18" s="240"/>
-      <c r="L18" s="235"/>
+      <c r="E18" s="238"/>
+      <c r="F18" s="235"/>
+      <c r="G18" s="235"/>
+      <c r="H18" s="235"/>
+      <c r="I18" s="239"/>
+      <c r="J18" s="239"/>
+      <c r="K18" s="241"/>
+      <c r="L18" s="239"/>
     </row>
     <row r="19" spans="1:14" ht="28.8">
       <c r="A19" s="125" t="s">
+        <v>200</v>
+      </c>
+      <c r="B19" s="74" t="s">
         <v>201</v>
       </c>
-      <c r="B19" s="74" t="s">
+      <c r="C19" s="125" t="s">
         <v>202</v>
-      </c>
-      <c r="C19" s="125" t="s">
-        <v>203</v>
       </c>
       <c r="D19" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E19" s="80" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F19" s="127" t="s">
         <v>17</v>
@@ -12310,35 +12311,35 @@
         <v>29</v>
       </c>
       <c r="K19" s="207" t="s">
+        <v>204</v>
+      </c>
+      <c r="L19" s="134" t="s">
         <v>205</v>
-      </c>
-      <c r="L19" s="134" t="s">
-        <v>206</v>
       </c>
       <c r="M19" s="129"/>
       <c r="N19" s="129"/>
     </row>
     <row r="20" spans="1:14" ht="86.4">
       <c r="A20" s="121" t="s">
+        <v>206</v>
+      </c>
+      <c r="B20" s="35" t="s">
         <v>207</v>
       </c>
-      <c r="B20" s="35" t="s">
+      <c r="C20" s="121" t="s">
         <v>208</v>
-      </c>
-      <c r="C20" s="121" t="s">
-        <v>209</v>
       </c>
       <c r="D20" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E20" s="79" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F20" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G20" s="124" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H20" s="124" t="s">
         <v>19</v>
@@ -12350,25 +12351,25 @@
         <v>66</v>
       </c>
       <c r="K20" s="106" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L20" s="107"/>
     </row>
     <row r="21" spans="1:14" ht="100.8">
       <c r="A21" s="125" t="s">
+        <v>211</v>
+      </c>
+      <c r="B21" s="74" t="s">
         <v>212</v>
       </c>
-      <c r="B21" s="74" t="s">
+      <c r="C21" s="125" t="s">
         <v>213</v>
-      </c>
-      <c r="C21" s="125" t="s">
-        <v>214</v>
       </c>
       <c r="D21" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E21" s="208" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>35</v>
@@ -12386,7 +12387,7 @@
         <v>37</v>
       </c>
       <c r="K21" s="130" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="L21" s="129"/>
       <c r="M21" s="129"/>
@@ -12394,25 +12395,25 @@
     </row>
     <row r="22" spans="1:14">
       <c r="A22" s="121" t="s">
+        <v>216</v>
+      </c>
+      <c r="B22" s="35" t="s">
         <v>217</v>
       </c>
-      <c r="B22" s="35" t="s">
+      <c r="C22" s="121" t="s">
         <v>218</v>
-      </c>
-      <c r="C22" s="121" t="s">
-        <v>219</v>
       </c>
       <c r="D22" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E22" s="132" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G22" s="128" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H22" s="124" t="s">
         <v>19</v>
@@ -12425,30 +12426,30 @@
       </c>
       <c r="K22" s="106"/>
       <c r="L22" s="141" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="43.2">
       <c r="A23" s="125" t="s">
+        <v>222</v>
+      </c>
+      <c r="B23" s="74" t="s">
         <v>223</v>
       </c>
-      <c r="B23" s="74" t="s">
+      <c r="C23" s="125" t="s">
         <v>224</v>
-      </c>
-      <c r="C23" s="125" t="s">
-        <v>225</v>
       </c>
       <c r="D23" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E23" s="74" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G23" s="127" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H23" s="127" t="s">
         <v>19</v>
@@ -12460,7 +12461,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="207" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="L23" s="129"/>
       <c r="M23" s="129"/>
@@ -12468,19 +12469,19 @@
     </row>
     <row r="24" spans="1:14" ht="43.2">
       <c r="A24" s="121" t="s">
+        <v>228</v>
+      </c>
+      <c r="B24" s="35" t="s">
         <v>229</v>
       </c>
-      <c r="B24" s="35" t="s">
+      <c r="C24" s="141" t="s">
         <v>230</v>
-      </c>
-      <c r="C24" s="141" t="s">
-        <v>231</v>
       </c>
       <c r="D24" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E24" s="71" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F24" s="124" t="s">
         <v>35</v>
@@ -12498,7 +12499,7 @@
         <v>29</v>
       </c>
       <c r="K24" s="106" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="L24" s="107"/>
     </row>
@@ -12516,7 +12517,7 @@
         <v>85</v>
       </c>
       <c r="E25" s="126" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F25" s="127" t="s">
         <v>17</v>
@@ -12540,27 +12541,27 @@
       <c r="M25" s="129"/>
       <c r="N25" s="129"/>
     </row>
-    <row r="26" spans="1:14" ht="115.2">
+    <row r="26" spans="1:14" ht="144">
       <c r="A26" s="121" t="s">
+        <v>234</v>
+      </c>
+      <c r="B26" s="35" t="s">
         <v>235</v>
       </c>
-      <c r="B26" s="35" t="s">
+      <c r="C26" s="141" t="s">
         <v>236</v>
       </c>
-      <c r="C26" s="141" t="s">
+      <c r="D26" s="122" t="s">
         <v>237</v>
       </c>
-      <c r="D26" s="122" t="s">
-        <v>238</v>
-      </c>
       <c r="E26" s="132" t="s">
-        <v>239</v>
+        <v>674</v>
       </c>
       <c r="F26" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G26" s="124" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H26" s="124" t="s">
         <v>19</v>
@@ -12572,31 +12573,31 @@
         <v>66</v>
       </c>
       <c r="K26" s="106" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="L26" s="107"/>
     </row>
     <row r="27" spans="1:14" ht="43.2">
       <c r="A27" s="125" t="s">
+        <v>240</v>
+      </c>
+      <c r="B27" s="74" t="s">
+        <v>241</v>
+      </c>
+      <c r="C27" s="125" t="s">
         <v>242</v>
-      </c>
-      <c r="B27" s="74" t="s">
-        <v>243</v>
-      </c>
-      <c r="C27" s="125" t="s">
-        <v>244</v>
       </c>
       <c r="D27" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E27" s="126" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="F27" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G27" s="127" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="H27" s="127" t="s">
         <v>81</v>
@@ -12608,7 +12609,7 @@
         <v>66</v>
       </c>
       <c r="K27" s="130" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L27" s="129"/>
       <c r="M27" s="129"/>
@@ -12616,25 +12617,25 @@
     </row>
     <row r="28" spans="1:14" ht="28.8">
       <c r="A28" s="121" t="s">
+        <v>246</v>
+      </c>
+      <c r="B28" s="35" t="s">
+        <v>247</v>
+      </c>
+      <c r="C28" s="141" t="s">
         <v>248</v>
-      </c>
-      <c r="B28" s="35" t="s">
-        <v>249</v>
-      </c>
-      <c r="C28" s="141" t="s">
-        <v>250</v>
       </c>
       <c r="D28" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E28" s="132" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F28" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G28" s="124" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="H28" s="124" t="s">
         <v>81</v>
@@ -12646,7 +12647,7 @@
         <v>66</v>
       </c>
       <c r="K28" s="106" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="L28" s="107"/>
     </row>
@@ -12664,7 +12665,7 @@
         <v>16</v>
       </c>
       <c r="E29" s="74" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="F29" s="127" t="s">
         <v>17</v>
@@ -12690,25 +12691,25 @@
     </row>
     <row r="30" spans="1:14" ht="28.8">
       <c r="A30" s="121" t="s">
+        <v>252</v>
+      </c>
+      <c r="B30" s="35" t="s">
+        <v>253</v>
+      </c>
+      <c r="C30" s="121" t="s">
         <v>254</v>
-      </c>
-      <c r="B30" s="35" t="s">
-        <v>255</v>
-      </c>
-      <c r="C30" s="121" t="s">
-        <v>256</v>
       </c>
       <c r="D30" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E30" s="132" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="F30" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G30" s="124" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="H30" s="124" t="s">
         <v>81</v>
@@ -12720,31 +12721,31 @@
         <v>66</v>
       </c>
       <c r="K30" s="106" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="L30" s="107"/>
     </row>
     <row r="31" spans="1:14" ht="28.8">
       <c r="A31" s="125" t="s">
+        <v>258</v>
+      </c>
+      <c r="B31" s="74" t="s">
+        <v>259</v>
+      </c>
+      <c r="C31" s="125" t="s">
         <v>260</v>
-      </c>
-      <c r="B31" s="74" t="s">
-        <v>261</v>
-      </c>
-      <c r="C31" s="125" t="s">
-        <v>262</v>
       </c>
       <c r="D31" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E31" s="74" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="F31" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G31" s="127" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="H31" s="127" t="s">
         <v>81</v>
@@ -12756,7 +12757,7 @@
         <v>66</v>
       </c>
       <c r="K31" s="130" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="L31" s="129"/>
       <c r="M31" s="129"/>
@@ -12764,25 +12765,25 @@
     </row>
     <row r="32" spans="1:14" ht="57.6">
       <c r="A32" s="121" t="s">
+        <v>263</v>
+      </c>
+      <c r="B32" s="35" t="s">
+        <v>264</v>
+      </c>
+      <c r="C32" s="121" t="s">
         <v>265</v>
-      </c>
-      <c r="B32" s="35" t="s">
-        <v>266</v>
-      </c>
-      <c r="C32" s="121" t="s">
-        <v>267</v>
       </c>
       <c r="D32" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E32" s="132" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="F32" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G32" s="124" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="H32" s="124" t="s">
         <v>19</v>
@@ -12794,31 +12795,31 @@
         <v>29</v>
       </c>
       <c r="K32" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="L32" s="107"/>
     </row>
     <row r="33" spans="1:14" ht="57.6">
       <c r="A33" s="125" t="s">
+        <v>269</v>
+      </c>
+      <c r="B33" s="74" t="s">
+        <v>270</v>
+      </c>
+      <c r="C33" s="125" t="s">
         <v>271</v>
       </c>
-      <c r="B33" s="74" t="s">
+      <c r="D33" s="142" t="s">
         <v>272</v>
       </c>
-      <c r="C33" s="125" t="s">
+      <c r="E33" s="80" t="s">
         <v>273</v>
-      </c>
-      <c r="D33" s="142" t="s">
-        <v>274</v>
-      </c>
-      <c r="E33" s="80" t="s">
-        <v>275</v>
       </c>
       <c r="F33" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G33" s="127" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="H33" s="127" t="s">
         <v>19</v>
@@ -12830,7 +12831,7 @@
         <v>66</v>
       </c>
       <c r="K33" s="130" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="L33" s="129"/>
       <c r="M33" s="129"/>
@@ -12838,19 +12839,19 @@
     </row>
     <row r="34" spans="1:14" ht="43.2">
       <c r="A34" s="121" t="s">
+        <v>276</v>
+      </c>
+      <c r="B34" s="35" t="s">
+        <v>277</v>
+      </c>
+      <c r="C34" s="121" t="s">
         <v>278</v>
-      </c>
-      <c r="B34" s="35" t="s">
-        <v>279</v>
-      </c>
-      <c r="C34" s="121" t="s">
-        <v>280</v>
       </c>
       <c r="D34" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E34" s="132" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="F34" s="124" t="s">
         <v>17</v>
@@ -12868,7 +12869,7 @@
         <v>66</v>
       </c>
       <c r="K34" s="106" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="L34" s="107"/>
     </row>
@@ -12886,7 +12887,7 @@
         <v>16</v>
       </c>
       <c r="E35" s="205" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="F35" s="127" t="s">
         <v>35</v>
@@ -12916,27 +12917,27 @@
         <v>46</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="43.2">
+    <row r="36" spans="1:14" ht="57.6">
       <c r="A36" s="121" t="s">
+        <v>282</v>
+      </c>
+      <c r="B36" s="35" t="s">
+        <v>283</v>
+      </c>
+      <c r="C36" s="121" t="s">
         <v>284</v>
       </c>
-      <c r="B36" s="35" t="s">
+      <c r="D36" s="122" t="s">
         <v>285</v>
       </c>
-      <c r="C36" s="121" t="s">
-        <v>286</v>
-      </c>
-      <c r="D36" s="122" t="s">
-        <v>287</v>
-      </c>
       <c r="E36" s="138" t="s">
-        <v>288</v>
+        <v>673</v>
       </c>
       <c r="F36" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G36" s="124" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="H36" s="124" t="s">
         <v>19</v>
@@ -12954,25 +12955,25 @@
     </row>
     <row r="37" spans="1:14" ht="228" customHeight="1">
       <c r="A37" s="125" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="B37" s="74" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="C37" s="134" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="D37" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E37" s="126" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="F37" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G37" s="128" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="H37" s="127" t="s">
         <v>19</v>
@@ -12985,36 +12986,36 @@
       </c>
       <c r="K37" s="130"/>
       <c r="L37" s="129" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="M37" s="129" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="N37" s="129" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
     <row r="38" spans="1:14" ht="57.6">
       <c r="A38" s="121" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="B38" s="35" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C38" s="121" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="D38" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E38" s="132" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="F38" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G38" s="128" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="H38" s="124" t="s">
         <v>19</v>
@@ -13029,36 +13030,36 @@
         <v>136</v>
       </c>
       <c r="L38" s="107" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="M38" s="107" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="N38" s="107" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="43.2">
       <c r="A39" s="125" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="B39" s="74" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="C39" s="125" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="D39" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E39" s="126" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="F39" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G39" s="128" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="H39" s="127" t="s">
         <v>19</v>
@@ -13071,13 +13072,13 @@
       </c>
       <c r="K39" s="130"/>
       <c r="L39" s="129" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="M39" s="129" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="N39" s="129" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
     </row>
     <row r="40" spans="1:14" ht="28.8">
@@ -13094,7 +13095,7 @@
         <v>16</v>
       </c>
       <c r="E40" s="132" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F40" s="124" t="s">
         <v>17</v>
@@ -13118,19 +13119,19 @@
     </row>
     <row r="41" spans="1:14" ht="28.8">
       <c r="A41" s="125" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B41" s="74" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C41" s="125" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="D41" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E41" s="74" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="F41" s="127" t="s">
         <v>17</v>
@@ -13151,30 +13152,30 @@
         <v>137</v>
       </c>
       <c r="L41" s="129" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="M41" s="129" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="N41" s="129" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="42" spans="1:14" ht="72">
       <c r="A42" s="121" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="B42" s="35" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="C42" s="121" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D42" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E42" s="132" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="F42" s="124" t="s">
         <v>17</v>
@@ -13195,26 +13196,26 @@
         <v>138</v>
       </c>
       <c r="L42" s="141" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="M42" s="107"/>
       <c r="N42" s="107"/>
     </row>
     <row r="43" spans="1:14" ht="28.8">
       <c r="A43" s="125" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="B43" s="74" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="C43" s="125" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="D43" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E43" s="205" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="F43" s="127" t="s">
         <v>17</v>
@@ -13235,32 +13236,32 @@
         <v>139</v>
       </c>
       <c r="L43" s="134" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="M43" s="129"/>
       <c r="N43" s="129"/>
     </row>
     <row r="44" spans="1:14" ht="57.6">
       <c r="A44" s="121" t="s">
+        <v>321</v>
+      </c>
+      <c r="B44" s="35" t="s">
+        <v>322</v>
+      </c>
+      <c r="C44" s="121" t="s">
+        <v>323</v>
+      </c>
+      <c r="D44" s="143" t="s">
         <v>324</v>
       </c>
-      <c r="B44" s="35" t="s">
+      <c r="E44" s="132" t="s">
         <v>325</v>
-      </c>
-      <c r="C44" s="121" t="s">
-        <v>326</v>
-      </c>
-      <c r="D44" s="143" t="s">
-        <v>327</v>
-      </c>
-      <c r="E44" s="132" t="s">
-        <v>328</v>
       </c>
       <c r="F44" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G44" s="124" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H44" s="124" t="s">
         <v>81</v>
@@ -13292,7 +13293,7 @@
         <v>16</v>
       </c>
       <c r="E45" s="74" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="F45" s="127" t="s">
         <v>17</v>
@@ -13313,36 +13314,36 @@
         <v>125</v>
       </c>
       <c r="L45" s="129" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="M45" s="129" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="N45" s="129" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="46" spans="1:14" ht="57.6">
       <c r="A46" s="121" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="B46" s="35" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="C46" s="141" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="D46" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E46" s="132" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="F46" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G46" s="124" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="H46" s="124" t="s">
         <v>81</v>
@@ -13362,25 +13363,25 @@
     </row>
     <row r="47" spans="1:14" ht="74.25" customHeight="1">
       <c r="A47" s="125" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="B47" s="74" t="s">
         <v>127</v>
       </c>
       <c r="C47" s="125" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="D47" s="142" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="E47" s="74" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="F47" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G47" s="127" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H47" s="127" t="s">
         <v>52</v>
@@ -13412,7 +13413,7 @@
         <v>16</v>
       </c>
       <c r="E48" s="132" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="F48" s="124" t="s">
         <v>35</v>
@@ -13438,25 +13439,25 @@
     </row>
     <row r="49" spans="1:14" ht="57.6">
       <c r="A49" s="125" t="s">
+        <v>337</v>
+      </c>
+      <c r="B49" s="74" t="s">
+        <v>338</v>
+      </c>
+      <c r="C49" s="125" t="s">
+        <v>339</v>
+      </c>
+      <c r="D49" s="217" t="s">
         <v>340</v>
       </c>
-      <c r="B49" s="74" t="s">
+      <c r="E49" s="83" t="s">
         <v>341</v>
-      </c>
-      <c r="C49" s="125" t="s">
-        <v>342</v>
-      </c>
-      <c r="D49" s="217" t="s">
-        <v>343</v>
-      </c>
-      <c r="E49" s="83" t="s">
-        <v>344</v>
       </c>
       <c r="F49" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G49" s="127" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H49" s="127" t="s">
         <v>19</v>
@@ -13476,19 +13477,19 @@
     </row>
     <row r="50" spans="1:14" ht="28.8">
       <c r="A50" s="121" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="B50" s="35" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="C50" s="121" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="D50" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E50" s="132" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="F50" s="124" t="s">
         <v>17</v>
@@ -13514,19 +13515,19 @@
     </row>
     <row r="51" spans="1:14" ht="28.8">
       <c r="A51" s="125" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="B51" s="74" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="C51" s="125" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="D51" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E51" s="74" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="F51" s="127" t="s">
         <v>17</v>
@@ -13552,13 +13553,13 @@
     </row>
     <row r="52" spans="1:14" ht="84.75" customHeight="1">
       <c r="A52" s="121" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="B52" s="35" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="C52" s="121" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="D52" s="132" t="s">
         <v>16</v>
@@ -13568,7 +13569,7 @@
         <v>17</v>
       </c>
       <c r="G52" s="124" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="H52" s="124" t="s">
         <v>19</v>
@@ -13604,17 +13605,17 @@
     <sortCondition ref="A2:A53"/>
   </sortState>
   <mergeCells count="11">
-    <mergeCell ref="A14:A18"/>
-    <mergeCell ref="B14:B18"/>
-    <mergeCell ref="C14:C18"/>
-    <mergeCell ref="F14:F18"/>
-    <mergeCell ref="E14:E18"/>
     <mergeCell ref="L14:L18"/>
     <mergeCell ref="K14:K18"/>
     <mergeCell ref="G14:G18"/>
     <mergeCell ref="H14:H18"/>
     <mergeCell ref="I14:I18"/>
     <mergeCell ref="J14:J18"/>
+    <mergeCell ref="A14:A18"/>
+    <mergeCell ref="B14:B18"/>
+    <mergeCell ref="C14:C18"/>
+    <mergeCell ref="F14:F18"/>
+    <mergeCell ref="E14:E18"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F14 F19:F53">
     <cfRule type="cellIs" dxfId="171" priority="8" operator="equal">
@@ -13781,42 +13782,42 @@
         <v>10</v>
       </c>
       <c r="L1" s="223" t="s">
+        <v>354</v>
+      </c>
+      <c r="M1" s="223" t="s">
+        <v>355</v>
+      </c>
+      <c r="N1" s="108" t="s">
+        <v>356</v>
+      </c>
+      <c r="O1" s="108" t="s">
         <v>357</v>
       </c>
-      <c r="M1" s="223" t="s">
+      <c r="P1" s="223" t="s">
         <v>358</v>
       </c>
-      <c r="N1" s="108" t="s">
+      <c r="Q1" s="223" t="s">
         <v>359</v>
       </c>
-      <c r="O1" s="108" t="s">
+      <c r="R1" s="224" t="s">
         <v>360</v>
       </c>
-      <c r="P1" s="223" t="s">
+      <c r="S1" s="224" t="s">
         <v>361</v>
       </c>
-      <c r="Q1" s="223" t="s">
+      <c r="T1" s="224" t="s">
         <v>362</v>
       </c>
-      <c r="R1" s="224" t="s">
+      <c r="U1" s="224" t="s">
         <v>363</v>
       </c>
-      <c r="S1" s="224" t="s">
+      <c r="V1" s="233" t="s">
         <v>364</v>
-      </c>
-      <c r="T1" s="224" t="s">
-        <v>365</v>
-      </c>
-      <c r="U1" s="224" t="s">
-        <v>366</v>
-      </c>
-      <c r="V1" s="233" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="28.8">
       <c r="A2" s="64" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="B2" s="157" t="s">
         <v>61</v>
@@ -13825,10 +13826,10 @@
         <v>62</v>
       </c>
       <c r="D2" s="152" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="E2" s="158" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="F2" s="159" t="s">
         <v>17</v>
@@ -13848,25 +13849,25 @@
     </row>
     <row r="3" spans="1:22" ht="115.2">
       <c r="A3" s="68" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="C3" s="68" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="D3" s="162" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="184" t="s">
-        <v>671</v>
+        <v>668</v>
       </c>
       <c r="F3" s="163" t="s">
         <v>35</v>
       </c>
       <c r="G3" s="163" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="H3" s="163">
         <v>1</v>
@@ -13878,7 +13879,7 @@
         <v>66</v>
       </c>
       <c r="K3" s="136" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="L3" s="129"/>
       <c r="M3" s="129"/>
@@ -13893,19 +13894,19 @@
     </row>
     <row r="4" spans="1:22" ht="129.6">
       <c r="A4" s="64" t="s">
+        <v>211</v>
+      </c>
+      <c r="B4" s="157" t="s">
         <v>212</v>
       </c>
-      <c r="B4" s="157" t="s">
+      <c r="C4" s="64" t="s">
         <v>213</v>
       </c>
-      <c r="C4" s="64" t="s">
-        <v>214</v>
-      </c>
       <c r="D4" s="71" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="E4" s="158" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="F4" s="159" t="s">
         <v>35</v>
@@ -13920,28 +13921,28 @@
         <v>28</v>
       </c>
       <c r="J4" s="160" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="K4" s="136" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="L4" s="107"/>
     </row>
     <row r="5" spans="1:22" ht="43.2">
       <c r="A5" s="165" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="B5" s="75" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="C5" s="165" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="D5" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="75" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="F5" s="166" t="s">
         <v>35</v>
@@ -13959,7 +13960,7 @@
         <v>29</v>
       </c>
       <c r="K5" s="136" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="L5" s="129"/>
       <c r="M5" s="129"/>
@@ -13974,19 +13975,19 @@
     </row>
     <row r="6" spans="1:22" ht="72">
       <c r="A6" s="168" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="B6" s="151" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="C6" s="168" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="D6" s="169" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="151" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="F6" s="133" t="s">
         <v>17</v>
@@ -14008,25 +14009,25 @@
     </row>
     <row r="7" spans="1:22" ht="115.2">
       <c r="A7" s="125" t="s">
+        <v>386</v>
+      </c>
+      <c r="B7" s="74" t="s">
+        <v>387</v>
+      </c>
+      <c r="C7" s="125" t="s">
+        <v>388</v>
+      </c>
+      <c r="D7" s="171" t="s">
         <v>389</v>
       </c>
-      <c r="B7" s="74" t="s">
+      <c r="E7" s="81" t="s">
         <v>390</v>
-      </c>
-      <c r="C7" s="125" t="s">
-        <v>391</v>
-      </c>
-      <c r="D7" s="171" t="s">
-        <v>392</v>
-      </c>
-      <c r="E7" s="81" t="s">
-        <v>393</v>
       </c>
       <c r="F7" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G7" s="127" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H7" s="127" t="s">
         <v>81</v>
@@ -14051,25 +14052,25 @@
     </row>
     <row r="8" spans="1:22" ht="28.8">
       <c r="A8" s="64" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="B8" s="157" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="C8" s="172" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="D8" s="143" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="E8" s="135" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="F8" s="159" t="s">
         <v>17</v>
       </c>
       <c r="G8" s="159" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H8" s="159" t="s">
         <v>81</v>
@@ -14081,13 +14082,13 @@
         <v>29</v>
       </c>
       <c r="K8" s="136" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="L8" s="107"/>
     </row>
     <row r="9" spans="1:22" ht="43.2">
       <c r="A9" s="165" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="B9" s="75" t="s">
         <v>77</v>
@@ -14099,13 +14100,13 @@
         <v>16</v>
       </c>
       <c r="E9" s="173" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="F9" s="166" t="s">
         <v>35</v>
       </c>
       <c r="G9" s="166" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H9" s="166">
         <v>1</v>
@@ -14117,7 +14118,7 @@
         <v>66</v>
       </c>
       <c r="K9" s="136" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="L9" s="129"/>
       <c r="M9" s="129"/>
@@ -14862,45 +14863,45 @@
         <v>10</v>
       </c>
       <c r="L1" s="225" t="s">
+        <v>396</v>
+      </c>
+      <c r="M1" s="108" t="s">
+        <v>397</v>
+      </c>
+      <c r="N1" s="223" t="s">
+        <v>398</v>
+      </c>
+      <c r="O1" s="224" t="s">
         <v>399</v>
       </c>
-      <c r="M1" s="108" t="s">
+      <c r="P1" s="232" t="s">
         <v>400</v>
       </c>
-      <c r="N1" s="223" t="s">
+      <c r="Q1" s="233" t="s">
         <v>401</v>
-      </c>
-      <c r="O1" s="224" t="s">
-        <v>402</v>
-      </c>
-      <c r="P1" s="232" t="s">
-        <v>403</v>
-      </c>
-      <c r="Q1" s="233" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="64.349999999999994" customHeight="1">
       <c r="A2" s="64" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="B2" s="45" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="C2" s="172" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="D2" s="64" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="88" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="F2" s="159" t="s">
         <v>17</v>
       </c>
       <c r="G2" s="159" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="H2" s="159" t="s">
         <v>19</v>
@@ -14912,31 +14913,31 @@
         <v>29</v>
       </c>
       <c r="K2" s="156" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="L2" s="136"/>
     </row>
     <row r="3" spans="1:17" ht="129.6">
       <c r="A3" s="68" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="C3" s="68" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="D3" s="183" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="184" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
       <c r="F3" s="163" t="s">
         <v>35</v>
       </c>
       <c r="G3" s="163" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="H3" s="163">
         <v>1</v>
@@ -14948,7 +14949,7 @@
         <v>29</v>
       </c>
       <c r="K3" s="156" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="L3" s="75"/>
       <c r="M3" s="61"/>
@@ -14958,25 +14959,25 @@
     </row>
     <row r="4" spans="1:17" ht="28.8">
       <c r="A4" s="64" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="B4" s="45" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="C4" s="64" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="D4" s="64" t="s">
         <v>16</v>
       </c>
       <c r="E4" s="88" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="F4" s="159" t="s">
         <v>35</v>
       </c>
       <c r="G4" s="159" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="H4" s="159">
         <v>1</v>
@@ -14988,7 +14989,7 @@
         <v>29</v>
       </c>
       <c r="K4" s="156" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="L4" s="136"/>
     </row>
@@ -15811,27 +15812,27 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="M1" s="223" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="28.8">
       <c r="A2" s="121" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="B2" s="35" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="C2" s="121" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="D2" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="35" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>17</v>
@@ -15849,36 +15850,36 @@
         <v>37</v>
       </c>
       <c r="K2" s="98" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="L2" s="141" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="M2" s="141" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="72">
       <c r="A3" s="125" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="B3" s="74" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="C3" s="125" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="D3" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="85" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="F3" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G3" s="127" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H3" s="127">
         <v>1</v>
@@ -15890,7 +15891,7 @@
         <v>37</v>
       </c>
       <c r="K3" s="98" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="L3" s="129"/>
       <c r="M3" s="129"/>
@@ -15909,7 +15910,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="35" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="F4" s="124" t="s">
         <v>17</v>
@@ -15934,25 +15935,25 @@
     </row>
     <row r="5" spans="1:13" ht="43.2">
       <c r="A5" s="125" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="B5" s="74" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="C5" s="134" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="D5" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="126" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="F5" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G5" s="127" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="H5" s="127">
         <v>1</v>
@@ -15964,32 +15965,32 @@
         <v>29</v>
       </c>
       <c r="K5" s="98" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="L5" s="129"/>
       <c r="M5" s="129"/>
     </row>
     <row r="6" spans="1:13" ht="57.6">
       <c r="A6" s="121" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="C6" s="121" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="D6" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="35" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="F6" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G6" s="128" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="H6" s="124" t="s">
         <v>81</v>
@@ -16001,36 +16002,36 @@
         <v>29</v>
       </c>
       <c r="K6" s="98" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="L6" s="107" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="M6" s="107" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="43.2">
       <c r="A7" s="125" t="s">
+        <v>444</v>
+      </c>
+      <c r="B7" s="74" t="s">
+        <v>445</v>
+      </c>
+      <c r="C7" s="134" t="s">
+        <v>446</v>
+      </c>
+      <c r="D7" s="185" t="s">
         <v>447</v>
       </c>
-      <c r="B7" s="74" t="s">
+      <c r="E7" s="126" t="s">
         <v>448</v>
-      </c>
-      <c r="C7" s="134" t="s">
-        <v>449</v>
-      </c>
-      <c r="D7" s="185" t="s">
-        <v>450</v>
-      </c>
-      <c r="E7" s="126" t="s">
-        <v>451</v>
       </c>
       <c r="F7" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G7" s="156" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="H7" s="127" t="s">
         <v>81</v>
@@ -16042,7 +16043,7 @@
         <v>29</v>
       </c>
       <c r="K7" s="98" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="L7" s="129"/>
       <c r="M7" s="129"/>
@@ -16061,7 +16062,7 @@
         <v>16</v>
       </c>
       <c r="E8" s="35" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="F8" s="124" t="s">
         <v>17</v>
@@ -16079,26 +16080,26 @@
         <v>29</v>
       </c>
       <c r="K8" s="98" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="L8" s="107"/>
       <c r="M8" s="107"/>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="125" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B9" s="74" t="s">
         <v>77</v>
       </c>
       <c r="C9" s="125" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D9" s="187" t="s">
         <v>16</v>
       </c>
       <c r="E9" s="126" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="F9" s="127" t="s">
         <v>17</v>
@@ -16116,32 +16117,32 @@
         <v>29</v>
       </c>
       <c r="K9" s="98" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="L9" s="129"/>
       <c r="M9" s="129"/>
     </row>
     <row r="10" spans="1:13" ht="57.6">
       <c r="A10" s="121" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="C10" s="141" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="D10" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="F10" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G10" s="124" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H10" s="124" t="s">
         <v>81</v>
@@ -16153,32 +16154,32 @@
         <v>37</v>
       </c>
       <c r="K10" s="98" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="L10" s="107"/>
       <c r="M10" s="107"/>
     </row>
     <row r="11" spans="1:13" ht="43.2">
       <c r="A11" s="125" t="s">
+        <v>460</v>
+      </c>
+      <c r="B11" s="74" t="s">
+        <v>461</v>
+      </c>
+      <c r="C11" s="125" t="s">
+        <v>462</v>
+      </c>
+      <c r="D11" s="154" t="s">
         <v>463</v>
       </c>
-      <c r="B11" s="74" t="s">
-        <v>464</v>
-      </c>
-      <c r="C11" s="125" t="s">
-        <v>465</v>
-      </c>
-      <c r="D11" s="154" t="s">
-        <v>466</v>
-      </c>
       <c r="E11" s="126" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="F11" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G11" s="127" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="H11" s="127">
         <v>1</v>
@@ -16190,7 +16191,7 @@
         <v>29</v>
       </c>
       <c r="K11" s="99" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="L11" s="129"/>
       <c r="M11" s="129"/>
@@ -16209,7 +16210,7 @@
         <v>85</v>
       </c>
       <c r="E12" s="138" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="F12" s="124" t="s">
         <v>17</v>
@@ -16227,14 +16228,14 @@
         <v>29</v>
       </c>
       <c r="K12" s="98" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="L12" s="107"/>
       <c r="M12" s="107"/>
     </row>
     <row r="13" spans="1:13" ht="72">
       <c r="A13" s="125" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="B13" s="74" t="s">
         <v>90</v>
@@ -16246,13 +16247,13 @@
         <v>92</v>
       </c>
       <c r="E13" s="80" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G13" s="127" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="H13" s="127">
         <v>1</v>
@@ -16264,32 +16265,32 @@
         <v>37</v>
       </c>
       <c r="K13" s="98" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="L13" s="129"/>
       <c r="M13" s="129"/>
     </row>
     <row r="14" spans="1:13" ht="72">
       <c r="A14" s="121" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="B14" s="35" t="s">
+        <v>175</v>
+      </c>
+      <c r="C14" s="121" t="s">
         <v>176</v>
-      </c>
-      <c r="C14" s="121" t="s">
-        <v>177</v>
       </c>
       <c r="D14" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="F14" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G14" s="124" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H14" s="124" t="s">
         <v>19</v>
@@ -16301,32 +16302,32 @@
         <v>29</v>
       </c>
       <c r="K14" s="98" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="L14" s="107"/>
       <c r="M14" s="107"/>
     </row>
     <row r="15" spans="1:13" ht="100.8">
       <c r="A15" s="125" t="s">
+        <v>475</v>
+      </c>
+      <c r="B15" s="74" t="s">
+        <v>476</v>
+      </c>
+      <c r="C15" s="125" t="s">
+        <v>477</v>
+      </c>
+      <c r="D15" s="185" t="s">
+        <v>447</v>
+      </c>
+      <c r="E15" s="80" t="s">
         <v>478</v>
-      </c>
-      <c r="B15" s="74" t="s">
-        <v>479</v>
-      </c>
-      <c r="C15" s="125" t="s">
-        <v>480</v>
-      </c>
-      <c r="D15" s="185" t="s">
-        <v>450</v>
-      </c>
-      <c r="E15" s="80" t="s">
-        <v>481</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G15" s="127" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="H15" s="127" t="s">
         <v>81</v>
@@ -16338,7 +16339,7 @@
         <v>29</v>
       </c>
       <c r="K15" s="98" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="L15" s="129"/>
       <c r="M15" s="129"/>
@@ -16373,32 +16374,32 @@
         <v>29</v>
       </c>
       <c r="K16" s="98" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="L16" s="107"/>
       <c r="M16" s="107"/>
     </row>
     <row r="17" spans="1:13" ht="57.6">
       <c r="A17" s="125" t="s">
+        <v>481</v>
+      </c>
+      <c r="B17" s="74" t="s">
+        <v>482</v>
+      </c>
+      <c r="C17" s="125" t="s">
+        <v>483</v>
+      </c>
+      <c r="D17" s="185" t="s">
+        <v>447</v>
+      </c>
+      <c r="E17" s="74" t="s">
         <v>484</v>
-      </c>
-      <c r="B17" s="74" t="s">
-        <v>485</v>
-      </c>
-      <c r="C17" s="125" t="s">
-        <v>486</v>
-      </c>
-      <c r="D17" s="185" t="s">
-        <v>450</v>
-      </c>
-      <c r="E17" s="74" t="s">
-        <v>487</v>
       </c>
       <c r="F17" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G17" s="127" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="H17" s="127" t="s">
         <v>81</v>
@@ -16410,7 +16411,7 @@
         <v>29</v>
       </c>
       <c r="K17" s="98" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="L17" s="129"/>
       <c r="M17" s="129"/>
@@ -16429,7 +16430,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="132" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="F18" s="124" t="s">
         <v>17</v>
@@ -16447,24 +16448,24 @@
         <v>29</v>
       </c>
       <c r="K18" s="98" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="L18" s="107"/>
       <c r="M18" s="107"/>
     </row>
     <row r="19" spans="1:13" ht="28.8">
       <c r="A19" s="125" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B19" s="126" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C19" s="125" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="D19" s="126"/>
       <c r="E19" s="80" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="F19" s="127" t="s">
         <v>17</v>
@@ -16483,10 +16484,10 @@
       </c>
       <c r="K19" s="104"/>
       <c r="L19" s="129" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="M19" s="129" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="129.6">
@@ -16503,7 +16504,7 @@
         <v>16</v>
       </c>
       <c r="E20" s="79" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="F20" s="190" t="s">
         <v>35</v>
@@ -16521,32 +16522,32 @@
         <v>29</v>
       </c>
       <c r="K20" s="99" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="L20" s="107"/>
       <c r="M20" s="107"/>
     </row>
     <row r="21" spans="1:13" ht="43.2">
       <c r="A21" s="125" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="B21" s="74" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="C21" s="125" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="D21" s="154" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="E21" s="81" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G21" s="127" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H21" s="127" t="s">
         <v>81</v>
@@ -16558,32 +16559,32 @@
         <v>29</v>
       </c>
       <c r="K21" s="98" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="L21" s="129"/>
       <c r="M21" s="129"/>
     </row>
     <row r="22" spans="1:13" ht="57.6">
       <c r="A22" s="121" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="B22" s="35" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="C22" s="121" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="D22" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E22" s="132" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G22" s="124" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="H22" s="124" t="s">
         <v>81</v>
@@ -16612,7 +16613,7 @@
         <v>16</v>
       </c>
       <c r="E23" s="126" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>17</v>
@@ -16630,7 +16631,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="98" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="L23" s="129"/>
       <c r="M23" s="129"/>
@@ -17112,7 +17113,7 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -17129,7 +17130,7 @@
         <v>16</v>
       </c>
       <c r="E2" s="74" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>17</v>
@@ -17147,7 +17148,7 @@
         <v>29</v>
       </c>
       <c r="K2" s="98" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="L2" s="129"/>
     </row>
@@ -17183,7 +17184,7 @@
         <v>29</v>
       </c>
       <c r="K3" s="98" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="L3" s="107" t="s">
         <v>39</v>
@@ -17203,7 +17204,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="126" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="F4" s="127" t="s">
         <v>35</v>
@@ -17221,31 +17222,31 @@
         <v>29</v>
       </c>
       <c r="K4" s="99" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="L4" s="129"/>
     </row>
     <row r="5" spans="1:12" ht="43.2">
       <c r="A5" s="121" t="s">
+        <v>193</v>
+      </c>
+      <c r="B5" s="35" t="s">
         <v>194</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="C5" s="121" t="s">
         <v>195</v>
       </c>
-      <c r="C5" s="121" t="s">
+      <c r="D5" s="122" t="s">
         <v>196</v>
       </c>
-      <c r="D5" s="122" t="s">
-        <v>197</v>
-      </c>
       <c r="E5" s="135" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="F5" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G5" s="124" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H5" s="124" t="s">
         <v>81</v>
@@ -17260,104 +17261,104 @@
       <c r="L5" s="107"/>
     </row>
     <row r="6" spans="1:12" ht="28.8">
-      <c r="A6" s="245" t="s">
+      <c r="A6" s="243" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="246" t="s">
+      <c r="B6" s="244" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="245" t="s">
+      <c r="C6" s="243" t="s">
         <v>62</v>
       </c>
       <c r="D6" s="215" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="247" t="s">
-        <v>200</v>
-      </c>
-      <c r="F6" s="244" t="s">
+      <c r="E6" s="245" t="s">
+        <v>199</v>
+      </c>
+      <c r="F6" s="242" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="244" t="s">
+      <c r="G6" s="242" t="s">
         <v>65</v>
       </c>
-      <c r="H6" s="244" t="s">
+      <c r="H6" s="242" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="242" t="s">
+      <c r="I6" s="246" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="235" t="s">
+      <c r="J6" s="239" t="s">
         <v>66</v>
       </c>
-      <c r="K6" s="243" t="s">
-        <v>508</v>
-      </c>
-      <c r="L6" s="242"/>
+      <c r="K6" s="247" t="s">
+        <v>505</v>
+      </c>
+      <c r="L6" s="246"/>
     </row>
     <row r="7" spans="1:12" ht="28.8">
-      <c r="A7" s="245"/>
-      <c r="B7" s="246"/>
-      <c r="C7" s="245"/>
+      <c r="A7" s="243"/>
+      <c r="B7" s="244"/>
+      <c r="C7" s="243"/>
       <c r="D7" s="216" t="s">
         <v>67</v>
       </c>
-      <c r="E7" s="247"/>
-      <c r="F7" s="244"/>
-      <c r="G7" s="244"/>
-      <c r="H7" s="244"/>
-      <c r="I7" s="242"/>
-      <c r="J7" s="235"/>
-      <c r="K7" s="243"/>
-      <c r="L7" s="242"/>
+      <c r="E7" s="245"/>
+      <c r="F7" s="242"/>
+      <c r="G7" s="242"/>
+      <c r="H7" s="242"/>
+      <c r="I7" s="246"/>
+      <c r="J7" s="239"/>
+      <c r="K7" s="247"/>
+      <c r="L7" s="246"/>
     </row>
     <row r="8" spans="1:12" ht="28.8">
-      <c r="A8" s="245"/>
-      <c r="B8" s="246"/>
-      <c r="C8" s="245"/>
+      <c r="A8" s="243"/>
+      <c r="B8" s="244"/>
+      <c r="C8" s="243"/>
       <c r="D8" s="216" t="s">
         <v>68</v>
       </c>
-      <c r="E8" s="247"/>
-      <c r="F8" s="244"/>
-      <c r="G8" s="244"/>
-      <c r="H8" s="244"/>
-      <c r="I8" s="242"/>
-      <c r="J8" s="235"/>
-      <c r="K8" s="243"/>
-      <c r="L8" s="242"/>
+      <c r="E8" s="245"/>
+      <c r="F8" s="242"/>
+      <c r="G8" s="242"/>
+      <c r="H8" s="242"/>
+      <c r="I8" s="246"/>
+      <c r="J8" s="239"/>
+      <c r="K8" s="247"/>
+      <c r="L8" s="246"/>
     </row>
     <row r="9" spans="1:12">
-      <c r="A9" s="245"/>
-      <c r="B9" s="246"/>
-      <c r="C9" s="245"/>
+      <c r="A9" s="243"/>
+      <c r="B9" s="244"/>
+      <c r="C9" s="243"/>
       <c r="D9" s="139" t="s">
         <v>69</v>
       </c>
-      <c r="E9" s="247"/>
-      <c r="F9" s="244"/>
-      <c r="G9" s="244"/>
-      <c r="H9" s="244"/>
-      <c r="I9" s="242"/>
-      <c r="J9" s="235"/>
-      <c r="K9" s="243"/>
-      <c r="L9" s="242"/>
+      <c r="E9" s="245"/>
+      <c r="F9" s="242"/>
+      <c r="G9" s="242"/>
+      <c r="H9" s="242"/>
+      <c r="I9" s="246"/>
+      <c r="J9" s="239"/>
+      <c r="K9" s="247"/>
+      <c r="L9" s="246"/>
     </row>
     <row r="10" spans="1:12">
-      <c r="A10" s="245"/>
-      <c r="B10" s="246"/>
-      <c r="C10" s="245"/>
+      <c r="A10" s="243"/>
+      <c r="B10" s="244"/>
+      <c r="C10" s="243"/>
       <c r="D10" s="139" t="s">
         <v>70</v>
       </c>
-      <c r="E10" s="247"/>
-      <c r="F10" s="244"/>
-      <c r="G10" s="244"/>
-      <c r="H10" s="244"/>
-      <c r="I10" s="242"/>
-      <c r="J10" s="235"/>
-      <c r="K10" s="243"/>
-      <c r="L10" s="242"/>
+      <c r="E10" s="245"/>
+      <c r="F10" s="242"/>
+      <c r="G10" s="242"/>
+      <c r="H10" s="242"/>
+      <c r="I10" s="246"/>
+      <c r="J10" s="239"/>
+      <c r="K10" s="247"/>
+      <c r="L10" s="246"/>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="121" t="s">
@@ -17373,7 +17374,7 @@
         <v>16</v>
       </c>
       <c r="E11" s="132" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="F11" s="124" t="s">
         <v>17</v>
@@ -17391,7 +17392,7 @@
         <v>29</v>
       </c>
       <c r="K11" s="99" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="L11" s="107"/>
     </row>
@@ -17409,7 +17410,7 @@
         <v>16</v>
       </c>
       <c r="E12" s="126" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="F12" s="124" t="s">
         <v>17</v>
@@ -17427,7 +17428,7 @@
         <v>29</v>
       </c>
       <c r="K12" s="98" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="L12" s="129" t="s">
         <v>46</v>
@@ -17447,7 +17448,7 @@
         <v>16</v>
       </c>
       <c r="E13" s="132" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>17</v>
@@ -17465,7 +17466,7 @@
         <v>29</v>
       </c>
       <c r="K13" s="98" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="L13" s="107"/>
     </row>
@@ -17483,7 +17484,7 @@
         <v>16</v>
       </c>
       <c r="E14" s="126" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="F14" s="124" t="s">
         <v>17</v>
@@ -17501,10 +17502,10 @@
         <v>29</v>
       </c>
       <c r="K14" s="98" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="L14" s="129" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -17521,7 +17522,7 @@
         <v>16</v>
       </c>
       <c r="E15" s="121" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>35</v>
@@ -17666,17 +17667,17 @@
   </sheetData>
   <autoFilter ref="A1:L15" xr:uid="{FBE7E653-2382-46E4-9C76-9C694EDC9195}"/>
   <mergeCells count="11">
+    <mergeCell ref="L6:L10"/>
+    <mergeCell ref="K6:K10"/>
+    <mergeCell ref="H6:H10"/>
+    <mergeCell ref="I6:I10"/>
+    <mergeCell ref="J6:J10"/>
     <mergeCell ref="G6:G10"/>
     <mergeCell ref="A6:A10"/>
     <mergeCell ref="B6:B10"/>
     <mergeCell ref="C6:C10"/>
     <mergeCell ref="E6:E10"/>
     <mergeCell ref="F6:F10"/>
-    <mergeCell ref="L6:L10"/>
-    <mergeCell ref="K6:K10"/>
-    <mergeCell ref="H6:H10"/>
-    <mergeCell ref="I6:I10"/>
-    <mergeCell ref="J6:J10"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F6 F11:F15">
     <cfRule type="cellIs" dxfId="127" priority="7" operator="equal">
@@ -17820,7 +17821,7 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="92.4">
@@ -17837,7 +17838,7 @@
         <v>152</v>
       </c>
       <c r="E2" s="82" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>35</v>
@@ -17855,7 +17856,7 @@
         <v>37</v>
       </c>
       <c r="K2" s="107" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="L2" s="186"/>
     </row>
@@ -17893,25 +17894,25 @@
     </row>
     <row r="4" spans="1:12" ht="92.25" customHeight="1">
       <c r="A4" s="121" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="B4" s="35" t="s">
+        <v>175</v>
+      </c>
+      <c r="C4" s="121" t="s">
         <v>176</v>
-      </c>
-      <c r="C4" s="121" t="s">
-        <v>177</v>
       </c>
       <c r="D4" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E4" s="194" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="F4" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G4" s="124" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H4" s="124" t="s">
         <v>19</v>
@@ -18043,7 +18044,7 @@
         <v>16</v>
       </c>
       <c r="E8" s="82" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="F8" s="124" t="s">
         <v>35</v>
@@ -18061,31 +18062,31 @@
         <v>37</v>
       </c>
       <c r="K8" s="107" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="L8" s="107"/>
     </row>
     <row r="9" spans="1:12" ht="43.2">
       <c r="A9" s="125" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="B9" s="74" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="C9" s="125" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="D9" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E9" s="212" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="F9" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G9" s="127" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="H9" s="127">
         <v>1</v>
@@ -18097,31 +18098,31 @@
         <v>37</v>
       </c>
       <c r="K9" s="106" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="L9" s="129"/>
     </row>
     <row r="10" spans="1:12" ht="43.2">
       <c r="A10" s="121" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="C10" s="121" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="D10" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="F10" s="124" t="s">
         <v>35</v>
       </c>
       <c r="G10" s="124" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="H10" s="133">
         <v>1</v>
@@ -18133,29 +18134,29 @@
         <v>37</v>
       </c>
       <c r="K10" s="106" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="L10" s="107"/>
     </row>
     <row r="11" spans="1:12" ht="43.2">
       <c r="A11" s="125" t="s">
+        <v>460</v>
+      </c>
+      <c r="B11" s="74" t="s">
+        <v>461</v>
+      </c>
+      <c r="C11" s="134" t="s">
+        <v>462</v>
+      </c>
+      <c r="D11" s="154" t="s">
         <v>463</v>
-      </c>
-      <c r="B11" s="74" t="s">
-        <v>464</v>
-      </c>
-      <c r="C11" s="134" t="s">
-        <v>465</v>
-      </c>
-      <c r="D11" s="154" t="s">
-        <v>466</v>
       </c>
       <c r="E11" s="126"/>
       <c r="F11" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G11" s="127" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="H11" s="127" t="s">
         <v>19</v>
@@ -18171,13 +18172,13 @@
     </row>
     <row r="12" spans="1:12" ht="28.8">
       <c r="A12" s="121" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="C12" s="121" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="D12" s="132" t="s">
         <v>16</v>
@@ -18187,7 +18188,7 @@
         <v>17</v>
       </c>
       <c r="G12" s="124" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H12" s="124" t="s">
         <v>19</v>
@@ -18203,19 +18204,19 @@
     </row>
     <row r="13" spans="1:12" ht="57.6">
       <c r="A13" s="191" t="s">
+        <v>211</v>
+      </c>
+      <c r="B13" s="74" t="s">
         <v>212</v>
       </c>
-      <c r="B13" s="74" t="s">
+      <c r="C13" s="134" t="s">
         <v>213</v>
-      </c>
-      <c r="C13" s="134" t="s">
-        <v>214</v>
       </c>
       <c r="D13" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E13" s="126" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>35</v>
@@ -18237,13 +18238,13 @@
     </row>
     <row r="14" spans="1:12" ht="28.8">
       <c r="A14" s="121" t="s">
+        <v>228</v>
+      </c>
+      <c r="B14" s="35" t="s">
         <v>229</v>
       </c>
-      <c r="B14" s="35" t="s">
+      <c r="C14" s="121" t="s">
         <v>230</v>
-      </c>
-      <c r="C14" s="121" t="s">
-        <v>231</v>
       </c>
       <c r="D14" s="132" t="s">
         <v>16</v>
@@ -18269,19 +18270,19 @@
     </row>
     <row r="15" spans="1:12" ht="57.6">
       <c r="A15" s="125" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="B15" s="74" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="C15" s="125" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="D15" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E15" s="126" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>17</v>
@@ -18315,7 +18316,7 @@
         <v>85</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="F16" s="124" t="s">
         <v>17</v>
@@ -18349,7 +18350,7 @@
         <v>92</v>
       </c>
       <c r="E17" s="80" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="F17" s="127" t="s">
         <v>35</v>
@@ -18367,7 +18368,7 @@
         <v>37</v>
       </c>
       <c r="K17" s="107" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="L17" s="129"/>
     </row>
@@ -18385,7 +18386,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="35" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="F18" s="124" t="s">
         <v>17</v>
@@ -18407,13 +18408,13 @@
     </row>
     <row r="19" spans="1:12" ht="28.8">
       <c r="A19" s="125" t="s">
+        <v>263</v>
+      </c>
+      <c r="B19" s="74" t="s">
+        <v>264</v>
+      </c>
+      <c r="C19" s="134" t="s">
         <v>265</v>
-      </c>
-      <c r="B19" s="74" t="s">
-        <v>266</v>
-      </c>
-      <c r="C19" s="134" t="s">
-        <v>267</v>
       </c>
       <c r="D19" s="126" t="s">
         <v>16</v>
@@ -18423,7 +18424,7 @@
         <v>17</v>
       </c>
       <c r="G19" s="128" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="H19" s="127" t="s">
         <v>19</v>
@@ -18436,7 +18437,7 @@
       </c>
       <c r="K19" s="106"/>
       <c r="L19" s="129" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="43.2">
@@ -18453,7 +18454,7 @@
         <v>16</v>
       </c>
       <c r="E20" s="35" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="F20" s="124" t="s">
         <v>35</v>
@@ -18477,19 +18478,19 @@
     </row>
     <row r="21" spans="1:12" ht="57.6">
       <c r="A21" s="125" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="B21" s="74" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="C21" s="125" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="D21" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E21" s="126" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>17</v>
@@ -18507,33 +18508,33 @@
         <v>29</v>
       </c>
       <c r="K21" s="107" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="L21" s="192" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="43.2">
       <c r="A22" s="121" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="B22" s="35" t="s">
         <v>127</v>
       </c>
       <c r="C22" s="121" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="D22" s="143" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="E22" s="35" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>35</v>
       </c>
       <c r="G22" s="124" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H22" s="124" t="s">
         <v>52</v>
@@ -18561,7 +18562,7 @@
         <v>16</v>
       </c>
       <c r="E23" s="126" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>35</v>
@@ -18579,7 +18580,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="106" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="L23" s="195"/>
     </row>
@@ -19062,15 +19063,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000B1A1CF98C819F4881BB4349588D0C85" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ff8ef391852eaca4511043a54bffd4a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cfc87205-1831-4b6c-a7b4-76d40079a43e" xmlns:ns3="221af607-abea-4d5e-830c-567dcc03c0ec" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="201dd8b781da46d5daa37e3355db44fe" ns2:_="" ns3:_="">
     <xsd:import namespace="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
@@ -19313,6 +19305,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -19326,14 +19327,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19A23828-4FF7-4569-837D-B1B2C775409F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19352,6 +19345,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16D2CAB5-B21B-4A93-9D82-49FE3E36CF14}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
docs: Anas and bot suggestions
</commit_message>
<xml_diff>
--- a/Documents/Metadata_CoreGenericHealth_v2.xlsx
+++ b/Documents/Metadata_CoreGenericHealth_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://healthri-my.sharepoint.com/personal/hannah_neikes_health-ri_nl/Documents/Documenten/GitHub/health-ri-metadata/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{B604F9AE-9787-411E-AB68-6C0D2821F0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A5D35E6-B235-466B-BAC2-6DE286A26D1D}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="8_{B604F9AE-9787-411E-AB68-6C0D2821F0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB2FDFB2-6BD5-4989-9906-EC23F51E3B08}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-12765" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2611,14 +2611,14 @@
 While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property (also in Datasets) described the legal basis for initial collection and processing of (personal) data.</t>
   </si>
   <si>
-    <t>One (or many) category or sub-category of the purposes can be chosen from the taxonomy provided by dpv (see controlled vocabulary column). Try to be as specific as possible.
-Example value could be: dpv:ResearchAndDevelopment.</t>
-  </si>
-  <si>
     <t>The legal basis can be provided as a value from the dpv taxonomy (see Controlled vocabulary column).
 While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property described the legal basis for initial collection and processing of (personal) data.
-This property should always be filled if the data contains personal data and the applicable legislation is GDPR.
+This property should always be filled if the dataset contains personal data and the applicable legislation is GDPR.
 Example value for this property could be: dpv:Consent</t>
+  </si>
+  <si>
+    <t>One (or many) categoiesy or sub-categories of the purposes can be chosen from the taxonomy provided by dpv (see controlled vocabulary column). Try to be as specific as possible.
+Example value could be: dpv:ResearchAndDevelopment.</t>
   </si>
 </sst>
 </file>
@@ -3766,24 +3766,30 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -3797,12 +3803,6 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -10606,107 +10606,107 @@
       <c r="M7" s="129"/>
     </row>
     <row r="8" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A8" s="236" t="s">
+      <c r="A8" s="238" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="237" t="s">
+      <c r="B8" s="241" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="236" t="s">
+      <c r="C8" s="238" t="s">
         <v>62</v>
       </c>
       <c r="D8" s="213" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="238" t="s">
+      <c r="E8" s="240" t="s">
         <v>64</v>
       </c>
-      <c r="F8" s="235" t="s">
+      <c r="F8" s="237" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="235" t="s">
+      <c r="G8" s="237" t="s">
         <v>65</v>
       </c>
-      <c r="H8" s="235" t="s">
+      <c r="H8" s="237" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="239" t="s">
+      <c r="I8" s="235" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="239" t="s">
+      <c r="J8" s="235" t="s">
         <v>66</v>
       </c>
       <c r="K8" s="137"/>
-      <c r="L8" s="239"/>
-      <c r="M8" s="239"/>
+      <c r="L8" s="235"/>
+      <c r="M8" s="235"/>
     </row>
     <row r="9" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A9" s="236"/>
-      <c r="B9" s="237"/>
-      <c r="C9" s="236"/>
+      <c r="A9" s="238"/>
+      <c r="B9" s="241"/>
+      <c r="C9" s="238"/>
       <c r="D9" s="214" t="s">
         <v>67</v>
       </c>
-      <c r="E9" s="238"/>
-      <c r="F9" s="235"/>
-      <c r="G9" s="235"/>
-      <c r="H9" s="235"/>
-      <c r="I9" s="239"/>
-      <c r="J9" s="239"/>
+      <c r="E9" s="240"/>
+      <c r="F9" s="237"/>
+      <c r="G9" s="237"/>
+      <c r="H9" s="237"/>
+      <c r="I9" s="235"/>
+      <c r="J9" s="235"/>
       <c r="K9" s="137"/>
-      <c r="L9" s="239"/>
-      <c r="M9" s="239"/>
+      <c r="L9" s="235"/>
+      <c r="M9" s="235"/>
     </row>
     <row r="10" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A10" s="236"/>
-      <c r="B10" s="237"/>
-      <c r="C10" s="236"/>
+      <c r="A10" s="238"/>
+      <c r="B10" s="241"/>
+      <c r="C10" s="238"/>
       <c r="D10" s="214" t="s">
         <v>68</v>
       </c>
-      <c r="E10" s="238"/>
-      <c r="F10" s="235"/>
-      <c r="G10" s="235"/>
-      <c r="H10" s="235"/>
-      <c r="I10" s="239"/>
-      <c r="J10" s="239"/>
+      <c r="E10" s="240"/>
+      <c r="F10" s="237"/>
+      <c r="G10" s="237"/>
+      <c r="H10" s="237"/>
+      <c r="I10" s="235"/>
+      <c r="J10" s="235"/>
       <c r="K10" s="137"/>
-      <c r="L10" s="239"/>
-      <c r="M10" s="239"/>
+      <c r="L10" s="235"/>
+      <c r="M10" s="235"/>
     </row>
     <row r="11" spans="1:13" ht="14.4" customHeight="1">
-      <c r="A11" s="236"/>
-      <c r="B11" s="237"/>
-      <c r="C11" s="236"/>
+      <c r="A11" s="238"/>
+      <c r="B11" s="241"/>
+      <c r="C11" s="238"/>
       <c r="D11" s="152" t="s">
         <v>69</v>
       </c>
-      <c r="E11" s="238"/>
-      <c r="F11" s="235"/>
-      <c r="G11" s="235"/>
-      <c r="H11" s="235"/>
-      <c r="I11" s="239"/>
-      <c r="J11" s="239"/>
+      <c r="E11" s="240"/>
+      <c r="F11" s="237"/>
+      <c r="G11" s="237"/>
+      <c r="H11" s="237"/>
+      <c r="I11" s="235"/>
+      <c r="J11" s="235"/>
       <c r="K11" s="153"/>
-      <c r="L11" s="239"/>
-      <c r="M11" s="239"/>
+      <c r="L11" s="235"/>
+      <c r="M11" s="235"/>
     </row>
     <row r="12" spans="1:13" ht="14.4" customHeight="1">
-      <c r="A12" s="236"/>
-      <c r="B12" s="237"/>
-      <c r="C12" s="236"/>
+      <c r="A12" s="238"/>
+      <c r="B12" s="241"/>
+      <c r="C12" s="238"/>
       <c r="D12" s="152" t="s">
         <v>70</v>
       </c>
-      <c r="E12" s="238"/>
-      <c r="F12" s="235"/>
-      <c r="G12" s="235"/>
-      <c r="H12" s="235"/>
-      <c r="I12" s="239"/>
-      <c r="J12" s="239"/>
+      <c r="E12" s="240"/>
+      <c r="F12" s="237"/>
+      <c r="G12" s="237"/>
+      <c r="H12" s="237"/>
+      <c r="I12" s="235"/>
+      <c r="J12" s="235"/>
       <c r="K12" s="137"/>
-      <c r="L12" s="239"/>
-      <c r="M12" s="239"/>
+      <c r="L12" s="235"/>
+      <c r="M12" s="235"/>
     </row>
     <row r="13" spans="1:13" ht="43.2">
       <c r="A13" s="125" t="s">
@@ -11525,17 +11525,17 @@
     <sortCondition ref="A2:A24"/>
   </sortState>
   <mergeCells count="11">
-    <mergeCell ref="M8:M12"/>
-    <mergeCell ref="L8:L12"/>
-    <mergeCell ref="H8:H12"/>
-    <mergeCell ref="I8:I12"/>
-    <mergeCell ref="J8:J12"/>
     <mergeCell ref="G8:G12"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="B8:B12"/>
     <mergeCell ref="C8:C12"/>
     <mergeCell ref="E8:E12"/>
     <mergeCell ref="F8:F12"/>
+    <mergeCell ref="M8:M12"/>
+    <mergeCell ref="L8:L12"/>
+    <mergeCell ref="H8:H12"/>
+    <mergeCell ref="I8:I12"/>
+    <mergeCell ref="J8:J12"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F8">
     <cfRule type="cellIs" dxfId="190" priority="16" operator="equal">
@@ -12182,102 +12182,102 @@
       <c r="N13" s="129"/>
     </row>
     <row r="14" spans="1:14" ht="43.2">
-      <c r="A14" s="236" t="s">
+      <c r="A14" s="238" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="240" t="s">
+      <c r="B14" s="239" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="236" t="s">
+      <c r="C14" s="238" t="s">
         <v>62</v>
       </c>
       <c r="D14" s="213" t="s">
         <v>63</v>
       </c>
-      <c r="E14" s="238" t="s">
+      <c r="E14" s="240" t="s">
         <v>199</v>
       </c>
-      <c r="F14" s="235" t="s">
+      <c r="F14" s="237" t="s">
         <v>17</v>
       </c>
-      <c r="G14" s="235" t="s">
+      <c r="G14" s="237" t="s">
         <v>65</v>
       </c>
-      <c r="H14" s="235" t="s">
+      <c r="H14" s="237" t="s">
         <v>19</v>
       </c>
-      <c r="I14" s="239" t="s">
+      <c r="I14" s="235" t="s">
         <v>20</v>
       </c>
-      <c r="J14" s="239" t="s">
+      <c r="J14" s="235" t="s">
         <v>66</v>
       </c>
-      <c r="K14" s="241"/>
-      <c r="L14" s="239"/>
+      <c r="K14" s="236"/>
+      <c r="L14" s="235"/>
     </row>
     <row r="15" spans="1:14" ht="43.2">
-      <c r="A15" s="236"/>
-      <c r="B15" s="240"/>
-      <c r="C15" s="236"/>
+      <c r="A15" s="238"/>
+      <c r="B15" s="239"/>
+      <c r="C15" s="238"/>
       <c r="D15" s="214" t="s">
         <v>67</v>
       </c>
-      <c r="E15" s="238"/>
-      <c r="F15" s="235"/>
-      <c r="G15" s="235"/>
-      <c r="H15" s="235"/>
-      <c r="I15" s="239"/>
-      <c r="J15" s="239"/>
-      <c r="K15" s="241"/>
-      <c r="L15" s="239"/>
+      <c r="E15" s="240"/>
+      <c r="F15" s="237"/>
+      <c r="G15" s="237"/>
+      <c r="H15" s="237"/>
+      <c r="I15" s="235"/>
+      <c r="J15" s="235"/>
+      <c r="K15" s="236"/>
+      <c r="L15" s="235"/>
     </row>
     <row r="16" spans="1:14" ht="28.8">
-      <c r="A16" s="236"/>
-      <c r="B16" s="240"/>
-      <c r="C16" s="236"/>
+      <c r="A16" s="238"/>
+      <c r="B16" s="239"/>
+      <c r="C16" s="238"/>
       <c r="D16" s="214" t="s">
         <v>68</v>
       </c>
-      <c r="E16" s="238"/>
-      <c r="F16" s="235"/>
-      <c r="G16" s="235"/>
-      <c r="H16" s="235"/>
-      <c r="I16" s="239"/>
-      <c r="J16" s="239"/>
-      <c r="K16" s="241"/>
-      <c r="L16" s="239"/>
+      <c r="E16" s="240"/>
+      <c r="F16" s="237"/>
+      <c r="G16" s="237"/>
+      <c r="H16" s="237"/>
+      <c r="I16" s="235"/>
+      <c r="J16" s="235"/>
+      <c r="K16" s="236"/>
+      <c r="L16" s="235"/>
     </row>
     <row r="17" spans="1:14">
-      <c r="A17" s="236"/>
-      <c r="B17" s="240"/>
-      <c r="C17" s="236"/>
+      <c r="A17" s="238"/>
+      <c r="B17" s="239"/>
+      <c r="C17" s="238"/>
       <c r="D17" s="152" t="s">
         <v>69</v>
       </c>
-      <c r="E17" s="238"/>
-      <c r="F17" s="235"/>
-      <c r="G17" s="235"/>
-      <c r="H17" s="235"/>
-      <c r="I17" s="239"/>
-      <c r="J17" s="239"/>
-      <c r="K17" s="241"/>
-      <c r="L17" s="239"/>
+      <c r="E17" s="240"/>
+      <c r="F17" s="237"/>
+      <c r="G17" s="237"/>
+      <c r="H17" s="237"/>
+      <c r="I17" s="235"/>
+      <c r="J17" s="235"/>
+      <c r="K17" s="236"/>
+      <c r="L17" s="235"/>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="236"/>
-      <c r="B18" s="240"/>
-      <c r="C18" s="236"/>
+      <c r="A18" s="238"/>
+      <c r="B18" s="239"/>
+      <c r="C18" s="238"/>
       <c r="D18" s="152" t="s">
         <v>70</v>
       </c>
-      <c r="E18" s="238"/>
-      <c r="F18" s="235"/>
-      <c r="G18" s="235"/>
-      <c r="H18" s="235"/>
-      <c r="I18" s="239"/>
-      <c r="J18" s="239"/>
-      <c r="K18" s="241"/>
-      <c r="L18" s="239"/>
+      <c r="E18" s="240"/>
+      <c r="F18" s="237"/>
+      <c r="G18" s="237"/>
+      <c r="H18" s="237"/>
+      <c r="I18" s="235"/>
+      <c r="J18" s="235"/>
+      <c r="K18" s="236"/>
+      <c r="L18" s="235"/>
     </row>
     <row r="19" spans="1:14" ht="28.8">
       <c r="A19" s="125" t="s">
@@ -12555,7 +12555,7 @@
         <v>237</v>
       </c>
       <c r="E26" s="132" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="F26" s="124" t="s">
         <v>17</v>
@@ -12931,7 +12931,7 @@
         <v>285</v>
       </c>
       <c r="E36" s="138" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="F36" s="124" t="s">
         <v>17</v>
@@ -13605,17 +13605,17 @@
     <sortCondition ref="A2:A53"/>
   </sortState>
   <mergeCells count="11">
+    <mergeCell ref="A14:A18"/>
+    <mergeCell ref="B14:B18"/>
+    <mergeCell ref="C14:C18"/>
+    <mergeCell ref="F14:F18"/>
+    <mergeCell ref="E14:E18"/>
     <mergeCell ref="L14:L18"/>
     <mergeCell ref="K14:K18"/>
     <mergeCell ref="G14:G18"/>
     <mergeCell ref="H14:H18"/>
     <mergeCell ref="I14:I18"/>
     <mergeCell ref="J14:J18"/>
-    <mergeCell ref="A14:A18"/>
-    <mergeCell ref="B14:B18"/>
-    <mergeCell ref="C14:C18"/>
-    <mergeCell ref="F14:F18"/>
-    <mergeCell ref="E14:E18"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F14 F19:F53">
     <cfRule type="cellIs" dxfId="171" priority="8" operator="equal">
@@ -17261,104 +17261,104 @@
       <c r="L5" s="107"/>
     </row>
     <row r="6" spans="1:12" ht="28.8">
-      <c r="A6" s="243" t="s">
+      <c r="A6" s="245" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="244" t="s">
+      <c r="B6" s="246" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="243" t="s">
+      <c r="C6" s="245" t="s">
         <v>62</v>
       </c>
       <c r="D6" s="215" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="245" t="s">
+      <c r="E6" s="247" t="s">
         <v>199</v>
       </c>
-      <c r="F6" s="242" t="s">
+      <c r="F6" s="244" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="242" t="s">
+      <c r="G6" s="244" t="s">
         <v>65</v>
       </c>
-      <c r="H6" s="242" t="s">
+      <c r="H6" s="244" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="246" t="s">
+      <c r="I6" s="242" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="239" t="s">
+      <c r="J6" s="235" t="s">
         <v>66</v>
       </c>
-      <c r="K6" s="247" t="s">
+      <c r="K6" s="243" t="s">
         <v>505</v>
       </c>
-      <c r="L6" s="246"/>
+      <c r="L6" s="242"/>
     </row>
     <row r="7" spans="1:12" ht="28.8">
-      <c r="A7" s="243"/>
-      <c r="B7" s="244"/>
-      <c r="C7" s="243"/>
+      <c r="A7" s="245"/>
+      <c r="B7" s="246"/>
+      <c r="C7" s="245"/>
       <c r="D7" s="216" t="s">
         <v>67</v>
       </c>
-      <c r="E7" s="245"/>
-      <c r="F7" s="242"/>
-      <c r="G7" s="242"/>
-      <c r="H7" s="242"/>
-      <c r="I7" s="246"/>
-      <c r="J7" s="239"/>
-      <c r="K7" s="247"/>
-      <c r="L7" s="246"/>
+      <c r="E7" s="247"/>
+      <c r="F7" s="244"/>
+      <c r="G7" s="244"/>
+      <c r="H7" s="244"/>
+      <c r="I7" s="242"/>
+      <c r="J7" s="235"/>
+      <c r="K7" s="243"/>
+      <c r="L7" s="242"/>
     </row>
     <row r="8" spans="1:12" ht="28.8">
-      <c r="A8" s="243"/>
-      <c r="B8" s="244"/>
-      <c r="C8" s="243"/>
+      <c r="A8" s="245"/>
+      <c r="B8" s="246"/>
+      <c r="C8" s="245"/>
       <c r="D8" s="216" t="s">
         <v>68</v>
       </c>
-      <c r="E8" s="245"/>
-      <c r="F8" s="242"/>
-      <c r="G8" s="242"/>
-      <c r="H8" s="242"/>
-      <c r="I8" s="246"/>
-      <c r="J8" s="239"/>
-      <c r="K8" s="247"/>
-      <c r="L8" s="246"/>
+      <c r="E8" s="247"/>
+      <c r="F8" s="244"/>
+      <c r="G8" s="244"/>
+      <c r="H8" s="244"/>
+      <c r="I8" s="242"/>
+      <c r="J8" s="235"/>
+      <c r="K8" s="243"/>
+      <c r="L8" s="242"/>
     </row>
     <row r="9" spans="1:12">
-      <c r="A9" s="243"/>
-      <c r="B9" s="244"/>
-      <c r="C9" s="243"/>
+      <c r="A9" s="245"/>
+      <c r="B9" s="246"/>
+      <c r="C9" s="245"/>
       <c r="D9" s="139" t="s">
         <v>69</v>
       </c>
-      <c r="E9" s="245"/>
-      <c r="F9" s="242"/>
-      <c r="G9" s="242"/>
-      <c r="H9" s="242"/>
-      <c r="I9" s="246"/>
-      <c r="J9" s="239"/>
-      <c r="K9" s="247"/>
-      <c r="L9" s="246"/>
+      <c r="E9" s="247"/>
+      <c r="F9" s="244"/>
+      <c r="G9" s="244"/>
+      <c r="H9" s="244"/>
+      <c r="I9" s="242"/>
+      <c r="J9" s="235"/>
+      <c r="K9" s="243"/>
+      <c r="L9" s="242"/>
     </row>
     <row r="10" spans="1:12">
-      <c r="A10" s="243"/>
-      <c r="B10" s="244"/>
-      <c r="C10" s="243"/>
+      <c r="A10" s="245"/>
+      <c r="B10" s="246"/>
+      <c r="C10" s="245"/>
       <c r="D10" s="139" t="s">
         <v>70</v>
       </c>
-      <c r="E10" s="245"/>
-      <c r="F10" s="242"/>
-      <c r="G10" s="242"/>
-      <c r="H10" s="242"/>
-      <c r="I10" s="246"/>
-      <c r="J10" s="239"/>
-      <c r="K10" s="247"/>
-      <c r="L10" s="246"/>
+      <c r="E10" s="247"/>
+      <c r="F10" s="244"/>
+      <c r="G10" s="244"/>
+      <c r="H10" s="244"/>
+      <c r="I10" s="242"/>
+      <c r="J10" s="235"/>
+      <c r="K10" s="243"/>
+      <c r="L10" s="242"/>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="121" t="s">
@@ -17667,17 +17667,17 @@
   </sheetData>
   <autoFilter ref="A1:L15" xr:uid="{FBE7E653-2382-46E4-9C76-9C694EDC9195}"/>
   <mergeCells count="11">
-    <mergeCell ref="L6:L10"/>
-    <mergeCell ref="K6:K10"/>
-    <mergeCell ref="H6:H10"/>
-    <mergeCell ref="I6:I10"/>
-    <mergeCell ref="J6:J10"/>
     <mergeCell ref="G6:G10"/>
     <mergeCell ref="A6:A10"/>
     <mergeCell ref="B6:B10"/>
     <mergeCell ref="C6:C10"/>
     <mergeCell ref="E6:E10"/>
     <mergeCell ref="F6:F10"/>
+    <mergeCell ref="L6:L10"/>
+    <mergeCell ref="K6:K10"/>
+    <mergeCell ref="H6:H10"/>
+    <mergeCell ref="I6:I10"/>
+    <mergeCell ref="J6:J10"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F6 F11:F15">
     <cfRule type="cellIs" dxfId="127" priority="7" operator="equal">
@@ -19063,6 +19063,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000B1A1CF98C819F4881BB4349588D0C85" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ff8ef391852eaca4511043a54bffd4a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cfc87205-1831-4b6c-a7b4-76d40079a43e" xmlns:ns3="221af607-abea-4d5e-830c-567dcc03c0ec" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="201dd8b781da46d5daa37e3355db44fe" ns2:_="" ns3:_="">
     <xsd:import namespace="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
@@ -19305,15 +19314,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -19327,6 +19327,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19A23828-4FF7-4569-837D-B1B2C775409F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19345,14 +19353,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16D2CAB5-B21B-4A93-9D82-49FE3E36CF14}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
docs: update usage notes after legal check (#258)
* docs: update usage notes after legal check

* docs: Anas and bot suggestions
</commit_message>
<xml_diff>
--- a/Documents/Metadata_CoreGenericHealth_v2.xlsx
+++ b/Documents/Metadata_CoreGenericHealth_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://healthri-my.sharepoint.com/personal/hannah_neikes_health-ri_nl/Documents/Documenten/GitHub/health-ri-metadata/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{B604F9AE-9787-411E-AB68-6C0D2821F0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75DD3E37-514C-4AE3-A673-1E268BD8AFB0}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="8_{B604F9AE-9787-411E-AB68-6C0D2821F0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB2FDFB2-6BD5-4989-9906-EC23F51E3B08}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-12765" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="14" r:id="rId1"/>
@@ -583,12 +583,6 @@
     <t>If available, add URI to analytics distribution here</t>
   </si>
   <si>
-    <t>The ELI of the EHDS was published in March 2025 and can now be included as the applicable legislation mandating that the dataset has to be made public.
-For health datasets, the value must include the ELI of the EHDS Regulation (http://data.europa.eu/eli/reg/2025/327/oj).
-As multiple legislations may apply to the resource the maximum cardinality is not limited.
-While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property (also in Datasets) described the legal basis for initial collection and processing of (personal) data.</t>
-  </si>
-  <si>
     <t>code values</t>
   </si>
   <si>
@@ -841,11 +835,6 @@
     <t>https://w3c.github.io/dpv/2.0/dpv/modules/legal_basis.html#vocab-legal-basis</t>
   </si>
   <si>
-    <t>The legal basis can be provided as a value from the dpv taxonomy (see Controlled vocabulary column).
-While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property described the legal basis for initial collection and processing of (personal) data.
-Example value for this property could be: dpv:Consent</t>
-  </si>
-  <si>
     <t>dpv:LegalBasis</t>
   </si>
   <si>
@@ -989,10 +978,6 @@
   </si>
   <si>
     <t>https://w3c.github.io/dpv/2.1/dpv/#vocab-purposes</t>
-  </si>
-  <si>
-    <t>One (or many) category or sub-category of the purposes can be chosen from the taxonomy provided by dpv (see controlled vocabulary column).
-Example value could be: dpv:ResearchAndDevelopment.</t>
   </si>
   <si>
     <t>dpv:Purpose</t>
@@ -2618,6 +2603,22 @@
   </si>
   <si>
     <t>This property can be used to describe a media format in more detail than "media type" (using IANA media type) when needed. Instances of this property should use a URL from the File Type vocabulary.</t>
+  </si>
+  <si>
+    <t>The ELI of the EHDS was published in March 2025 and can now be included as the applicable legislation mandating that the dataset has to be made public.
+For health datasets, the value must include the ELI of the EHDS Regulation (http://data.europa.eu/eli/reg/2025/327/oj).
+As multiple legislations may apply to the resource the maximum cardinality is not limited. Note that the relation with other legislations is complex and is being looked into by legal experts.
+While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property (also in Datasets) described the legal basis for initial collection and processing of (personal) data.</t>
+  </si>
+  <si>
+    <t>The legal basis can be provided as a value from the dpv taxonomy (see Controlled vocabulary column).
+While the applicable legislation indicates which legislation mandates the publication of the dataset, the legal basis property described the legal basis for initial collection and processing of (personal) data.
+This property should always be filled if the dataset contains personal data and the applicable legislation is GDPR.
+Example value for this property could be: dpv:Consent</t>
+  </si>
+  <si>
+    <t>One (or many) categoiesy or sub-categories of the purposes can be chosen from the taxonomy provided by dpv (see controlled vocabulary column). Try to be as specific as possible.
+Example value could be: dpv:ResearchAndDevelopment.</t>
   </si>
 </sst>
 </file>
@@ -3767,22 +3768,22 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -7438,33 +7439,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>554</v>
+      </c>
+      <c r="M1" s="226" t="s">
+        <v>555</v>
+      </c>
+      <c r="N1" s="227" t="s">
+        <v>556</v>
+      </c>
+      <c r="O1" s="233" t="s">
         <v>557</v>
-      </c>
-      <c r="M1" s="226" t="s">
-        <v>558</v>
-      </c>
-      <c r="N1" s="227" t="s">
-        <v>559</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>560</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="72">
       <c r="A2" s="196" t="s">
-        <v>561</v>
+        <v>558</v>
       </c>
       <c r="B2" s="45" t="s">
-        <v>562</v>
+        <v>559</v>
       </c>
       <c r="C2" s="76" t="s">
-        <v>563</v>
+        <v>560</v>
       </c>
       <c r="D2" s="196" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="197" t="s">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="F2" s="198" t="s">
         <v>35</v>
@@ -7473,7 +7474,7 @@
         <v>58</v>
       </c>
       <c r="H2" s="198" t="s">
-        <v>565</v>
+        <v>562</v>
       </c>
       <c r="I2" s="160" t="s">
         <v>20</v>
@@ -7488,13 +7489,13 @@
     </row>
     <row r="3" spans="1:15" ht="28.8">
       <c r="A3" s="68" t="s">
-        <v>566</v>
+        <v>563</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>567</v>
+        <v>564</v>
       </c>
       <c r="C3" s="77" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="D3" s="68" t="s">
         <v>16</v>
@@ -7633,36 +7634,36 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>566</v>
+      </c>
+      <c r="M1" s="220" t="s">
+        <v>567</v>
+      </c>
+      <c r="N1" s="226" t="s">
+        <v>568</v>
+      </c>
+      <c r="O1" s="230" t="s">
         <v>569</v>
       </c>
-      <c r="M1" s="220" t="s">
+      <c r="P1" s="227" t="s">
         <v>570</v>
       </c>
-      <c r="N1" s="226" t="s">
+      <c r="Q1" s="231" t="s">
         <v>571</v>
       </c>
-      <c r="O1" s="230" t="s">
+      <c r="R1" s="233" t="s">
         <v>572</v>
-      </c>
-      <c r="P1" s="227" t="s">
-        <v>573</v>
-      </c>
-      <c r="Q1" s="231" t="s">
-        <v>574</v>
-      </c>
-      <c r="R1" s="233" t="s">
-        <v>575</v>
       </c>
     </row>
     <row r="2" spans="1:18">
       <c r="A2" s="58" t="s">
-        <v>576</v>
+        <v>573</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>577</v>
+        <v>574</v>
       </c>
       <c r="C2" s="76" t="s">
-        <v>578</v>
+        <v>575</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
@@ -7690,13 +7691,13 @@
     </row>
     <row r="3" spans="1:18">
       <c r="A3" s="48" t="s">
-        <v>579</v>
+        <v>576</v>
       </c>
       <c r="B3" s="49" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="C3" s="77" t="s">
-        <v>581</v>
+        <v>578</v>
       </c>
       <c r="D3" s="48" t="s">
         <v>16</v>
@@ -8358,33 +8359,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>579</v>
+      </c>
+      <c r="M1" s="226" t="s">
+        <v>580</v>
+      </c>
+      <c r="N1" s="227" t="s">
+        <v>581</v>
+      </c>
+      <c r="O1" s="233" t="s">
         <v>582</v>
-      </c>
-      <c r="M1" s="226" t="s">
-        <v>583</v>
-      </c>
-      <c r="N1" s="227" t="s">
-        <v>584</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>585</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="43.2">
       <c r="A2" s="84" t="s">
-        <v>586</v>
+        <v>583</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>587</v>
+        <v>584</v>
       </c>
       <c r="C2" s="58" t="s">
-        <v>588</v>
+        <v>585</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>589</v>
+        <v>586</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>17</v>
@@ -8414,25 +8415,25 @@
     </row>
     <row r="3" spans="1:15" ht="129.6">
       <c r="A3" s="48" t="s">
+        <v>587</v>
+      </c>
+      <c r="B3" s="49" t="s">
+        <v>588</v>
+      </c>
+      <c r="C3" s="77" t="s">
+        <v>589</v>
+      </c>
+      <c r="D3" s="234" t="s">
         <v>590</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="E3" s="50" t="s">
         <v>591</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>592</v>
-      </c>
-      <c r="D3" s="234" t="s">
-        <v>593</v>
-      </c>
-      <c r="E3" s="50" t="s">
-        <v>594</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>17</v>
       </c>
       <c r="G3" s="51" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H3" s="51" t="s">
         <v>81</v>
@@ -8552,39 +8553,39 @@
         <v>10</v>
       </c>
       <c r="L1" s="218" t="s">
+        <v>592</v>
+      </c>
+      <c r="M1" s="229" t="s">
+        <v>593</v>
+      </c>
+      <c r="N1" s="228" t="s">
+        <v>594</v>
+      </c>
+      <c r="O1" s="233" t="s">
         <v>595</v>
-      </c>
-      <c r="M1" s="229" t="s">
-        <v>596</v>
-      </c>
-      <c r="N1" s="228" t="s">
-        <v>597</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>598</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="158.4">
       <c r="A2" s="84" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>591</v>
+        <v>588</v>
       </c>
       <c r="C2" s="58" t="s">
-        <v>592</v>
+        <v>589</v>
       </c>
       <c r="D2" s="59" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>35</v>
       </c>
       <c r="G2" s="115" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H2" s="60" t="s">
         <v>52</v>
@@ -8599,25 +8600,25 @@
     </row>
     <row r="3" spans="1:15" ht="43.2">
       <c r="A3" s="48" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="B3" s="49" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="C3" s="77" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
       <c r="D3" s="116" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>35</v>
       </c>
       <c r="G3" s="51" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H3" s="51" t="s">
         <v>52</v>
@@ -8737,39 +8738,39 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>603</v>
+      </c>
+      <c r="M1" s="226" t="s">
+        <v>604</v>
+      </c>
+      <c r="N1" s="227" t="s">
+        <v>605</v>
+      </c>
+      <c r="O1" s="233" t="s">
         <v>606</v>
-      </c>
-      <c r="M1" s="226" t="s">
-        <v>607</v>
-      </c>
-      <c r="N1" s="227" t="s">
-        <v>608</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>609</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="100.8">
       <c r="A2" s="84" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="C2" s="58" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>17</v>
       </c>
       <c r="G2" s="46" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H2" s="60" t="s">
         <v>81</v>
@@ -8784,25 +8785,25 @@
     </row>
     <row r="3" spans="1:15" ht="57.6">
       <c r="A3" s="48" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="B3" s="49" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="C3" s="77" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
       <c r="D3" s="116" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>17</v>
       </c>
       <c r="G3" s="51" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H3" s="51" t="s">
         <v>81</v>
@@ -8900,7 +8901,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="56" t="s">
-        <v>618</v>
+        <v>615</v>
       </c>
       <c r="E1" s="56" t="s">
         <v>4</v>
@@ -8923,13 +8924,13 @@
     </row>
     <row r="2" spans="1:10" ht="28.8">
       <c r="A2" s="63" t="s">
-        <v>619</v>
+        <v>616</v>
       </c>
       <c r="B2" s="53" t="s">
-        <v>620</v>
+        <v>617</v>
       </c>
       <c r="C2" s="44" t="s">
-        <v>621</v>
+        <v>618</v>
       </c>
       <c r="D2" s="43" t="s">
         <v>16</v>
@@ -8937,7 +8938,7 @@
       <c r="E2" s="45"/>
       <c r="F2" s="64"/>
       <c r="G2" s="63" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="H2" s="65" t="s">
         <v>81</v>
@@ -8951,13 +8952,13 @@
     </row>
     <row r="3" spans="1:10" ht="43.2">
       <c r="A3" s="67" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="B3" s="50" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="C3" s="49" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="D3" s="48" t="s">
         <v>16</v>
@@ -8965,10 +8966,10 @@
       <c r="E3" s="50"/>
       <c r="F3" s="68"/>
       <c r="G3" s="69" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="H3" s="48" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="I3" s="69" t="s">
         <v>20</v>
@@ -8979,13 +8980,13 @@
     </row>
     <row r="4" spans="1:10" ht="43.2">
       <c r="A4" s="63" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="B4" s="53" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="C4" s="44" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
       <c r="D4" s="43" t="s">
         <v>16</v>
@@ -8993,10 +8994,10 @@
       <c r="E4" s="53"/>
       <c r="F4" s="64"/>
       <c r="G4" s="63" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="H4" s="65" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="I4" s="66" t="s">
         <v>20</v>
@@ -9007,26 +9008,26 @@
     </row>
     <row r="5" spans="1:10" ht="43.2">
       <c r="A5" s="67" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="B5" s="50" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="C5" s="49" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
       <c r="D5" s="48" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="49" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="F5" s="68"/>
       <c r="G5" s="67" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="H5" s="48" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="I5" s="69" t="s">
         <v>20</v>
@@ -9037,13 +9038,13 @@
     </row>
     <row r="6" spans="1:10" ht="28.8">
       <c r="A6" s="63" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="B6" s="73" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="C6" s="44" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
       <c r="D6" s="43" t="s">
         <v>16</v>
@@ -9054,7 +9055,7 @@
         <v>98</v>
       </c>
       <c r="H6" s="65" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="I6" s="66" t="s">
         <v>20</v>
@@ -9065,13 +9066,13 @@
     </row>
     <row r="7" spans="1:10" ht="28.8">
       <c r="A7" s="67" t="s">
-        <v>642</v>
+        <v>639</v>
       </c>
       <c r="B7" s="50" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="C7" s="49" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
       <c r="D7" s="48" t="s">
         <v>16</v>
@@ -9093,23 +9094,23 @@
     </row>
     <row r="8" spans="1:10" ht="86.4">
       <c r="A8" s="63" t="s">
-        <v>645</v>
+        <v>642</v>
       </c>
       <c r="B8" s="53" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="C8" s="44" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="D8" s="43" t="s">
         <v>16</v>
       </c>
       <c r="E8" s="71" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
       <c r="F8" s="47"/>
       <c r="G8" s="63" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
       <c r="H8" s="65">
         <v>1</v>
@@ -9123,13 +9124,13 @@
     </row>
     <row r="9" spans="1:10" ht="28.8">
       <c r="A9" s="67" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
       <c r="B9" s="50" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="C9" s="49" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
       <c r="D9" s="48" t="s">
         <v>16</v>
@@ -9137,7 +9138,7 @@
       <c r="E9" s="50"/>
       <c r="F9" s="68"/>
       <c r="G9" s="69" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
       <c r="H9" s="48" t="s">
         <v>81</v>
@@ -9151,23 +9152,23 @@
     </row>
     <row r="10" spans="1:10" ht="28.8">
       <c r="A10" s="63" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
       <c r="B10" s="72" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
       <c r="C10" s="44" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
       <c r="D10" s="43" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="72" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
       <c r="F10" s="64"/>
       <c r="G10" s="63" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="H10" s="65" t="s">
         <v>19</v>
@@ -9632,36 +9633,36 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
       <c r="M1" s="226" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="N1" s="233" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="72">
       <c r="A2" s="44" t="s">
+        <v>658</v>
+      </c>
+      <c r="B2" s="57" t="s">
+        <v>659</v>
+      </c>
+      <c r="C2" s="58" t="s">
+        <v>660</v>
+      </c>
+      <c r="D2" s="78" t="s">
         <v>661</v>
       </c>
-      <c r="B2" s="57" t="s">
+      <c r="E2" s="197" t="s">
         <v>662</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>663</v>
-      </c>
-      <c r="D2" s="78" t="s">
-        <v>664</v>
-      </c>
-      <c r="E2" s="197" t="s">
-        <v>665</v>
       </c>
       <c r="F2" s="46" t="s">
         <v>35</v>
       </c>
       <c r="G2" s="204" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
       <c r="H2" s="47">
         <v>1</v>
@@ -9675,13 +9676,13 @@
     </row>
     <row r="3" spans="1:14" ht="71.25" customHeight="1">
       <c r="A3" s="49" t="s">
-        <v>667</v>
+        <v>664</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>668</v>
+        <v>665</v>
       </c>
       <c r="C3" s="48" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="D3" s="50" t="s">
         <v>16</v>
@@ -9691,7 +9692,7 @@
         <v>35</v>
       </c>
       <c r="G3" s="51" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="H3" s="52">
         <v>1</v>
@@ -10605,28 +10606,28 @@
       <c r="M7" s="129"/>
     </row>
     <row r="8" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A8" s="237" t="s">
+      <c r="A8" s="238" t="s">
         <v>60</v>
       </c>
-      <c r="B8" s="238" t="s">
+      <c r="B8" s="241" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="237" t="s">
+      <c r="C8" s="238" t="s">
         <v>62</v>
       </c>
       <c r="D8" s="213" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="239" t="s">
+      <c r="E8" s="240" t="s">
         <v>64</v>
       </c>
-      <c r="F8" s="236" t="s">
+      <c r="F8" s="237" t="s">
         <v>17</v>
       </c>
-      <c r="G8" s="236" t="s">
+      <c r="G8" s="237" t="s">
         <v>65</v>
       </c>
-      <c r="H8" s="236" t="s">
+      <c r="H8" s="237" t="s">
         <v>19</v>
       </c>
       <c r="I8" s="235" t="s">
@@ -10640,16 +10641,16 @@
       <c r="M8" s="235"/>
     </row>
     <row r="9" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A9" s="237"/>
-      <c r="B9" s="238"/>
-      <c r="C9" s="237"/>
+      <c r="A9" s="238"/>
+      <c r="B9" s="241"/>
+      <c r="C9" s="238"/>
       <c r="D9" s="214" t="s">
         <v>67</v>
       </c>
-      <c r="E9" s="239"/>
-      <c r="F9" s="236"/>
-      <c r="G9" s="236"/>
-      <c r="H9" s="236"/>
+      <c r="E9" s="240"/>
+      <c r="F9" s="237"/>
+      <c r="G9" s="237"/>
+      <c r="H9" s="237"/>
       <c r="I9" s="235"/>
       <c r="J9" s="235"/>
       <c r="K9" s="137"/>
@@ -10657,16 +10658,16 @@
       <c r="M9" s="235"/>
     </row>
     <row r="10" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A10" s="237"/>
-      <c r="B10" s="238"/>
-      <c r="C10" s="237"/>
+      <c r="A10" s="238"/>
+      <c r="B10" s="241"/>
+      <c r="C10" s="238"/>
       <c r="D10" s="214" t="s">
         <v>68</v>
       </c>
-      <c r="E10" s="239"/>
-      <c r="F10" s="236"/>
-      <c r="G10" s="236"/>
-      <c r="H10" s="236"/>
+      <c r="E10" s="240"/>
+      <c r="F10" s="237"/>
+      <c r="G10" s="237"/>
+      <c r="H10" s="237"/>
       <c r="I10" s="235"/>
       <c r="J10" s="235"/>
       <c r="K10" s="137"/>
@@ -10674,16 +10675,16 @@
       <c r="M10" s="235"/>
     </row>
     <row r="11" spans="1:13" ht="14.4" customHeight="1">
-      <c r="A11" s="237"/>
-      <c r="B11" s="238"/>
-      <c r="C11" s="237"/>
+      <c r="A11" s="238"/>
+      <c r="B11" s="241"/>
+      <c r="C11" s="238"/>
       <c r="D11" s="152" t="s">
         <v>69</v>
       </c>
-      <c r="E11" s="239"/>
-      <c r="F11" s="236"/>
-      <c r="G11" s="236"/>
-      <c r="H11" s="236"/>
+      <c r="E11" s="240"/>
+      <c r="F11" s="237"/>
+      <c r="G11" s="237"/>
+      <c r="H11" s="237"/>
       <c r="I11" s="235"/>
       <c r="J11" s="235"/>
       <c r="K11" s="153"/>
@@ -10691,16 +10692,16 @@
       <c r="M11" s="235"/>
     </row>
     <row r="12" spans="1:13" ht="14.4" customHeight="1">
-      <c r="A12" s="237"/>
-      <c r="B12" s="238"/>
-      <c r="C12" s="237"/>
+      <c r="A12" s="238"/>
+      <c r="B12" s="241"/>
+      <c r="C12" s="238"/>
       <c r="D12" s="152" t="s">
         <v>70</v>
       </c>
-      <c r="E12" s="239"/>
-      <c r="F12" s="236"/>
-      <c r="G12" s="236"/>
-      <c r="H12" s="236"/>
+      <c r="E12" s="240"/>
+      <c r="F12" s="237"/>
+      <c r="G12" s="237"/>
+      <c r="H12" s="237"/>
       <c r="I12" s="235"/>
       <c r="J12" s="235"/>
       <c r="K12" s="137"/>
@@ -10830,7 +10831,7 @@
         <v>92</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>673</v>
+        <v>670</v>
       </c>
       <c r="F16" s="124" t="s">
         <v>17</v>
@@ -11792,7 +11793,7 @@
       <c r="M3" s="129"/>
       <c r="N3" s="129"/>
     </row>
-    <row r="4" spans="1:14" s="117" customFormat="1" ht="144">
+    <row r="4" spans="1:14" s="117" customFormat="1" ht="158.4">
       <c r="A4" s="131" t="s">
         <v>13</v>
       </c>
@@ -11806,7 +11807,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="132" t="s">
-        <v>162</v>
+        <v>672</v>
       </c>
       <c r="F4" s="124" t="s">
         <v>35</v>
@@ -11830,25 +11831,25 @@
     </row>
     <row r="5" spans="1:14" ht="57.6">
       <c r="A5" s="125" t="s">
+        <v>162</v>
+      </c>
+      <c r="B5" s="74" t="s">
         <v>163</v>
       </c>
-      <c r="B5" s="74" t="s">
+      <c r="C5" s="134" t="s">
         <v>164</v>
-      </c>
-      <c r="C5" s="134" t="s">
-        <v>165</v>
       </c>
       <c r="D5" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="126" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F5" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G5" s="127" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H5" s="127" t="s">
         <v>19</v>
@@ -11860,7 +11861,7 @@
         <v>66</v>
       </c>
       <c r="K5" s="130" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="L5" s="129"/>
       <c r="M5" s="129"/>
@@ -11868,25 +11869,25 @@
     </row>
     <row r="6" spans="1:14" ht="28.8">
       <c r="A6" s="121" t="s">
+        <v>168</v>
+      </c>
+      <c r="B6" s="35" t="s">
         <v>169</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="C6" s="121" t="s">
         <v>170</v>
-      </c>
-      <c r="C6" s="121" t="s">
-        <v>171</v>
       </c>
       <c r="D6" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="132" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F6" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G6" s="124" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H6" s="124" t="s">
         <v>19</v>
@@ -11898,31 +11899,31 @@
         <v>66</v>
       </c>
       <c r="K6" s="106" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="L6" s="107"/>
     </row>
     <row r="7" spans="1:14" ht="43.2">
       <c r="A7" s="125" t="s">
+        <v>174</v>
+      </c>
+      <c r="B7" s="74" t="s">
         <v>175</v>
       </c>
-      <c r="B7" s="74" t="s">
+      <c r="C7" s="125" t="s">
         <v>176</v>
-      </c>
-      <c r="C7" s="125" t="s">
-        <v>177</v>
       </c>
       <c r="D7" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E7" s="74" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F7" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G7" s="127" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H7" s="127" t="s">
         <v>19</v>
@@ -11934,7 +11935,7 @@
         <v>66</v>
       </c>
       <c r="K7" s="130" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="L7" s="129"/>
       <c r="M7" s="129"/>
@@ -11972,7 +11973,7 @@
         <v>37</v>
       </c>
       <c r="K8" s="106" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="L8" s="107" t="s">
         <v>39</v>
@@ -11998,7 +11999,7 @@
         <v>16</v>
       </c>
       <c r="E9" s="74" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F9" s="127" t="s">
         <v>35</v>
@@ -12016,7 +12017,7 @@
         <v>37</v>
       </c>
       <c r="K9" s="130" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="L9" s="129" t="s">
         <v>46</v>
@@ -12042,7 +12043,7 @@
         <v>16</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F10" s="124" t="s">
         <v>35</v>
@@ -12066,19 +12067,19 @@
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="125" t="s">
+        <v>183</v>
+      </c>
+      <c r="B11" s="74" t="s">
         <v>184</v>
       </c>
-      <c r="B11" s="74" t="s">
+      <c r="C11" s="125" t="s">
         <v>185</v>
-      </c>
-      <c r="C11" s="125" t="s">
-        <v>186</v>
       </c>
       <c r="D11" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E11" s="140" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F11" s="127" t="s">
         <v>17</v>
@@ -12097,30 +12098,30 @@
       </c>
       <c r="K11" s="130"/>
       <c r="L11" s="129" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="M11" s="129" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="N11" s="129" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="28.8">
       <c r="A12" s="121" t="s">
+        <v>188</v>
+      </c>
+      <c r="B12" s="35" t="s">
         <v>189</v>
       </c>
-      <c r="B12" s="35" t="s">
+      <c r="C12" s="121" t="s">
         <v>190</v>
-      </c>
-      <c r="C12" s="121" t="s">
-        <v>191</v>
       </c>
       <c r="D12" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E12" s="132" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F12" s="124" t="s">
         <v>17</v>
@@ -12138,31 +12139,31 @@
         <v>66</v>
       </c>
       <c r="K12" s="106" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="L12" s="107"/>
     </row>
     <row r="13" spans="1:14" ht="69.75" customHeight="1">
       <c r="A13" s="125" t="s">
+        <v>193</v>
+      </c>
+      <c r="B13" s="74" t="s">
         <v>194</v>
       </c>
-      <c r="B13" s="74" t="s">
+      <c r="C13" s="125" t="s">
         <v>195</v>
       </c>
-      <c r="C13" s="125" t="s">
+      <c r="D13" s="142" t="s">
         <v>196</v>
       </c>
-      <c r="D13" s="142" t="s">
+      <c r="E13" s="80" t="s">
         <v>197</v>
-      </c>
-      <c r="E13" s="80" t="s">
-        <v>198</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G13" s="127" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H13" s="127" t="s">
         <v>81</v>
@@ -12174,35 +12175,35 @@
         <v>66</v>
       </c>
       <c r="K13" s="130" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="L13" s="129"/>
       <c r="M13" s="129"/>
       <c r="N13" s="129"/>
     </row>
     <row r="14" spans="1:14" ht="43.2">
-      <c r="A14" s="237" t="s">
+      <c r="A14" s="238" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="241" t="s">
+      <c r="B14" s="239" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="237" t="s">
+      <c r="C14" s="238" t="s">
         <v>62</v>
       </c>
       <c r="D14" s="213" t="s">
         <v>63</v>
       </c>
-      <c r="E14" s="239" t="s">
-        <v>200</v>
-      </c>
-      <c r="F14" s="236" t="s">
+      <c r="E14" s="240" t="s">
+        <v>199</v>
+      </c>
+      <c r="F14" s="237" t="s">
         <v>17</v>
       </c>
-      <c r="G14" s="236" t="s">
+      <c r="G14" s="237" t="s">
         <v>65</v>
       </c>
-      <c r="H14" s="236" t="s">
+      <c r="H14" s="237" t="s">
         <v>19</v>
       </c>
       <c r="I14" s="235" t="s">
@@ -12211,88 +12212,88 @@
       <c r="J14" s="235" t="s">
         <v>66</v>
       </c>
-      <c r="K14" s="240"/>
+      <c r="K14" s="236"/>
       <c r="L14" s="235"/>
     </row>
     <row r="15" spans="1:14" ht="43.2">
-      <c r="A15" s="237"/>
-      <c r="B15" s="241"/>
-      <c r="C15" s="237"/>
+      <c r="A15" s="238"/>
+      <c r="B15" s="239"/>
+      <c r="C15" s="238"/>
       <c r="D15" s="214" t="s">
         <v>67</v>
       </c>
-      <c r="E15" s="239"/>
-      <c r="F15" s="236"/>
-      <c r="G15" s="236"/>
-      <c r="H15" s="236"/>
+      <c r="E15" s="240"/>
+      <c r="F15" s="237"/>
+      <c r="G15" s="237"/>
+      <c r="H15" s="237"/>
       <c r="I15" s="235"/>
       <c r="J15" s="235"/>
-      <c r="K15" s="240"/>
+      <c r="K15" s="236"/>
       <c r="L15" s="235"/>
     </row>
     <row r="16" spans="1:14" ht="28.8">
-      <c r="A16" s="237"/>
-      <c r="B16" s="241"/>
-      <c r="C16" s="237"/>
+      <c r="A16" s="238"/>
+      <c r="B16" s="239"/>
+      <c r="C16" s="238"/>
       <c r="D16" s="214" t="s">
         <v>68</v>
       </c>
-      <c r="E16" s="239"/>
-      <c r="F16" s="236"/>
-      <c r="G16" s="236"/>
-      <c r="H16" s="236"/>
+      <c r="E16" s="240"/>
+      <c r="F16" s="237"/>
+      <c r="G16" s="237"/>
+      <c r="H16" s="237"/>
       <c r="I16" s="235"/>
       <c r="J16" s="235"/>
-      <c r="K16" s="240"/>
+      <c r="K16" s="236"/>
       <c r="L16" s="235"/>
     </row>
     <row r="17" spans="1:14">
-      <c r="A17" s="237"/>
-      <c r="B17" s="241"/>
-      <c r="C17" s="237"/>
+      <c r="A17" s="238"/>
+      <c r="B17" s="239"/>
+      <c r="C17" s="238"/>
       <c r="D17" s="152" t="s">
         <v>69</v>
       </c>
-      <c r="E17" s="239"/>
-      <c r="F17" s="236"/>
-      <c r="G17" s="236"/>
-      <c r="H17" s="236"/>
+      <c r="E17" s="240"/>
+      <c r="F17" s="237"/>
+      <c r="G17" s="237"/>
+      <c r="H17" s="237"/>
       <c r="I17" s="235"/>
       <c r="J17" s="235"/>
-      <c r="K17" s="240"/>
+      <c r="K17" s="236"/>
       <c r="L17" s="235"/>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="237"/>
-      <c r="B18" s="241"/>
-      <c r="C18" s="237"/>
+      <c r="A18" s="238"/>
+      <c r="B18" s="239"/>
+      <c r="C18" s="238"/>
       <c r="D18" s="152" t="s">
         <v>70</v>
       </c>
-      <c r="E18" s="239"/>
-      <c r="F18" s="236"/>
-      <c r="G18" s="236"/>
-      <c r="H18" s="236"/>
+      <c r="E18" s="240"/>
+      <c r="F18" s="237"/>
+      <c r="G18" s="237"/>
+      <c r="H18" s="237"/>
       <c r="I18" s="235"/>
       <c r="J18" s="235"/>
-      <c r="K18" s="240"/>
+      <c r="K18" s="236"/>
       <c r="L18" s="235"/>
     </row>
     <row r="19" spans="1:14" ht="28.8">
       <c r="A19" s="125" t="s">
+        <v>200</v>
+      </c>
+      <c r="B19" s="74" t="s">
         <v>201</v>
       </c>
-      <c r="B19" s="74" t="s">
+      <c r="C19" s="125" t="s">
         <v>202</v>
-      </c>
-      <c r="C19" s="125" t="s">
-        <v>203</v>
       </c>
       <c r="D19" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E19" s="80" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F19" s="127" t="s">
         <v>17</v>
@@ -12310,35 +12311,35 @@
         <v>29</v>
       </c>
       <c r="K19" s="207" t="s">
+        <v>204</v>
+      </c>
+      <c r="L19" s="134" t="s">
         <v>205</v>
-      </c>
-      <c r="L19" s="134" t="s">
-        <v>206</v>
       </c>
       <c r="M19" s="129"/>
       <c r="N19" s="129"/>
     </row>
     <row r="20" spans="1:14" ht="86.4">
       <c r="A20" s="121" t="s">
+        <v>206</v>
+      </c>
+      <c r="B20" s="35" t="s">
         <v>207</v>
       </c>
-      <c r="B20" s="35" t="s">
+      <c r="C20" s="121" t="s">
         <v>208</v>
-      </c>
-      <c r="C20" s="121" t="s">
-        <v>209</v>
       </c>
       <c r="D20" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E20" s="79" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F20" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G20" s="124" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H20" s="124" t="s">
         <v>19</v>
@@ -12350,25 +12351,25 @@
         <v>66</v>
       </c>
       <c r="K20" s="106" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L20" s="107"/>
     </row>
     <row r="21" spans="1:14" ht="100.8">
       <c r="A21" s="125" t="s">
+        <v>211</v>
+      </c>
+      <c r="B21" s="74" t="s">
         <v>212</v>
       </c>
-      <c r="B21" s="74" t="s">
+      <c r="C21" s="125" t="s">
         <v>213</v>
-      </c>
-      <c r="C21" s="125" t="s">
-        <v>214</v>
       </c>
       <c r="D21" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E21" s="208" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>35</v>
@@ -12386,7 +12387,7 @@
         <v>37</v>
       </c>
       <c r="K21" s="130" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="L21" s="129"/>
       <c r="M21" s="129"/>
@@ -12394,25 +12395,25 @@
     </row>
     <row r="22" spans="1:14">
       <c r="A22" s="121" t="s">
+        <v>216</v>
+      </c>
+      <c r="B22" s="35" t="s">
         <v>217</v>
       </c>
-      <c r="B22" s="35" t="s">
+      <c r="C22" s="121" t="s">
         <v>218</v>
-      </c>
-      <c r="C22" s="121" t="s">
-        <v>219</v>
       </c>
       <c r="D22" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E22" s="132" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G22" s="128" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H22" s="124" t="s">
         <v>19</v>
@@ -12425,30 +12426,30 @@
       </c>
       <c r="K22" s="106"/>
       <c r="L22" s="141" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="43.2">
       <c r="A23" s="125" t="s">
+        <v>222</v>
+      </c>
+      <c r="B23" s="74" t="s">
         <v>223</v>
       </c>
-      <c r="B23" s="74" t="s">
+      <c r="C23" s="125" t="s">
         <v>224</v>
-      </c>
-      <c r="C23" s="125" t="s">
-        <v>225</v>
       </c>
       <c r="D23" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E23" s="74" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G23" s="127" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H23" s="127" t="s">
         <v>19</v>
@@ -12460,7 +12461,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="207" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="L23" s="129"/>
       <c r="M23" s="129"/>
@@ -12468,19 +12469,19 @@
     </row>
     <row r="24" spans="1:14" ht="43.2">
       <c r="A24" s="121" t="s">
+        <v>228</v>
+      </c>
+      <c r="B24" s="35" t="s">
         <v>229</v>
       </c>
-      <c r="B24" s="35" t="s">
+      <c r="C24" s="141" t="s">
         <v>230</v>
-      </c>
-      <c r="C24" s="141" t="s">
-        <v>231</v>
       </c>
       <c r="D24" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E24" s="71" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F24" s="124" t="s">
         <v>35</v>
@@ -12498,7 +12499,7 @@
         <v>29</v>
       </c>
       <c r="K24" s="106" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="L24" s="107"/>
     </row>
@@ -12516,7 +12517,7 @@
         <v>85</v>
       </c>
       <c r="E25" s="126" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F25" s="127" t="s">
         <v>17</v>
@@ -12540,27 +12541,27 @@
       <c r="M25" s="129"/>
       <c r="N25" s="129"/>
     </row>
-    <row r="26" spans="1:14" ht="115.2">
+    <row r="26" spans="1:14" ht="144">
       <c r="A26" s="121" t="s">
+        <v>234</v>
+      </c>
+      <c r="B26" s="35" t="s">
         <v>235</v>
       </c>
-      <c r="B26" s="35" t="s">
+      <c r="C26" s="141" t="s">
         <v>236</v>
       </c>
-      <c r="C26" s="141" t="s">
+      <c r="D26" s="122" t="s">
         <v>237</v>
       </c>
-      <c r="D26" s="122" t="s">
-        <v>238</v>
-      </c>
       <c r="E26" s="132" t="s">
-        <v>239</v>
+        <v>673</v>
       </c>
       <c r="F26" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G26" s="124" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H26" s="124" t="s">
         <v>19</v>
@@ -12572,31 +12573,31 @@
         <v>66</v>
       </c>
       <c r="K26" s="106" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="L26" s="107"/>
     </row>
     <row r="27" spans="1:14" ht="43.2">
       <c r="A27" s="125" t="s">
+        <v>240</v>
+      </c>
+      <c r="B27" s="74" t="s">
+        <v>241</v>
+      </c>
+      <c r="C27" s="125" t="s">
         <v>242</v>
-      </c>
-      <c r="B27" s="74" t="s">
-        <v>243</v>
-      </c>
-      <c r="C27" s="125" t="s">
-        <v>244</v>
       </c>
       <c r="D27" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E27" s="126" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="F27" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G27" s="127" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="H27" s="127" t="s">
         <v>81</v>
@@ -12608,7 +12609,7 @@
         <v>66</v>
       </c>
       <c r="K27" s="130" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="L27" s="129"/>
       <c r="M27" s="129"/>
@@ -12616,25 +12617,25 @@
     </row>
     <row r="28" spans="1:14" ht="28.8">
       <c r="A28" s="121" t="s">
+        <v>246</v>
+      </c>
+      <c r="B28" s="35" t="s">
+        <v>247</v>
+      </c>
+      <c r="C28" s="141" t="s">
         <v>248</v>
-      </c>
-      <c r="B28" s="35" t="s">
-        <v>249</v>
-      </c>
-      <c r="C28" s="141" t="s">
-        <v>250</v>
       </c>
       <c r="D28" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E28" s="132" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F28" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G28" s="124" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="H28" s="124" t="s">
         <v>81</v>
@@ -12646,7 +12647,7 @@
         <v>66</v>
       </c>
       <c r="K28" s="106" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="L28" s="107"/>
     </row>
@@ -12664,7 +12665,7 @@
         <v>16</v>
       </c>
       <c r="E29" s="74" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="F29" s="127" t="s">
         <v>17</v>
@@ -12690,25 +12691,25 @@
     </row>
     <row r="30" spans="1:14" ht="28.8">
       <c r="A30" s="121" t="s">
+        <v>252</v>
+      </c>
+      <c r="B30" s="35" t="s">
+        <v>253</v>
+      </c>
+      <c r="C30" s="121" t="s">
         <v>254</v>
-      </c>
-      <c r="B30" s="35" t="s">
-        <v>255</v>
-      </c>
-      <c r="C30" s="121" t="s">
-        <v>256</v>
       </c>
       <c r="D30" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E30" s="132" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="F30" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G30" s="124" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="H30" s="124" t="s">
         <v>81</v>
@@ -12720,31 +12721,31 @@
         <v>66</v>
       </c>
       <c r="K30" s="106" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="L30" s="107"/>
     </row>
     <row r="31" spans="1:14" ht="28.8">
       <c r="A31" s="125" t="s">
+        <v>258</v>
+      </c>
+      <c r="B31" s="74" t="s">
+        <v>259</v>
+      </c>
+      <c r="C31" s="125" t="s">
         <v>260</v>
-      </c>
-      <c r="B31" s="74" t="s">
-        <v>261</v>
-      </c>
-      <c r="C31" s="125" t="s">
-        <v>262</v>
       </c>
       <c r="D31" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E31" s="74" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="F31" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G31" s="127" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="H31" s="127" t="s">
         <v>81</v>
@@ -12756,7 +12757,7 @@
         <v>66</v>
       </c>
       <c r="K31" s="130" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="L31" s="129"/>
       <c r="M31" s="129"/>
@@ -12764,25 +12765,25 @@
     </row>
     <row r="32" spans="1:14" ht="57.6">
       <c r="A32" s="121" t="s">
+        <v>263</v>
+      </c>
+      <c r="B32" s="35" t="s">
+        <v>264</v>
+      </c>
+      <c r="C32" s="121" t="s">
         <v>265</v>
-      </c>
-      <c r="B32" s="35" t="s">
-        <v>266</v>
-      </c>
-      <c r="C32" s="121" t="s">
-        <v>267</v>
       </c>
       <c r="D32" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E32" s="132" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="F32" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G32" s="124" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="H32" s="124" t="s">
         <v>19</v>
@@ -12794,31 +12795,31 @@
         <v>29</v>
       </c>
       <c r="K32" s="106" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="L32" s="107"/>
     </row>
     <row r="33" spans="1:14" ht="57.6">
       <c r="A33" s="125" t="s">
+        <v>269</v>
+      </c>
+      <c r="B33" s="74" t="s">
+        <v>270</v>
+      </c>
+      <c r="C33" s="125" t="s">
         <v>271</v>
       </c>
-      <c r="B33" s="74" t="s">
+      <c r="D33" s="142" t="s">
         <v>272</v>
       </c>
-      <c r="C33" s="125" t="s">
+      <c r="E33" s="80" t="s">
         <v>273</v>
-      </c>
-      <c r="D33" s="142" t="s">
-        <v>274</v>
-      </c>
-      <c r="E33" s="80" t="s">
-        <v>275</v>
       </c>
       <c r="F33" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G33" s="127" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="H33" s="127" t="s">
         <v>19</v>
@@ -12830,7 +12831,7 @@
         <v>66</v>
       </c>
       <c r="K33" s="130" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="L33" s="129"/>
       <c r="M33" s="129"/>
@@ -12838,19 +12839,19 @@
     </row>
     <row r="34" spans="1:14" ht="43.2">
       <c r="A34" s="121" t="s">
+        <v>276</v>
+      </c>
+      <c r="B34" s="35" t="s">
+        <v>277</v>
+      </c>
+      <c r="C34" s="121" t="s">
         <v>278</v>
-      </c>
-      <c r="B34" s="35" t="s">
-        <v>279</v>
-      </c>
-      <c r="C34" s="121" t="s">
-        <v>280</v>
       </c>
       <c r="D34" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E34" s="132" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="F34" s="124" t="s">
         <v>17</v>
@@ -12868,7 +12869,7 @@
         <v>66</v>
       </c>
       <c r="K34" s="106" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="L34" s="107"/>
     </row>
@@ -12886,7 +12887,7 @@
         <v>16</v>
       </c>
       <c r="E35" s="205" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="F35" s="127" t="s">
         <v>35</v>
@@ -12916,27 +12917,27 @@
         <v>46</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="43.2">
+    <row r="36" spans="1:14" ht="57.6">
       <c r="A36" s="121" t="s">
+        <v>282</v>
+      </c>
+      <c r="B36" s="35" t="s">
+        <v>283</v>
+      </c>
+      <c r="C36" s="121" t="s">
         <v>284</v>
       </c>
-      <c r="B36" s="35" t="s">
+      <c r="D36" s="122" t="s">
         <v>285</v>
       </c>
-      <c r="C36" s="121" t="s">
-        <v>286</v>
-      </c>
-      <c r="D36" s="122" t="s">
-        <v>287</v>
-      </c>
       <c r="E36" s="138" t="s">
-        <v>288</v>
+        <v>674</v>
       </c>
       <c r="F36" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G36" s="124" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="H36" s="124" t="s">
         <v>19</v>
@@ -12954,25 +12955,25 @@
     </row>
     <row r="37" spans="1:14" ht="228" customHeight="1">
       <c r="A37" s="125" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="B37" s="74" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="C37" s="134" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="D37" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E37" s="126" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="F37" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G37" s="128" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="H37" s="127" t="s">
         <v>19</v>
@@ -12985,36 +12986,36 @@
       </c>
       <c r="K37" s="130"/>
       <c r="L37" s="129" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="M37" s="129" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="N37" s="129" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
     <row r="38" spans="1:14" ht="57.6">
       <c r="A38" s="121" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="B38" s="35" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C38" s="121" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="D38" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E38" s="132" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="F38" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G38" s="128" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="H38" s="124" t="s">
         <v>19</v>
@@ -13029,36 +13030,36 @@
         <v>136</v>
       </c>
       <c r="L38" s="107" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="M38" s="107" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="N38" s="107" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="43.2">
       <c r="A39" s="125" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="B39" s="74" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="C39" s="125" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="D39" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E39" s="126" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="F39" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G39" s="128" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="H39" s="127" t="s">
         <v>19</v>
@@ -13071,13 +13072,13 @@
       </c>
       <c r="K39" s="130"/>
       <c r="L39" s="129" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="M39" s="129" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="N39" s="129" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
     </row>
     <row r="40" spans="1:14" ht="28.8">
@@ -13094,7 +13095,7 @@
         <v>16</v>
       </c>
       <c r="E40" s="132" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F40" s="124" t="s">
         <v>17</v>
@@ -13118,19 +13119,19 @@
     </row>
     <row r="41" spans="1:14" ht="28.8">
       <c r="A41" s="125" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B41" s="74" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C41" s="125" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="D41" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E41" s="74" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="F41" s="127" t="s">
         <v>17</v>
@@ -13151,30 +13152,30 @@
         <v>137</v>
       </c>
       <c r="L41" s="129" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="M41" s="129" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="N41" s="129" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="42" spans="1:14" ht="72">
       <c r="A42" s="121" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="B42" s="35" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="C42" s="121" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D42" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E42" s="132" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="F42" s="124" t="s">
         <v>17</v>
@@ -13195,26 +13196,26 @@
         <v>138</v>
       </c>
       <c r="L42" s="141" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="M42" s="107"/>
       <c r="N42" s="107"/>
     </row>
     <row r="43" spans="1:14" ht="28.8">
       <c r="A43" s="125" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="B43" s="74" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="C43" s="125" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="D43" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E43" s="205" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="F43" s="127" t="s">
         <v>17</v>
@@ -13235,32 +13236,32 @@
         <v>139</v>
       </c>
       <c r="L43" s="134" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="M43" s="129"/>
       <c r="N43" s="129"/>
     </row>
     <row r="44" spans="1:14" ht="57.6">
       <c r="A44" s="121" t="s">
+        <v>321</v>
+      </c>
+      <c r="B44" s="35" t="s">
+        <v>322</v>
+      </c>
+      <c r="C44" s="121" t="s">
+        <v>323</v>
+      </c>
+      <c r="D44" s="143" t="s">
         <v>324</v>
       </c>
-      <c r="B44" s="35" t="s">
+      <c r="E44" s="132" t="s">
         <v>325</v>
-      </c>
-      <c r="C44" s="121" t="s">
-        <v>326</v>
-      </c>
-      <c r="D44" s="143" t="s">
-        <v>327</v>
-      </c>
-      <c r="E44" s="132" t="s">
-        <v>328</v>
       </c>
       <c r="F44" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G44" s="124" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H44" s="124" t="s">
         <v>81</v>
@@ -13292,7 +13293,7 @@
         <v>16</v>
       </c>
       <c r="E45" s="74" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="F45" s="127" t="s">
         <v>17</v>
@@ -13313,36 +13314,36 @@
         <v>125</v>
       </c>
       <c r="L45" s="129" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="M45" s="129" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="N45" s="129" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="46" spans="1:14" ht="57.6">
       <c r="A46" s="121" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="B46" s="35" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="C46" s="141" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="D46" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E46" s="132" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="F46" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G46" s="124" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="H46" s="124" t="s">
         <v>81</v>
@@ -13362,25 +13363,25 @@
     </row>
     <row r="47" spans="1:14" ht="74.25" customHeight="1">
       <c r="A47" s="125" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="B47" s="74" t="s">
         <v>127</v>
       </c>
       <c r="C47" s="125" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="D47" s="142" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="E47" s="74" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="F47" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G47" s="127" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H47" s="127" t="s">
         <v>52</v>
@@ -13412,7 +13413,7 @@
         <v>16</v>
       </c>
       <c r="E48" s="132" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="F48" s="124" t="s">
         <v>35</v>
@@ -13438,25 +13439,25 @@
     </row>
     <row r="49" spans="1:14" ht="57.6">
       <c r="A49" s="125" t="s">
+        <v>337</v>
+      </c>
+      <c r="B49" s="74" t="s">
+        <v>338</v>
+      </c>
+      <c r="C49" s="125" t="s">
+        <v>339</v>
+      </c>
+      <c r="D49" s="217" t="s">
         <v>340</v>
       </c>
-      <c r="B49" s="74" t="s">
+      <c r="E49" s="83" t="s">
         <v>341</v>
-      </c>
-      <c r="C49" s="125" t="s">
-        <v>342</v>
-      </c>
-      <c r="D49" s="217" t="s">
-        <v>343</v>
-      </c>
-      <c r="E49" s="83" t="s">
-        <v>344</v>
       </c>
       <c r="F49" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G49" s="127" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H49" s="127" t="s">
         <v>19</v>
@@ -13476,19 +13477,19 @@
     </row>
     <row r="50" spans="1:14" ht="28.8">
       <c r="A50" s="121" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="B50" s="35" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="C50" s="121" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="D50" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E50" s="132" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="F50" s="124" t="s">
         <v>17</v>
@@ -13514,19 +13515,19 @@
     </row>
     <row r="51" spans="1:14" ht="28.8">
       <c r="A51" s="125" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="B51" s="74" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="C51" s="125" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="D51" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E51" s="74" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="F51" s="127" t="s">
         <v>17</v>
@@ -13552,13 +13553,13 @@
     </row>
     <row r="52" spans="1:14" ht="84.75" customHeight="1">
       <c r="A52" s="121" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="B52" s="35" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="C52" s="121" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="D52" s="132" t="s">
         <v>16</v>
@@ -13568,7 +13569,7 @@
         <v>17</v>
       </c>
       <c r="G52" s="124" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="H52" s="124" t="s">
         <v>19</v>
@@ -13781,42 +13782,42 @@
         <v>10</v>
       </c>
       <c r="L1" s="223" t="s">
+        <v>354</v>
+      </c>
+      <c r="M1" s="223" t="s">
+        <v>355</v>
+      </c>
+      <c r="N1" s="108" t="s">
+        <v>356</v>
+      </c>
+      <c r="O1" s="108" t="s">
         <v>357</v>
       </c>
-      <c r="M1" s="223" t="s">
+      <c r="P1" s="223" t="s">
         <v>358</v>
       </c>
-      <c r="N1" s="108" t="s">
+      <c r="Q1" s="223" t="s">
         <v>359</v>
       </c>
-      <c r="O1" s="108" t="s">
+      <c r="R1" s="224" t="s">
         <v>360</v>
       </c>
-      <c r="P1" s="223" t="s">
+      <c r="S1" s="224" t="s">
         <v>361</v>
       </c>
-      <c r="Q1" s="223" t="s">
+      <c r="T1" s="224" t="s">
         <v>362</v>
       </c>
-      <c r="R1" s="224" t="s">
+      <c r="U1" s="224" t="s">
         <v>363</v>
       </c>
-      <c r="S1" s="224" t="s">
+      <c r="V1" s="233" t="s">
         <v>364</v>
-      </c>
-      <c r="T1" s="224" t="s">
-        <v>365</v>
-      </c>
-      <c r="U1" s="224" t="s">
-        <v>366</v>
-      </c>
-      <c r="V1" s="233" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="28.8">
       <c r="A2" s="64" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="B2" s="157" t="s">
         <v>61</v>
@@ -13825,10 +13826,10 @@
         <v>62</v>
       </c>
       <c r="D2" s="152" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="E2" s="158" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="F2" s="159" t="s">
         <v>17</v>
@@ -13848,25 +13849,25 @@
     </row>
     <row r="3" spans="1:22" ht="115.2">
       <c r="A3" s="68" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="C3" s="68" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="D3" s="162" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="184" t="s">
-        <v>671</v>
+        <v>668</v>
       </c>
       <c r="F3" s="163" t="s">
         <v>35</v>
       </c>
       <c r="G3" s="163" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="H3" s="163">
         <v>1</v>
@@ -13878,7 +13879,7 @@
         <v>66</v>
       </c>
       <c r="K3" s="136" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="L3" s="129"/>
       <c r="M3" s="129"/>
@@ -13893,19 +13894,19 @@
     </row>
     <row r="4" spans="1:22" ht="129.6">
       <c r="A4" s="64" t="s">
+        <v>211</v>
+      </c>
+      <c r="B4" s="157" t="s">
         <v>212</v>
       </c>
-      <c r="B4" s="157" t="s">
+      <c r="C4" s="64" t="s">
         <v>213</v>
       </c>
-      <c r="C4" s="64" t="s">
-        <v>214</v>
-      </c>
       <c r="D4" s="71" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="E4" s="158" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="F4" s="159" t="s">
         <v>35</v>
@@ -13920,28 +13921,28 @@
         <v>28</v>
       </c>
       <c r="J4" s="160" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="K4" s="136" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="L4" s="107"/>
     </row>
     <row r="5" spans="1:22" ht="43.2">
       <c r="A5" s="165" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="B5" s="75" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="C5" s="165" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="D5" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="75" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="F5" s="166" t="s">
         <v>35</v>
@@ -13959,7 +13960,7 @@
         <v>29</v>
       </c>
       <c r="K5" s="136" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="L5" s="129"/>
       <c r="M5" s="129"/>
@@ -13974,19 +13975,19 @@
     </row>
     <row r="6" spans="1:22" ht="72">
       <c r="A6" s="168" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="B6" s="151" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="C6" s="168" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="D6" s="169" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="151" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="F6" s="133" t="s">
         <v>17</v>
@@ -14008,25 +14009,25 @@
     </row>
     <row r="7" spans="1:22" ht="115.2">
       <c r="A7" s="125" t="s">
+        <v>386</v>
+      </c>
+      <c r="B7" s="74" t="s">
+        <v>387</v>
+      </c>
+      <c r="C7" s="125" t="s">
+        <v>388</v>
+      </c>
+      <c r="D7" s="171" t="s">
         <v>389</v>
       </c>
-      <c r="B7" s="74" t="s">
+      <c r="E7" s="81" t="s">
         <v>390</v>
-      </c>
-      <c r="C7" s="125" t="s">
-        <v>391</v>
-      </c>
-      <c r="D7" s="171" t="s">
-        <v>392</v>
-      </c>
-      <c r="E7" s="81" t="s">
-        <v>393</v>
       </c>
       <c r="F7" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G7" s="127" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H7" s="127" t="s">
         <v>81</v>
@@ -14051,25 +14052,25 @@
     </row>
     <row r="8" spans="1:22" ht="28.8">
       <c r="A8" s="64" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="B8" s="157" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="C8" s="172" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="D8" s="143" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="E8" s="135" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="F8" s="159" t="s">
         <v>17</v>
       </c>
       <c r="G8" s="159" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H8" s="159" t="s">
         <v>81</v>
@@ -14081,13 +14082,13 @@
         <v>29</v>
       </c>
       <c r="K8" s="136" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="L8" s="107"/>
     </row>
     <row r="9" spans="1:22" ht="43.2">
       <c r="A9" s="165" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="B9" s="75" t="s">
         <v>77</v>
@@ -14099,13 +14100,13 @@
         <v>16</v>
       </c>
       <c r="E9" s="173" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="F9" s="166" t="s">
         <v>35</v>
       </c>
       <c r="G9" s="166" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H9" s="166">
         <v>1</v>
@@ -14117,7 +14118,7 @@
         <v>66</v>
       </c>
       <c r="K9" s="136" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="L9" s="129"/>
       <c r="M9" s="129"/>
@@ -14862,45 +14863,45 @@
         <v>10</v>
       </c>
       <c r="L1" s="225" t="s">
+        <v>396</v>
+      </c>
+      <c r="M1" s="108" t="s">
+        <v>397</v>
+      </c>
+      <c r="N1" s="223" t="s">
+        <v>398</v>
+      </c>
+      <c r="O1" s="224" t="s">
         <v>399</v>
       </c>
-      <c r="M1" s="108" t="s">
+      <c r="P1" s="232" t="s">
         <v>400</v>
       </c>
-      <c r="N1" s="223" t="s">
+      <c r="Q1" s="233" t="s">
         <v>401</v>
-      </c>
-      <c r="O1" s="224" t="s">
-        <v>402</v>
-      </c>
-      <c r="P1" s="232" t="s">
-        <v>403</v>
-      </c>
-      <c r="Q1" s="233" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="64.349999999999994" customHeight="1">
       <c r="A2" s="64" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="B2" s="45" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="C2" s="172" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="D2" s="64" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="88" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="F2" s="159" t="s">
         <v>17</v>
       </c>
       <c r="G2" s="159" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="H2" s="159" t="s">
         <v>19</v>
@@ -14912,31 +14913,31 @@
         <v>29</v>
       </c>
       <c r="K2" s="156" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="L2" s="136"/>
     </row>
     <row r="3" spans="1:17" ht="129.6">
       <c r="A3" s="68" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="B3" s="61" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="C3" s="68" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="D3" s="183" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="184" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
       <c r="F3" s="163" t="s">
         <v>35</v>
       </c>
       <c r="G3" s="163" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="H3" s="163">
         <v>1</v>
@@ -14948,7 +14949,7 @@
         <v>29</v>
       </c>
       <c r="K3" s="156" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="L3" s="75"/>
       <c r="M3" s="61"/>
@@ -14958,25 +14959,25 @@
     </row>
     <row r="4" spans="1:17" ht="28.8">
       <c r="A4" s="64" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="B4" s="45" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="C4" s="64" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="D4" s="64" t="s">
         <v>16</v>
       </c>
       <c r="E4" s="88" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="F4" s="159" t="s">
         <v>35</v>
       </c>
       <c r="G4" s="159" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="H4" s="159">
         <v>1</v>
@@ -14988,7 +14989,7 @@
         <v>29</v>
       </c>
       <c r="K4" s="156" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="L4" s="136"/>
     </row>
@@ -15811,27 +15812,27 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="M1" s="223" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="28.8">
       <c r="A2" s="121" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="B2" s="35" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="C2" s="121" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="D2" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="35" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>17</v>
@@ -15849,36 +15850,36 @@
         <v>37</v>
       </c>
       <c r="K2" s="98" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="L2" s="141" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="M2" s="141" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="72">
       <c r="A3" s="125" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="B3" s="74" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="C3" s="125" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="D3" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="85" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
       <c r="F3" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G3" s="127" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H3" s="127">
         <v>1</v>
@@ -15890,7 +15891,7 @@
         <v>37</v>
       </c>
       <c r="K3" s="98" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
       <c r="L3" s="129"/>
       <c r="M3" s="129"/>
@@ -15909,7 +15910,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="35" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
       <c r="F4" s="124" t="s">
         <v>17</v>
@@ -15934,25 +15935,25 @@
     </row>
     <row r="5" spans="1:13" ht="43.2">
       <c r="A5" s="125" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
       <c r="B5" s="74" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
       <c r="C5" s="134" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
       <c r="D5" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="126" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
       <c r="F5" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G5" s="127" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
       <c r="H5" s="127">
         <v>1</v>
@@ -15964,32 +15965,32 @@
         <v>29</v>
       </c>
       <c r="K5" s="98" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
       <c r="L5" s="129"/>
       <c r="M5" s="129"/>
     </row>
     <row r="6" spans="1:13" ht="57.6">
       <c r="A6" s="121" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="C6" s="121" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="D6" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="35" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="F6" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G6" s="128" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="H6" s="124" t="s">
         <v>81</v>
@@ -16001,36 +16002,36 @@
         <v>29</v>
       </c>
       <c r="K6" s="98" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="L6" s="107" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="M6" s="107" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="43.2">
       <c r="A7" s="125" t="s">
+        <v>444</v>
+      </c>
+      <c r="B7" s="74" t="s">
+        <v>445</v>
+      </c>
+      <c r="C7" s="134" t="s">
+        <v>446</v>
+      </c>
+      <c r="D7" s="185" t="s">
         <v>447</v>
       </c>
-      <c r="B7" s="74" t="s">
+      <c r="E7" s="126" t="s">
         <v>448</v>
-      </c>
-      <c r="C7" s="134" t="s">
-        <v>449</v>
-      </c>
-      <c r="D7" s="185" t="s">
-        <v>450</v>
-      </c>
-      <c r="E7" s="126" t="s">
-        <v>451</v>
       </c>
       <c r="F7" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G7" s="156" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="H7" s="127" t="s">
         <v>81</v>
@@ -16042,7 +16043,7 @@
         <v>29</v>
       </c>
       <c r="K7" s="98" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="L7" s="129"/>
       <c r="M7" s="129"/>
@@ -16061,7 +16062,7 @@
         <v>16</v>
       </c>
       <c r="E8" s="35" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="F8" s="124" t="s">
         <v>17</v>
@@ -16079,26 +16080,26 @@
         <v>29</v>
       </c>
       <c r="K8" s="98" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="L8" s="107"/>
       <c r="M8" s="107"/>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" s="125" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B9" s="74" t="s">
         <v>77</v>
       </c>
       <c r="C9" s="125" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D9" s="187" t="s">
         <v>16</v>
       </c>
       <c r="E9" s="126" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="F9" s="127" t="s">
         <v>17</v>
@@ -16116,32 +16117,32 @@
         <v>29</v>
       </c>
       <c r="K9" s="98" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="L9" s="129"/>
       <c r="M9" s="129"/>
     </row>
     <row r="10" spans="1:13" ht="57.6">
       <c r="A10" s="121" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="C10" s="141" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="D10" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="F10" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G10" s="124" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H10" s="124" t="s">
         <v>81</v>
@@ -16153,32 +16154,32 @@
         <v>37</v>
       </c>
       <c r="K10" s="98" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
       <c r="L10" s="107"/>
       <c r="M10" s="107"/>
     </row>
     <row r="11" spans="1:13" ht="43.2">
       <c r="A11" s="125" t="s">
+        <v>460</v>
+      </c>
+      <c r="B11" s="74" t="s">
+        <v>461</v>
+      </c>
+      <c r="C11" s="125" t="s">
+        <v>462</v>
+      </c>
+      <c r="D11" s="154" t="s">
         <v>463</v>
       </c>
-      <c r="B11" s="74" t="s">
-        <v>464</v>
-      </c>
-      <c r="C11" s="125" t="s">
-        <v>465</v>
-      </c>
-      <c r="D11" s="154" t="s">
-        <v>466</v>
-      </c>
       <c r="E11" s="126" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
       <c r="F11" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G11" s="127" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="H11" s="127">
         <v>1</v>
@@ -16190,7 +16191,7 @@
         <v>29</v>
       </c>
       <c r="K11" s="99" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="L11" s="129"/>
       <c r="M11" s="129"/>
@@ -16209,7 +16210,7 @@
         <v>85</v>
       </c>
       <c r="E12" s="138" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="F12" s="124" t="s">
         <v>17</v>
@@ -16227,14 +16228,14 @@
         <v>29</v>
       </c>
       <c r="K12" s="98" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="L12" s="107"/>
       <c r="M12" s="107"/>
     </row>
     <row r="13" spans="1:13" ht="72">
       <c r="A13" s="125" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="B13" s="74" t="s">
         <v>90</v>
@@ -16246,13 +16247,13 @@
         <v>92</v>
       </c>
       <c r="E13" s="80" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G13" s="127" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="H13" s="127">
         <v>1</v>
@@ -16264,32 +16265,32 @@
         <v>37</v>
       </c>
       <c r="K13" s="98" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="L13" s="129"/>
       <c r="M13" s="129"/>
     </row>
     <row r="14" spans="1:13" ht="72">
       <c r="A14" s="121" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="B14" s="35" t="s">
+        <v>175</v>
+      </c>
+      <c r="C14" s="121" t="s">
         <v>176</v>
-      </c>
-      <c r="C14" s="121" t="s">
-        <v>177</v>
       </c>
       <c r="D14" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="F14" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G14" s="124" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H14" s="124" t="s">
         <v>19</v>
@@ -16301,32 +16302,32 @@
         <v>29</v>
       </c>
       <c r="K14" s="98" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="L14" s="107"/>
       <c r="M14" s="107"/>
     </row>
     <row r="15" spans="1:13" ht="100.8">
       <c r="A15" s="125" t="s">
+        <v>475</v>
+      </c>
+      <c r="B15" s="74" t="s">
+        <v>476</v>
+      </c>
+      <c r="C15" s="125" t="s">
+        <v>477</v>
+      </c>
+      <c r="D15" s="185" t="s">
+        <v>447</v>
+      </c>
+      <c r="E15" s="80" t="s">
         <v>478</v>
-      </c>
-      <c r="B15" s="74" t="s">
-        <v>479</v>
-      </c>
-      <c r="C15" s="125" t="s">
-        <v>480</v>
-      </c>
-      <c r="D15" s="185" t="s">
-        <v>450</v>
-      </c>
-      <c r="E15" s="80" t="s">
-        <v>481</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G15" s="127" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="H15" s="127" t="s">
         <v>81</v>
@@ -16338,7 +16339,7 @@
         <v>29</v>
       </c>
       <c r="K15" s="98" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="L15" s="129"/>
       <c r="M15" s="129"/>
@@ -16373,32 +16374,32 @@
         <v>29</v>
       </c>
       <c r="K16" s="98" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="L16" s="107"/>
       <c r="M16" s="107"/>
     </row>
     <row r="17" spans="1:13" ht="57.6">
       <c r="A17" s="125" t="s">
+        <v>481</v>
+      </c>
+      <c r="B17" s="74" t="s">
+        <v>482</v>
+      </c>
+      <c r="C17" s="125" t="s">
+        <v>483</v>
+      </c>
+      <c r="D17" s="185" t="s">
+        <v>447</v>
+      </c>
+      <c r="E17" s="74" t="s">
         <v>484</v>
-      </c>
-      <c r="B17" s="74" t="s">
-        <v>485</v>
-      </c>
-      <c r="C17" s="125" t="s">
-        <v>486</v>
-      </c>
-      <c r="D17" s="185" t="s">
-        <v>450</v>
-      </c>
-      <c r="E17" s="74" t="s">
-        <v>487</v>
       </c>
       <c r="F17" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G17" s="127" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="H17" s="127" t="s">
         <v>81</v>
@@ -16410,7 +16411,7 @@
         <v>29</v>
       </c>
       <c r="K17" s="98" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="L17" s="129"/>
       <c r="M17" s="129"/>
@@ -16429,7 +16430,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="132" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="F18" s="124" t="s">
         <v>17</v>
@@ -16447,24 +16448,24 @@
         <v>29</v>
       </c>
       <c r="K18" s="98" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="L18" s="107"/>
       <c r="M18" s="107"/>
     </row>
     <row r="19" spans="1:13" ht="28.8">
       <c r="A19" s="125" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="B19" s="126" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C19" s="125" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="D19" s="126"/>
       <c r="E19" s="80" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="F19" s="127" t="s">
         <v>17</v>
@@ -16483,10 +16484,10 @@
       </c>
       <c r="K19" s="104"/>
       <c r="L19" s="129" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="M19" s="129" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="129.6">
@@ -16503,7 +16504,7 @@
         <v>16</v>
       </c>
       <c r="E20" s="79" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
       <c r="F20" s="190" t="s">
         <v>35</v>
@@ -16521,32 +16522,32 @@
         <v>29</v>
       </c>
       <c r="K20" s="99" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="L20" s="107"/>
       <c r="M20" s="107"/>
     </row>
     <row r="21" spans="1:13" ht="43.2">
       <c r="A21" s="125" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="B21" s="74" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="C21" s="125" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="D21" s="154" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="E21" s="81" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G21" s="127" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H21" s="127" t="s">
         <v>81</v>
@@ -16558,32 +16559,32 @@
         <v>29</v>
       </c>
       <c r="K21" s="98" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="L21" s="129"/>
       <c r="M21" s="129"/>
     </row>
     <row r="22" spans="1:13" ht="57.6">
       <c r="A22" s="121" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="B22" s="35" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="C22" s="121" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="D22" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E22" s="132" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G22" s="124" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="H22" s="124" t="s">
         <v>81</v>
@@ -16612,7 +16613,7 @@
         <v>16</v>
       </c>
       <c r="E23" s="126" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>17</v>
@@ -16630,7 +16631,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="98" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
       <c r="L23" s="129"/>
       <c r="M23" s="129"/>
@@ -17112,7 +17113,7 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -17129,7 +17130,7 @@
         <v>16</v>
       </c>
       <c r="E2" s="74" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>17</v>
@@ -17147,7 +17148,7 @@
         <v>29</v>
       </c>
       <c r="K2" s="98" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
       <c r="L2" s="129"/>
     </row>
@@ -17183,7 +17184,7 @@
         <v>29</v>
       </c>
       <c r="K3" s="98" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
       <c r="L3" s="107" t="s">
         <v>39</v>
@@ -17203,7 +17204,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="126" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="F4" s="127" t="s">
         <v>35</v>
@@ -17221,31 +17222,31 @@
         <v>29</v>
       </c>
       <c r="K4" s="99" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="L4" s="129"/>
     </row>
     <row r="5" spans="1:12" ht="43.2">
       <c r="A5" s="121" t="s">
+        <v>193</v>
+      </c>
+      <c r="B5" s="35" t="s">
         <v>194</v>
       </c>
-      <c r="B5" s="35" t="s">
+      <c r="C5" s="121" t="s">
         <v>195</v>
       </c>
-      <c r="C5" s="121" t="s">
+      <c r="D5" s="122" t="s">
         <v>196</v>
       </c>
-      <c r="D5" s="122" t="s">
-        <v>197</v>
-      </c>
       <c r="E5" s="135" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
       <c r="F5" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G5" s="124" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H5" s="124" t="s">
         <v>81</v>
@@ -17273,7 +17274,7 @@
         <v>63</v>
       </c>
       <c r="E6" s="247" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F6" s="244" t="s">
         <v>17</v>
@@ -17291,7 +17292,7 @@
         <v>66</v>
       </c>
       <c r="K6" s="243" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="L6" s="242"/>
     </row>
@@ -17373,7 +17374,7 @@
         <v>16</v>
       </c>
       <c r="E11" s="132" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="F11" s="124" t="s">
         <v>17</v>
@@ -17391,7 +17392,7 @@
         <v>29</v>
       </c>
       <c r="K11" s="99" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
       <c r="L11" s="107"/>
     </row>
@@ -17409,7 +17410,7 @@
         <v>16</v>
       </c>
       <c r="E12" s="126" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="F12" s="124" t="s">
         <v>17</v>
@@ -17427,7 +17428,7 @@
         <v>29</v>
       </c>
       <c r="K12" s="98" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="L12" s="129" t="s">
         <v>46</v>
@@ -17447,7 +17448,7 @@
         <v>16</v>
       </c>
       <c r="E13" s="132" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>17</v>
@@ -17465,7 +17466,7 @@
         <v>29</v>
       </c>
       <c r="K13" s="98" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="L13" s="107"/>
     </row>
@@ -17483,7 +17484,7 @@
         <v>16</v>
       </c>
       <c r="E14" s="126" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
       <c r="F14" s="124" t="s">
         <v>17</v>
@@ -17501,10 +17502,10 @@
         <v>29</v>
       </c>
       <c r="K14" s="98" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="L14" s="129" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -17521,7 +17522,7 @@
         <v>16</v>
       </c>
       <c r="E15" s="121" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>35</v>
@@ -17820,7 +17821,7 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="92.4">
@@ -17837,7 +17838,7 @@
         <v>152</v>
       </c>
       <c r="E2" s="82" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>35</v>
@@ -17855,7 +17856,7 @@
         <v>37</v>
       </c>
       <c r="K2" s="107" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="L2" s="186"/>
     </row>
@@ -17893,25 +17894,25 @@
     </row>
     <row r="4" spans="1:12" ht="92.25" customHeight="1">
       <c r="A4" s="121" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="B4" s="35" t="s">
+        <v>175</v>
+      </c>
+      <c r="C4" s="121" t="s">
         <v>176</v>
-      </c>
-      <c r="C4" s="121" t="s">
-        <v>177</v>
       </c>
       <c r="D4" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E4" s="194" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="F4" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G4" s="124" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H4" s="124" t="s">
         <v>19</v>
@@ -18043,7 +18044,7 @@
         <v>16</v>
       </c>
       <c r="E8" s="82" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="F8" s="124" t="s">
         <v>35</v>
@@ -18061,31 +18062,31 @@
         <v>37</v>
       </c>
       <c r="K8" s="107" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="L8" s="107"/>
     </row>
     <row r="9" spans="1:12" ht="43.2">
       <c r="A9" s="125" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="B9" s="74" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="C9" s="125" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="D9" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E9" s="212" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="F9" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G9" s="127" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="H9" s="127">
         <v>1</v>
@@ -18097,31 +18098,31 @@
         <v>37</v>
       </c>
       <c r="K9" s="106" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="L9" s="129"/>
     </row>
     <row r="10" spans="1:12" ht="43.2">
       <c r="A10" s="121" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="B10" s="35" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="C10" s="121" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="D10" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="F10" s="124" t="s">
         <v>35</v>
       </c>
       <c r="G10" s="124" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="H10" s="133">
         <v>1</v>
@@ -18133,29 +18134,29 @@
         <v>37</v>
       </c>
       <c r="K10" s="106" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="L10" s="107"/>
     </row>
     <row r="11" spans="1:12" ht="43.2">
       <c r="A11" s="125" t="s">
+        <v>460</v>
+      </c>
+      <c r="B11" s="74" t="s">
+        <v>461</v>
+      </c>
+      <c r="C11" s="134" t="s">
+        <v>462</v>
+      </c>
+      <c r="D11" s="154" t="s">
         <v>463</v>
-      </c>
-      <c r="B11" s="74" t="s">
-        <v>464</v>
-      </c>
-      <c r="C11" s="134" t="s">
-        <v>465</v>
-      </c>
-      <c r="D11" s="154" t="s">
-        <v>466</v>
       </c>
       <c r="E11" s="126"/>
       <c r="F11" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G11" s="127" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="H11" s="127" t="s">
         <v>19</v>
@@ -18171,13 +18172,13 @@
     </row>
     <row r="12" spans="1:12" ht="28.8">
       <c r="A12" s="121" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="B12" s="35" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="C12" s="121" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="D12" s="132" t="s">
         <v>16</v>
@@ -18187,7 +18188,7 @@
         <v>17</v>
       </c>
       <c r="G12" s="124" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H12" s="124" t="s">
         <v>19</v>
@@ -18203,19 +18204,19 @@
     </row>
     <row r="13" spans="1:12" ht="57.6">
       <c r="A13" s="191" t="s">
+        <v>211</v>
+      </c>
+      <c r="B13" s="74" t="s">
         <v>212</v>
       </c>
-      <c r="B13" s="74" t="s">
+      <c r="C13" s="134" t="s">
         <v>213</v>
-      </c>
-      <c r="C13" s="134" t="s">
-        <v>214</v>
       </c>
       <c r="D13" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E13" s="126" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>35</v>
@@ -18237,13 +18238,13 @@
     </row>
     <row r="14" spans="1:12" ht="28.8">
       <c r="A14" s="121" t="s">
+        <v>228</v>
+      </c>
+      <c r="B14" s="35" t="s">
         <v>229</v>
       </c>
-      <c r="B14" s="35" t="s">
+      <c r="C14" s="121" t="s">
         <v>230</v>
-      </c>
-      <c r="C14" s="121" t="s">
-        <v>231</v>
       </c>
       <c r="D14" s="132" t="s">
         <v>16</v>
@@ -18269,19 +18270,19 @@
     </row>
     <row r="15" spans="1:12" ht="57.6">
       <c r="A15" s="125" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="B15" s="74" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="C15" s="125" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="D15" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E15" s="126" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>17</v>
@@ -18315,7 +18316,7 @@
         <v>85</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="F16" s="124" t="s">
         <v>17</v>
@@ -18349,7 +18350,7 @@
         <v>92</v>
       </c>
       <c r="E17" s="80" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="F17" s="127" t="s">
         <v>35</v>
@@ -18367,7 +18368,7 @@
         <v>37</v>
       </c>
       <c r="K17" s="107" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="L17" s="129"/>
     </row>
@@ -18385,7 +18386,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="35" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="F18" s="124" t="s">
         <v>17</v>
@@ -18407,13 +18408,13 @@
     </row>
     <row r="19" spans="1:12" ht="28.8">
       <c r="A19" s="125" t="s">
+        <v>263</v>
+      </c>
+      <c r="B19" s="74" t="s">
+        <v>264</v>
+      </c>
+      <c r="C19" s="134" t="s">
         <v>265</v>
-      </c>
-      <c r="B19" s="74" t="s">
-        <v>266</v>
-      </c>
-      <c r="C19" s="134" t="s">
-        <v>267</v>
       </c>
       <c r="D19" s="126" t="s">
         <v>16</v>
@@ -18423,7 +18424,7 @@
         <v>17</v>
       </c>
       <c r="G19" s="128" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="H19" s="127" t="s">
         <v>19</v>
@@ -18436,7 +18437,7 @@
       </c>
       <c r="K19" s="106"/>
       <c r="L19" s="129" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="43.2">
@@ -18453,7 +18454,7 @@
         <v>16</v>
       </c>
       <c r="E20" s="35" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="F20" s="124" t="s">
         <v>35</v>
@@ -18477,19 +18478,19 @@
     </row>
     <row r="21" spans="1:12" ht="57.6">
       <c r="A21" s="125" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="B21" s="74" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="C21" s="125" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="D21" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E21" s="126" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>17</v>
@@ -18507,33 +18508,33 @@
         <v>29</v>
       </c>
       <c r="K21" s="107" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="L21" s="192" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="43.2">
       <c r="A22" s="121" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="B22" s="35" t="s">
         <v>127</v>
       </c>
       <c r="C22" s="121" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="D22" s="143" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="E22" s="35" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>35</v>
       </c>
       <c r="G22" s="124" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H22" s="124" t="s">
         <v>52</v>
@@ -18561,7 +18562,7 @@
         <v>16</v>
       </c>
       <c r="E23" s="126" t="s">
-        <v>555</v>
+        <v>552</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>35</v>
@@ -18579,7 +18580,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="106" t="s">
-        <v>556</v>
+        <v>553</v>
       </c>
       <c r="L23" s="195"/>
     </row>

</xml_diff>

<commit_message>
doc update retention period
usage note of retention period property in Dataset and Distribution class was updated to clarify what it is for.
</commit_message>
<xml_diff>
--- a/Documents/Metadata_CoreGenericHealth_v2.xlsx
+++ b/Documents/Metadata_CoreGenericHealth_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://healthri-my.sharepoint.com/personal/hannah_neikes_health-ri_nl/Documents/Documenten/GitHub/health-ri-metadata/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{B604F9AE-9787-411E-AB68-6C0D2821F0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB2FDFB2-6BD5-4989-9906-EC23F51E3B08}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="8_{B604F9AE-9787-411E-AB68-6C0D2821F0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56501FCB-3D8B-4B1A-811D-B69BAEFCE65B}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-12765" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5295" yWindow="-16320" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="14" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1846" uniqueCount="675">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1846" uniqueCount="676">
   <si>
     <t>Property label</t>
   </si>
@@ -1145,9 +1145,6 @@
     <t>healthdcatap:retentionPeriod</t>
   </si>
   <si>
-    <t>This property makes use of the class dct:PeriodOfTime, in which a start and end date should be provided.</t>
-  </si>
-  <si>
     <t>fill in in 'Period of Time' tab</t>
   </si>
   <si>
@@ -2619,6 +2616,20 @@
   <si>
     <t>One (or many) categoiesy or sub-categories of the purposes can be chosen from the taxonomy provided by dpv (see controlled vocabulary column). Try to be as specific as possible.
 Example value could be: dpv:ResearchAndDevelopment.</t>
+  </si>
+  <si>
+    <t>Indicate with this property in case the Dataset is only available for secondary use for a specific period of time (e.g. due to data protection, contractual, or project constraints).
+This property makes use of the class dct:PeriodOfTime, in which a start and end date can be provided.
+If the Dataset is available indefinitely, leave the property empty (cardinality is 0..1; it is only meaningful when a retention limit applies).
+If only a start is known, provide dcat:startDate only (open-ended interval, as allowed by dct:PeriodOfTime).
+If a limit is known, provide both dcat:startDate and dcat:endDate.</t>
+  </si>
+  <si>
+    <t>Indicate with this property in case the Distribution is only available for secondary use for a specific period of time (e.g. due to data protection, contractual, or project constraints).
+This property makes use of the class dct:PeriodOfTime, in which a start and end date can be provided.
+If the Distribution is available indefinitely, leave the property empty (cardinality is 0..1; it is only meaningful when a retention limit applies).
+If only a start is known, provide dcat:startDate only (open-ended interval, as allowed by dct:PeriodOfTime).
+If a limit is known, provide both dcat:startDate and dcat:endDate.</t>
   </si>
 </sst>
 </file>
@@ -3766,43 +3777,43 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -7439,33 +7450,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>553</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>554</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="227" t="s">
         <v>555</v>
       </c>
-      <c r="N1" s="227" t="s">
+      <c r="O1" s="233" t="s">
         <v>556</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>557</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="72">
       <c r="A2" s="196" t="s">
+        <v>557</v>
+      </c>
+      <c r="B2" s="45" t="s">
         <v>558</v>
       </c>
-      <c r="B2" s="45" t="s">
+      <c r="C2" s="76" t="s">
         <v>559</v>
-      </c>
-      <c r="C2" s="76" t="s">
-        <v>560</v>
       </c>
       <c r="D2" s="196" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="197" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="F2" s="198" t="s">
         <v>35</v>
@@ -7474,7 +7485,7 @@
         <v>58</v>
       </c>
       <c r="H2" s="198" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="I2" s="160" t="s">
         <v>20</v>
@@ -7489,13 +7500,13 @@
     </row>
     <row r="3" spans="1:15" ht="28.8">
       <c r="A3" s="68" t="s">
+        <v>562</v>
+      </c>
+      <c r="B3" s="61" t="s">
         <v>563</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="C3" s="77" t="s">
         <v>564</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>565</v>
       </c>
       <c r="D3" s="68" t="s">
         <v>16</v>
@@ -7634,36 +7645,36 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>565</v>
+      </c>
+      <c r="M1" s="220" t="s">
         <v>566</v>
       </c>
-      <c r="M1" s="220" t="s">
+      <c r="N1" s="226" t="s">
         <v>567</v>
       </c>
-      <c r="N1" s="226" t="s">
+      <c r="O1" s="230" t="s">
         <v>568</v>
       </c>
-      <c r="O1" s="230" t="s">
+      <c r="P1" s="227" t="s">
         <v>569</v>
       </c>
-      <c r="P1" s="227" t="s">
+      <c r="Q1" s="231" t="s">
         <v>570</v>
       </c>
-      <c r="Q1" s="231" t="s">
+      <c r="R1" s="233" t="s">
         <v>571</v>
-      </c>
-      <c r="R1" s="233" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="2" spans="1:18">
       <c r="A2" s="58" t="s">
+        <v>572</v>
+      </c>
+      <c r="B2" s="44" t="s">
         <v>573</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="C2" s="76" t="s">
         <v>574</v>
-      </c>
-      <c r="C2" s="76" t="s">
-        <v>575</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
@@ -7691,13 +7702,13 @@
     </row>
     <row r="3" spans="1:18">
       <c r="A3" s="48" t="s">
+        <v>575</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>576</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>577</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>578</v>
       </c>
       <c r="D3" s="48" t="s">
         <v>16</v>
@@ -8359,33 +8370,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>578</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>579</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="227" t="s">
         <v>580</v>
       </c>
-      <c r="N1" s="227" t="s">
+      <c r="O1" s="233" t="s">
         <v>581</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>582</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="43.2">
       <c r="A2" s="84" t="s">
+        <v>582</v>
+      </c>
+      <c r="B2" s="44" t="s">
         <v>583</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="C2" s="58" t="s">
         <v>584</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>585</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>17</v>
@@ -8415,19 +8426,19 @@
     </row>
     <row r="3" spans="1:15" ht="129.6">
       <c r="A3" s="48" t="s">
+        <v>586</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>587</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>588</v>
       </c>
-      <c r="C3" s="77" t="s">
+      <c r="D3" s="234" t="s">
         <v>589</v>
       </c>
-      <c r="D3" s="234" t="s">
+      <c r="E3" s="50" t="s">
         <v>590</v>
-      </c>
-      <c r="E3" s="50" t="s">
-        <v>591</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>17</v>
@@ -8553,33 +8564,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="218" t="s">
+        <v>591</v>
+      </c>
+      <c r="M1" s="229" t="s">
         <v>592</v>
       </c>
-      <c r="M1" s="229" t="s">
+      <c r="N1" s="228" t="s">
         <v>593</v>
       </c>
-      <c r="N1" s="228" t="s">
+      <c r="O1" s="233" t="s">
         <v>594</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>595</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="158.4">
       <c r="A2" s="84" t="s">
+        <v>595</v>
+      </c>
+      <c r="B2" s="44" t="s">
+        <v>587</v>
+      </c>
+      <c r="C2" s="58" t="s">
+        <v>588</v>
+      </c>
+      <c r="D2" s="59" t="s">
         <v>596</v>
       </c>
-      <c r="B2" s="44" t="s">
-        <v>588</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>589</v>
-      </c>
-      <c r="D2" s="59" t="s">
+      <c r="E2" s="59" t="s">
         <v>597</v>
-      </c>
-      <c r="E2" s="59" t="s">
-        <v>598</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>35</v>
@@ -8600,19 +8611,19 @@
     </row>
     <row r="3" spans="1:15" ht="43.2">
       <c r="A3" s="48" t="s">
+        <v>598</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>599</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>600</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>601</v>
       </c>
       <c r="D3" s="116" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>35</v>
@@ -8738,33 +8749,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>602</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>603</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="227" t="s">
         <v>604</v>
       </c>
-      <c r="N1" s="227" t="s">
+      <c r="O1" s="233" t="s">
         <v>605</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>606</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="100.8">
       <c r="A2" s="84" t="s">
+        <v>606</v>
+      </c>
+      <c r="B2" s="44" t="s">
         <v>607</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="C2" s="58" t="s">
         <v>608</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>609</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>17</v>
@@ -8785,19 +8796,19 @@
     </row>
     <row r="3" spans="1:15" ht="57.6">
       <c r="A3" s="48" t="s">
+        <v>610</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>611</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>612</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>613</v>
       </c>
       <c r="D3" s="116" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>17</v>
@@ -8901,7 +8912,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="56" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="E1" s="56" t="s">
         <v>4</v>
@@ -8924,13 +8935,13 @@
     </row>
     <row r="2" spans="1:10" ht="28.8">
       <c r="A2" s="63" t="s">
+        <v>615</v>
+      </c>
+      <c r="B2" s="53" t="s">
         <v>616</v>
       </c>
-      <c r="B2" s="53" t="s">
+      <c r="C2" s="44" t="s">
         <v>617</v>
-      </c>
-      <c r="C2" s="44" t="s">
-        <v>618</v>
       </c>
       <c r="D2" s="43" t="s">
         <v>16</v>
@@ -8938,7 +8949,7 @@
       <c r="E2" s="45"/>
       <c r="F2" s="64"/>
       <c r="G2" s="63" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="H2" s="65" t="s">
         <v>81</v>
@@ -8952,13 +8963,13 @@
     </row>
     <row r="3" spans="1:10" ht="43.2">
       <c r="A3" s="67" t="s">
+        <v>619</v>
+      </c>
+      <c r="B3" s="50" t="s">
         <v>620</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="C3" s="49" t="s">
         <v>621</v>
-      </c>
-      <c r="C3" s="49" t="s">
-        <v>622</v>
       </c>
       <c r="D3" s="48" t="s">
         <v>16</v>
@@ -8966,10 +8977,10 @@
       <c r="E3" s="50"/>
       <c r="F3" s="68"/>
       <c r="G3" s="69" t="s">
+        <v>622</v>
+      </c>
+      <c r="H3" s="48" t="s">
         <v>623</v>
-      </c>
-      <c r="H3" s="48" t="s">
-        <v>624</v>
       </c>
       <c r="I3" s="69" t="s">
         <v>20</v>
@@ -8980,13 +8991,13 @@
     </row>
     <row r="4" spans="1:10" ht="43.2">
       <c r="A4" s="63" t="s">
+        <v>624</v>
+      </c>
+      <c r="B4" s="53" t="s">
         <v>625</v>
       </c>
-      <c r="B4" s="53" t="s">
+      <c r="C4" s="44" t="s">
         <v>626</v>
-      </c>
-      <c r="C4" s="44" t="s">
-        <v>627</v>
       </c>
       <c r="D4" s="43" t="s">
         <v>16</v>
@@ -8994,10 +9005,10 @@
       <c r="E4" s="53"/>
       <c r="F4" s="64"/>
       <c r="G4" s="63" t="s">
+        <v>627</v>
+      </c>
+      <c r="H4" s="65" t="s">
         <v>628</v>
-      </c>
-      <c r="H4" s="65" t="s">
-        <v>629</v>
       </c>
       <c r="I4" s="66" t="s">
         <v>20</v>
@@ -9008,26 +9019,26 @@
     </row>
     <row r="5" spans="1:10" ht="43.2">
       <c r="A5" s="67" t="s">
+        <v>629</v>
+      </c>
+      <c r="B5" s="50" t="s">
         <v>630</v>
       </c>
-      <c r="B5" s="50" t="s">
+      <c r="C5" s="49" t="s">
         <v>631</v>
-      </c>
-      <c r="C5" s="49" t="s">
-        <v>632</v>
       </c>
       <c r="D5" s="48" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="49" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="F5" s="68"/>
       <c r="G5" s="67" t="s">
+        <v>633</v>
+      </c>
+      <c r="H5" s="48" t="s">
         <v>634</v>
-      </c>
-      <c r="H5" s="48" t="s">
-        <v>635</v>
       </c>
       <c r="I5" s="69" t="s">
         <v>20</v>
@@ -9038,13 +9049,13 @@
     </row>
     <row r="6" spans="1:10" ht="28.8">
       <c r="A6" s="63" t="s">
+        <v>635</v>
+      </c>
+      <c r="B6" s="73" t="s">
         <v>636</v>
       </c>
-      <c r="B6" s="73" t="s">
+      <c r="C6" s="44" t="s">
         <v>637</v>
-      </c>
-      <c r="C6" s="44" t="s">
-        <v>638</v>
       </c>
       <c r="D6" s="43" t="s">
         <v>16</v>
@@ -9055,7 +9066,7 @@
         <v>98</v>
       </c>
       <c r="H6" s="65" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="I6" s="66" t="s">
         <v>20</v>
@@ -9066,13 +9077,13 @@
     </row>
     <row r="7" spans="1:10" ht="28.8">
       <c r="A7" s="67" t="s">
+        <v>638</v>
+      </c>
+      <c r="B7" s="50" t="s">
         <v>639</v>
       </c>
-      <c r="B7" s="50" t="s">
+      <c r="C7" s="49" t="s">
         <v>640</v>
-      </c>
-      <c r="C7" s="49" t="s">
-        <v>641</v>
       </c>
       <c r="D7" s="48" t="s">
         <v>16</v>
@@ -9094,23 +9105,23 @@
     </row>
     <row r="8" spans="1:10" ht="86.4">
       <c r="A8" s="63" t="s">
+        <v>641</v>
+      </c>
+      <c r="B8" s="53" t="s">
         <v>642</v>
       </c>
-      <c r="B8" s="53" t="s">
+      <c r="C8" s="44" t="s">
         <v>643</v>
-      </c>
-      <c r="C8" s="44" t="s">
-        <v>644</v>
       </c>
       <c r="D8" s="43" t="s">
         <v>16</v>
       </c>
       <c r="E8" s="71" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="F8" s="47"/>
       <c r="G8" s="63" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="H8" s="65">
         <v>1</v>
@@ -9124,13 +9135,13 @@
     </row>
     <row r="9" spans="1:10" ht="28.8">
       <c r="A9" s="67" t="s">
+        <v>646</v>
+      </c>
+      <c r="B9" s="50" t="s">
         <v>647</v>
       </c>
-      <c r="B9" s="50" t="s">
+      <c r="C9" s="49" t="s">
         <v>648</v>
-      </c>
-      <c r="C9" s="49" t="s">
-        <v>649</v>
       </c>
       <c r="D9" s="48" t="s">
         <v>16</v>
@@ -9138,7 +9149,7 @@
       <c r="E9" s="50"/>
       <c r="F9" s="68"/>
       <c r="G9" s="69" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="H9" s="48" t="s">
         <v>81</v>
@@ -9152,23 +9163,23 @@
     </row>
     <row r="10" spans="1:10" ht="28.8">
       <c r="A10" s="63" t="s">
+        <v>650</v>
+      </c>
+      <c r="B10" s="72" t="s">
         <v>651</v>
       </c>
-      <c r="B10" s="72" t="s">
+      <c r="C10" s="44" t="s">
         <v>652</v>
-      </c>
-      <c r="C10" s="44" t="s">
-        <v>653</v>
       </c>
       <c r="D10" s="43" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="72" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="F10" s="64"/>
       <c r="G10" s="63" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="H10" s="65" t="s">
         <v>19</v>
@@ -9633,36 +9644,36 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>654</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>655</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="233" t="s">
         <v>656</v>
-      </c>
-      <c r="N1" s="233" t="s">
-        <v>657</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="72">
       <c r="A2" s="44" t="s">
+        <v>657</v>
+      </c>
+      <c r="B2" s="57" t="s">
         <v>658</v>
       </c>
-      <c r="B2" s="57" t="s">
+      <c r="C2" s="58" t="s">
         <v>659</v>
       </c>
-      <c r="C2" s="58" t="s">
+      <c r="D2" s="78" t="s">
         <v>660</v>
       </c>
-      <c r="D2" s="78" t="s">
+      <c r="E2" s="197" t="s">
         <v>661</v>
-      </c>
-      <c r="E2" s="197" t="s">
-        <v>662</v>
       </c>
       <c r="F2" s="46" t="s">
         <v>35</v>
       </c>
       <c r="G2" s="204" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="H2" s="47">
         <v>1</v>
@@ -9676,13 +9687,13 @@
     </row>
     <row r="3" spans="1:14" ht="71.25" customHeight="1">
       <c r="A3" s="49" t="s">
+        <v>663</v>
+      </c>
+      <c r="B3" s="61" t="s">
         <v>664</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="C3" s="48" t="s">
         <v>665</v>
-      </c>
-      <c r="C3" s="48" t="s">
-        <v>666</v>
       </c>
       <c r="D3" s="50" t="s">
         <v>16</v>
@@ -9692,7 +9703,7 @@
         <v>35</v>
       </c>
       <c r="G3" s="51" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="H3" s="52">
         <v>1</v>
@@ -10606,19 +10617,19 @@
       <c r="M7" s="129"/>
     </row>
     <row r="8" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A8" s="238" t="s">
+      <c r="A8" s="235" t="s">
         <v>60</v>
       </c>
       <c r="B8" s="241" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="238" t="s">
+      <c r="C8" s="235" t="s">
         <v>62</v>
       </c>
       <c r="D8" s="213" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="240" t="s">
+      <c r="E8" s="238" t="s">
         <v>64</v>
       </c>
       <c r="F8" s="237" t="s">
@@ -10630,83 +10641,83 @@
       <c r="H8" s="237" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="235" t="s">
+      <c r="I8" s="239" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="235" t="s">
+      <c r="J8" s="239" t="s">
         <v>66</v>
       </c>
       <c r="K8" s="137"/>
-      <c r="L8" s="235"/>
-      <c r="M8" s="235"/>
+      <c r="L8" s="239"/>
+      <c r="M8" s="239"/>
     </row>
     <row r="9" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A9" s="238"/>
+      <c r="A9" s="235"/>
       <c r="B9" s="241"/>
-      <c r="C9" s="238"/>
+      <c r="C9" s="235"/>
       <c r="D9" s="214" t="s">
         <v>67</v>
       </c>
-      <c r="E9" s="240"/>
+      <c r="E9" s="238"/>
       <c r="F9" s="237"/>
       <c r="G9" s="237"/>
       <c r="H9" s="237"/>
-      <c r="I9" s="235"/>
-      <c r="J9" s="235"/>
+      <c r="I9" s="239"/>
+      <c r="J9" s="239"/>
       <c r="K9" s="137"/>
-      <c r="L9" s="235"/>
-      <c r="M9" s="235"/>
+      <c r="L9" s="239"/>
+      <c r="M9" s="239"/>
     </row>
     <row r="10" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A10" s="238"/>
+      <c r="A10" s="235"/>
       <c r="B10" s="241"/>
-      <c r="C10" s="238"/>
+      <c r="C10" s="235"/>
       <c r="D10" s="214" t="s">
         <v>68</v>
       </c>
-      <c r="E10" s="240"/>
+      <c r="E10" s="238"/>
       <c r="F10" s="237"/>
       <c r="G10" s="237"/>
       <c r="H10" s="237"/>
-      <c r="I10" s="235"/>
-      <c r="J10" s="235"/>
+      <c r="I10" s="239"/>
+      <c r="J10" s="239"/>
       <c r="K10" s="137"/>
-      <c r="L10" s="235"/>
-      <c r="M10" s="235"/>
+      <c r="L10" s="239"/>
+      <c r="M10" s="239"/>
     </row>
     <row r="11" spans="1:13" ht="14.4" customHeight="1">
-      <c r="A11" s="238"/>
+      <c r="A11" s="235"/>
       <c r="B11" s="241"/>
-      <c r="C11" s="238"/>
+      <c r="C11" s="235"/>
       <c r="D11" s="152" t="s">
         <v>69</v>
       </c>
-      <c r="E11" s="240"/>
+      <c r="E11" s="238"/>
       <c r="F11" s="237"/>
       <c r="G11" s="237"/>
       <c r="H11" s="237"/>
-      <c r="I11" s="235"/>
-      <c r="J11" s="235"/>
+      <c r="I11" s="239"/>
+      <c r="J11" s="239"/>
       <c r="K11" s="153"/>
-      <c r="L11" s="235"/>
-      <c r="M11" s="235"/>
+      <c r="L11" s="239"/>
+      <c r="M11" s="239"/>
     </row>
     <row r="12" spans="1:13" ht="14.4" customHeight="1">
-      <c r="A12" s="238"/>
+      <c r="A12" s="235"/>
       <c r="B12" s="241"/>
-      <c r="C12" s="238"/>
+      <c r="C12" s="235"/>
       <c r="D12" s="152" t="s">
         <v>70</v>
       </c>
-      <c r="E12" s="240"/>
+      <c r="E12" s="238"/>
       <c r="F12" s="237"/>
       <c r="G12" s="237"/>
       <c r="H12" s="237"/>
-      <c r="I12" s="235"/>
-      <c r="J12" s="235"/>
+      <c r="I12" s="239"/>
+      <c r="J12" s="239"/>
       <c r="K12" s="137"/>
-      <c r="L12" s="235"/>
-      <c r="M12" s="235"/>
+      <c r="L12" s="239"/>
+      <c r="M12" s="239"/>
     </row>
     <row r="13" spans="1:13" ht="43.2">
       <c r="A13" s="125" t="s">
@@ -10831,7 +10842,7 @@
         <v>92</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="F16" s="124" t="s">
         <v>17</v>
@@ -11525,17 +11536,17 @@
     <sortCondition ref="A2:A24"/>
   </sortState>
   <mergeCells count="11">
+    <mergeCell ref="M8:M12"/>
+    <mergeCell ref="L8:L12"/>
+    <mergeCell ref="H8:H12"/>
+    <mergeCell ref="I8:I12"/>
+    <mergeCell ref="J8:J12"/>
     <mergeCell ref="G8:G12"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="B8:B12"/>
     <mergeCell ref="C8:C12"/>
     <mergeCell ref="E8:E12"/>
     <mergeCell ref="F8:F12"/>
-    <mergeCell ref="M8:M12"/>
-    <mergeCell ref="L8:L12"/>
-    <mergeCell ref="H8:H12"/>
-    <mergeCell ref="I8:I12"/>
-    <mergeCell ref="J8:J12"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F8">
     <cfRule type="cellIs" dxfId="190" priority="16" operator="equal">
@@ -11807,7 +11818,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="132" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="F4" s="124" t="s">
         <v>35</v>
@@ -12182,19 +12193,19 @@
       <c r="N13" s="129"/>
     </row>
     <row r="14" spans="1:14" ht="43.2">
-      <c r="A14" s="238" t="s">
+      <c r="A14" s="235" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="239" t="s">
+      <c r="B14" s="236" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="238" t="s">
+      <c r="C14" s="235" t="s">
         <v>62</v>
       </c>
       <c r="D14" s="213" t="s">
         <v>63</v>
       </c>
-      <c r="E14" s="240" t="s">
+      <c r="E14" s="238" t="s">
         <v>199</v>
       </c>
       <c r="F14" s="237" t="s">
@@ -12206,78 +12217,78 @@
       <c r="H14" s="237" t="s">
         <v>19</v>
       </c>
-      <c r="I14" s="235" t="s">
+      <c r="I14" s="239" t="s">
         <v>20</v>
       </c>
-      <c r="J14" s="235" t="s">
+      <c r="J14" s="239" t="s">
         <v>66</v>
       </c>
-      <c r="K14" s="236"/>
-      <c r="L14" s="235"/>
+      <c r="K14" s="240"/>
+      <c r="L14" s="239"/>
     </row>
     <row r="15" spans="1:14" ht="43.2">
-      <c r="A15" s="238"/>
-      <c r="B15" s="239"/>
-      <c r="C15" s="238"/>
+      <c r="A15" s="235"/>
+      <c r="B15" s="236"/>
+      <c r="C15" s="235"/>
       <c r="D15" s="214" t="s">
         <v>67</v>
       </c>
-      <c r="E15" s="240"/>
+      <c r="E15" s="238"/>
       <c r="F15" s="237"/>
       <c r="G15" s="237"/>
       <c r="H15" s="237"/>
-      <c r="I15" s="235"/>
-      <c r="J15" s="235"/>
-      <c r="K15" s="236"/>
-      <c r="L15" s="235"/>
+      <c r="I15" s="239"/>
+      <c r="J15" s="239"/>
+      <c r="K15" s="240"/>
+      <c r="L15" s="239"/>
     </row>
     <row r="16" spans="1:14" ht="28.8">
-      <c r="A16" s="238"/>
-      <c r="B16" s="239"/>
-      <c r="C16" s="238"/>
+      <c r="A16" s="235"/>
+      <c r="B16" s="236"/>
+      <c r="C16" s="235"/>
       <c r="D16" s="214" t="s">
         <v>68</v>
       </c>
-      <c r="E16" s="240"/>
+      <c r="E16" s="238"/>
       <c r="F16" s="237"/>
       <c r="G16" s="237"/>
       <c r="H16" s="237"/>
-      <c r="I16" s="235"/>
-      <c r="J16" s="235"/>
-      <c r="K16" s="236"/>
-      <c r="L16" s="235"/>
+      <c r="I16" s="239"/>
+      <c r="J16" s="239"/>
+      <c r="K16" s="240"/>
+      <c r="L16" s="239"/>
     </row>
     <row r="17" spans="1:14">
-      <c r="A17" s="238"/>
-      <c r="B17" s="239"/>
-      <c r="C17" s="238"/>
+      <c r="A17" s="235"/>
+      <c r="B17" s="236"/>
+      <c r="C17" s="235"/>
       <c r="D17" s="152" t="s">
         <v>69</v>
       </c>
-      <c r="E17" s="240"/>
+      <c r="E17" s="238"/>
       <c r="F17" s="237"/>
       <c r="G17" s="237"/>
       <c r="H17" s="237"/>
-      <c r="I17" s="235"/>
-      <c r="J17" s="235"/>
-      <c r="K17" s="236"/>
-      <c r="L17" s="235"/>
+      <c r="I17" s="239"/>
+      <c r="J17" s="239"/>
+      <c r="K17" s="240"/>
+      <c r="L17" s="239"/>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="238"/>
-      <c r="B18" s="239"/>
-      <c r="C18" s="238"/>
+      <c r="A18" s="235"/>
+      <c r="B18" s="236"/>
+      <c r="C18" s="235"/>
       <c r="D18" s="152" t="s">
         <v>70</v>
       </c>
-      <c r="E18" s="240"/>
+      <c r="E18" s="238"/>
       <c r="F18" s="237"/>
       <c r="G18" s="237"/>
       <c r="H18" s="237"/>
-      <c r="I18" s="235"/>
-      <c r="J18" s="235"/>
-      <c r="K18" s="236"/>
-      <c r="L18" s="235"/>
+      <c r="I18" s="239"/>
+      <c r="J18" s="239"/>
+      <c r="K18" s="240"/>
+      <c r="L18" s="239"/>
     </row>
     <row r="19" spans="1:14" ht="28.8">
       <c r="A19" s="125" t="s">
@@ -12555,7 +12566,7 @@
         <v>237</v>
       </c>
       <c r="E26" s="132" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="F26" s="124" t="s">
         <v>17</v>
@@ -12931,7 +12942,7 @@
         <v>285</v>
       </c>
       <c r="E36" s="138" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="F36" s="124" t="s">
         <v>17</v>
@@ -13117,7 +13128,7 @@
       </c>
       <c r="L40" s="107"/>
     </row>
-    <row r="41" spans="1:14" ht="28.8">
+    <row r="41" spans="1:14" ht="158.4">
       <c r="A41" s="125" t="s">
         <v>306</v>
       </c>
@@ -13131,7 +13142,7 @@
         <v>16</v>
       </c>
       <c r="E41" s="74" t="s">
-        <v>309</v>
+        <v>674</v>
       </c>
       <c r="F41" s="127" t="s">
         <v>17</v>
@@ -13152,30 +13163,30 @@
         <v>137</v>
       </c>
       <c r="L41" s="129" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="M41" s="129" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="N41" s="129" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="42" spans="1:14" ht="72">
       <c r="A42" s="121" t="s">
+        <v>310</v>
+      </c>
+      <c r="B42" s="35" t="s">
         <v>311</v>
       </c>
-      <c r="B42" s="35" t="s">
+      <c r="C42" s="121" t="s">
         <v>312</v>
-      </c>
-      <c r="C42" s="121" t="s">
-        <v>313</v>
       </c>
       <c r="D42" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E42" s="132" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F42" s="124" t="s">
         <v>17</v>
@@ -13196,26 +13207,26 @@
         <v>138</v>
       </c>
       <c r="L42" s="141" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M42" s="107"/>
       <c r="N42" s="107"/>
     </row>
     <row r="43" spans="1:14" ht="28.8">
       <c r="A43" s="125" t="s">
+        <v>315</v>
+      </c>
+      <c r="B43" s="74" t="s">
         <v>316</v>
       </c>
-      <c r="B43" s="74" t="s">
+      <c r="C43" s="125" t="s">
         <v>317</v>
-      </c>
-      <c r="C43" s="125" t="s">
-        <v>318</v>
       </c>
       <c r="D43" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E43" s="205" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="F43" s="127" t="s">
         <v>17</v>
@@ -13236,26 +13247,26 @@
         <v>139</v>
       </c>
       <c r="L43" s="134" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="M43" s="129"/>
       <c r="N43" s="129"/>
     </row>
     <row r="44" spans="1:14" ht="57.6">
       <c r="A44" s="121" t="s">
+        <v>320</v>
+      </c>
+      <c r="B44" s="35" t="s">
         <v>321</v>
       </c>
-      <c r="B44" s="35" t="s">
+      <c r="C44" s="121" t="s">
         <v>322</v>
       </c>
-      <c r="C44" s="121" t="s">
+      <c r="D44" s="143" t="s">
         <v>323</v>
       </c>
-      <c r="D44" s="143" t="s">
+      <c r="E44" s="132" t="s">
         <v>324</v>
-      </c>
-      <c r="E44" s="132" t="s">
-        <v>325</v>
       </c>
       <c r="F44" s="124" t="s">
         <v>17</v>
@@ -13293,7 +13304,7 @@
         <v>16</v>
       </c>
       <c r="E45" s="74" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="F45" s="127" t="s">
         <v>17</v>
@@ -13314,36 +13325,36 @@
         <v>125</v>
       </c>
       <c r="L45" s="129" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="M45" s="129" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="N45" s="129" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="46" spans="1:14" ht="57.6">
       <c r="A46" s="121" t="s">
+        <v>326</v>
+      </c>
+      <c r="B46" s="35" t="s">
         <v>327</v>
       </c>
-      <c r="B46" s="35" t="s">
+      <c r="C46" s="141" t="s">
         <v>328</v>
-      </c>
-      <c r="C46" s="141" t="s">
-        <v>329</v>
       </c>
       <c r="D46" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E46" s="132" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F46" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G46" s="124" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="H46" s="124" t="s">
         <v>81</v>
@@ -13363,19 +13374,19 @@
     </row>
     <row r="47" spans="1:14" ht="74.25" customHeight="1">
       <c r="A47" s="125" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B47" s="74" t="s">
         <v>127</v>
       </c>
       <c r="C47" s="125" t="s">
+        <v>332</v>
+      </c>
+      <c r="D47" s="142" t="s">
         <v>333</v>
       </c>
-      <c r="D47" s="142" t="s">
+      <c r="E47" s="74" t="s">
         <v>334</v>
-      </c>
-      <c r="E47" s="74" t="s">
-        <v>335</v>
       </c>
       <c r="F47" s="127" t="s">
         <v>35</v>
@@ -13413,7 +13424,7 @@
         <v>16</v>
       </c>
       <c r="E48" s="132" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F48" s="124" t="s">
         <v>35</v>
@@ -13439,19 +13450,19 @@
     </row>
     <row r="49" spans="1:14" ht="57.6">
       <c r="A49" s="125" t="s">
+        <v>336</v>
+      </c>
+      <c r="B49" s="74" t="s">
         <v>337</v>
       </c>
-      <c r="B49" s="74" t="s">
+      <c r="C49" s="125" t="s">
         <v>338</v>
       </c>
-      <c r="C49" s="125" t="s">
+      <c r="D49" s="217" t="s">
         <v>339</v>
       </c>
-      <c r="D49" s="217" t="s">
+      <c r="E49" s="83" t="s">
         <v>340</v>
-      </c>
-      <c r="E49" s="83" t="s">
-        <v>341</v>
       </c>
       <c r="F49" s="127" t="s">
         <v>17</v>
@@ -13477,19 +13488,19 @@
     </row>
     <row r="50" spans="1:14" ht="28.8">
       <c r="A50" s="121" t="s">
+        <v>341</v>
+      </c>
+      <c r="B50" s="35" t="s">
         <v>342</v>
       </c>
-      <c r="B50" s="35" t="s">
+      <c r="C50" s="121" t="s">
         <v>343</v>
-      </c>
-      <c r="C50" s="121" t="s">
-        <v>344</v>
       </c>
       <c r="D50" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E50" s="132" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="F50" s="124" t="s">
         <v>17</v>
@@ -13515,19 +13526,19 @@
     </row>
     <row r="51" spans="1:14" ht="28.8">
       <c r="A51" s="125" t="s">
+        <v>345</v>
+      </c>
+      <c r="B51" s="74" t="s">
         <v>346</v>
       </c>
-      <c r="B51" s="74" t="s">
+      <c r="C51" s="125" t="s">
         <v>347</v>
-      </c>
-      <c r="C51" s="125" t="s">
-        <v>348</v>
       </c>
       <c r="D51" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E51" s="74" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="F51" s="127" t="s">
         <v>17</v>
@@ -13553,13 +13564,13 @@
     </row>
     <row r="52" spans="1:14" ht="84.75" customHeight="1">
       <c r="A52" s="121" t="s">
+        <v>349</v>
+      </c>
+      <c r="B52" s="35" t="s">
         <v>350</v>
       </c>
-      <c r="B52" s="35" t="s">
+      <c r="C52" s="121" t="s">
         <v>351</v>
-      </c>
-      <c r="C52" s="121" t="s">
-        <v>352</v>
       </c>
       <c r="D52" s="132" t="s">
         <v>16</v>
@@ -13569,7 +13580,7 @@
         <v>17</v>
       </c>
       <c r="G52" s="124" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="H52" s="124" t="s">
         <v>19</v>
@@ -13605,17 +13616,17 @@
     <sortCondition ref="A2:A53"/>
   </sortState>
   <mergeCells count="11">
-    <mergeCell ref="A14:A18"/>
-    <mergeCell ref="B14:B18"/>
-    <mergeCell ref="C14:C18"/>
-    <mergeCell ref="F14:F18"/>
-    <mergeCell ref="E14:E18"/>
     <mergeCell ref="L14:L18"/>
     <mergeCell ref="K14:K18"/>
     <mergeCell ref="G14:G18"/>
     <mergeCell ref="H14:H18"/>
     <mergeCell ref="I14:I18"/>
     <mergeCell ref="J14:J18"/>
+    <mergeCell ref="A14:A18"/>
+    <mergeCell ref="B14:B18"/>
+    <mergeCell ref="C14:C18"/>
+    <mergeCell ref="F14:F18"/>
+    <mergeCell ref="E14:E18"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F14 F19:F53">
     <cfRule type="cellIs" dxfId="171" priority="8" operator="equal">
@@ -13782,42 +13793,42 @@
         <v>10</v>
       </c>
       <c r="L1" s="223" t="s">
+        <v>353</v>
+      </c>
+      <c r="M1" s="223" t="s">
         <v>354</v>
       </c>
-      <c r="M1" s="223" t="s">
+      <c r="N1" s="108" t="s">
         <v>355</v>
       </c>
-      <c r="N1" s="108" t="s">
+      <c r="O1" s="108" t="s">
         <v>356</v>
       </c>
-      <c r="O1" s="108" t="s">
+      <c r="P1" s="223" t="s">
         <v>357</v>
       </c>
-      <c r="P1" s="223" t="s">
+      <c r="Q1" s="223" t="s">
         <v>358</v>
       </c>
-      <c r="Q1" s="223" t="s">
+      <c r="R1" s="224" t="s">
         <v>359</v>
       </c>
-      <c r="R1" s="224" t="s">
+      <c r="S1" s="224" t="s">
         <v>360</v>
       </c>
-      <c r="S1" s="224" t="s">
+      <c r="T1" s="224" t="s">
         <v>361</v>
       </c>
-      <c r="T1" s="224" t="s">
+      <c r="U1" s="224" t="s">
         <v>362</v>
       </c>
-      <c r="U1" s="224" t="s">
+      <c r="V1" s="233" t="s">
         <v>363</v>
-      </c>
-      <c r="V1" s="233" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="28.8">
       <c r="A2" s="64" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B2" s="157" t="s">
         <v>61</v>
@@ -13826,10 +13837,10 @@
         <v>62</v>
       </c>
       <c r="D2" s="152" t="s">
+        <v>365</v>
+      </c>
+      <c r="E2" s="158" t="s">
         <v>366</v>
-      </c>
-      <c r="E2" s="158" t="s">
-        <v>367</v>
       </c>
       <c r="F2" s="159" t="s">
         <v>17</v>
@@ -13849,25 +13860,25 @@
     </row>
     <row r="3" spans="1:22" ht="115.2">
       <c r="A3" s="68" t="s">
+        <v>367</v>
+      </c>
+      <c r="B3" s="61" t="s">
         <v>368</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="C3" s="68" t="s">
         <v>369</v>
-      </c>
-      <c r="C3" s="68" t="s">
-        <v>370</v>
       </c>
       <c r="D3" s="162" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="184" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="F3" s="163" t="s">
         <v>35</v>
       </c>
       <c r="G3" s="163" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H3" s="163">
         <v>1</v>
@@ -13879,7 +13890,7 @@
         <v>66</v>
       </c>
       <c r="K3" s="136" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="L3" s="129"/>
       <c r="M3" s="129"/>
@@ -13903,10 +13914,10 @@
         <v>213</v>
       </c>
       <c r="D4" s="71" t="s">
+        <v>372</v>
+      </c>
+      <c r="E4" s="158" t="s">
         <v>373</v>
-      </c>
-      <c r="E4" s="158" t="s">
-        <v>374</v>
       </c>
       <c r="F4" s="159" t="s">
         <v>35</v>
@@ -13921,28 +13932,28 @@
         <v>28</v>
       </c>
       <c r="J4" s="160" t="s">
+        <v>374</v>
+      </c>
+      <c r="K4" s="136" t="s">
         <v>375</v>
-      </c>
-      <c r="K4" s="136" t="s">
-        <v>376</v>
       </c>
       <c r="L4" s="107"/>
     </row>
     <row r="5" spans="1:22" ht="43.2">
       <c r="A5" s="165" t="s">
+        <v>376</v>
+      </c>
+      <c r="B5" s="75" t="s">
         <v>377</v>
       </c>
-      <c r="B5" s="75" t="s">
+      <c r="C5" s="165" t="s">
         <v>378</v>
-      </c>
-      <c r="C5" s="165" t="s">
-        <v>379</v>
       </c>
       <c r="D5" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="75" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F5" s="166" t="s">
         <v>35</v>
@@ -13960,7 +13971,7 @@
         <v>29</v>
       </c>
       <c r="K5" s="136" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="L5" s="129"/>
       <c r="M5" s="129"/>
@@ -13975,19 +13986,19 @@
     </row>
     <row r="6" spans="1:22" ht="72">
       <c r="A6" s="168" t="s">
+        <v>381</v>
+      </c>
+      <c r="B6" s="151" t="s">
         <v>382</v>
       </c>
-      <c r="B6" s="151" t="s">
+      <c r="C6" s="168" t="s">
         <v>383</v>
-      </c>
-      <c r="C6" s="168" t="s">
-        <v>384</v>
       </c>
       <c r="D6" s="169" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="151" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F6" s="133" t="s">
         <v>17</v>
@@ -14009,19 +14020,19 @@
     </row>
     <row r="7" spans="1:22" ht="115.2">
       <c r="A7" s="125" t="s">
+        <v>385</v>
+      </c>
+      <c r="B7" s="74" t="s">
         <v>386</v>
       </c>
-      <c r="B7" s="74" t="s">
+      <c r="C7" s="125" t="s">
         <v>387</v>
       </c>
-      <c r="C7" s="125" t="s">
+      <c r="D7" s="171" t="s">
         <v>388</v>
       </c>
-      <c r="D7" s="171" t="s">
+      <c r="E7" s="81" t="s">
         <v>389</v>
-      </c>
-      <c r="E7" s="81" t="s">
-        <v>390</v>
       </c>
       <c r="F7" s="127" t="s">
         <v>17</v>
@@ -14052,19 +14063,19 @@
     </row>
     <row r="8" spans="1:22" ht="28.8">
       <c r="A8" s="64" t="s">
+        <v>336</v>
+      </c>
+      <c r="B8" s="157" t="s">
         <v>337</v>
       </c>
-      <c r="B8" s="157" t="s">
+      <c r="C8" s="172" t="s">
         <v>338</v>
       </c>
-      <c r="C8" s="172" t="s">
-        <v>339</v>
-      </c>
       <c r="D8" s="143" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E8" s="135" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="F8" s="159" t="s">
         <v>17</v>
@@ -14082,13 +14093,13 @@
         <v>29</v>
       </c>
       <c r="K8" s="136" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="L8" s="107"/>
     </row>
     <row r="9" spans="1:22" ht="43.2">
       <c r="A9" s="165" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B9" s="75" t="s">
         <v>77</v>
@@ -14100,7 +14111,7 @@
         <v>16</v>
       </c>
       <c r="E9" s="173" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F9" s="166" t="s">
         <v>35</v>
@@ -14118,7 +14129,7 @@
         <v>66</v>
       </c>
       <c r="K9" s="136" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="L9" s="129"/>
       <c r="M9" s="129"/>
@@ -14863,45 +14874,45 @@
         <v>10</v>
       </c>
       <c r="L1" s="225" t="s">
+        <v>395</v>
+      </c>
+      <c r="M1" s="108" t="s">
         <v>396</v>
       </c>
-      <c r="M1" s="108" t="s">
+      <c r="N1" s="223" t="s">
         <v>397</v>
       </c>
-      <c r="N1" s="223" t="s">
+      <c r="O1" s="224" t="s">
         <v>398</v>
       </c>
-      <c r="O1" s="224" t="s">
+      <c r="P1" s="232" t="s">
         <v>399</v>
       </c>
-      <c r="P1" s="232" t="s">
+      <c r="Q1" s="233" t="s">
         <v>400</v>
-      </c>
-      <c r="Q1" s="233" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="64.349999999999994" customHeight="1">
       <c r="A2" s="64" t="s">
+        <v>401</v>
+      </c>
+      <c r="B2" s="45" t="s">
         <v>402</v>
       </c>
-      <c r="B2" s="45" t="s">
+      <c r="C2" s="172" t="s">
         <v>403</v>
-      </c>
-      <c r="C2" s="172" t="s">
-        <v>404</v>
       </c>
       <c r="D2" s="64" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="88" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="F2" s="159" t="s">
         <v>17</v>
       </c>
       <c r="G2" s="159" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H2" s="159" t="s">
         <v>19</v>
@@ -14913,31 +14924,31 @@
         <v>29</v>
       </c>
       <c r="K2" s="156" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="L2" s="136"/>
     </row>
     <row r="3" spans="1:17" ht="129.6">
       <c r="A3" s="68" t="s">
+        <v>406</v>
+      </c>
+      <c r="B3" s="61" t="s">
         <v>407</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="C3" s="68" t="s">
         <v>408</v>
-      </c>
-      <c r="C3" s="68" t="s">
-        <v>409</v>
       </c>
       <c r="D3" s="183" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="184" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="F3" s="163" t="s">
         <v>35</v>
       </c>
       <c r="G3" s="163" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H3" s="163">
         <v>1</v>
@@ -14949,7 +14960,7 @@
         <v>29</v>
       </c>
       <c r="K3" s="156" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="L3" s="75"/>
       <c r="M3" s="61"/>
@@ -14959,25 +14970,25 @@
     </row>
     <row r="4" spans="1:17" ht="28.8">
       <c r="A4" s="64" t="s">
+        <v>410</v>
+      </c>
+      <c r="B4" s="45" t="s">
         <v>411</v>
       </c>
-      <c r="B4" s="45" t="s">
+      <c r="C4" s="64" t="s">
         <v>412</v>
-      </c>
-      <c r="C4" s="64" t="s">
-        <v>413</v>
       </c>
       <c r="D4" s="64" t="s">
         <v>16</v>
       </c>
       <c r="E4" s="88" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F4" s="159" t="s">
         <v>35</v>
       </c>
       <c r="G4" s="159" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H4" s="159">
         <v>1</v>
@@ -14989,7 +15000,7 @@
         <v>29</v>
       </c>
       <c r="K4" s="156" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="L4" s="136"/>
     </row>
@@ -15812,27 +15823,27 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
+        <v>416</v>
+      </c>
+      <c r="M1" s="223" t="s">
         <v>417</v>
-      </c>
-      <c r="M1" s="223" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="28.8">
       <c r="A2" s="121" t="s">
+        <v>418</v>
+      </c>
+      <c r="B2" s="35" t="s">
         <v>419</v>
       </c>
-      <c r="B2" s="35" t="s">
+      <c r="C2" s="121" t="s">
         <v>420</v>
-      </c>
-      <c r="C2" s="121" t="s">
-        <v>421</v>
       </c>
       <c r="D2" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="35" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>17</v>
@@ -15850,30 +15861,30 @@
         <v>37</v>
       </c>
       <c r="K2" s="98" t="s">
+        <v>422</v>
+      </c>
+      <c r="L2" s="141" t="s">
         <v>423</v>
       </c>
-      <c r="L2" s="141" t="s">
-        <v>424</v>
-      </c>
       <c r="M2" s="141" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="72">
       <c r="A3" s="125" t="s">
+        <v>424</v>
+      </c>
+      <c r="B3" s="74" t="s">
         <v>425</v>
       </c>
-      <c r="B3" s="74" t="s">
+      <c r="C3" s="125" t="s">
         <v>426</v>
-      </c>
-      <c r="C3" s="125" t="s">
-        <v>427</v>
       </c>
       <c r="D3" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="85" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F3" s="127" t="s">
         <v>35</v>
@@ -15891,7 +15902,7 @@
         <v>37</v>
       </c>
       <c r="K3" s="98" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="L3" s="129"/>
       <c r="M3" s="129"/>
@@ -15910,7 +15921,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="35" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="F4" s="124" t="s">
         <v>17</v>
@@ -15935,25 +15946,25 @@
     </row>
     <row r="5" spans="1:13" ht="43.2">
       <c r="A5" s="125" t="s">
+        <v>430</v>
+      </c>
+      <c r="B5" s="74" t="s">
         <v>431</v>
       </c>
-      <c r="B5" s="74" t="s">
+      <c r="C5" s="134" t="s">
         <v>432</v>
-      </c>
-      <c r="C5" s="134" t="s">
-        <v>433</v>
       </c>
       <c r="D5" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="126" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="F5" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G5" s="127" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="H5" s="127">
         <v>1</v>
@@ -15965,32 +15976,32 @@
         <v>29</v>
       </c>
       <c r="K5" s="98" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="L5" s="129"/>
       <c r="M5" s="129"/>
     </row>
     <row r="6" spans="1:13" ht="57.6">
       <c r="A6" s="121" t="s">
+        <v>436</v>
+      </c>
+      <c r="B6" s="35" t="s">
         <v>437</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="C6" s="121" t="s">
         <v>438</v>
-      </c>
-      <c r="C6" s="121" t="s">
-        <v>439</v>
       </c>
       <c r="D6" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="35" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="F6" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G6" s="128" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="H6" s="124" t="s">
         <v>81</v>
@@ -16002,36 +16013,36 @@
         <v>29</v>
       </c>
       <c r="K6" s="98" t="s">
+        <v>441</v>
+      </c>
+      <c r="L6" s="107" t="s">
         <v>442</v>
       </c>
-      <c r="L6" s="107" t="s">
-        <v>443</v>
-      </c>
       <c r="M6" s="107" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="43.2">
       <c r="A7" s="125" t="s">
+        <v>443</v>
+      </c>
+      <c r="B7" s="74" t="s">
         <v>444</v>
       </c>
-      <c r="B7" s="74" t="s">
+      <c r="C7" s="134" t="s">
         <v>445</v>
       </c>
-      <c r="C7" s="134" t="s">
+      <c r="D7" s="185" t="s">
         <v>446</v>
       </c>
-      <c r="D7" s="185" t="s">
+      <c r="E7" s="126" t="s">
         <v>447</v>
-      </c>
-      <c r="E7" s="126" t="s">
-        <v>448</v>
       </c>
       <c r="F7" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G7" s="156" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="H7" s="127" t="s">
         <v>81</v>
@@ -16043,7 +16054,7 @@
         <v>29</v>
       </c>
       <c r="K7" s="98" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="L7" s="129"/>
       <c r="M7" s="129"/>
@@ -16062,7 +16073,7 @@
         <v>16</v>
       </c>
       <c r="E8" s="35" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F8" s="124" t="s">
         <v>17</v>
@@ -16080,7 +16091,7 @@
         <v>29</v>
       </c>
       <c r="K8" s="98" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="L8" s="107"/>
       <c r="M8" s="107"/>
@@ -16099,7 +16110,7 @@
         <v>16</v>
       </c>
       <c r="E9" s="126" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="F9" s="127" t="s">
         <v>17</v>
@@ -16117,26 +16128,26 @@
         <v>29</v>
       </c>
       <c r="K9" s="98" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="L9" s="129"/>
       <c r="M9" s="129"/>
     </row>
     <row r="10" spans="1:13" ht="57.6">
       <c r="A10" s="121" t="s">
+        <v>454</v>
+      </c>
+      <c r="B10" s="35" t="s">
         <v>455</v>
       </c>
-      <c r="B10" s="35" t="s">
+      <c r="C10" s="141" t="s">
         <v>456</v>
-      </c>
-      <c r="C10" s="141" t="s">
-        <v>457</v>
       </c>
       <c r="D10" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F10" s="124" t="s">
         <v>17</v>
@@ -16154,32 +16165,32 @@
         <v>37</v>
       </c>
       <c r="K10" s="98" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="L10" s="107"/>
       <c r="M10" s="107"/>
     </row>
     <row r="11" spans="1:13" ht="43.2">
       <c r="A11" s="125" t="s">
+        <v>459</v>
+      </c>
+      <c r="B11" s="74" t="s">
         <v>460</v>
       </c>
-      <c r="B11" s="74" t="s">
+      <c r="C11" s="125" t="s">
         <v>461</v>
       </c>
-      <c r="C11" s="125" t="s">
+      <c r="D11" s="154" t="s">
         <v>462</v>
       </c>
-      <c r="D11" s="154" t="s">
-        <v>463</v>
-      </c>
       <c r="E11" s="126" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="F11" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G11" s="127" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="H11" s="127">
         <v>1</v>
@@ -16191,7 +16202,7 @@
         <v>29</v>
       </c>
       <c r="K11" s="99" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="L11" s="129"/>
       <c r="M11" s="129"/>
@@ -16210,7 +16221,7 @@
         <v>85</v>
       </c>
       <c r="E12" s="138" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="F12" s="124" t="s">
         <v>17</v>
@@ -16228,14 +16239,14 @@
         <v>29</v>
       </c>
       <c r="K12" s="98" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="L12" s="107"/>
       <c r="M12" s="107"/>
     </row>
     <row r="13" spans="1:13" ht="72">
       <c r="A13" s="125" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B13" s="74" t="s">
         <v>90</v>
@@ -16247,13 +16258,13 @@
         <v>92</v>
       </c>
       <c r="E13" s="80" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G13" s="127" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="H13" s="127">
         <v>1</v>
@@ -16265,14 +16276,14 @@
         <v>37</v>
       </c>
       <c r="K13" s="98" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="L13" s="129"/>
       <c r="M13" s="129"/>
     </row>
     <row r="14" spans="1:13" ht="72">
       <c r="A14" s="121" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B14" s="35" t="s">
         <v>175</v>
@@ -16284,7 +16295,7 @@
         <v>16</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="F14" s="124" t="s">
         <v>17</v>
@@ -16302,32 +16313,32 @@
         <v>29</v>
       </c>
       <c r="K14" s="98" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="L14" s="107"/>
       <c r="M14" s="107"/>
     </row>
     <row r="15" spans="1:13" ht="100.8">
       <c r="A15" s="125" t="s">
+        <v>474</v>
+      </c>
+      <c r="B15" s="74" t="s">
         <v>475</v>
       </c>
-      <c r="B15" s="74" t="s">
+      <c r="C15" s="125" t="s">
         <v>476</v>
       </c>
-      <c r="C15" s="125" t="s">
+      <c r="D15" s="185" t="s">
+        <v>446</v>
+      </c>
+      <c r="E15" s="80" t="s">
         <v>477</v>
-      </c>
-      <c r="D15" s="185" t="s">
-        <v>447</v>
-      </c>
-      <c r="E15" s="80" t="s">
-        <v>478</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G15" s="127" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="H15" s="127" t="s">
         <v>81</v>
@@ -16339,7 +16350,7 @@
         <v>29</v>
       </c>
       <c r="K15" s="98" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L15" s="129"/>
       <c r="M15" s="129"/>
@@ -16374,32 +16385,32 @@
         <v>29</v>
       </c>
       <c r="K16" s="98" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L16" s="107"/>
       <c r="M16" s="107"/>
     </row>
     <row r="17" spans="1:13" ht="57.6">
       <c r="A17" s="125" t="s">
+        <v>480</v>
+      </c>
+      <c r="B17" s="74" t="s">
         <v>481</v>
       </c>
-      <c r="B17" s="74" t="s">
+      <c r="C17" s="125" t="s">
         <v>482</v>
       </c>
-      <c r="C17" s="125" t="s">
+      <c r="D17" s="185" t="s">
+        <v>446</v>
+      </c>
+      <c r="E17" s="74" t="s">
         <v>483</v>
-      </c>
-      <c r="D17" s="185" t="s">
-        <v>447</v>
-      </c>
-      <c r="E17" s="74" t="s">
-        <v>484</v>
       </c>
       <c r="F17" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G17" s="127" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="H17" s="127" t="s">
         <v>81</v>
@@ -16411,7 +16422,7 @@
         <v>29</v>
       </c>
       <c r="K17" s="98" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="L17" s="129"/>
       <c r="M17" s="129"/>
@@ -16430,7 +16441,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="132" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="F18" s="124" t="s">
         <v>17</v>
@@ -16448,12 +16459,12 @@
         <v>29</v>
       </c>
       <c r="K18" s="98" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="L18" s="107"/>
       <c r="M18" s="107"/>
     </row>
-    <row r="19" spans="1:13" ht="28.8">
+    <row r="19" spans="1:13" ht="185.4" customHeight="1">
       <c r="A19" s="125" t="s">
         <v>306</v>
       </c>
@@ -16461,11 +16472,11 @@
         <v>307</v>
       </c>
       <c r="C19" s="125" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D19" s="126"/>
-      <c r="E19" s="80" t="s">
-        <v>309</v>
+      <c r="E19" s="74" t="s">
+        <v>675</v>
       </c>
       <c r="F19" s="127" t="s">
         <v>17</v>
@@ -16484,10 +16495,10 @@
       </c>
       <c r="K19" s="104"/>
       <c r="L19" s="129" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="M19" s="129" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="129.6">
@@ -16504,7 +16515,7 @@
         <v>16</v>
       </c>
       <c r="E20" s="79" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="F20" s="190" t="s">
         <v>35</v>
@@ -16522,26 +16533,26 @@
         <v>29</v>
       </c>
       <c r="K20" s="99" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="L20" s="107"/>
       <c r="M20" s="107"/>
     </row>
     <row r="21" spans="1:13" ht="43.2">
       <c r="A21" s="125" t="s">
+        <v>320</v>
+      </c>
+      <c r="B21" s="74" t="s">
         <v>321</v>
       </c>
-      <c r="B21" s="74" t="s">
+      <c r="C21" s="125" t="s">
         <v>322</v>
       </c>
-      <c r="C21" s="125" t="s">
-        <v>323</v>
-      </c>
       <c r="D21" s="154" t="s">
+        <v>491</v>
+      </c>
+      <c r="E21" s="81" t="s">
         <v>492</v>
-      </c>
-      <c r="E21" s="81" t="s">
-        <v>493</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>17</v>
@@ -16559,32 +16570,32 @@
         <v>29</v>
       </c>
       <c r="K21" s="98" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="L21" s="129"/>
       <c r="M21" s="129"/>
     </row>
     <row r="22" spans="1:13" ht="57.6">
       <c r="A22" s="121" t="s">
+        <v>326</v>
+      </c>
+      <c r="B22" s="35" t="s">
         <v>327</v>
       </c>
-      <c r="B22" s="35" t="s">
+      <c r="C22" s="121" t="s">
         <v>328</v>
-      </c>
-      <c r="C22" s="121" t="s">
-        <v>329</v>
       </c>
       <c r="D22" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E22" s="132" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G22" s="124" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="H22" s="124" t="s">
         <v>81</v>
@@ -16613,7 +16624,7 @@
         <v>16</v>
       </c>
       <c r="E23" s="126" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>17</v>
@@ -16631,7 +16642,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="98" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="L23" s="129"/>
       <c r="M23" s="129"/>
@@ -17113,7 +17124,7 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -17130,7 +17141,7 @@
         <v>16</v>
       </c>
       <c r="E2" s="74" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>17</v>
@@ -17148,7 +17159,7 @@
         <v>29</v>
       </c>
       <c r="K2" s="98" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="L2" s="129"/>
     </row>
@@ -17184,7 +17195,7 @@
         <v>29</v>
       </c>
       <c r="K3" s="98" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="L3" s="107" t="s">
         <v>39</v>
@@ -17204,7 +17215,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="126" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="F4" s="127" t="s">
         <v>35</v>
@@ -17222,7 +17233,7 @@
         <v>29</v>
       </c>
       <c r="K4" s="99" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="L4" s="129"/>
     </row>
@@ -17240,7 +17251,7 @@
         <v>196</v>
       </c>
       <c r="E5" s="135" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="F5" s="124" t="s">
         <v>17</v>
@@ -17261,104 +17272,104 @@
       <c r="L5" s="107"/>
     </row>
     <row r="6" spans="1:12" ht="28.8">
-      <c r="A6" s="245" t="s">
+      <c r="A6" s="243" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="246" t="s">
+      <c r="B6" s="244" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="245" t="s">
+      <c r="C6" s="243" t="s">
         <v>62</v>
       </c>
       <c r="D6" s="215" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="247" t="s">
+      <c r="E6" s="245" t="s">
         <v>199</v>
       </c>
-      <c r="F6" s="244" t="s">
+      <c r="F6" s="242" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="244" t="s">
+      <c r="G6" s="242" t="s">
         <v>65</v>
       </c>
-      <c r="H6" s="244" t="s">
+      <c r="H6" s="242" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="242" t="s">
+      <c r="I6" s="246" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="235" t="s">
+      <c r="J6" s="239" t="s">
         <v>66</v>
       </c>
-      <c r="K6" s="243" t="s">
-        <v>505</v>
-      </c>
-      <c r="L6" s="242"/>
+      <c r="K6" s="247" t="s">
+        <v>504</v>
+      </c>
+      <c r="L6" s="246"/>
     </row>
     <row r="7" spans="1:12" ht="28.8">
-      <c r="A7" s="245"/>
-      <c r="B7" s="246"/>
-      <c r="C7" s="245"/>
+      <c r="A7" s="243"/>
+      <c r="B7" s="244"/>
+      <c r="C7" s="243"/>
       <c r="D7" s="216" t="s">
         <v>67</v>
       </c>
-      <c r="E7" s="247"/>
-      <c r="F7" s="244"/>
-      <c r="G7" s="244"/>
-      <c r="H7" s="244"/>
-      <c r="I7" s="242"/>
-      <c r="J7" s="235"/>
-      <c r="K7" s="243"/>
-      <c r="L7" s="242"/>
+      <c r="E7" s="245"/>
+      <c r="F7" s="242"/>
+      <c r="G7" s="242"/>
+      <c r="H7" s="242"/>
+      <c r="I7" s="246"/>
+      <c r="J7" s="239"/>
+      <c r="K7" s="247"/>
+      <c r="L7" s="246"/>
     </row>
     <row r="8" spans="1:12" ht="28.8">
-      <c r="A8" s="245"/>
-      <c r="B8" s="246"/>
-      <c r="C8" s="245"/>
+      <c r="A8" s="243"/>
+      <c r="B8" s="244"/>
+      <c r="C8" s="243"/>
       <c r="D8" s="216" t="s">
         <v>68</v>
       </c>
-      <c r="E8" s="247"/>
-      <c r="F8" s="244"/>
-      <c r="G8" s="244"/>
-      <c r="H8" s="244"/>
-      <c r="I8" s="242"/>
-      <c r="J8" s="235"/>
-      <c r="K8" s="243"/>
-      <c r="L8" s="242"/>
+      <c r="E8" s="245"/>
+      <c r="F8" s="242"/>
+      <c r="G8" s="242"/>
+      <c r="H8" s="242"/>
+      <c r="I8" s="246"/>
+      <c r="J8" s="239"/>
+      <c r="K8" s="247"/>
+      <c r="L8" s="246"/>
     </row>
     <row r="9" spans="1:12">
-      <c r="A9" s="245"/>
-      <c r="B9" s="246"/>
-      <c r="C9" s="245"/>
+      <c r="A9" s="243"/>
+      <c r="B9" s="244"/>
+      <c r="C9" s="243"/>
       <c r="D9" s="139" t="s">
         <v>69</v>
       </c>
-      <c r="E9" s="247"/>
-      <c r="F9" s="244"/>
-      <c r="G9" s="244"/>
-      <c r="H9" s="244"/>
-      <c r="I9" s="242"/>
-      <c r="J9" s="235"/>
-      <c r="K9" s="243"/>
-      <c r="L9" s="242"/>
+      <c r="E9" s="245"/>
+      <c r="F9" s="242"/>
+      <c r="G9" s="242"/>
+      <c r="H9" s="242"/>
+      <c r="I9" s="246"/>
+      <c r="J9" s="239"/>
+      <c r="K9" s="247"/>
+      <c r="L9" s="246"/>
     </row>
     <row r="10" spans="1:12">
-      <c r="A10" s="245"/>
-      <c r="B10" s="246"/>
-      <c r="C10" s="245"/>
+      <c r="A10" s="243"/>
+      <c r="B10" s="244"/>
+      <c r="C10" s="243"/>
       <c r="D10" s="139" t="s">
         <v>70</v>
       </c>
-      <c r="E10" s="247"/>
-      <c r="F10" s="244"/>
-      <c r="G10" s="244"/>
-      <c r="H10" s="244"/>
-      <c r="I10" s="242"/>
-      <c r="J10" s="235"/>
-      <c r="K10" s="243"/>
-      <c r="L10" s="242"/>
+      <c r="E10" s="245"/>
+      <c r="F10" s="242"/>
+      <c r="G10" s="242"/>
+      <c r="H10" s="242"/>
+      <c r="I10" s="246"/>
+      <c r="J10" s="239"/>
+      <c r="K10" s="247"/>
+      <c r="L10" s="246"/>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="121" t="s">
@@ -17374,7 +17385,7 @@
         <v>16</v>
       </c>
       <c r="E11" s="132" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="F11" s="124" t="s">
         <v>17</v>
@@ -17392,7 +17403,7 @@
         <v>29</v>
       </c>
       <c r="K11" s="99" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="L11" s="107"/>
     </row>
@@ -17410,7 +17421,7 @@
         <v>16</v>
       </c>
       <c r="E12" s="126" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="F12" s="124" t="s">
         <v>17</v>
@@ -17428,7 +17439,7 @@
         <v>29</v>
       </c>
       <c r="K12" s="98" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="L12" s="129" t="s">
         <v>46</v>
@@ -17448,7 +17459,7 @@
         <v>16</v>
       </c>
       <c r="E13" s="132" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>17</v>
@@ -17466,7 +17477,7 @@
         <v>29</v>
       </c>
       <c r="K13" s="98" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="L13" s="107"/>
     </row>
@@ -17484,7 +17495,7 @@
         <v>16</v>
       </c>
       <c r="E14" s="126" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="F14" s="124" t="s">
         <v>17</v>
@@ -17502,10 +17513,10 @@
         <v>29</v>
       </c>
       <c r="K14" s="98" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="L14" s="129" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -17522,7 +17533,7 @@
         <v>16</v>
       </c>
       <c r="E15" s="121" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>35</v>
@@ -17667,17 +17678,17 @@
   </sheetData>
   <autoFilter ref="A1:L15" xr:uid="{FBE7E653-2382-46E4-9C76-9C694EDC9195}"/>
   <mergeCells count="11">
+    <mergeCell ref="L6:L10"/>
+    <mergeCell ref="K6:K10"/>
+    <mergeCell ref="H6:H10"/>
+    <mergeCell ref="I6:I10"/>
+    <mergeCell ref="J6:J10"/>
     <mergeCell ref="G6:G10"/>
     <mergeCell ref="A6:A10"/>
     <mergeCell ref="B6:B10"/>
     <mergeCell ref="C6:C10"/>
     <mergeCell ref="E6:E10"/>
     <mergeCell ref="F6:F10"/>
-    <mergeCell ref="L6:L10"/>
-    <mergeCell ref="K6:K10"/>
-    <mergeCell ref="H6:H10"/>
-    <mergeCell ref="I6:I10"/>
-    <mergeCell ref="J6:J10"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F6 F11:F15">
     <cfRule type="cellIs" dxfId="127" priority="7" operator="equal">
@@ -17821,7 +17832,7 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="92.4">
@@ -17838,7 +17849,7 @@
         <v>152</v>
       </c>
       <c r="E2" s="82" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>35</v>
@@ -17856,7 +17867,7 @@
         <v>37</v>
       </c>
       <c r="K2" s="107" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="L2" s="186"/>
     </row>
@@ -17894,7 +17905,7 @@
     </row>
     <row r="4" spans="1:12" ht="92.25" customHeight="1">
       <c r="A4" s="121" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B4" s="35" t="s">
         <v>175</v>
@@ -17906,7 +17917,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="194" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="F4" s="124" t="s">
         <v>17</v>
@@ -18044,7 +18055,7 @@
         <v>16</v>
       </c>
       <c r="E8" s="82" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="F8" s="124" t="s">
         <v>35</v>
@@ -18062,31 +18073,31 @@
         <v>37</v>
       </c>
       <c r="K8" s="107" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="L8" s="107"/>
     </row>
     <row r="9" spans="1:12" ht="43.2">
       <c r="A9" s="125" t="s">
+        <v>520</v>
+      </c>
+      <c r="B9" s="74" t="s">
         <v>521</v>
       </c>
-      <c r="B9" s="74" t="s">
+      <c r="C9" s="125" t="s">
         <v>522</v>
-      </c>
-      <c r="C9" s="125" t="s">
-        <v>523</v>
       </c>
       <c r="D9" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E9" s="212" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="F9" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G9" s="127" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H9" s="127">
         <v>1</v>
@@ -18098,31 +18109,31 @@
         <v>37</v>
       </c>
       <c r="K9" s="106" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="L9" s="129"/>
     </row>
     <row r="10" spans="1:12" ht="43.2">
       <c r="A10" s="121" t="s">
+        <v>525</v>
+      </c>
+      <c r="B10" s="35" t="s">
         <v>526</v>
       </c>
-      <c r="B10" s="35" t="s">
+      <c r="C10" s="121" t="s">
         <v>527</v>
-      </c>
-      <c r="C10" s="121" t="s">
-        <v>528</v>
       </c>
       <c r="D10" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="F10" s="124" t="s">
         <v>35</v>
       </c>
       <c r="G10" s="124" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H10" s="133">
         <v>1</v>
@@ -18134,29 +18145,29 @@
         <v>37</v>
       </c>
       <c r="K10" s="106" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="L10" s="107"/>
     </row>
     <row r="11" spans="1:12" ht="43.2">
       <c r="A11" s="125" t="s">
+        <v>459</v>
+      </c>
+      <c r="B11" s="74" t="s">
         <v>460</v>
       </c>
-      <c r="B11" s="74" t="s">
+      <c r="C11" s="134" t="s">
         <v>461</v>
       </c>
-      <c r="C11" s="134" t="s">
+      <c r="D11" s="154" t="s">
         <v>462</v>
-      </c>
-      <c r="D11" s="154" t="s">
-        <v>463</v>
       </c>
       <c r="E11" s="126"/>
       <c r="F11" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G11" s="127" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="H11" s="127" t="s">
         <v>19</v>
@@ -18172,13 +18183,13 @@
     </row>
     <row r="12" spans="1:12" ht="28.8">
       <c r="A12" s="121" t="s">
+        <v>530</v>
+      </c>
+      <c r="B12" s="35" t="s">
         <v>531</v>
       </c>
-      <c r="B12" s="35" t="s">
+      <c r="C12" s="121" t="s">
         <v>532</v>
-      </c>
-      <c r="C12" s="121" t="s">
-        <v>533</v>
       </c>
       <c r="D12" s="132" t="s">
         <v>16</v>
@@ -18216,7 +18227,7 @@
         <v>16</v>
       </c>
       <c r="E13" s="126" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>35</v>
@@ -18270,19 +18281,19 @@
     </row>
     <row r="15" spans="1:12" ht="57.6">
       <c r="A15" s="125" t="s">
+        <v>534</v>
+      </c>
+      <c r="B15" s="74" t="s">
         <v>535</v>
       </c>
-      <c r="B15" s="74" t="s">
+      <c r="C15" s="125" t="s">
         <v>536</v>
-      </c>
-      <c r="C15" s="125" t="s">
-        <v>537</v>
       </c>
       <c r="D15" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E15" s="126" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>17</v>
@@ -18316,7 +18327,7 @@
         <v>85</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="F16" s="124" t="s">
         <v>17</v>
@@ -18350,7 +18361,7 @@
         <v>92</v>
       </c>
       <c r="E17" s="80" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="F17" s="127" t="s">
         <v>35</v>
@@ -18368,7 +18379,7 @@
         <v>37</v>
       </c>
       <c r="K17" s="107" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="L17" s="129"/>
     </row>
@@ -18386,7 +18397,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="35" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F18" s="124" t="s">
         <v>17</v>
@@ -18437,7 +18448,7 @@
       </c>
       <c r="K19" s="106"/>
       <c r="L19" s="129" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="43.2">
@@ -18454,7 +18465,7 @@
         <v>16</v>
       </c>
       <c r="E20" s="35" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="F20" s="124" t="s">
         <v>35</v>
@@ -18478,19 +18489,19 @@
     </row>
     <row r="21" spans="1:12" ht="57.6">
       <c r="A21" s="125" t="s">
+        <v>544</v>
+      </c>
+      <c r="B21" s="74" t="s">
         <v>545</v>
       </c>
-      <c r="B21" s="74" t="s">
+      <c r="C21" s="125" t="s">
         <v>546</v>
-      </c>
-      <c r="C21" s="125" t="s">
-        <v>547</v>
       </c>
       <c r="D21" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E21" s="126" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>17</v>
@@ -18508,27 +18519,27 @@
         <v>29</v>
       </c>
       <c r="K21" s="107" t="s">
+        <v>548</v>
+      </c>
+      <c r="L21" s="192" t="s">
         <v>549</v>
-      </c>
-      <c r="L21" s="192" t="s">
-        <v>550</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="43.2">
       <c r="A22" s="121" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B22" s="35" t="s">
         <v>127</v>
       </c>
       <c r="C22" s="121" t="s">
+        <v>332</v>
+      </c>
+      <c r="D22" s="143" t="s">
         <v>333</v>
       </c>
-      <c r="D22" s="143" t="s">
-        <v>334</v>
-      </c>
       <c r="E22" s="35" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>35</v>
@@ -18562,7 +18573,7 @@
         <v>16</v>
       </c>
       <c r="E23" s="126" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>35</v>
@@ -18580,7 +18591,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="106" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="L23" s="195"/>
     </row>
@@ -19063,15 +19074,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000B1A1CF98C819F4881BB4349588D0C85" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ff8ef391852eaca4511043a54bffd4a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cfc87205-1831-4b6c-a7b4-76d40079a43e" xmlns:ns3="221af607-abea-4d5e-830c-567dcc03c0ec" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="201dd8b781da46d5daa37e3355db44fe" ns2:_="" ns3:_="">
     <xsd:import namespace="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
@@ -19314,6 +19316,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -19327,14 +19338,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19A23828-4FF7-4569-837D-B1B2C775409F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19353,6 +19356,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16D2CAB5-B21B-4A93-9D82-49FE3E36CF14}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
doc update retention period (#273)
usage note of retention period property in Dataset and Distribution class was updated to clarify what it is for.
</commit_message>
<xml_diff>
--- a/Documents/Metadata_CoreGenericHealth_v2.xlsx
+++ b/Documents/Metadata_CoreGenericHealth_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://healthri-my.sharepoint.com/personal/hannah_neikes_health-ri_nl/Documents/Documenten/GitHub/health-ri-metadata/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{B604F9AE-9787-411E-AB68-6C0D2821F0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB2FDFB2-6BD5-4989-9906-EC23F51E3B08}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="8_{B604F9AE-9787-411E-AB68-6C0D2821F0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56501FCB-3D8B-4B1A-811D-B69BAEFCE65B}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-12765" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5295" yWindow="-16320" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="14" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1846" uniqueCount="675">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1846" uniqueCount="676">
   <si>
     <t>Property label</t>
   </si>
@@ -1145,9 +1145,6 @@
     <t>healthdcatap:retentionPeriod</t>
   </si>
   <si>
-    <t>This property makes use of the class dct:PeriodOfTime, in which a start and end date should be provided.</t>
-  </si>
-  <si>
     <t>fill in in 'Period of Time' tab</t>
   </si>
   <si>
@@ -2619,6 +2616,20 @@
   <si>
     <t>One (or many) categoiesy or sub-categories of the purposes can be chosen from the taxonomy provided by dpv (see controlled vocabulary column). Try to be as specific as possible.
 Example value could be: dpv:ResearchAndDevelopment.</t>
+  </si>
+  <si>
+    <t>Indicate with this property in case the Dataset is only available for secondary use for a specific period of time (e.g. due to data protection, contractual, or project constraints).
+This property makes use of the class dct:PeriodOfTime, in which a start and end date can be provided.
+If the Dataset is available indefinitely, leave the property empty (cardinality is 0..1; it is only meaningful when a retention limit applies).
+If only a start is known, provide dcat:startDate only (open-ended interval, as allowed by dct:PeriodOfTime).
+If a limit is known, provide both dcat:startDate and dcat:endDate.</t>
+  </si>
+  <si>
+    <t>Indicate with this property in case the Distribution is only available for secondary use for a specific period of time (e.g. due to data protection, contractual, or project constraints).
+This property makes use of the class dct:PeriodOfTime, in which a start and end date can be provided.
+If the Distribution is available indefinitely, leave the property empty (cardinality is 0..1; it is only meaningful when a retention limit applies).
+If only a start is known, provide dcat:startDate only (open-ended interval, as allowed by dct:PeriodOfTime).
+If a limit is known, provide both dcat:startDate and dcat:endDate.</t>
   </si>
 </sst>
 </file>
@@ -3766,43 +3777,43 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -7439,33 +7450,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>553</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>554</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="227" t="s">
         <v>555</v>
       </c>
-      <c r="N1" s="227" t="s">
+      <c r="O1" s="233" t="s">
         <v>556</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>557</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="72">
       <c r="A2" s="196" t="s">
+        <v>557</v>
+      </c>
+      <c r="B2" s="45" t="s">
         <v>558</v>
       </c>
-      <c r="B2" s="45" t="s">
+      <c r="C2" s="76" t="s">
         <v>559</v>
-      </c>
-      <c r="C2" s="76" t="s">
-        <v>560</v>
       </c>
       <c r="D2" s="196" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="197" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="F2" s="198" t="s">
         <v>35</v>
@@ -7474,7 +7485,7 @@
         <v>58</v>
       </c>
       <c r="H2" s="198" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="I2" s="160" t="s">
         <v>20</v>
@@ -7489,13 +7500,13 @@
     </row>
     <row r="3" spans="1:15" ht="28.8">
       <c r="A3" s="68" t="s">
+        <v>562</v>
+      </c>
+      <c r="B3" s="61" t="s">
         <v>563</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="C3" s="77" t="s">
         <v>564</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>565</v>
       </c>
       <c r="D3" s="68" t="s">
         <v>16</v>
@@ -7634,36 +7645,36 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>565</v>
+      </c>
+      <c r="M1" s="220" t="s">
         <v>566</v>
       </c>
-      <c r="M1" s="220" t="s">
+      <c r="N1" s="226" t="s">
         <v>567</v>
       </c>
-      <c r="N1" s="226" t="s">
+      <c r="O1" s="230" t="s">
         <v>568</v>
       </c>
-      <c r="O1" s="230" t="s">
+      <c r="P1" s="227" t="s">
         <v>569</v>
       </c>
-      <c r="P1" s="227" t="s">
+      <c r="Q1" s="231" t="s">
         <v>570</v>
       </c>
-      <c r="Q1" s="231" t="s">
+      <c r="R1" s="233" t="s">
         <v>571</v>
-      </c>
-      <c r="R1" s="233" t="s">
-        <v>572</v>
       </c>
     </row>
     <row r="2" spans="1:18">
       <c r="A2" s="58" t="s">
+        <v>572</v>
+      </c>
+      <c r="B2" s="44" t="s">
         <v>573</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="C2" s="76" t="s">
         <v>574</v>
-      </c>
-      <c r="C2" s="76" t="s">
-        <v>575</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
@@ -7691,13 +7702,13 @@
     </row>
     <row r="3" spans="1:18">
       <c r="A3" s="48" t="s">
+        <v>575</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>576</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>577</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>578</v>
       </c>
       <c r="D3" s="48" t="s">
         <v>16</v>
@@ -8359,33 +8370,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>578</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>579</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="227" t="s">
         <v>580</v>
       </c>
-      <c r="N1" s="227" t="s">
+      <c r="O1" s="233" t="s">
         <v>581</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>582</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="43.2">
       <c r="A2" s="84" t="s">
+        <v>582</v>
+      </c>
+      <c r="B2" s="44" t="s">
         <v>583</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="C2" s="58" t="s">
         <v>584</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>585</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>17</v>
@@ -8415,19 +8426,19 @@
     </row>
     <row r="3" spans="1:15" ht="129.6">
       <c r="A3" s="48" t="s">
+        <v>586</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>587</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>588</v>
       </c>
-      <c r="C3" s="77" t="s">
+      <c r="D3" s="234" t="s">
         <v>589</v>
       </c>
-      <c r="D3" s="234" t="s">
+      <c r="E3" s="50" t="s">
         <v>590</v>
-      </c>
-      <c r="E3" s="50" t="s">
-        <v>591</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>17</v>
@@ -8553,33 +8564,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="218" t="s">
+        <v>591</v>
+      </c>
+      <c r="M1" s="229" t="s">
         <v>592</v>
       </c>
-      <c r="M1" s="229" t="s">
+      <c r="N1" s="228" t="s">
         <v>593</v>
       </c>
-      <c r="N1" s="228" t="s">
+      <c r="O1" s="233" t="s">
         <v>594</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>595</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="158.4">
       <c r="A2" s="84" t="s">
+        <v>595</v>
+      </c>
+      <c r="B2" s="44" t="s">
+        <v>587</v>
+      </c>
+      <c r="C2" s="58" t="s">
+        <v>588</v>
+      </c>
+      <c r="D2" s="59" t="s">
         <v>596</v>
       </c>
-      <c r="B2" s="44" t="s">
-        <v>588</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>589</v>
-      </c>
-      <c r="D2" s="59" t="s">
+      <c r="E2" s="59" t="s">
         <v>597</v>
-      </c>
-      <c r="E2" s="59" t="s">
-        <v>598</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>35</v>
@@ -8600,19 +8611,19 @@
     </row>
     <row r="3" spans="1:15" ht="43.2">
       <c r="A3" s="48" t="s">
+        <v>598</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>599</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>600</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>601</v>
       </c>
       <c r="D3" s="116" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>35</v>
@@ -8738,33 +8749,33 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>602</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>603</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="227" t="s">
         <v>604</v>
       </c>
-      <c r="N1" s="227" t="s">
+      <c r="O1" s="233" t="s">
         <v>605</v>
-      </c>
-      <c r="O1" s="233" t="s">
-        <v>606</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="100.8">
       <c r="A2" s="84" t="s">
+        <v>606</v>
+      </c>
+      <c r="B2" s="44" t="s">
         <v>607</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="C2" s="58" t="s">
         <v>608</v>
-      </c>
-      <c r="C2" s="58" t="s">
-        <v>609</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="59" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="F2" s="60" t="s">
         <v>17</v>
@@ -8785,19 +8796,19 @@
     </row>
     <row r="3" spans="1:15" ht="57.6">
       <c r="A3" s="48" t="s">
+        <v>610</v>
+      </c>
+      <c r="B3" s="49" t="s">
         <v>611</v>
       </c>
-      <c r="B3" s="49" t="s">
+      <c r="C3" s="77" t="s">
         <v>612</v>
-      </c>
-      <c r="C3" s="77" t="s">
-        <v>613</v>
       </c>
       <c r="D3" s="116" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="F3" s="51" t="s">
         <v>17</v>
@@ -8901,7 +8912,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="56" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="E1" s="56" t="s">
         <v>4</v>
@@ -8924,13 +8935,13 @@
     </row>
     <row r="2" spans="1:10" ht="28.8">
       <c r="A2" s="63" t="s">
+        <v>615</v>
+      </c>
+      <c r="B2" s="53" t="s">
         <v>616</v>
       </c>
-      <c r="B2" s="53" t="s">
+      <c r="C2" s="44" t="s">
         <v>617</v>
-      </c>
-      <c r="C2" s="44" t="s">
-        <v>618</v>
       </c>
       <c r="D2" s="43" t="s">
         <v>16</v>
@@ -8938,7 +8949,7 @@
       <c r="E2" s="45"/>
       <c r="F2" s="64"/>
       <c r="G2" s="63" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="H2" s="65" t="s">
         <v>81</v>
@@ -8952,13 +8963,13 @@
     </row>
     <row r="3" spans="1:10" ht="43.2">
       <c r="A3" s="67" t="s">
+        <v>619</v>
+      </c>
+      <c r="B3" s="50" t="s">
         <v>620</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="C3" s="49" t="s">
         <v>621</v>
-      </c>
-      <c r="C3" s="49" t="s">
-        <v>622</v>
       </c>
       <c r="D3" s="48" t="s">
         <v>16</v>
@@ -8966,10 +8977,10 @@
       <c r="E3" s="50"/>
       <c r="F3" s="68"/>
       <c r="G3" s="69" t="s">
+        <v>622</v>
+      </c>
+      <c r="H3" s="48" t="s">
         <v>623</v>
-      </c>
-      <c r="H3" s="48" t="s">
-        <v>624</v>
       </c>
       <c r="I3" s="69" t="s">
         <v>20</v>
@@ -8980,13 +8991,13 @@
     </row>
     <row r="4" spans="1:10" ht="43.2">
       <c r="A4" s="63" t="s">
+        <v>624</v>
+      </c>
+      <c r="B4" s="53" t="s">
         <v>625</v>
       </c>
-      <c r="B4" s="53" t="s">
+      <c r="C4" s="44" t="s">
         <v>626</v>
-      </c>
-      <c r="C4" s="44" t="s">
-        <v>627</v>
       </c>
       <c r="D4" s="43" t="s">
         <v>16</v>
@@ -8994,10 +9005,10 @@
       <c r="E4" s="53"/>
       <c r="F4" s="64"/>
       <c r="G4" s="63" t="s">
+        <v>627</v>
+      </c>
+      <c r="H4" s="65" t="s">
         <v>628</v>
-      </c>
-      <c r="H4" s="65" t="s">
-        <v>629</v>
       </c>
       <c r="I4" s="66" t="s">
         <v>20</v>
@@ -9008,26 +9019,26 @@
     </row>
     <row r="5" spans="1:10" ht="43.2">
       <c r="A5" s="67" t="s">
+        <v>629</v>
+      </c>
+      <c r="B5" s="50" t="s">
         <v>630</v>
       </c>
-      <c r="B5" s="50" t="s">
+      <c r="C5" s="49" t="s">
         <v>631</v>
-      </c>
-      <c r="C5" s="49" t="s">
-        <v>632</v>
       </c>
       <c r="D5" s="48" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="49" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="F5" s="68"/>
       <c r="G5" s="67" t="s">
+        <v>633</v>
+      </c>
+      <c r="H5" s="48" t="s">
         <v>634</v>
-      </c>
-      <c r="H5" s="48" t="s">
-        <v>635</v>
       </c>
       <c r="I5" s="69" t="s">
         <v>20</v>
@@ -9038,13 +9049,13 @@
     </row>
     <row r="6" spans="1:10" ht="28.8">
       <c r="A6" s="63" t="s">
+        <v>635</v>
+      </c>
+      <c r="B6" s="73" t="s">
         <v>636</v>
       </c>
-      <c r="B6" s="73" t="s">
+      <c r="C6" s="44" t="s">
         <v>637</v>
-      </c>
-      <c r="C6" s="44" t="s">
-        <v>638</v>
       </c>
       <c r="D6" s="43" t="s">
         <v>16</v>
@@ -9055,7 +9066,7 @@
         <v>98</v>
       </c>
       <c r="H6" s="65" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="I6" s="66" t="s">
         <v>20</v>
@@ -9066,13 +9077,13 @@
     </row>
     <row r="7" spans="1:10" ht="28.8">
       <c r="A7" s="67" t="s">
+        <v>638</v>
+      </c>
+      <c r="B7" s="50" t="s">
         <v>639</v>
       </c>
-      <c r="B7" s="50" t="s">
+      <c r="C7" s="49" t="s">
         <v>640</v>
-      </c>
-      <c r="C7" s="49" t="s">
-        <v>641</v>
       </c>
       <c r="D7" s="48" t="s">
         <v>16</v>
@@ -9094,23 +9105,23 @@
     </row>
     <row r="8" spans="1:10" ht="86.4">
       <c r="A8" s="63" t="s">
+        <v>641</v>
+      </c>
+      <c r="B8" s="53" t="s">
         <v>642</v>
       </c>
-      <c r="B8" s="53" t="s">
+      <c r="C8" s="44" t="s">
         <v>643</v>
-      </c>
-      <c r="C8" s="44" t="s">
-        <v>644</v>
       </c>
       <c r="D8" s="43" t="s">
         <v>16</v>
       </c>
       <c r="E8" s="71" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="F8" s="47"/>
       <c r="G8" s="63" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="H8" s="65">
         <v>1</v>
@@ -9124,13 +9135,13 @@
     </row>
     <row r="9" spans="1:10" ht="28.8">
       <c r="A9" s="67" t="s">
+        <v>646</v>
+      </c>
+      <c r="B9" s="50" t="s">
         <v>647</v>
       </c>
-      <c r="B9" s="50" t="s">
+      <c r="C9" s="49" t="s">
         <v>648</v>
-      </c>
-      <c r="C9" s="49" t="s">
-        <v>649</v>
       </c>
       <c r="D9" s="48" t="s">
         <v>16</v>
@@ -9138,7 +9149,7 @@
       <c r="E9" s="50"/>
       <c r="F9" s="68"/>
       <c r="G9" s="69" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="H9" s="48" t="s">
         <v>81</v>
@@ -9152,23 +9163,23 @@
     </row>
     <row r="10" spans="1:10" ht="28.8">
       <c r="A10" s="63" t="s">
+        <v>650</v>
+      </c>
+      <c r="B10" s="72" t="s">
         <v>651</v>
       </c>
-      <c r="B10" s="72" t="s">
+      <c r="C10" s="44" t="s">
         <v>652</v>
-      </c>
-      <c r="C10" s="44" t="s">
-        <v>653</v>
       </c>
       <c r="D10" s="43" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="72" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
       <c r="F10" s="64"/>
       <c r="G10" s="63" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="H10" s="65" t="s">
         <v>19</v>
@@ -9633,36 +9644,36 @@
         <v>10</v>
       </c>
       <c r="L1" s="219" t="s">
+        <v>654</v>
+      </c>
+      <c r="M1" s="226" t="s">
         <v>655</v>
       </c>
-      <c r="M1" s="226" t="s">
+      <c r="N1" s="233" t="s">
         <v>656</v>
-      </c>
-      <c r="N1" s="233" t="s">
-        <v>657</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="72">
       <c r="A2" s="44" t="s">
+        <v>657</v>
+      </c>
+      <c r="B2" s="57" t="s">
         <v>658</v>
       </c>
-      <c r="B2" s="57" t="s">
+      <c r="C2" s="58" t="s">
         <v>659</v>
       </c>
-      <c r="C2" s="58" t="s">
+      <c r="D2" s="78" t="s">
         <v>660</v>
       </c>
-      <c r="D2" s="78" t="s">
+      <c r="E2" s="197" t="s">
         <v>661</v>
-      </c>
-      <c r="E2" s="197" t="s">
-        <v>662</v>
       </c>
       <c r="F2" s="46" t="s">
         <v>35</v>
       </c>
       <c r="G2" s="204" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="H2" s="47">
         <v>1</v>
@@ -9676,13 +9687,13 @@
     </row>
     <row r="3" spans="1:14" ht="71.25" customHeight="1">
       <c r="A3" s="49" t="s">
+        <v>663</v>
+      </c>
+      <c r="B3" s="61" t="s">
         <v>664</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="C3" s="48" t="s">
         <v>665</v>
-      </c>
-      <c r="C3" s="48" t="s">
-        <v>666</v>
       </c>
       <c r="D3" s="50" t="s">
         <v>16</v>
@@ -9692,7 +9703,7 @@
         <v>35</v>
       </c>
       <c r="G3" s="51" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="H3" s="52">
         <v>1</v>
@@ -10606,19 +10617,19 @@
       <c r="M7" s="129"/>
     </row>
     <row r="8" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A8" s="238" t="s">
+      <c r="A8" s="235" t="s">
         <v>60</v>
       </c>
       <c r="B8" s="241" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="238" t="s">
+      <c r="C8" s="235" t="s">
         <v>62</v>
       </c>
       <c r="D8" s="213" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="240" t="s">
+      <c r="E8" s="238" t="s">
         <v>64</v>
       </c>
       <c r="F8" s="237" t="s">
@@ -10630,83 +10641,83 @@
       <c r="H8" s="237" t="s">
         <v>19</v>
       </c>
-      <c r="I8" s="235" t="s">
+      <c r="I8" s="239" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="235" t="s">
+      <c r="J8" s="239" t="s">
         <v>66</v>
       </c>
       <c r="K8" s="137"/>
-      <c r="L8" s="235"/>
-      <c r="M8" s="235"/>
+      <c r="L8" s="239"/>
+      <c r="M8" s="239"/>
     </row>
     <row r="9" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A9" s="238"/>
+      <c r="A9" s="235"/>
       <c r="B9" s="241"/>
-      <c r="C9" s="238"/>
+      <c r="C9" s="235"/>
       <c r="D9" s="214" t="s">
         <v>67</v>
       </c>
-      <c r="E9" s="240"/>
+      <c r="E9" s="238"/>
       <c r="F9" s="237"/>
       <c r="G9" s="237"/>
       <c r="H9" s="237"/>
-      <c r="I9" s="235"/>
-      <c r="J9" s="235"/>
+      <c r="I9" s="239"/>
+      <c r="J9" s="239"/>
       <c r="K9" s="137"/>
-      <c r="L9" s="235"/>
-      <c r="M9" s="235"/>
+      <c r="L9" s="239"/>
+      <c r="M9" s="239"/>
     </row>
     <row r="10" spans="1:13" ht="29.1" customHeight="1">
-      <c r="A10" s="238"/>
+      <c r="A10" s="235"/>
       <c r="B10" s="241"/>
-      <c r="C10" s="238"/>
+      <c r="C10" s="235"/>
       <c r="D10" s="214" t="s">
         <v>68</v>
       </c>
-      <c r="E10" s="240"/>
+      <c r="E10" s="238"/>
       <c r="F10" s="237"/>
       <c r="G10" s="237"/>
       <c r="H10" s="237"/>
-      <c r="I10" s="235"/>
-      <c r="J10" s="235"/>
+      <c r="I10" s="239"/>
+      <c r="J10" s="239"/>
       <c r="K10" s="137"/>
-      <c r="L10" s="235"/>
-      <c r="M10" s="235"/>
+      <c r="L10" s="239"/>
+      <c r="M10" s="239"/>
     </row>
     <row r="11" spans="1:13" ht="14.4" customHeight="1">
-      <c r="A11" s="238"/>
+      <c r="A11" s="235"/>
       <c r="B11" s="241"/>
-      <c r="C11" s="238"/>
+      <c r="C11" s="235"/>
       <c r="D11" s="152" t="s">
         <v>69</v>
       </c>
-      <c r="E11" s="240"/>
+      <c r="E11" s="238"/>
       <c r="F11" s="237"/>
       <c r="G11" s="237"/>
       <c r="H11" s="237"/>
-      <c r="I11" s="235"/>
-      <c r="J11" s="235"/>
+      <c r="I11" s="239"/>
+      <c r="J11" s="239"/>
       <c r="K11" s="153"/>
-      <c r="L11" s="235"/>
-      <c r="M11" s="235"/>
+      <c r="L11" s="239"/>
+      <c r="M11" s="239"/>
     </row>
     <row r="12" spans="1:13" ht="14.4" customHeight="1">
-      <c r="A12" s="238"/>
+      <c r="A12" s="235"/>
       <c r="B12" s="241"/>
-      <c r="C12" s="238"/>
+      <c r="C12" s="235"/>
       <c r="D12" s="152" t="s">
         <v>70</v>
       </c>
-      <c r="E12" s="240"/>
+      <c r="E12" s="238"/>
       <c r="F12" s="237"/>
       <c r="G12" s="237"/>
       <c r="H12" s="237"/>
-      <c r="I12" s="235"/>
-      <c r="J12" s="235"/>
+      <c r="I12" s="239"/>
+      <c r="J12" s="239"/>
       <c r="K12" s="137"/>
-      <c r="L12" s="235"/>
-      <c r="M12" s="235"/>
+      <c r="L12" s="239"/>
+      <c r="M12" s="239"/>
     </row>
     <row r="13" spans="1:13" ht="43.2">
       <c r="A13" s="125" t="s">
@@ -10831,7 +10842,7 @@
         <v>92</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
       <c r="F16" s="124" t="s">
         <v>17</v>
@@ -11525,17 +11536,17 @@
     <sortCondition ref="A2:A24"/>
   </sortState>
   <mergeCells count="11">
+    <mergeCell ref="M8:M12"/>
+    <mergeCell ref="L8:L12"/>
+    <mergeCell ref="H8:H12"/>
+    <mergeCell ref="I8:I12"/>
+    <mergeCell ref="J8:J12"/>
     <mergeCell ref="G8:G12"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="B8:B12"/>
     <mergeCell ref="C8:C12"/>
     <mergeCell ref="E8:E12"/>
     <mergeCell ref="F8:F12"/>
-    <mergeCell ref="M8:M12"/>
-    <mergeCell ref="L8:L12"/>
-    <mergeCell ref="H8:H12"/>
-    <mergeCell ref="I8:I12"/>
-    <mergeCell ref="J8:J12"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F8">
     <cfRule type="cellIs" dxfId="190" priority="16" operator="equal">
@@ -11807,7 +11818,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="132" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="F4" s="124" t="s">
         <v>35</v>
@@ -12182,19 +12193,19 @@
       <c r="N13" s="129"/>
     </row>
     <row r="14" spans="1:14" ht="43.2">
-      <c r="A14" s="238" t="s">
+      <c r="A14" s="235" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="239" t="s">
+      <c r="B14" s="236" t="s">
         <v>61</v>
       </c>
-      <c r="C14" s="238" t="s">
+      <c r="C14" s="235" t="s">
         <v>62</v>
       </c>
       <c r="D14" s="213" t="s">
         <v>63</v>
       </c>
-      <c r="E14" s="240" t="s">
+      <c r="E14" s="238" t="s">
         <v>199</v>
       </c>
       <c r="F14" s="237" t="s">
@@ -12206,78 +12217,78 @@
       <c r="H14" s="237" t="s">
         <v>19</v>
       </c>
-      <c r="I14" s="235" t="s">
+      <c r="I14" s="239" t="s">
         <v>20</v>
       </c>
-      <c r="J14" s="235" t="s">
+      <c r="J14" s="239" t="s">
         <v>66</v>
       </c>
-      <c r="K14" s="236"/>
-      <c r="L14" s="235"/>
+      <c r="K14" s="240"/>
+      <c r="L14" s="239"/>
     </row>
     <row r="15" spans="1:14" ht="43.2">
-      <c r="A15" s="238"/>
-      <c r="B15" s="239"/>
-      <c r="C15" s="238"/>
+      <c r="A15" s="235"/>
+      <c r="B15" s="236"/>
+      <c r="C15" s="235"/>
       <c r="D15" s="214" t="s">
         <v>67</v>
       </c>
-      <c r="E15" s="240"/>
+      <c r="E15" s="238"/>
       <c r="F15" s="237"/>
       <c r="G15" s="237"/>
       <c r="H15" s="237"/>
-      <c r="I15" s="235"/>
-      <c r="J15" s="235"/>
-      <c r="K15" s="236"/>
-      <c r="L15" s="235"/>
+      <c r="I15" s="239"/>
+      <c r="J15" s="239"/>
+      <c r="K15" s="240"/>
+      <c r="L15" s="239"/>
     </row>
     <row r="16" spans="1:14" ht="28.8">
-      <c r="A16" s="238"/>
-      <c r="B16" s="239"/>
-      <c r="C16" s="238"/>
+      <c r="A16" s="235"/>
+      <c r="B16" s="236"/>
+      <c r="C16" s="235"/>
       <c r="D16" s="214" t="s">
         <v>68</v>
       </c>
-      <c r="E16" s="240"/>
+      <c r="E16" s="238"/>
       <c r="F16" s="237"/>
       <c r="G16" s="237"/>
       <c r="H16" s="237"/>
-      <c r="I16" s="235"/>
-      <c r="J16" s="235"/>
-      <c r="K16" s="236"/>
-      <c r="L16" s="235"/>
+      <c r="I16" s="239"/>
+      <c r="J16" s="239"/>
+      <c r="K16" s="240"/>
+      <c r="L16" s="239"/>
     </row>
     <row r="17" spans="1:14">
-      <c r="A17" s="238"/>
-      <c r="B17" s="239"/>
-      <c r="C17" s="238"/>
+      <c r="A17" s="235"/>
+      <c r="B17" s="236"/>
+      <c r="C17" s="235"/>
       <c r="D17" s="152" t="s">
         <v>69</v>
       </c>
-      <c r="E17" s="240"/>
+      <c r="E17" s="238"/>
       <c r="F17" s="237"/>
       <c r="G17" s="237"/>
       <c r="H17" s="237"/>
-      <c r="I17" s="235"/>
-      <c r="J17" s="235"/>
-      <c r="K17" s="236"/>
-      <c r="L17" s="235"/>
+      <c r="I17" s="239"/>
+      <c r="J17" s="239"/>
+      <c r="K17" s="240"/>
+      <c r="L17" s="239"/>
     </row>
     <row r="18" spans="1:14">
-      <c r="A18" s="238"/>
-      <c r="B18" s="239"/>
-      <c r="C18" s="238"/>
+      <c r="A18" s="235"/>
+      <c r="B18" s="236"/>
+      <c r="C18" s="235"/>
       <c r="D18" s="152" t="s">
         <v>70</v>
       </c>
-      <c r="E18" s="240"/>
+      <c r="E18" s="238"/>
       <c r="F18" s="237"/>
       <c r="G18" s="237"/>
       <c r="H18" s="237"/>
-      <c r="I18" s="235"/>
-      <c r="J18" s="235"/>
-      <c r="K18" s="236"/>
-      <c r="L18" s="235"/>
+      <c r="I18" s="239"/>
+      <c r="J18" s="239"/>
+      <c r="K18" s="240"/>
+      <c r="L18" s="239"/>
     </row>
     <row r="19" spans="1:14" ht="28.8">
       <c r="A19" s="125" t="s">
@@ -12555,7 +12566,7 @@
         <v>237</v>
       </c>
       <c r="E26" s="132" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
       <c r="F26" s="124" t="s">
         <v>17</v>
@@ -12931,7 +12942,7 @@
         <v>285</v>
       </c>
       <c r="E36" s="138" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
       <c r="F36" s="124" t="s">
         <v>17</v>
@@ -13117,7 +13128,7 @@
       </c>
       <c r="L40" s="107"/>
     </row>
-    <row r="41" spans="1:14" ht="28.8">
+    <row r="41" spans="1:14" ht="158.4">
       <c r="A41" s="125" t="s">
         <v>306</v>
       </c>
@@ -13131,7 +13142,7 @@
         <v>16</v>
       </c>
       <c r="E41" s="74" t="s">
-        <v>309</v>
+        <v>674</v>
       </c>
       <c r="F41" s="127" t="s">
         <v>17</v>
@@ -13152,30 +13163,30 @@
         <v>137</v>
       </c>
       <c r="L41" s="129" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="M41" s="129" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="N41" s="129" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="42" spans="1:14" ht="72">
       <c r="A42" s="121" t="s">
+        <v>310</v>
+      </c>
+      <c r="B42" s="35" t="s">
         <v>311</v>
       </c>
-      <c r="B42" s="35" t="s">
+      <c r="C42" s="121" t="s">
         <v>312</v>
-      </c>
-      <c r="C42" s="121" t="s">
-        <v>313</v>
       </c>
       <c r="D42" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E42" s="132" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F42" s="124" t="s">
         <v>17</v>
@@ -13196,26 +13207,26 @@
         <v>138</v>
       </c>
       <c r="L42" s="141" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="M42" s="107"/>
       <c r="N42" s="107"/>
     </row>
     <row r="43" spans="1:14" ht="28.8">
       <c r="A43" s="125" t="s">
+        <v>315</v>
+      </c>
+      <c r="B43" s="74" t="s">
         <v>316</v>
       </c>
-      <c r="B43" s="74" t="s">
+      <c r="C43" s="125" t="s">
         <v>317</v>
-      </c>
-      <c r="C43" s="125" t="s">
-        <v>318</v>
       </c>
       <c r="D43" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E43" s="205" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="F43" s="127" t="s">
         <v>17</v>
@@ -13236,26 +13247,26 @@
         <v>139</v>
       </c>
       <c r="L43" s="134" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="M43" s="129"/>
       <c r="N43" s="129"/>
     </row>
     <row r="44" spans="1:14" ht="57.6">
       <c r="A44" s="121" t="s">
+        <v>320</v>
+      </c>
+      <c r="B44" s="35" t="s">
         <v>321</v>
       </c>
-      <c r="B44" s="35" t="s">
+      <c r="C44" s="121" t="s">
         <v>322</v>
       </c>
-      <c r="C44" s="121" t="s">
+      <c r="D44" s="143" t="s">
         <v>323</v>
       </c>
-      <c r="D44" s="143" t="s">
+      <c r="E44" s="132" t="s">
         <v>324</v>
-      </c>
-      <c r="E44" s="132" t="s">
-        <v>325</v>
       </c>
       <c r="F44" s="124" t="s">
         <v>17</v>
@@ -13293,7 +13304,7 @@
         <v>16</v>
       </c>
       <c r="E45" s="74" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="F45" s="127" t="s">
         <v>17</v>
@@ -13314,36 +13325,36 @@
         <v>125</v>
       </c>
       <c r="L45" s="129" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="M45" s="129" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="N45" s="129" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="46" spans="1:14" ht="57.6">
       <c r="A46" s="121" t="s">
+        <v>326</v>
+      </c>
+      <c r="B46" s="35" t="s">
         <v>327</v>
       </c>
-      <c r="B46" s="35" t="s">
+      <c r="C46" s="141" t="s">
         <v>328</v>
-      </c>
-      <c r="C46" s="141" t="s">
-        <v>329</v>
       </c>
       <c r="D46" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E46" s="132" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="F46" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G46" s="124" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="H46" s="124" t="s">
         <v>81</v>
@@ -13363,19 +13374,19 @@
     </row>
     <row r="47" spans="1:14" ht="74.25" customHeight="1">
       <c r="A47" s="125" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B47" s="74" t="s">
         <v>127</v>
       </c>
       <c r="C47" s="125" t="s">
+        <v>332</v>
+      </c>
+      <c r="D47" s="142" t="s">
         <v>333</v>
       </c>
-      <c r="D47" s="142" t="s">
+      <c r="E47" s="74" t="s">
         <v>334</v>
-      </c>
-      <c r="E47" s="74" t="s">
-        <v>335</v>
       </c>
       <c r="F47" s="127" t="s">
         <v>35</v>
@@ -13413,7 +13424,7 @@
         <v>16</v>
       </c>
       <c r="E48" s="132" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F48" s="124" t="s">
         <v>35</v>
@@ -13439,19 +13450,19 @@
     </row>
     <row r="49" spans="1:14" ht="57.6">
       <c r="A49" s="125" t="s">
+        <v>336</v>
+      </c>
+      <c r="B49" s="74" t="s">
         <v>337</v>
       </c>
-      <c r="B49" s="74" t="s">
+      <c r="C49" s="125" t="s">
         <v>338</v>
       </c>
-      <c r="C49" s="125" t="s">
+      <c r="D49" s="217" t="s">
         <v>339</v>
       </c>
-      <c r="D49" s="217" t="s">
+      <c r="E49" s="83" t="s">
         <v>340</v>
-      </c>
-      <c r="E49" s="83" t="s">
-        <v>341</v>
       </c>
       <c r="F49" s="127" t="s">
         <v>17</v>
@@ -13477,19 +13488,19 @@
     </row>
     <row r="50" spans="1:14" ht="28.8">
       <c r="A50" s="121" t="s">
+        <v>341</v>
+      </c>
+      <c r="B50" s="35" t="s">
         <v>342</v>
       </c>
-      <c r="B50" s="35" t="s">
+      <c r="C50" s="121" t="s">
         <v>343</v>
-      </c>
-      <c r="C50" s="121" t="s">
-        <v>344</v>
       </c>
       <c r="D50" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E50" s="132" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="F50" s="124" t="s">
         <v>17</v>
@@ -13515,19 +13526,19 @@
     </row>
     <row r="51" spans="1:14" ht="28.8">
       <c r="A51" s="125" t="s">
+        <v>345</v>
+      </c>
+      <c r="B51" s="74" t="s">
         <v>346</v>
       </c>
-      <c r="B51" s="74" t="s">
+      <c r="C51" s="125" t="s">
         <v>347</v>
-      </c>
-      <c r="C51" s="125" t="s">
-        <v>348</v>
       </c>
       <c r="D51" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E51" s="74" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="F51" s="127" t="s">
         <v>17</v>
@@ -13553,13 +13564,13 @@
     </row>
     <row r="52" spans="1:14" ht="84.75" customHeight="1">
       <c r="A52" s="121" t="s">
+        <v>349</v>
+      </c>
+      <c r="B52" s="35" t="s">
         <v>350</v>
       </c>
-      <c r="B52" s="35" t="s">
+      <c r="C52" s="121" t="s">
         <v>351</v>
-      </c>
-      <c r="C52" s="121" t="s">
-        <v>352</v>
       </c>
       <c r="D52" s="132" t="s">
         <v>16</v>
@@ -13569,7 +13580,7 @@
         <v>17</v>
       </c>
       <c r="G52" s="124" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="H52" s="124" t="s">
         <v>19</v>
@@ -13605,17 +13616,17 @@
     <sortCondition ref="A2:A53"/>
   </sortState>
   <mergeCells count="11">
-    <mergeCell ref="A14:A18"/>
-    <mergeCell ref="B14:B18"/>
-    <mergeCell ref="C14:C18"/>
-    <mergeCell ref="F14:F18"/>
-    <mergeCell ref="E14:E18"/>
     <mergeCell ref="L14:L18"/>
     <mergeCell ref="K14:K18"/>
     <mergeCell ref="G14:G18"/>
     <mergeCell ref="H14:H18"/>
     <mergeCell ref="I14:I18"/>
     <mergeCell ref="J14:J18"/>
+    <mergeCell ref="A14:A18"/>
+    <mergeCell ref="B14:B18"/>
+    <mergeCell ref="C14:C18"/>
+    <mergeCell ref="F14:F18"/>
+    <mergeCell ref="E14:E18"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F14 F19:F53">
     <cfRule type="cellIs" dxfId="171" priority="8" operator="equal">
@@ -13782,42 +13793,42 @@
         <v>10</v>
       </c>
       <c r="L1" s="223" t="s">
+        <v>353</v>
+      </c>
+      <c r="M1" s="223" t="s">
         <v>354</v>
       </c>
-      <c r="M1" s="223" t="s">
+      <c r="N1" s="108" t="s">
         <v>355</v>
       </c>
-      <c r="N1" s="108" t="s">
+      <c r="O1" s="108" t="s">
         <v>356</v>
       </c>
-      <c r="O1" s="108" t="s">
+      <c r="P1" s="223" t="s">
         <v>357</v>
       </c>
-      <c r="P1" s="223" t="s">
+      <c r="Q1" s="223" t="s">
         <v>358</v>
       </c>
-      <c r="Q1" s="223" t="s">
+      <c r="R1" s="224" t="s">
         <v>359</v>
       </c>
-      <c r="R1" s="224" t="s">
+      <c r="S1" s="224" t="s">
         <v>360</v>
       </c>
-      <c r="S1" s="224" t="s">
+      <c r="T1" s="224" t="s">
         <v>361</v>
       </c>
-      <c r="T1" s="224" t="s">
+      <c r="U1" s="224" t="s">
         <v>362</v>
       </c>
-      <c r="U1" s="224" t="s">
+      <c r="V1" s="233" t="s">
         <v>363</v>
-      </c>
-      <c r="V1" s="233" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="28.8">
       <c r="A2" s="64" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="B2" s="157" t="s">
         <v>61</v>
@@ -13826,10 +13837,10 @@
         <v>62</v>
       </c>
       <c r="D2" s="152" t="s">
+        <v>365</v>
+      </c>
+      <c r="E2" s="158" t="s">
         <v>366</v>
-      </c>
-      <c r="E2" s="158" t="s">
-        <v>367</v>
       </c>
       <c r="F2" s="159" t="s">
         <v>17</v>
@@ -13849,25 +13860,25 @@
     </row>
     <row r="3" spans="1:22" ht="115.2">
       <c r="A3" s="68" t="s">
+        <v>367</v>
+      </c>
+      <c r="B3" s="61" t="s">
         <v>368</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="C3" s="68" t="s">
         <v>369</v>
-      </c>
-      <c r="C3" s="68" t="s">
-        <v>370</v>
       </c>
       <c r="D3" s="162" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="184" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="F3" s="163" t="s">
         <v>35</v>
       </c>
       <c r="G3" s="163" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H3" s="163">
         <v>1</v>
@@ -13879,7 +13890,7 @@
         <v>66</v>
       </c>
       <c r="K3" s="136" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="L3" s="129"/>
       <c r="M3" s="129"/>
@@ -13903,10 +13914,10 @@
         <v>213</v>
       </c>
       <c r="D4" s="71" t="s">
+        <v>372</v>
+      </c>
+      <c r="E4" s="158" t="s">
         <v>373</v>
-      </c>
-      <c r="E4" s="158" t="s">
-        <v>374</v>
       </c>
       <c r="F4" s="159" t="s">
         <v>35</v>
@@ -13921,28 +13932,28 @@
         <v>28</v>
       </c>
       <c r="J4" s="160" t="s">
+        <v>374</v>
+      </c>
+      <c r="K4" s="136" t="s">
         <v>375</v>
-      </c>
-      <c r="K4" s="136" t="s">
-        <v>376</v>
       </c>
       <c r="L4" s="107"/>
     </row>
     <row r="5" spans="1:22" ht="43.2">
       <c r="A5" s="165" t="s">
+        <v>376</v>
+      </c>
+      <c r="B5" s="75" t="s">
         <v>377</v>
       </c>
-      <c r="B5" s="75" t="s">
+      <c r="C5" s="165" t="s">
         <v>378</v>
-      </c>
-      <c r="C5" s="165" t="s">
-        <v>379</v>
       </c>
       <c r="D5" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="75" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="F5" s="166" t="s">
         <v>35</v>
@@ -13960,7 +13971,7 @@
         <v>29</v>
       </c>
       <c r="K5" s="136" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="L5" s="129"/>
       <c r="M5" s="129"/>
@@ -13975,19 +13986,19 @@
     </row>
     <row r="6" spans="1:22" ht="72">
       <c r="A6" s="168" t="s">
+        <v>381</v>
+      </c>
+      <c r="B6" s="151" t="s">
         <v>382</v>
       </c>
-      <c r="B6" s="151" t="s">
+      <c r="C6" s="168" t="s">
         <v>383</v>
-      </c>
-      <c r="C6" s="168" t="s">
-        <v>384</v>
       </c>
       <c r="D6" s="169" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="151" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="F6" s="133" t="s">
         <v>17</v>
@@ -14009,19 +14020,19 @@
     </row>
     <row r="7" spans="1:22" ht="115.2">
       <c r="A7" s="125" t="s">
+        <v>385</v>
+      </c>
+      <c r="B7" s="74" t="s">
         <v>386</v>
       </c>
-      <c r="B7" s="74" t="s">
+      <c r="C7" s="125" t="s">
         <v>387</v>
       </c>
-      <c r="C7" s="125" t="s">
+      <c r="D7" s="171" t="s">
         <v>388</v>
       </c>
-      <c r="D7" s="171" t="s">
+      <c r="E7" s="81" t="s">
         <v>389</v>
-      </c>
-      <c r="E7" s="81" t="s">
-        <v>390</v>
       </c>
       <c r="F7" s="127" t="s">
         <v>17</v>
@@ -14052,19 +14063,19 @@
     </row>
     <row r="8" spans="1:22" ht="28.8">
       <c r="A8" s="64" t="s">
+        <v>336</v>
+      </c>
+      <c r="B8" s="157" t="s">
         <v>337</v>
       </c>
-      <c r="B8" s="157" t="s">
+      <c r="C8" s="172" t="s">
         <v>338</v>
       </c>
-      <c r="C8" s="172" t="s">
-        <v>339</v>
-      </c>
       <c r="D8" s="143" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E8" s="135" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="F8" s="159" t="s">
         <v>17</v>
@@ -14082,13 +14093,13 @@
         <v>29</v>
       </c>
       <c r="K8" s="136" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="L8" s="107"/>
     </row>
     <row r="9" spans="1:22" ht="43.2">
       <c r="A9" s="165" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="B9" s="75" t="s">
         <v>77</v>
@@ -14100,7 +14111,7 @@
         <v>16</v>
       </c>
       <c r="E9" s="173" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="F9" s="166" t="s">
         <v>35</v>
@@ -14118,7 +14129,7 @@
         <v>66</v>
       </c>
       <c r="K9" s="136" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="L9" s="129"/>
       <c r="M9" s="129"/>
@@ -14863,45 +14874,45 @@
         <v>10</v>
       </c>
       <c r="L1" s="225" t="s">
+        <v>395</v>
+      </c>
+      <c r="M1" s="108" t="s">
         <v>396</v>
       </c>
-      <c r="M1" s="108" t="s">
+      <c r="N1" s="223" t="s">
         <v>397</v>
       </c>
-      <c r="N1" s="223" t="s">
+      <c r="O1" s="224" t="s">
         <v>398</v>
       </c>
-      <c r="O1" s="224" t="s">
+      <c r="P1" s="232" t="s">
         <v>399</v>
       </c>
-      <c r="P1" s="232" t="s">
+      <c r="Q1" s="233" t="s">
         <v>400</v>
-      </c>
-      <c r="Q1" s="233" t="s">
-        <v>401</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="64.349999999999994" customHeight="1">
       <c r="A2" s="64" t="s">
+        <v>401</v>
+      </c>
+      <c r="B2" s="45" t="s">
         <v>402</v>
       </c>
-      <c r="B2" s="45" t="s">
+      <c r="C2" s="172" t="s">
         <v>403</v>
-      </c>
-      <c r="C2" s="172" t="s">
-        <v>404</v>
       </c>
       <c r="D2" s="64" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="88" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="F2" s="159" t="s">
         <v>17</v>
       </c>
       <c r="G2" s="159" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H2" s="159" t="s">
         <v>19</v>
@@ -14913,31 +14924,31 @@
         <v>29</v>
       </c>
       <c r="K2" s="156" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="L2" s="136"/>
     </row>
     <row r="3" spans="1:17" ht="129.6">
       <c r="A3" s="68" t="s">
+        <v>406</v>
+      </c>
+      <c r="B3" s="61" t="s">
         <v>407</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="C3" s="68" t="s">
         <v>408</v>
-      </c>
-      <c r="C3" s="68" t="s">
-        <v>409</v>
       </c>
       <c r="D3" s="183" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="184" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="F3" s="163" t="s">
         <v>35</v>
       </c>
       <c r="G3" s="163" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H3" s="163">
         <v>1</v>
@@ -14949,7 +14960,7 @@
         <v>29</v>
       </c>
       <c r="K3" s="156" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="L3" s="75"/>
       <c r="M3" s="61"/>
@@ -14959,25 +14970,25 @@
     </row>
     <row r="4" spans="1:17" ht="28.8">
       <c r="A4" s="64" t="s">
+        <v>410</v>
+      </c>
+      <c r="B4" s="45" t="s">
         <v>411</v>
       </c>
-      <c r="B4" s="45" t="s">
+      <c r="C4" s="64" t="s">
         <v>412</v>
-      </c>
-      <c r="C4" s="64" t="s">
-        <v>413</v>
       </c>
       <c r="D4" s="64" t="s">
         <v>16</v>
       </c>
       <c r="E4" s="88" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="F4" s="159" t="s">
         <v>35</v>
       </c>
       <c r="G4" s="159" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="H4" s="159">
         <v>1</v>
@@ -14989,7 +15000,7 @@
         <v>29</v>
       </c>
       <c r="K4" s="156" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="L4" s="136"/>
     </row>
@@ -15812,27 +15823,27 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
+        <v>416</v>
+      </c>
+      <c r="M1" s="223" t="s">
         <v>417</v>
-      </c>
-      <c r="M1" s="223" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="28.8">
       <c r="A2" s="121" t="s">
+        <v>418</v>
+      </c>
+      <c r="B2" s="35" t="s">
         <v>419</v>
       </c>
-      <c r="B2" s="35" t="s">
+      <c r="C2" s="121" t="s">
         <v>420</v>
-      </c>
-      <c r="C2" s="121" t="s">
-        <v>421</v>
       </c>
       <c r="D2" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E2" s="35" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>17</v>
@@ -15850,30 +15861,30 @@
         <v>37</v>
       </c>
       <c r="K2" s="98" t="s">
+        <v>422</v>
+      </c>
+      <c r="L2" s="141" t="s">
         <v>423</v>
       </c>
-      <c r="L2" s="141" t="s">
-        <v>424</v>
-      </c>
       <c r="M2" s="141" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="72">
       <c r="A3" s="125" t="s">
+        <v>424</v>
+      </c>
+      <c r="B3" s="74" t="s">
         <v>425</v>
       </c>
-      <c r="B3" s="74" t="s">
+      <c r="C3" s="125" t="s">
         <v>426</v>
-      </c>
-      <c r="C3" s="125" t="s">
-        <v>427</v>
       </c>
       <c r="D3" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E3" s="85" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="F3" s="127" t="s">
         <v>35</v>
@@ -15891,7 +15902,7 @@
         <v>37</v>
       </c>
       <c r="K3" s="98" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="L3" s="129"/>
       <c r="M3" s="129"/>
@@ -15910,7 +15921,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="35" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="F4" s="124" t="s">
         <v>17</v>
@@ -15935,25 +15946,25 @@
     </row>
     <row r="5" spans="1:13" ht="43.2">
       <c r="A5" s="125" t="s">
+        <v>430</v>
+      </c>
+      <c r="B5" s="74" t="s">
         <v>431</v>
       </c>
-      <c r="B5" s="74" t="s">
+      <c r="C5" s="134" t="s">
         <v>432</v>
-      </c>
-      <c r="C5" s="134" t="s">
-        <v>433</v>
       </c>
       <c r="D5" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E5" s="126" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="F5" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G5" s="127" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="H5" s="127">
         <v>1</v>
@@ -15965,32 +15976,32 @@
         <v>29</v>
       </c>
       <c r="K5" s="98" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="L5" s="129"/>
       <c r="M5" s="129"/>
     </row>
     <row r="6" spans="1:13" ht="57.6">
       <c r="A6" s="121" t="s">
+        <v>436</v>
+      </c>
+      <c r="B6" s="35" t="s">
         <v>437</v>
       </c>
-      <c r="B6" s="35" t="s">
+      <c r="C6" s="121" t="s">
         <v>438</v>
-      </c>
-      <c r="C6" s="121" t="s">
-        <v>439</v>
       </c>
       <c r="D6" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="35" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="F6" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G6" s="128" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="H6" s="124" t="s">
         <v>81</v>
@@ -16002,36 +16013,36 @@
         <v>29</v>
       </c>
       <c r="K6" s="98" t="s">
+        <v>441</v>
+      </c>
+      <c r="L6" s="107" t="s">
         <v>442</v>
       </c>
-      <c r="L6" s="107" t="s">
-        <v>443</v>
-      </c>
       <c r="M6" s="107" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="43.2">
       <c r="A7" s="125" t="s">
+        <v>443</v>
+      </c>
+      <c r="B7" s="74" t="s">
         <v>444</v>
       </c>
-      <c r="B7" s="74" t="s">
+      <c r="C7" s="134" t="s">
         <v>445</v>
       </c>
-      <c r="C7" s="134" t="s">
+      <c r="D7" s="185" t="s">
         <v>446</v>
       </c>
-      <c r="D7" s="185" t="s">
+      <c r="E7" s="126" t="s">
         <v>447</v>
-      </c>
-      <c r="E7" s="126" t="s">
-        <v>448</v>
       </c>
       <c r="F7" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G7" s="156" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="H7" s="127" t="s">
         <v>81</v>
@@ -16043,7 +16054,7 @@
         <v>29</v>
       </c>
       <c r="K7" s="98" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="L7" s="129"/>
       <c r="M7" s="129"/>
@@ -16062,7 +16073,7 @@
         <v>16</v>
       </c>
       <c r="E8" s="35" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="F8" s="124" t="s">
         <v>17</v>
@@ -16080,7 +16091,7 @@
         <v>29</v>
       </c>
       <c r="K8" s="98" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="L8" s="107"/>
       <c r="M8" s="107"/>
@@ -16099,7 +16110,7 @@
         <v>16</v>
       </c>
       <c r="E9" s="126" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="F9" s="127" t="s">
         <v>17</v>
@@ -16117,26 +16128,26 @@
         <v>29</v>
       </c>
       <c r="K9" s="98" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="L9" s="129"/>
       <c r="M9" s="129"/>
     </row>
     <row r="10" spans="1:13" ht="57.6">
       <c r="A10" s="121" t="s">
+        <v>454</v>
+      </c>
+      <c r="B10" s="35" t="s">
         <v>455</v>
       </c>
-      <c r="B10" s="35" t="s">
+      <c r="C10" s="141" t="s">
         <v>456</v>
-      </c>
-      <c r="C10" s="141" t="s">
-        <v>457</v>
       </c>
       <c r="D10" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="F10" s="124" t="s">
         <v>17</v>
@@ -16154,32 +16165,32 @@
         <v>37</v>
       </c>
       <c r="K10" s="98" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="L10" s="107"/>
       <c r="M10" s="107"/>
     </row>
     <row r="11" spans="1:13" ht="43.2">
       <c r="A11" s="125" t="s">
+        <v>459</v>
+      </c>
+      <c r="B11" s="74" t="s">
         <v>460</v>
       </c>
-      <c r="B11" s="74" t="s">
+      <c r="C11" s="125" t="s">
         <v>461</v>
       </c>
-      <c r="C11" s="125" t="s">
+      <c r="D11" s="154" t="s">
         <v>462</v>
       </c>
-      <c r="D11" s="154" t="s">
-        <v>463</v>
-      </c>
       <c r="E11" s="126" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="F11" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G11" s="127" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="H11" s="127">
         <v>1</v>
@@ -16191,7 +16202,7 @@
         <v>29</v>
       </c>
       <c r="K11" s="99" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="L11" s="129"/>
       <c r="M11" s="129"/>
@@ -16210,7 +16221,7 @@
         <v>85</v>
       </c>
       <c r="E12" s="138" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="F12" s="124" t="s">
         <v>17</v>
@@ -16228,14 +16239,14 @@
         <v>29</v>
       </c>
       <c r="K12" s="98" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="L12" s="107"/>
       <c r="M12" s="107"/>
     </row>
     <row r="13" spans="1:13" ht="72">
       <c r="A13" s="125" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B13" s="74" t="s">
         <v>90</v>
@@ -16247,13 +16258,13 @@
         <v>92</v>
       </c>
       <c r="E13" s="80" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G13" s="127" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="H13" s="127">
         <v>1</v>
@@ -16265,14 +16276,14 @@
         <v>37</v>
       </c>
       <c r="K13" s="98" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="L13" s="129"/>
       <c r="M13" s="129"/>
     </row>
     <row r="14" spans="1:13" ht="72">
       <c r="A14" s="121" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B14" s="35" t="s">
         <v>175</v>
@@ -16284,7 +16295,7 @@
         <v>16</v>
       </c>
       <c r="E14" s="35" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="F14" s="124" t="s">
         <v>17</v>
@@ -16302,32 +16313,32 @@
         <v>29</v>
       </c>
       <c r="K14" s="98" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="L14" s="107"/>
       <c r="M14" s="107"/>
     </row>
     <row r="15" spans="1:13" ht="100.8">
       <c r="A15" s="125" t="s">
+        <v>474</v>
+      </c>
+      <c r="B15" s="74" t="s">
         <v>475</v>
       </c>
-      <c r="B15" s="74" t="s">
+      <c r="C15" s="125" t="s">
         <v>476</v>
       </c>
-      <c r="C15" s="125" t="s">
+      <c r="D15" s="185" t="s">
+        <v>446</v>
+      </c>
+      <c r="E15" s="80" t="s">
         <v>477</v>
-      </c>
-      <c r="D15" s="185" t="s">
-        <v>447</v>
-      </c>
-      <c r="E15" s="80" t="s">
-        <v>478</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G15" s="127" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="H15" s="127" t="s">
         <v>81</v>
@@ -16339,7 +16350,7 @@
         <v>29</v>
       </c>
       <c r="K15" s="98" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="L15" s="129"/>
       <c r="M15" s="129"/>
@@ -16374,32 +16385,32 @@
         <v>29</v>
       </c>
       <c r="K16" s="98" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="L16" s="107"/>
       <c r="M16" s="107"/>
     </row>
     <row r="17" spans="1:13" ht="57.6">
       <c r="A17" s="125" t="s">
+        <v>480</v>
+      </c>
+      <c r="B17" s="74" t="s">
         <v>481</v>
       </c>
-      <c r="B17" s="74" t="s">
+      <c r="C17" s="125" t="s">
         <v>482</v>
       </c>
-      <c r="C17" s="125" t="s">
+      <c r="D17" s="185" t="s">
+        <v>446</v>
+      </c>
+      <c r="E17" s="74" t="s">
         <v>483</v>
-      </c>
-      <c r="D17" s="185" t="s">
-        <v>447</v>
-      </c>
-      <c r="E17" s="74" t="s">
-        <v>484</v>
       </c>
       <c r="F17" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G17" s="127" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="H17" s="127" t="s">
         <v>81</v>
@@ -16411,7 +16422,7 @@
         <v>29</v>
       </c>
       <c r="K17" s="98" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="L17" s="129"/>
       <c r="M17" s="129"/>
@@ -16430,7 +16441,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="132" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="F18" s="124" t="s">
         <v>17</v>
@@ -16448,12 +16459,12 @@
         <v>29</v>
       </c>
       <c r="K18" s="98" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="L18" s="107"/>
       <c r="M18" s="107"/>
     </row>
-    <row r="19" spans="1:13" ht="28.8">
+    <row r="19" spans="1:13" ht="185.4" customHeight="1">
       <c r="A19" s="125" t="s">
         <v>306</v>
       </c>
@@ -16461,11 +16472,11 @@
         <v>307</v>
       </c>
       <c r="C19" s="125" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="D19" s="126"/>
-      <c r="E19" s="80" t="s">
-        <v>309</v>
+      <c r="E19" s="74" t="s">
+        <v>675</v>
       </c>
       <c r="F19" s="127" t="s">
         <v>17</v>
@@ -16484,10 +16495,10 @@
       </c>
       <c r="K19" s="104"/>
       <c r="L19" s="129" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="M19" s="129" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="129.6">
@@ -16504,7 +16515,7 @@
         <v>16</v>
       </c>
       <c r="E20" s="79" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="F20" s="190" t="s">
         <v>35</v>
@@ -16522,26 +16533,26 @@
         <v>29</v>
       </c>
       <c r="K20" s="99" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="L20" s="107"/>
       <c r="M20" s="107"/>
     </row>
     <row r="21" spans="1:13" ht="43.2">
       <c r="A21" s="125" t="s">
+        <v>320</v>
+      </c>
+      <c r="B21" s="74" t="s">
         <v>321</v>
       </c>
-      <c r="B21" s="74" t="s">
+      <c r="C21" s="125" t="s">
         <v>322</v>
       </c>
-      <c r="C21" s="125" t="s">
-        <v>323</v>
-      </c>
       <c r="D21" s="154" t="s">
+        <v>491</v>
+      </c>
+      <c r="E21" s="81" t="s">
         <v>492</v>
-      </c>
-      <c r="E21" s="81" t="s">
-        <v>493</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>17</v>
@@ -16559,32 +16570,32 @@
         <v>29</v>
       </c>
       <c r="K21" s="98" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="L21" s="129"/>
       <c r="M21" s="129"/>
     </row>
     <row r="22" spans="1:13" ht="57.6">
       <c r="A22" s="121" t="s">
+        <v>326</v>
+      </c>
+      <c r="B22" s="35" t="s">
         <v>327</v>
       </c>
-      <c r="B22" s="35" t="s">
+      <c r="C22" s="121" t="s">
         <v>328</v>
-      </c>
-      <c r="C22" s="121" t="s">
-        <v>329</v>
       </c>
       <c r="D22" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E22" s="132" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>17</v>
       </c>
       <c r="G22" s="124" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="H22" s="124" t="s">
         <v>81</v>
@@ -16613,7 +16624,7 @@
         <v>16</v>
       </c>
       <c r="E23" s="126" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>17</v>
@@ -16631,7 +16642,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="98" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="L23" s="129"/>
       <c r="M23" s="129"/>
@@ -17113,7 +17124,7 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="2" spans="1:12">
@@ -17130,7 +17141,7 @@
         <v>16</v>
       </c>
       <c r="E2" s="74" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>17</v>
@@ -17148,7 +17159,7 @@
         <v>29</v>
       </c>
       <c r="K2" s="98" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="L2" s="129"/>
     </row>
@@ -17184,7 +17195,7 @@
         <v>29</v>
       </c>
       <c r="K3" s="98" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="L3" s="107" t="s">
         <v>39</v>
@@ -17204,7 +17215,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="126" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="F4" s="127" t="s">
         <v>35</v>
@@ -17222,7 +17233,7 @@
         <v>29</v>
       </c>
       <c r="K4" s="99" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="L4" s="129"/>
     </row>
@@ -17240,7 +17251,7 @@
         <v>196</v>
       </c>
       <c r="E5" s="135" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="F5" s="124" t="s">
         <v>17</v>
@@ -17261,104 +17272,104 @@
       <c r="L5" s="107"/>
     </row>
     <row r="6" spans="1:12" ht="28.8">
-      <c r="A6" s="245" t="s">
+      <c r="A6" s="243" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="246" t="s">
+      <c r="B6" s="244" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="245" t="s">
+      <c r="C6" s="243" t="s">
         <v>62</v>
       </c>
       <c r="D6" s="215" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="247" t="s">
+      <c r="E6" s="245" t="s">
         <v>199</v>
       </c>
-      <c r="F6" s="244" t="s">
+      <c r="F6" s="242" t="s">
         <v>17</v>
       </c>
-      <c r="G6" s="244" t="s">
+      <c r="G6" s="242" t="s">
         <v>65</v>
       </c>
-      <c r="H6" s="244" t="s">
+      <c r="H6" s="242" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="242" t="s">
+      <c r="I6" s="246" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="235" t="s">
+      <c r="J6" s="239" t="s">
         <v>66</v>
       </c>
-      <c r="K6" s="243" t="s">
-        <v>505</v>
-      </c>
-      <c r="L6" s="242"/>
+      <c r="K6" s="247" t="s">
+        <v>504</v>
+      </c>
+      <c r="L6" s="246"/>
     </row>
     <row r="7" spans="1:12" ht="28.8">
-      <c r="A7" s="245"/>
-      <c r="B7" s="246"/>
-      <c r="C7" s="245"/>
+      <c r="A7" s="243"/>
+      <c r="B7" s="244"/>
+      <c r="C7" s="243"/>
       <c r="D7" s="216" t="s">
         <v>67</v>
       </c>
-      <c r="E7" s="247"/>
-      <c r="F7" s="244"/>
-      <c r="G7" s="244"/>
-      <c r="H7" s="244"/>
-      <c r="I7" s="242"/>
-      <c r="J7" s="235"/>
-      <c r="K7" s="243"/>
-      <c r="L7" s="242"/>
+      <c r="E7" s="245"/>
+      <c r="F7" s="242"/>
+      <c r="G7" s="242"/>
+      <c r="H7" s="242"/>
+      <c r="I7" s="246"/>
+      <c r="J7" s="239"/>
+      <c r="K7" s="247"/>
+      <c r="L7" s="246"/>
     </row>
     <row r="8" spans="1:12" ht="28.8">
-      <c r="A8" s="245"/>
-      <c r="B8" s="246"/>
-      <c r="C8" s="245"/>
+      <c r="A8" s="243"/>
+      <c r="B8" s="244"/>
+      <c r="C8" s="243"/>
       <c r="D8" s="216" t="s">
         <v>68</v>
       </c>
-      <c r="E8" s="247"/>
-      <c r="F8" s="244"/>
-      <c r="G8" s="244"/>
-      <c r="H8" s="244"/>
-      <c r="I8" s="242"/>
-      <c r="J8" s="235"/>
-      <c r="K8" s="243"/>
-      <c r="L8" s="242"/>
+      <c r="E8" s="245"/>
+      <c r="F8" s="242"/>
+      <c r="G8" s="242"/>
+      <c r="H8" s="242"/>
+      <c r="I8" s="246"/>
+      <c r="J8" s="239"/>
+      <c r="K8" s="247"/>
+      <c r="L8" s="246"/>
     </row>
     <row r="9" spans="1:12">
-      <c r="A9" s="245"/>
-      <c r="B9" s="246"/>
-      <c r="C9" s="245"/>
+      <c r="A9" s="243"/>
+      <c r="B9" s="244"/>
+      <c r="C9" s="243"/>
       <c r="D9" s="139" t="s">
         <v>69</v>
       </c>
-      <c r="E9" s="247"/>
-      <c r="F9" s="244"/>
-      <c r="G9" s="244"/>
-      <c r="H9" s="244"/>
-      <c r="I9" s="242"/>
-      <c r="J9" s="235"/>
-      <c r="K9" s="243"/>
-      <c r="L9" s="242"/>
+      <c r="E9" s="245"/>
+      <c r="F9" s="242"/>
+      <c r="G9" s="242"/>
+      <c r="H9" s="242"/>
+      <c r="I9" s="246"/>
+      <c r="J9" s="239"/>
+      <c r="K9" s="247"/>
+      <c r="L9" s="246"/>
     </row>
     <row r="10" spans="1:12">
-      <c r="A10" s="245"/>
-      <c r="B10" s="246"/>
-      <c r="C10" s="245"/>
+      <c r="A10" s="243"/>
+      <c r="B10" s="244"/>
+      <c r="C10" s="243"/>
       <c r="D10" s="139" t="s">
         <v>70</v>
       </c>
-      <c r="E10" s="247"/>
-      <c r="F10" s="244"/>
-      <c r="G10" s="244"/>
-      <c r="H10" s="244"/>
-      <c r="I10" s="242"/>
-      <c r="J10" s="235"/>
-      <c r="K10" s="243"/>
-      <c r="L10" s="242"/>
+      <c r="E10" s="245"/>
+      <c r="F10" s="242"/>
+      <c r="G10" s="242"/>
+      <c r="H10" s="242"/>
+      <c r="I10" s="246"/>
+      <c r="J10" s="239"/>
+      <c r="K10" s="247"/>
+      <c r="L10" s="246"/>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" s="121" t="s">
@@ -17374,7 +17385,7 @@
         <v>16</v>
       </c>
       <c r="E11" s="132" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="F11" s="124" t="s">
         <v>17</v>
@@ -17392,7 +17403,7 @@
         <v>29</v>
       </c>
       <c r="K11" s="99" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="L11" s="107"/>
     </row>
@@ -17410,7 +17421,7 @@
         <v>16</v>
       </c>
       <c r="E12" s="126" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="F12" s="124" t="s">
         <v>17</v>
@@ -17428,7 +17439,7 @@
         <v>29</v>
       </c>
       <c r="K12" s="98" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="L12" s="129" t="s">
         <v>46</v>
@@ -17448,7 +17459,7 @@
         <v>16</v>
       </c>
       <c r="E13" s="132" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>17</v>
@@ -17466,7 +17477,7 @@
         <v>29</v>
       </c>
       <c r="K13" s="98" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="L13" s="107"/>
     </row>
@@ -17484,7 +17495,7 @@
         <v>16</v>
       </c>
       <c r="E14" s="126" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="F14" s="124" t="s">
         <v>17</v>
@@ -17502,10 +17513,10 @@
         <v>29</v>
       </c>
       <c r="K14" s="98" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="L14" s="129" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="15" spans="1:12">
@@ -17522,7 +17533,7 @@
         <v>16</v>
       </c>
       <c r="E15" s="121" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>35</v>
@@ -17667,17 +17678,17 @@
   </sheetData>
   <autoFilter ref="A1:L15" xr:uid="{FBE7E653-2382-46E4-9C76-9C694EDC9195}"/>
   <mergeCells count="11">
+    <mergeCell ref="L6:L10"/>
+    <mergeCell ref="K6:K10"/>
+    <mergeCell ref="H6:H10"/>
+    <mergeCell ref="I6:I10"/>
+    <mergeCell ref="J6:J10"/>
     <mergeCell ref="G6:G10"/>
     <mergeCell ref="A6:A10"/>
     <mergeCell ref="B6:B10"/>
     <mergeCell ref="C6:C10"/>
     <mergeCell ref="E6:E10"/>
     <mergeCell ref="F6:F10"/>
-    <mergeCell ref="L6:L10"/>
-    <mergeCell ref="K6:K10"/>
-    <mergeCell ref="H6:H10"/>
-    <mergeCell ref="I6:I10"/>
-    <mergeCell ref="J6:J10"/>
   </mergeCells>
   <conditionalFormatting sqref="F2:F6 F11:F15">
     <cfRule type="cellIs" dxfId="127" priority="7" operator="equal">
@@ -17821,7 +17832,7 @@
         <v>10</v>
       </c>
       <c r="L1" s="108" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="92.4">
@@ -17838,7 +17849,7 @@
         <v>152</v>
       </c>
       <c r="E2" s="82" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="F2" s="124" t="s">
         <v>35</v>
@@ -17856,7 +17867,7 @@
         <v>37</v>
       </c>
       <c r="K2" s="107" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="L2" s="186"/>
     </row>
@@ -17894,7 +17905,7 @@
     </row>
     <row r="4" spans="1:12" ht="92.25" customHeight="1">
       <c r="A4" s="121" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B4" s="35" t="s">
         <v>175</v>
@@ -17906,7 +17917,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="194" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="F4" s="124" t="s">
         <v>17</v>
@@ -18044,7 +18055,7 @@
         <v>16</v>
       </c>
       <c r="E8" s="82" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="F8" s="124" t="s">
         <v>35</v>
@@ -18062,31 +18073,31 @@
         <v>37</v>
       </c>
       <c r="K8" s="107" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="L8" s="107"/>
     </row>
     <row r="9" spans="1:12" ht="43.2">
       <c r="A9" s="125" t="s">
+        <v>520</v>
+      </c>
+      <c r="B9" s="74" t="s">
         <v>521</v>
       </c>
-      <c r="B9" s="74" t="s">
+      <c r="C9" s="125" t="s">
         <v>522</v>
-      </c>
-      <c r="C9" s="125" t="s">
-        <v>523</v>
       </c>
       <c r="D9" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E9" s="212" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="F9" s="127" t="s">
         <v>35</v>
       </c>
       <c r="G9" s="127" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H9" s="127">
         <v>1</v>
@@ -18098,31 +18109,31 @@
         <v>37</v>
       </c>
       <c r="K9" s="106" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="L9" s="129"/>
     </row>
     <row r="10" spans="1:12" ht="43.2">
       <c r="A10" s="121" t="s">
+        <v>525</v>
+      </c>
+      <c r="B10" s="35" t="s">
         <v>526</v>
       </c>
-      <c r="B10" s="35" t="s">
+      <c r="C10" s="121" t="s">
         <v>527</v>
-      </c>
-      <c r="C10" s="121" t="s">
-        <v>528</v>
       </c>
       <c r="D10" s="132" t="s">
         <v>16</v>
       </c>
       <c r="E10" s="35" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="F10" s="124" t="s">
         <v>35</v>
       </c>
       <c r="G10" s="124" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="H10" s="133">
         <v>1</v>
@@ -18134,29 +18145,29 @@
         <v>37</v>
       </c>
       <c r="K10" s="106" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="L10" s="107"/>
     </row>
     <row r="11" spans="1:12" ht="43.2">
       <c r="A11" s="125" t="s">
+        <v>459</v>
+      </c>
+      <c r="B11" s="74" t="s">
         <v>460</v>
       </c>
-      <c r="B11" s="74" t="s">
+      <c r="C11" s="134" t="s">
         <v>461</v>
       </c>
-      <c r="C11" s="134" t="s">
+      <c r="D11" s="154" t="s">
         <v>462</v>
-      </c>
-      <c r="D11" s="154" t="s">
-        <v>463</v>
       </c>
       <c r="E11" s="126"/>
       <c r="F11" s="127" t="s">
         <v>17</v>
       </c>
       <c r="G11" s="127" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="H11" s="127" t="s">
         <v>19</v>
@@ -18172,13 +18183,13 @@
     </row>
     <row r="12" spans="1:12" ht="28.8">
       <c r="A12" s="121" t="s">
+        <v>530</v>
+      </c>
+      <c r="B12" s="35" t="s">
         <v>531</v>
       </c>
-      <c r="B12" s="35" t="s">
+      <c r="C12" s="121" t="s">
         <v>532</v>
-      </c>
-      <c r="C12" s="121" t="s">
-        <v>533</v>
       </c>
       <c r="D12" s="132" t="s">
         <v>16</v>
@@ -18216,7 +18227,7 @@
         <v>16</v>
       </c>
       <c r="E13" s="126" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F13" s="127" t="s">
         <v>35</v>
@@ -18270,19 +18281,19 @@
     </row>
     <row r="15" spans="1:12" ht="57.6">
       <c r="A15" s="125" t="s">
+        <v>534</v>
+      </c>
+      <c r="B15" s="74" t="s">
         <v>535</v>
       </c>
-      <c r="B15" s="74" t="s">
+      <c r="C15" s="125" t="s">
         <v>536</v>
-      </c>
-      <c r="C15" s="125" t="s">
-        <v>537</v>
       </c>
       <c r="D15" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E15" s="126" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="F15" s="127" t="s">
         <v>17</v>
@@ -18316,7 +18327,7 @@
         <v>85</v>
       </c>
       <c r="E16" s="35" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="F16" s="124" t="s">
         <v>17</v>
@@ -18350,7 +18361,7 @@
         <v>92</v>
       </c>
       <c r="E17" s="80" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="F17" s="127" t="s">
         <v>35</v>
@@ -18368,7 +18379,7 @@
         <v>37</v>
       </c>
       <c r="K17" s="107" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="L17" s="129"/>
     </row>
@@ -18386,7 +18397,7 @@
         <v>16</v>
       </c>
       <c r="E18" s="35" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="F18" s="124" t="s">
         <v>17</v>
@@ -18437,7 +18448,7 @@
       </c>
       <c r="K19" s="106"/>
       <c r="L19" s="129" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
     </row>
     <row r="20" spans="1:12" ht="43.2">
@@ -18454,7 +18465,7 @@
         <v>16</v>
       </c>
       <c r="E20" s="35" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="F20" s="124" t="s">
         <v>35</v>
@@ -18478,19 +18489,19 @@
     </row>
     <row r="21" spans="1:12" ht="57.6">
       <c r="A21" s="125" t="s">
+        <v>544</v>
+      </c>
+      <c r="B21" s="74" t="s">
         <v>545</v>
       </c>
-      <c r="B21" s="74" t="s">
+      <c r="C21" s="125" t="s">
         <v>546</v>
-      </c>
-      <c r="C21" s="125" t="s">
-        <v>547</v>
       </c>
       <c r="D21" s="126" t="s">
         <v>16</v>
       </c>
       <c r="E21" s="126" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="F21" s="127" t="s">
         <v>17</v>
@@ -18508,27 +18519,27 @@
         <v>29</v>
       </c>
       <c r="K21" s="107" t="s">
+        <v>548</v>
+      </c>
+      <c r="L21" s="192" t="s">
         <v>549</v>
-      </c>
-      <c r="L21" s="192" t="s">
-        <v>550</v>
       </c>
     </row>
     <row r="22" spans="1:12" ht="43.2">
       <c r="A22" s="121" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="B22" s="35" t="s">
         <v>127</v>
       </c>
       <c r="C22" s="121" t="s">
+        <v>332</v>
+      </c>
+      <c r="D22" s="143" t="s">
         <v>333</v>
       </c>
-      <c r="D22" s="143" t="s">
-        <v>334</v>
-      </c>
       <c r="E22" s="35" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="F22" s="124" t="s">
         <v>35</v>
@@ -18562,7 +18573,7 @@
         <v>16</v>
       </c>
       <c r="E23" s="126" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="F23" s="127" t="s">
         <v>35</v>
@@ -18580,7 +18591,7 @@
         <v>29</v>
       </c>
       <c r="K23" s="106" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="L23" s="195"/>
     </row>
@@ -19063,15 +19074,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000B1A1CF98C819F4881BB4349588D0C85" ma:contentTypeVersion="17" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ff8ef391852eaca4511043a54bffd4a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cfc87205-1831-4b6c-a7b4-76d40079a43e" xmlns:ns3="221af607-abea-4d5e-830c-567dcc03c0ec" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="201dd8b781da46d5daa37e3355db44fe" ns2:_="" ns3:_="">
     <xsd:import namespace="cfc87205-1831-4b6c-a7b4-76d40079a43e"/>
@@ -19314,6 +19316,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -19327,14 +19338,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19A23828-4FF7-4569-837D-B1B2C775409F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19353,6 +19356,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1A00443-9B7C-473F-A198-CBEB23A0BCC5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16D2CAB5-B21B-4A93-9D82-49FE3E36CF14}">
   <ds:schemaRefs>

</xml_diff>